<commit_message>
Updating the model fore Necaluxan with the lastest production data
</commit_message>
<xml_diff>
--- a/Astro/Results_Production_Astro_xgb.xlsx
+++ b/Astro/Results_Production_Astro_xgb.xlsx
@@ -28,511 +28,511 @@
     <t>Lookup</t>
   </si>
   <si>
-    <t>20.02.202620</t>
-  </si>
-  <si>
-    <t>20.02.202621</t>
-  </si>
-  <si>
-    <t>20.02.202622</t>
-  </si>
-  <si>
-    <t>20.02.202623</t>
-  </si>
-  <si>
-    <t>20.02.202624</t>
-  </si>
-  <si>
-    <t>21.02.20261</t>
-  </si>
-  <si>
-    <t>21.02.20262</t>
-  </si>
-  <si>
-    <t>21.02.20263</t>
-  </si>
-  <si>
-    <t>21.02.20264</t>
-  </si>
-  <si>
-    <t>21.02.20265</t>
-  </si>
-  <si>
-    <t>21.02.20266</t>
-  </si>
-  <si>
-    <t>21.02.20267</t>
-  </si>
-  <si>
-    <t>21.02.20268</t>
-  </si>
-  <si>
-    <t>21.02.20269</t>
-  </si>
-  <si>
-    <t>21.02.202610</t>
-  </si>
-  <si>
-    <t>21.02.202611</t>
-  </si>
-  <si>
-    <t>21.02.202612</t>
-  </si>
-  <si>
-    <t>21.02.202613</t>
-  </si>
-  <si>
-    <t>21.02.202614</t>
-  </si>
-  <si>
-    <t>21.02.202615</t>
-  </si>
-  <si>
-    <t>21.02.202616</t>
-  </si>
-  <si>
-    <t>21.02.202617</t>
-  </si>
-  <si>
-    <t>21.02.202618</t>
-  </si>
-  <si>
-    <t>21.02.202619</t>
-  </si>
-  <si>
-    <t>21.02.202620</t>
-  </si>
-  <si>
-    <t>21.02.202621</t>
-  </si>
-  <si>
-    <t>21.02.202622</t>
-  </si>
-  <si>
-    <t>21.02.202623</t>
-  </si>
-  <si>
-    <t>21.02.202624</t>
-  </si>
-  <si>
-    <t>22.02.20261</t>
-  </si>
-  <si>
-    <t>22.02.20262</t>
-  </si>
-  <si>
-    <t>22.02.20263</t>
-  </si>
-  <si>
-    <t>22.02.20264</t>
-  </si>
-  <si>
-    <t>22.02.20265</t>
-  </si>
-  <si>
-    <t>22.02.20266</t>
-  </si>
-  <si>
-    <t>22.02.20267</t>
-  </si>
-  <si>
-    <t>22.02.20268</t>
-  </si>
-  <si>
-    <t>22.02.20269</t>
-  </si>
-  <si>
-    <t>22.02.202610</t>
-  </si>
-  <si>
-    <t>22.02.202611</t>
-  </si>
-  <si>
-    <t>22.02.202612</t>
-  </si>
-  <si>
-    <t>22.02.202613</t>
-  </si>
-  <si>
-    <t>22.02.202614</t>
-  </si>
-  <si>
-    <t>22.02.202615</t>
-  </si>
-  <si>
-    <t>22.02.202616</t>
-  </si>
-  <si>
-    <t>22.02.202617</t>
-  </si>
-  <si>
-    <t>22.02.202618</t>
-  </si>
-  <si>
-    <t>22.02.202619</t>
-  </si>
-  <si>
-    <t>22.02.202620</t>
-  </si>
-  <si>
-    <t>22.02.202621</t>
-  </si>
-  <si>
-    <t>22.02.202622</t>
-  </si>
-  <si>
-    <t>22.02.202623</t>
-  </si>
-  <si>
-    <t>22.02.202624</t>
-  </si>
-  <si>
-    <t>23.02.20261</t>
-  </si>
-  <si>
-    <t>23.02.20262</t>
-  </si>
-  <si>
-    <t>23.02.20263</t>
-  </si>
-  <si>
-    <t>23.02.20264</t>
-  </si>
-  <si>
-    <t>23.02.20265</t>
-  </si>
-  <si>
-    <t>23.02.20266</t>
-  </si>
-  <si>
-    <t>23.02.20267</t>
-  </si>
-  <si>
-    <t>23.02.20268</t>
-  </si>
-  <si>
-    <t>23.02.20269</t>
-  </si>
-  <si>
-    <t>23.02.202610</t>
-  </si>
-  <si>
-    <t>23.02.202611</t>
-  </si>
-  <si>
-    <t>23.02.202612</t>
-  </si>
-  <si>
-    <t>23.02.202613</t>
-  </si>
-  <si>
-    <t>23.02.202614</t>
-  </si>
-  <si>
-    <t>23.02.202615</t>
-  </si>
-  <si>
-    <t>23.02.202616</t>
-  </si>
-  <si>
-    <t>23.02.202617</t>
-  </si>
-  <si>
-    <t>23.02.202618</t>
-  </si>
-  <si>
-    <t>23.02.202619</t>
-  </si>
-  <si>
-    <t>23.02.202620</t>
-  </si>
-  <si>
-    <t>23.02.202621</t>
-  </si>
-  <si>
-    <t>23.02.202622</t>
-  </si>
-  <si>
-    <t>23.02.202623</t>
-  </si>
-  <si>
-    <t>23.02.202624</t>
-  </si>
-  <si>
-    <t>24.02.20261</t>
-  </si>
-  <si>
-    <t>24.02.20262</t>
-  </si>
-  <si>
-    <t>24.02.20263</t>
-  </si>
-  <si>
-    <t>24.02.20264</t>
-  </si>
-  <si>
-    <t>24.02.20265</t>
-  </si>
-  <si>
-    <t>24.02.20266</t>
-  </si>
-  <si>
-    <t>24.02.20267</t>
-  </si>
-  <si>
-    <t>24.02.20268</t>
-  </si>
-  <si>
-    <t>24.02.20269</t>
-  </si>
-  <si>
-    <t>24.02.202610</t>
-  </si>
-  <si>
-    <t>24.02.202611</t>
-  </si>
-  <si>
-    <t>24.02.202612</t>
-  </si>
-  <si>
-    <t>24.02.202613</t>
-  </si>
-  <si>
-    <t>24.02.202614</t>
-  </si>
-  <si>
-    <t>24.02.202615</t>
-  </si>
-  <si>
-    <t>24.02.202616</t>
-  </si>
-  <si>
-    <t>24.02.202617</t>
-  </si>
-  <si>
-    <t>24.02.202618</t>
-  </si>
-  <si>
-    <t>24.02.202619</t>
-  </si>
-  <si>
-    <t>24.02.202620</t>
-  </si>
-  <si>
-    <t>24.02.202621</t>
-  </si>
-  <si>
-    <t>24.02.202622</t>
-  </si>
-  <si>
-    <t>24.02.202623</t>
-  </si>
-  <si>
-    <t>24.02.202624</t>
-  </si>
-  <si>
-    <t>25.02.20261</t>
-  </si>
-  <si>
-    <t>25.02.20262</t>
-  </si>
-  <si>
-    <t>25.02.20263</t>
-  </si>
-  <si>
-    <t>25.02.20264</t>
-  </si>
-  <si>
-    <t>25.02.20265</t>
-  </si>
-  <si>
-    <t>25.02.20266</t>
-  </si>
-  <si>
-    <t>25.02.20267</t>
-  </si>
-  <si>
-    <t>25.02.20268</t>
-  </si>
-  <si>
-    <t>25.02.20269</t>
-  </si>
-  <si>
-    <t>25.02.202610</t>
-  </si>
-  <si>
-    <t>25.02.202611</t>
-  </si>
-  <si>
-    <t>25.02.202612</t>
-  </si>
-  <si>
-    <t>25.02.202613</t>
-  </si>
-  <si>
-    <t>25.02.202614</t>
-  </si>
-  <si>
-    <t>25.02.202615</t>
-  </si>
-  <si>
-    <t>25.02.202616</t>
-  </si>
-  <si>
-    <t>25.02.202617</t>
-  </si>
-  <si>
-    <t>25.02.202618</t>
-  </si>
-  <si>
-    <t>25.02.202619</t>
-  </si>
-  <si>
-    <t>25.02.202620</t>
-  </si>
-  <si>
-    <t>25.02.202621</t>
-  </si>
-  <si>
-    <t>25.02.202622</t>
-  </si>
-  <si>
-    <t>25.02.202623</t>
-  </si>
-  <si>
-    <t>25.02.202624</t>
-  </si>
-  <si>
-    <t>26.02.20261</t>
-  </si>
-  <si>
-    <t>26.02.20262</t>
-  </si>
-  <si>
-    <t>26.02.20263</t>
-  </si>
-  <si>
-    <t>26.02.20264</t>
-  </si>
-  <si>
-    <t>26.02.20265</t>
-  </si>
-  <si>
-    <t>26.02.20266</t>
-  </si>
-  <si>
-    <t>26.02.20267</t>
-  </si>
-  <si>
-    <t>26.02.20268</t>
-  </si>
-  <si>
-    <t>26.02.20269</t>
-  </si>
-  <si>
-    <t>26.02.202610</t>
-  </si>
-  <si>
-    <t>26.02.202611</t>
-  </si>
-  <si>
-    <t>26.02.202612</t>
-  </si>
-  <si>
-    <t>26.02.202613</t>
-  </si>
-  <si>
-    <t>26.02.202614</t>
-  </si>
-  <si>
-    <t>26.02.202615</t>
-  </si>
-  <si>
-    <t>26.02.202616</t>
-  </si>
-  <si>
-    <t>26.02.202617</t>
-  </si>
-  <si>
-    <t>26.02.202618</t>
-  </si>
-  <si>
-    <t>26.02.202619</t>
-  </si>
-  <si>
-    <t>26.02.202620</t>
-  </si>
-  <si>
-    <t>26.02.202621</t>
-  </si>
-  <si>
-    <t>26.02.202622</t>
-  </si>
-  <si>
-    <t>26.02.202623</t>
-  </si>
-  <si>
-    <t>26.02.202624</t>
-  </si>
-  <si>
-    <t>27.02.20261</t>
-  </si>
-  <si>
-    <t>27.02.20262</t>
-  </si>
-  <si>
-    <t>27.02.20263</t>
-  </si>
-  <si>
-    <t>27.02.20264</t>
-  </si>
-  <si>
-    <t>27.02.20265</t>
-  </si>
-  <si>
-    <t>27.02.20266</t>
-  </si>
-  <si>
-    <t>27.02.20267</t>
-  </si>
-  <si>
-    <t>27.02.20268</t>
-  </si>
-  <si>
-    <t>27.02.20269</t>
-  </si>
-  <si>
-    <t>27.02.202610</t>
-  </si>
-  <si>
-    <t>27.02.202611</t>
-  </si>
-  <si>
-    <t>27.02.202612</t>
-  </si>
-  <si>
-    <t>27.02.202613</t>
-  </si>
-  <si>
-    <t>27.02.202614</t>
-  </si>
-  <si>
-    <t>27.02.202615</t>
-  </si>
-  <si>
-    <t>27.02.202616</t>
-  </si>
-  <si>
-    <t>27.02.202617</t>
-  </si>
-  <si>
-    <t>27.02.202618</t>
-  </si>
-  <si>
-    <t>27.02.202619</t>
-  </si>
-  <si>
-    <t>27.02.202620</t>
+    <t>17.03.202610</t>
+  </si>
+  <si>
+    <t>17.03.202611</t>
+  </si>
+  <si>
+    <t>17.03.202612</t>
+  </si>
+  <si>
+    <t>17.03.202613</t>
+  </si>
+  <si>
+    <t>17.03.202614</t>
+  </si>
+  <si>
+    <t>17.03.202615</t>
+  </si>
+  <si>
+    <t>17.03.202616</t>
+  </si>
+  <si>
+    <t>17.03.202617</t>
+  </si>
+  <si>
+    <t>17.03.202618</t>
+  </si>
+  <si>
+    <t>17.03.202619</t>
+  </si>
+  <si>
+    <t>17.03.202620</t>
+  </si>
+  <si>
+    <t>17.03.202621</t>
+  </si>
+  <si>
+    <t>17.03.202622</t>
+  </si>
+  <si>
+    <t>17.03.202623</t>
+  </si>
+  <si>
+    <t>17.03.202624</t>
+  </si>
+  <si>
+    <t>18.03.20261</t>
+  </si>
+  <si>
+    <t>18.03.20262</t>
+  </si>
+  <si>
+    <t>18.03.20263</t>
+  </si>
+  <si>
+    <t>18.03.20264</t>
+  </si>
+  <si>
+    <t>18.03.20265</t>
+  </si>
+  <si>
+    <t>18.03.20266</t>
+  </si>
+  <si>
+    <t>18.03.20267</t>
+  </si>
+  <si>
+    <t>18.03.20268</t>
+  </si>
+  <si>
+    <t>18.03.20269</t>
+  </si>
+  <si>
+    <t>18.03.202610</t>
+  </si>
+  <si>
+    <t>18.03.202611</t>
+  </si>
+  <si>
+    <t>18.03.202612</t>
+  </si>
+  <si>
+    <t>18.03.202613</t>
+  </si>
+  <si>
+    <t>18.03.202614</t>
+  </si>
+  <si>
+    <t>18.03.202615</t>
+  </si>
+  <si>
+    <t>18.03.202616</t>
+  </si>
+  <si>
+    <t>18.03.202617</t>
+  </si>
+  <si>
+    <t>18.03.202618</t>
+  </si>
+  <si>
+    <t>18.03.202619</t>
+  </si>
+  <si>
+    <t>18.03.202620</t>
+  </si>
+  <si>
+    <t>18.03.202621</t>
+  </si>
+  <si>
+    <t>18.03.202622</t>
+  </si>
+  <si>
+    <t>18.03.202623</t>
+  </si>
+  <si>
+    <t>18.03.202624</t>
+  </si>
+  <si>
+    <t>19.03.20261</t>
+  </si>
+  <si>
+    <t>19.03.20262</t>
+  </si>
+  <si>
+    <t>19.03.20263</t>
+  </si>
+  <si>
+    <t>19.03.20264</t>
+  </si>
+  <si>
+    <t>19.03.20265</t>
+  </si>
+  <si>
+    <t>19.03.20266</t>
+  </si>
+  <si>
+    <t>19.03.20267</t>
+  </si>
+  <si>
+    <t>19.03.20268</t>
+  </si>
+  <si>
+    <t>19.03.20269</t>
+  </si>
+  <si>
+    <t>19.03.202610</t>
+  </si>
+  <si>
+    <t>19.03.202611</t>
+  </si>
+  <si>
+    <t>19.03.202612</t>
+  </si>
+  <si>
+    <t>19.03.202613</t>
+  </si>
+  <si>
+    <t>19.03.202614</t>
+  </si>
+  <si>
+    <t>19.03.202615</t>
+  </si>
+  <si>
+    <t>19.03.202616</t>
+  </si>
+  <si>
+    <t>19.03.202617</t>
+  </si>
+  <si>
+    <t>19.03.202618</t>
+  </si>
+  <si>
+    <t>19.03.202619</t>
+  </si>
+  <si>
+    <t>19.03.202620</t>
+  </si>
+  <si>
+    <t>19.03.202621</t>
+  </si>
+  <si>
+    <t>19.03.202622</t>
+  </si>
+  <si>
+    <t>19.03.202623</t>
+  </si>
+  <si>
+    <t>19.03.202624</t>
+  </si>
+  <si>
+    <t>20.03.20261</t>
+  </si>
+  <si>
+    <t>20.03.20262</t>
+  </si>
+  <si>
+    <t>20.03.20263</t>
+  </si>
+  <si>
+    <t>20.03.20264</t>
+  </si>
+  <si>
+    <t>20.03.20265</t>
+  </si>
+  <si>
+    <t>20.03.20266</t>
+  </si>
+  <si>
+    <t>20.03.20267</t>
+  </si>
+  <si>
+    <t>20.03.20268</t>
+  </si>
+  <si>
+    <t>20.03.20269</t>
+  </si>
+  <si>
+    <t>20.03.202610</t>
+  </si>
+  <si>
+    <t>20.03.202611</t>
+  </si>
+  <si>
+    <t>20.03.202612</t>
+  </si>
+  <si>
+    <t>20.03.202613</t>
+  </si>
+  <si>
+    <t>20.03.202614</t>
+  </si>
+  <si>
+    <t>20.03.202615</t>
+  </si>
+  <si>
+    <t>20.03.202616</t>
+  </si>
+  <si>
+    <t>20.03.202617</t>
+  </si>
+  <si>
+    <t>20.03.202618</t>
+  </si>
+  <si>
+    <t>20.03.202619</t>
+  </si>
+  <si>
+    <t>20.03.202620</t>
+  </si>
+  <si>
+    <t>20.03.202621</t>
+  </si>
+  <si>
+    <t>20.03.202622</t>
+  </si>
+  <si>
+    <t>20.03.202623</t>
+  </si>
+  <si>
+    <t>20.03.202624</t>
+  </si>
+  <si>
+    <t>21.03.20261</t>
+  </si>
+  <si>
+    <t>21.03.20262</t>
+  </si>
+  <si>
+    <t>21.03.20263</t>
+  </si>
+  <si>
+    <t>21.03.20264</t>
+  </si>
+  <si>
+    <t>21.03.20265</t>
+  </si>
+  <si>
+    <t>21.03.20266</t>
+  </si>
+  <si>
+    <t>21.03.20267</t>
+  </si>
+  <si>
+    <t>21.03.20268</t>
+  </si>
+  <si>
+    <t>21.03.20269</t>
+  </si>
+  <si>
+    <t>21.03.202610</t>
+  </si>
+  <si>
+    <t>21.03.202611</t>
+  </si>
+  <si>
+    <t>21.03.202612</t>
+  </si>
+  <si>
+    <t>21.03.202613</t>
+  </si>
+  <si>
+    <t>21.03.202614</t>
+  </si>
+  <si>
+    <t>21.03.202615</t>
+  </si>
+  <si>
+    <t>21.03.202616</t>
+  </si>
+  <si>
+    <t>21.03.202617</t>
+  </si>
+  <si>
+    <t>21.03.202618</t>
+  </si>
+  <si>
+    <t>21.03.202619</t>
+  </si>
+  <si>
+    <t>21.03.202620</t>
+  </si>
+  <si>
+    <t>21.03.202621</t>
+  </si>
+  <si>
+    <t>21.03.202622</t>
+  </si>
+  <si>
+    <t>21.03.202623</t>
+  </si>
+  <si>
+    <t>21.03.202624</t>
+  </si>
+  <si>
+    <t>22.03.20261</t>
+  </si>
+  <si>
+    <t>22.03.20262</t>
+  </si>
+  <si>
+    <t>22.03.20263</t>
+  </si>
+  <si>
+    <t>22.03.20264</t>
+  </si>
+  <si>
+    <t>22.03.20265</t>
+  </si>
+  <si>
+    <t>22.03.20266</t>
+  </si>
+  <si>
+    <t>22.03.20267</t>
+  </si>
+  <si>
+    <t>22.03.20268</t>
+  </si>
+  <si>
+    <t>22.03.20269</t>
+  </si>
+  <si>
+    <t>22.03.202610</t>
+  </si>
+  <si>
+    <t>22.03.202611</t>
+  </si>
+  <si>
+    <t>22.03.202612</t>
+  </si>
+  <si>
+    <t>22.03.202613</t>
+  </si>
+  <si>
+    <t>22.03.202614</t>
+  </si>
+  <si>
+    <t>22.03.202615</t>
+  </si>
+  <si>
+    <t>22.03.202616</t>
+  </si>
+  <si>
+    <t>22.03.202617</t>
+  </si>
+  <si>
+    <t>22.03.202618</t>
+  </si>
+  <si>
+    <t>22.03.202619</t>
+  </si>
+  <si>
+    <t>22.03.202620</t>
+  </si>
+  <si>
+    <t>22.03.202621</t>
+  </si>
+  <si>
+    <t>22.03.202622</t>
+  </si>
+  <si>
+    <t>22.03.202623</t>
+  </si>
+  <si>
+    <t>22.03.202624</t>
+  </si>
+  <si>
+    <t>23.03.20261</t>
+  </si>
+  <si>
+    <t>23.03.20262</t>
+  </si>
+  <si>
+    <t>23.03.20263</t>
+  </si>
+  <si>
+    <t>23.03.20264</t>
+  </si>
+  <si>
+    <t>23.03.20265</t>
+  </si>
+  <si>
+    <t>23.03.20266</t>
+  </si>
+  <si>
+    <t>23.03.20267</t>
+  </si>
+  <si>
+    <t>23.03.20268</t>
+  </si>
+  <si>
+    <t>23.03.20269</t>
+  </si>
+  <si>
+    <t>23.03.202610</t>
+  </si>
+  <si>
+    <t>23.03.202611</t>
+  </si>
+  <si>
+    <t>23.03.202612</t>
+  </si>
+  <si>
+    <t>23.03.202613</t>
+  </si>
+  <si>
+    <t>23.03.202614</t>
+  </si>
+  <si>
+    <t>23.03.202615</t>
+  </si>
+  <si>
+    <t>23.03.202616</t>
+  </si>
+  <si>
+    <t>23.03.202617</t>
+  </si>
+  <si>
+    <t>23.03.202618</t>
+  </si>
+  <si>
+    <t>23.03.202619</t>
+  </si>
+  <si>
+    <t>23.03.202620</t>
+  </si>
+  <si>
+    <t>23.03.202621</t>
+  </si>
+  <si>
+    <t>23.03.202622</t>
+  </si>
+  <si>
+    <t>23.03.202623</t>
+  </si>
+  <si>
+    <t>23.03.202624</t>
+  </si>
+  <si>
+    <t>24.03.20261</t>
+  </si>
+  <si>
+    <t>24.03.20262</t>
+  </si>
+  <si>
+    <t>24.03.20263</t>
+  </si>
+  <si>
+    <t>24.03.20264</t>
+  </si>
+  <si>
+    <t>24.03.20265</t>
+  </si>
+  <si>
+    <t>24.03.20266</t>
+  </si>
+  <si>
+    <t>24.03.20267</t>
+  </si>
+  <si>
+    <t>24.03.20268</t>
+  </si>
+  <si>
+    <t>24.03.20269</t>
+  </si>
+  <si>
+    <t>24.03.202610</t>
   </si>
 </sst>
 </file>
@@ -913,10 +913,10 @@
     </row>
     <row r="2" spans="1:4">
       <c r="A2" s="2">
-        <v>46073</v>
+        <v>46098</v>
       </c>
       <c r="B2">
-        <v>20</v>
+        <v>10</v>
       </c>
       <c r="C2">
         <v>0</v>
@@ -927,10 +927,10 @@
     </row>
     <row r="3" spans="1:4">
       <c r="A3" s="2">
-        <v>46073</v>
+        <v>46098</v>
       </c>
       <c r="B3">
-        <v>21</v>
+        <v>11</v>
       </c>
       <c r="C3">
         <v>0</v>
@@ -941,13 +941,13 @@
     </row>
     <row r="4" spans="1:4">
       <c r="A4" s="2">
-        <v>46073</v>
+        <v>46098</v>
       </c>
       <c r="B4">
-        <v>22</v>
+        <v>12</v>
       </c>
       <c r="C4">
-        <v>0</v>
+        <v>2.792</v>
       </c>
       <c r="D4" t="s">
         <v>6</v>
@@ -955,13 +955,13 @@
     </row>
     <row r="5" spans="1:4">
       <c r="A5" s="2">
-        <v>46073</v>
+        <v>46098</v>
       </c>
       <c r="B5">
-        <v>23</v>
+        <v>13</v>
       </c>
       <c r="C5">
-        <v>0</v>
+        <v>2.664</v>
       </c>
       <c r="D5" t="s">
         <v>7</v>
@@ -969,13 +969,13 @@
     </row>
     <row r="6" spans="1:4">
       <c r="A6" s="2">
-        <v>46073</v>
+        <v>46098</v>
       </c>
       <c r="B6">
-        <v>24</v>
+        <v>14</v>
       </c>
       <c r="C6">
-        <v>0</v>
+        <v>2.792</v>
       </c>
       <c r="D6" t="s">
         <v>8</v>
@@ -983,13 +983,13 @@
     </row>
     <row r="7" spans="1:4">
       <c r="A7" s="2">
-        <v>46074</v>
+        <v>46098</v>
       </c>
       <c r="B7">
-        <v>1</v>
+        <v>15</v>
       </c>
       <c r="C7">
-        <v>0</v>
+        <v>2.674</v>
       </c>
       <c r="D7" t="s">
         <v>9</v>
@@ -997,13 +997,13 @@
     </row>
     <row r="8" spans="1:4">
       <c r="A8" s="2">
-        <v>46074</v>
+        <v>46098</v>
       </c>
       <c r="B8">
-        <v>2</v>
+        <v>16</v>
       </c>
       <c r="C8">
-        <v>0</v>
+        <v>2.399</v>
       </c>
       <c r="D8" t="s">
         <v>10</v>
@@ -1011,13 +1011,13 @@
     </row>
     <row r="9" spans="1:4">
       <c r="A9" s="2">
-        <v>46074</v>
+        <v>46098</v>
       </c>
       <c r="B9">
-        <v>3</v>
+        <v>17</v>
       </c>
       <c r="C9">
-        <v>0</v>
+        <v>1.623</v>
       </c>
       <c r="D9" t="s">
         <v>11</v>
@@ -1025,13 +1025,13 @@
     </row>
     <row r="10" spans="1:4">
       <c r="A10" s="2">
-        <v>46074</v>
+        <v>46098</v>
       </c>
       <c r="B10">
-        <v>4</v>
+        <v>18</v>
       </c>
       <c r="C10">
-        <v>0</v>
+        <v>0.927</v>
       </c>
       <c r="D10" t="s">
         <v>12</v>
@@ -1039,13 +1039,13 @@
     </row>
     <row r="11" spans="1:4">
       <c r="A11" s="2">
-        <v>46074</v>
+        <v>46098</v>
       </c>
       <c r="B11">
-        <v>5</v>
+        <v>19</v>
       </c>
       <c r="C11">
-        <v>0</v>
+        <v>0.185</v>
       </c>
       <c r="D11" t="s">
         <v>13</v>
@@ -1053,10 +1053,10 @@
     </row>
     <row r="12" spans="1:4">
       <c r="A12" s="2">
-        <v>46074</v>
+        <v>46098</v>
       </c>
       <c r="B12">
-        <v>6</v>
+        <v>20</v>
       </c>
       <c r="C12">
         <v>0</v>
@@ -1067,10 +1067,10 @@
     </row>
     <row r="13" spans="1:4">
       <c r="A13" s="2">
-        <v>46074</v>
+        <v>46098</v>
       </c>
       <c r="B13">
-        <v>7</v>
+        <v>21</v>
       </c>
       <c r="C13">
         <v>0</v>
@@ -1081,10 +1081,10 @@
     </row>
     <row r="14" spans="1:4">
       <c r="A14" s="2">
-        <v>46074</v>
+        <v>46098</v>
       </c>
       <c r="B14">
-        <v>8</v>
+        <v>22</v>
       </c>
       <c r="C14">
         <v>0</v>
@@ -1095,13 +1095,13 @@
     </row>
     <row r="15" spans="1:4">
       <c r="A15" s="2">
-        <v>46074</v>
+        <v>46098</v>
       </c>
       <c r="B15">
-        <v>9</v>
+        <v>23</v>
       </c>
       <c r="C15">
-        <v>0.012</v>
+        <v>0</v>
       </c>
       <c r="D15" t="s">
         <v>17</v>
@@ -1109,13 +1109,13 @@
     </row>
     <row r="16" spans="1:4">
       <c r="A16" s="2">
-        <v>46074</v>
+        <v>46098</v>
       </c>
       <c r="B16">
-        <v>10</v>
+        <v>24</v>
       </c>
       <c r="C16">
-        <v>0.112</v>
+        <v>0</v>
       </c>
       <c r="D16" t="s">
         <v>18</v>
@@ -1123,13 +1123,13 @@
     </row>
     <row r="17" spans="1:4">
       <c r="A17" s="2">
-        <v>46074</v>
+        <v>46099</v>
       </c>
       <c r="B17">
-        <v>11</v>
+        <v>1</v>
       </c>
       <c r="C17">
-        <v>0.416</v>
+        <v>0</v>
       </c>
       <c r="D17" t="s">
         <v>19</v>
@@ -1137,13 +1137,13 @@
     </row>
     <row r="18" spans="1:4">
       <c r="A18" s="2">
-        <v>46074</v>
+        <v>46099</v>
       </c>
       <c r="B18">
-        <v>12</v>
+        <v>2</v>
       </c>
       <c r="C18">
-        <v>0.736</v>
+        <v>0</v>
       </c>
       <c r="D18" t="s">
         <v>20</v>
@@ -1151,13 +1151,13 @@
     </row>
     <row r="19" spans="1:4">
       <c r="A19" s="2">
-        <v>46074</v>
+        <v>46099</v>
       </c>
       <c r="B19">
-        <v>13</v>
+        <v>3</v>
       </c>
       <c r="C19">
-        <v>0.845</v>
+        <v>0</v>
       </c>
       <c r="D19" t="s">
         <v>21</v>
@@ -1165,13 +1165,13 @@
     </row>
     <row r="20" spans="1:4">
       <c r="A20" s="2">
-        <v>46074</v>
+        <v>46099</v>
       </c>
       <c r="B20">
-        <v>14</v>
+        <v>4</v>
       </c>
       <c r="C20">
-        <v>0.823</v>
+        <v>0</v>
       </c>
       <c r="D20" t="s">
         <v>22</v>
@@ -1179,13 +1179,13 @@
     </row>
     <row r="21" spans="1:4">
       <c r="A21" s="2">
-        <v>46074</v>
+        <v>46099</v>
       </c>
       <c r="B21">
-        <v>15</v>
+        <v>5</v>
       </c>
       <c r="C21">
-        <v>0.792</v>
+        <v>0</v>
       </c>
       <c r="D21" t="s">
         <v>23</v>
@@ -1193,13 +1193,13 @@
     </row>
     <row r="22" spans="1:4">
       <c r="A22" s="2">
-        <v>46074</v>
+        <v>46099</v>
       </c>
       <c r="B22">
-        <v>16</v>
+        <v>6</v>
       </c>
       <c r="C22">
-        <v>0.4</v>
+        <v>0</v>
       </c>
       <c r="D22" t="s">
         <v>24</v>
@@ -1207,13 +1207,13 @@
     </row>
     <row r="23" spans="1:4">
       <c r="A23" s="2">
-        <v>46074</v>
+        <v>46099</v>
       </c>
       <c r="B23">
-        <v>17</v>
+        <v>7</v>
       </c>
       <c r="C23">
-        <v>0.248</v>
+        <v>0</v>
       </c>
       <c r="D23" t="s">
         <v>25</v>
@@ -1221,13 +1221,13 @@
     </row>
     <row r="24" spans="1:4">
       <c r="A24" s="2">
-        <v>46074</v>
+        <v>46099</v>
       </c>
       <c r="B24">
-        <v>18</v>
+        <v>8</v>
       </c>
       <c r="C24">
-        <v>0.099</v>
+        <v>0</v>
       </c>
       <c r="D24" t="s">
         <v>26</v>
@@ -1235,13 +1235,13 @@
     </row>
     <row r="25" spans="1:4">
       <c r="A25" s="2">
-        <v>46074</v>
+        <v>46099</v>
       </c>
       <c r="B25">
-        <v>19</v>
+        <v>9</v>
       </c>
       <c r="C25">
-        <v>0.015</v>
+        <v>0.346</v>
       </c>
       <c r="D25" t="s">
         <v>27</v>
@@ -1249,13 +1249,13 @@
     </row>
     <row r="26" spans="1:4">
       <c r="A26" s="2">
-        <v>46074</v>
+        <v>46099</v>
       </c>
       <c r="B26">
-        <v>20</v>
+        <v>10</v>
       </c>
       <c r="C26">
-        <v>0</v>
+        <v>1.107</v>
       </c>
       <c r="D26" t="s">
         <v>28</v>
@@ -1263,13 +1263,13 @@
     </row>
     <row r="27" spans="1:4">
       <c r="A27" s="2">
-        <v>46074</v>
+        <v>46099</v>
       </c>
       <c r="B27">
-        <v>21</v>
+        <v>11</v>
       </c>
       <c r="C27">
-        <v>0</v>
+        <v>1.967</v>
       </c>
       <c r="D27" t="s">
         <v>29</v>
@@ -1277,13 +1277,13 @@
     </row>
     <row r="28" spans="1:4">
       <c r="A28" s="2">
-        <v>46074</v>
+        <v>46099</v>
       </c>
       <c r="B28">
-        <v>22</v>
+        <v>12</v>
       </c>
       <c r="C28">
-        <v>0</v>
+        <v>2.674</v>
       </c>
       <c r="D28" t="s">
         <v>30</v>
@@ -1291,13 +1291,13 @@
     </row>
     <row r="29" spans="1:4">
       <c r="A29" s="2">
-        <v>46074</v>
+        <v>46099</v>
       </c>
       <c r="B29">
-        <v>23</v>
+        <v>13</v>
       </c>
       <c r="C29">
-        <v>0</v>
+        <v>2.783</v>
       </c>
       <c r="D29" t="s">
         <v>31</v>
@@ -1305,13 +1305,13 @@
     </row>
     <row r="30" spans="1:4">
       <c r="A30" s="2">
-        <v>46074</v>
+        <v>46099</v>
       </c>
       <c r="B30">
-        <v>24</v>
+        <v>14</v>
       </c>
       <c r="C30">
-        <v>0</v>
+        <v>2.878</v>
       </c>
       <c r="D30" t="s">
         <v>32</v>
@@ -1319,13 +1319,13 @@
     </row>
     <row r="31" spans="1:4">
       <c r="A31" s="2">
-        <v>46075</v>
+        <v>46099</v>
       </c>
       <c r="B31">
-        <v>1</v>
+        <v>15</v>
       </c>
       <c r="C31">
-        <v>0</v>
+        <v>2.514</v>
       </c>
       <c r="D31" t="s">
         <v>33</v>
@@ -1333,13 +1333,13 @@
     </row>
     <row r="32" spans="1:4">
       <c r="A32" s="2">
-        <v>46075</v>
+        <v>46099</v>
       </c>
       <c r="B32">
-        <v>2</v>
+        <v>16</v>
       </c>
       <c r="C32">
-        <v>0</v>
+        <v>2.297</v>
       </c>
       <c r="D32" t="s">
         <v>34</v>
@@ -1347,13 +1347,13 @@
     </row>
     <row r="33" spans="1:4">
       <c r="A33" s="2">
-        <v>46075</v>
+        <v>46099</v>
       </c>
       <c r="B33">
-        <v>3</v>
+        <v>17</v>
       </c>
       <c r="C33">
-        <v>0</v>
+        <v>1.733</v>
       </c>
       <c r="D33" t="s">
         <v>35</v>
@@ -1361,13 +1361,13 @@
     </row>
     <row r="34" spans="1:4">
       <c r="A34" s="2">
-        <v>46075</v>
+        <v>46099</v>
       </c>
       <c r="B34">
-        <v>4</v>
+        <v>18</v>
       </c>
       <c r="C34">
-        <v>0</v>
+        <v>1.129</v>
       </c>
       <c r="D34" t="s">
         <v>36</v>
@@ -1375,13 +1375,13 @@
     </row>
     <row r="35" spans="1:4">
       <c r="A35" s="2">
-        <v>46075</v>
+        <v>46099</v>
       </c>
       <c r="B35">
-        <v>5</v>
+        <v>19</v>
       </c>
       <c r="C35">
-        <v>0</v>
+        <v>0.3</v>
       </c>
       <c r="D35" t="s">
         <v>37</v>
@@ -1389,13 +1389,13 @@
     </row>
     <row r="36" spans="1:4">
       <c r="A36" s="2">
-        <v>46075</v>
+        <v>46099</v>
       </c>
       <c r="B36">
-        <v>6</v>
+        <v>20</v>
       </c>
       <c r="C36">
-        <v>0</v>
+        <v>0.015</v>
       </c>
       <c r="D36" t="s">
         <v>38</v>
@@ -1403,10 +1403,10 @@
     </row>
     <row r="37" spans="1:4">
       <c r="A37" s="2">
-        <v>46075</v>
+        <v>46099</v>
       </c>
       <c r="B37">
-        <v>7</v>
+        <v>21</v>
       </c>
       <c r="C37">
         <v>0</v>
@@ -1417,10 +1417,10 @@
     </row>
     <row r="38" spans="1:4">
       <c r="A38" s="2">
-        <v>46075</v>
+        <v>46099</v>
       </c>
       <c r="B38">
-        <v>8</v>
+        <v>22</v>
       </c>
       <c r="C38">
         <v>0</v>
@@ -1431,13 +1431,13 @@
     </row>
     <row r="39" spans="1:4">
       <c r="A39" s="2">
-        <v>46075</v>
+        <v>46099</v>
       </c>
       <c r="B39">
-        <v>9</v>
+        <v>23</v>
       </c>
       <c r="C39">
-        <v>0.012</v>
+        <v>0</v>
       </c>
       <c r="D39" t="s">
         <v>41</v>
@@ -1445,13 +1445,13 @@
     </row>
     <row r="40" spans="1:4">
       <c r="A40" s="2">
-        <v>46075</v>
+        <v>46099</v>
       </c>
       <c r="B40">
-        <v>10</v>
+        <v>24</v>
       </c>
       <c r="C40">
-        <v>0.139</v>
+        <v>0</v>
       </c>
       <c r="D40" t="s">
         <v>42</v>
@@ -1459,13 +1459,13 @@
     </row>
     <row r="41" spans="1:4">
       <c r="A41" s="2">
-        <v>46075</v>
+        <v>46100</v>
       </c>
       <c r="B41">
-        <v>11</v>
+        <v>1</v>
       </c>
       <c r="C41">
-        <v>0.472</v>
+        <v>0</v>
       </c>
       <c r="D41" t="s">
         <v>43</v>
@@ -1473,13 +1473,13 @@
     </row>
     <row r="42" spans="1:4">
       <c r="A42" s="2">
-        <v>46075</v>
+        <v>46100</v>
       </c>
       <c r="B42">
-        <v>12</v>
+        <v>2</v>
       </c>
       <c r="C42">
-        <v>1.05</v>
+        <v>0</v>
       </c>
       <c r="D42" t="s">
         <v>44</v>
@@ -1487,13 +1487,13 @@
     </row>
     <row r="43" spans="1:4">
       <c r="A43" s="2">
-        <v>46075</v>
+        <v>46100</v>
       </c>
       <c r="B43">
-        <v>13</v>
+        <v>3</v>
       </c>
       <c r="C43">
-        <v>1.265</v>
+        <v>0</v>
       </c>
       <c r="D43" t="s">
         <v>45</v>
@@ -1501,13 +1501,13 @@
     </row>
     <row r="44" spans="1:4">
       <c r="A44" s="2">
-        <v>46075</v>
+        <v>46100</v>
       </c>
       <c r="B44">
-        <v>14</v>
+        <v>4</v>
       </c>
       <c r="C44">
-        <v>1.466</v>
+        <v>0</v>
       </c>
       <c r="D44" t="s">
         <v>46</v>
@@ -1515,13 +1515,13 @@
     </row>
     <row r="45" spans="1:4">
       <c r="A45" s="2">
-        <v>46075</v>
+        <v>46100</v>
       </c>
       <c r="B45">
-        <v>15</v>
+        <v>5</v>
       </c>
       <c r="C45">
-        <v>1.47</v>
+        <v>0</v>
       </c>
       <c r="D45" t="s">
         <v>47</v>
@@ -1529,13 +1529,13 @@
     </row>
     <row r="46" spans="1:4">
       <c r="A46" s="2">
-        <v>46075</v>
+        <v>46100</v>
       </c>
       <c r="B46">
-        <v>16</v>
+        <v>6</v>
       </c>
       <c r="C46">
-        <v>1.194</v>
+        <v>0</v>
       </c>
       <c r="D46" t="s">
         <v>48</v>
@@ -1543,13 +1543,13 @@
     </row>
     <row r="47" spans="1:4">
       <c r="A47" s="2">
-        <v>46075</v>
+        <v>46100</v>
       </c>
       <c r="B47">
-        <v>17</v>
+        <v>7</v>
       </c>
       <c r="C47">
-        <v>0.741</v>
+        <v>0</v>
       </c>
       <c r="D47" t="s">
         <v>49</v>
@@ -1557,13 +1557,13 @@
     </row>
     <row r="48" spans="1:4">
       <c r="A48" s="2">
-        <v>46075</v>
+        <v>46100</v>
       </c>
       <c r="B48">
-        <v>18</v>
+        <v>8</v>
       </c>
       <c r="C48">
-        <v>0.252</v>
+        <v>0</v>
       </c>
       <c r="D48" t="s">
         <v>50</v>
@@ -1571,13 +1571,13 @@
     </row>
     <row r="49" spans="1:4">
       <c r="A49" s="2">
-        <v>46075</v>
+        <v>46100</v>
       </c>
       <c r="B49">
-        <v>19</v>
+        <v>9</v>
       </c>
       <c r="C49">
-        <v>0.033</v>
+        <v>0.312</v>
       </c>
       <c r="D49" t="s">
         <v>51</v>
@@ -1585,13 +1585,13 @@
     </row>
     <row r="50" spans="1:4">
       <c r="A50" s="2">
-        <v>46075</v>
+        <v>46100</v>
       </c>
       <c r="B50">
-        <v>20</v>
+        <v>10</v>
       </c>
       <c r="C50">
-        <v>0</v>
+        <v>0.853</v>
       </c>
       <c r="D50" t="s">
         <v>52</v>
@@ -1599,13 +1599,13 @@
     </row>
     <row r="51" spans="1:4">
       <c r="A51" s="2">
-        <v>46075</v>
+        <v>46100</v>
       </c>
       <c r="B51">
-        <v>21</v>
+        <v>11</v>
       </c>
       <c r="C51">
-        <v>0</v>
+        <v>1.469</v>
       </c>
       <c r="D51" t="s">
         <v>53</v>
@@ -1613,13 +1613,13 @@
     </row>
     <row r="52" spans="1:4">
       <c r="A52" s="2">
-        <v>46075</v>
+        <v>46100</v>
       </c>
       <c r="B52">
-        <v>22</v>
+        <v>12</v>
       </c>
       <c r="C52">
-        <v>0</v>
+        <v>1.788</v>
       </c>
       <c r="D52" t="s">
         <v>54</v>
@@ -1627,13 +1627,13 @@
     </row>
     <row r="53" spans="1:4">
       <c r="A53" s="2">
-        <v>46075</v>
+        <v>46100</v>
       </c>
       <c r="B53">
-        <v>23</v>
+        <v>13</v>
       </c>
       <c r="C53">
-        <v>0</v>
+        <v>1.987</v>
       </c>
       <c r="D53" t="s">
         <v>55</v>
@@ -1641,13 +1641,13 @@
     </row>
     <row r="54" spans="1:4">
       <c r="A54" s="2">
-        <v>46075</v>
+        <v>46100</v>
       </c>
       <c r="B54">
-        <v>24</v>
+        <v>14</v>
       </c>
       <c r="C54">
-        <v>0</v>
+        <v>2.032</v>
       </c>
       <c r="D54" t="s">
         <v>56</v>
@@ -1655,13 +1655,13 @@
     </row>
     <row r="55" spans="1:4">
       <c r="A55" s="2">
-        <v>46076</v>
+        <v>46100</v>
       </c>
       <c r="B55">
-        <v>1</v>
+        <v>15</v>
       </c>
       <c r="C55">
-        <v>0</v>
+        <v>1.982</v>
       </c>
       <c r="D55" t="s">
         <v>57</v>
@@ -1669,13 +1669,13 @@
     </row>
     <row r="56" spans="1:4">
       <c r="A56" s="2">
-        <v>46076</v>
+        <v>46100</v>
       </c>
       <c r="B56">
-        <v>2</v>
+        <v>16</v>
       </c>
       <c r="C56">
-        <v>0</v>
+        <v>1.603</v>
       </c>
       <c r="D56" t="s">
         <v>58</v>
@@ -1683,13 +1683,13 @@
     </row>
     <row r="57" spans="1:4">
       <c r="A57" s="2">
-        <v>46076</v>
+        <v>46100</v>
       </c>
       <c r="B57">
-        <v>3</v>
+        <v>17</v>
       </c>
       <c r="C57">
-        <v>0</v>
+        <v>1.224</v>
       </c>
       <c r="D57" t="s">
         <v>59</v>
@@ -1697,13 +1697,13 @@
     </row>
     <row r="58" spans="1:4">
       <c r="A58" s="2">
-        <v>46076</v>
+        <v>46100</v>
       </c>
       <c r="B58">
-        <v>4</v>
+        <v>18</v>
       </c>
       <c r="C58">
-        <v>0</v>
+        <v>0.706</v>
       </c>
       <c r="D58" t="s">
         <v>60</v>
@@ -1711,13 +1711,13 @@
     </row>
     <row r="59" spans="1:4">
       <c r="A59" s="2">
-        <v>46076</v>
+        <v>46100</v>
       </c>
       <c r="B59">
-        <v>5</v>
+        <v>19</v>
       </c>
       <c r="C59">
-        <v>0</v>
+        <v>0.19</v>
       </c>
       <c r="D59" t="s">
         <v>61</v>
@@ -1725,13 +1725,13 @@
     </row>
     <row r="60" spans="1:4">
       <c r="A60" s="2">
-        <v>46076</v>
+        <v>46100</v>
       </c>
       <c r="B60">
-        <v>6</v>
+        <v>20</v>
       </c>
       <c r="C60">
-        <v>0</v>
+        <v>0.013</v>
       </c>
       <c r="D60" t="s">
         <v>62</v>
@@ -1739,10 +1739,10 @@
     </row>
     <row r="61" spans="1:4">
       <c r="A61" s="2">
-        <v>46076</v>
+        <v>46100</v>
       </c>
       <c r="B61">
-        <v>7</v>
+        <v>21</v>
       </c>
       <c r="C61">
         <v>0</v>
@@ -1753,10 +1753,10 @@
     </row>
     <row r="62" spans="1:4">
       <c r="A62" s="2">
-        <v>46076</v>
+        <v>46100</v>
       </c>
       <c r="B62">
-        <v>8</v>
+        <v>22</v>
       </c>
       <c r="C62">
         <v>0</v>
@@ -1767,13 +1767,13 @@
     </row>
     <row r="63" spans="1:4">
       <c r="A63" s="2">
-        <v>46076</v>
+        <v>46100</v>
       </c>
       <c r="B63">
-        <v>9</v>
+        <v>23</v>
       </c>
       <c r="C63">
-        <v>0.011</v>
+        <v>0</v>
       </c>
       <c r="D63" t="s">
         <v>65</v>
@@ -1781,13 +1781,13 @@
     </row>
     <row r="64" spans="1:4">
       <c r="A64" s="2">
-        <v>46076</v>
+        <v>46100</v>
       </c>
       <c r="B64">
-        <v>10</v>
+        <v>24</v>
       </c>
       <c r="C64">
-        <v>0.093</v>
+        <v>0</v>
       </c>
       <c r="D64" t="s">
         <v>66</v>
@@ -1795,13 +1795,13 @@
     </row>
     <row r="65" spans="1:4">
       <c r="A65" s="2">
-        <v>46076</v>
+        <v>46101</v>
       </c>
       <c r="B65">
-        <v>11</v>
+        <v>1</v>
       </c>
       <c r="C65">
-        <v>0.252</v>
+        <v>0</v>
       </c>
       <c r="D65" t="s">
         <v>67</v>
@@ -1809,13 +1809,13 @@
     </row>
     <row r="66" spans="1:4">
       <c r="A66" s="2">
-        <v>46076</v>
+        <v>46101</v>
       </c>
       <c r="B66">
-        <v>12</v>
+        <v>2</v>
       </c>
       <c r="C66">
-        <v>0.354</v>
+        <v>0</v>
       </c>
       <c r="D66" t="s">
         <v>68</v>
@@ -1823,13 +1823,13 @@
     </row>
     <row r="67" spans="1:4">
       <c r="A67" s="2">
-        <v>46076</v>
+        <v>46101</v>
       </c>
       <c r="B67">
-        <v>13</v>
+        <v>3</v>
       </c>
       <c r="C67">
-        <v>0.411</v>
+        <v>0</v>
       </c>
       <c r="D67" t="s">
         <v>69</v>
@@ -1837,13 +1837,13 @@
     </row>
     <row r="68" spans="1:4">
       <c r="A68" s="2">
-        <v>46076</v>
+        <v>46101</v>
       </c>
       <c r="B68">
-        <v>14</v>
+        <v>4</v>
       </c>
       <c r="C68">
-        <v>0.469</v>
+        <v>0</v>
       </c>
       <c r="D68" t="s">
         <v>70</v>
@@ -1851,13 +1851,13 @@
     </row>
     <row r="69" spans="1:4">
       <c r="A69" s="2">
-        <v>46076</v>
+        <v>46101</v>
       </c>
       <c r="B69">
-        <v>15</v>
+        <v>5</v>
       </c>
       <c r="C69">
-        <v>0.425</v>
+        <v>0</v>
       </c>
       <c r="D69" t="s">
         <v>71</v>
@@ -1865,13 +1865,13 @@
     </row>
     <row r="70" spans="1:4">
       <c r="A70" s="2">
-        <v>46076</v>
+        <v>46101</v>
       </c>
       <c r="B70">
-        <v>16</v>
+        <v>6</v>
       </c>
       <c r="C70">
-        <v>0.347</v>
+        <v>0</v>
       </c>
       <c r="D70" t="s">
         <v>72</v>
@@ -1879,13 +1879,13 @@
     </row>
     <row r="71" spans="1:4">
       <c r="A71" s="2">
-        <v>46076</v>
+        <v>46101</v>
       </c>
       <c r="B71">
-        <v>17</v>
+        <v>7</v>
       </c>
       <c r="C71">
-        <v>0.213</v>
+        <v>0</v>
       </c>
       <c r="D71" t="s">
         <v>73</v>
@@ -1893,13 +1893,13 @@
     </row>
     <row r="72" spans="1:4">
       <c r="A72" s="2">
-        <v>46076</v>
+        <v>46101</v>
       </c>
       <c r="B72">
-        <v>18</v>
+        <v>8</v>
       </c>
       <c r="C72">
-        <v>0.126</v>
+        <v>0</v>
       </c>
       <c r="D72" t="s">
         <v>74</v>
@@ -1907,13 +1907,13 @@
     </row>
     <row r="73" spans="1:4">
       <c r="A73" s="2">
-        <v>46076</v>
+        <v>46101</v>
       </c>
       <c r="B73">
-        <v>19</v>
+        <v>9</v>
       </c>
       <c r="C73">
-        <v>0.021</v>
+        <v>0.219</v>
       </c>
       <c r="D73" t="s">
         <v>75</v>
@@ -1921,13 +1921,13 @@
     </row>
     <row r="74" spans="1:4">
       <c r="A74" s="2">
-        <v>46076</v>
+        <v>46101</v>
       </c>
       <c r="B74">
-        <v>20</v>
+        <v>10</v>
       </c>
       <c r="C74">
-        <v>0</v>
+        <v>0.678</v>
       </c>
       <c r="D74" t="s">
         <v>76</v>
@@ -1935,13 +1935,13 @@
     </row>
     <row r="75" spans="1:4">
       <c r="A75" s="2">
-        <v>46076</v>
+        <v>46101</v>
       </c>
       <c r="B75">
-        <v>21</v>
+        <v>11</v>
       </c>
       <c r="C75">
-        <v>0</v>
+        <v>1.056</v>
       </c>
       <c r="D75" t="s">
         <v>77</v>
@@ -1949,13 +1949,13 @@
     </row>
     <row r="76" spans="1:4">
       <c r="A76" s="2">
-        <v>46076</v>
+        <v>46101</v>
       </c>
       <c r="B76">
-        <v>22</v>
+        <v>12</v>
       </c>
       <c r="C76">
-        <v>0</v>
+        <v>1.524</v>
       </c>
       <c r="D76" t="s">
         <v>78</v>
@@ -1963,13 +1963,13 @@
     </row>
     <row r="77" spans="1:4">
       <c r="A77" s="2">
-        <v>46076</v>
+        <v>46101</v>
       </c>
       <c r="B77">
-        <v>23</v>
+        <v>13</v>
       </c>
       <c r="C77">
-        <v>0</v>
+        <v>1.794</v>
       </c>
       <c r="D77" t="s">
         <v>79</v>
@@ -1977,13 +1977,13 @@
     </row>
     <row r="78" spans="1:4">
       <c r="A78" s="2">
-        <v>46076</v>
+        <v>46101</v>
       </c>
       <c r="B78">
-        <v>24</v>
+        <v>14</v>
       </c>
       <c r="C78">
-        <v>0</v>
+        <v>1.794</v>
       </c>
       <c r="D78" t="s">
         <v>80</v>
@@ -1991,13 +1991,13 @@
     </row>
     <row r="79" spans="1:4">
       <c r="A79" s="2">
-        <v>46077</v>
+        <v>46101</v>
       </c>
       <c r="B79">
-        <v>1</v>
+        <v>15</v>
       </c>
       <c r="C79">
-        <v>0</v>
+        <v>1.616</v>
       </c>
       <c r="D79" t="s">
         <v>81</v>
@@ -2005,13 +2005,13 @@
     </row>
     <row r="80" spans="1:4">
       <c r="A80" s="2">
-        <v>46077</v>
+        <v>46101</v>
       </c>
       <c r="B80">
-        <v>2</v>
+        <v>16</v>
       </c>
       <c r="C80">
-        <v>0</v>
+        <v>1.35</v>
       </c>
       <c r="D80" t="s">
         <v>82</v>
@@ -2019,13 +2019,13 @@
     </row>
     <row r="81" spans="1:4">
       <c r="A81" s="2">
-        <v>46077</v>
+        <v>46101</v>
       </c>
       <c r="B81">
-        <v>3</v>
+        <v>17</v>
       </c>
       <c r="C81">
-        <v>0</v>
+        <v>0.967</v>
       </c>
       <c r="D81" t="s">
         <v>83</v>
@@ -2033,13 +2033,13 @@
     </row>
     <row r="82" spans="1:4">
       <c r="A82" s="2">
-        <v>46077</v>
+        <v>46101</v>
       </c>
       <c r="B82">
-        <v>4</v>
+        <v>18</v>
       </c>
       <c r="C82">
-        <v>0</v>
+        <v>0.456</v>
       </c>
       <c r="D82" t="s">
         <v>84</v>
@@ -2047,13 +2047,13 @@
     </row>
     <row r="83" spans="1:4">
       <c r="A83" s="2">
-        <v>46077</v>
+        <v>46101</v>
       </c>
       <c r="B83">
-        <v>5</v>
+        <v>19</v>
       </c>
       <c r="C83">
-        <v>0</v>
+        <v>0.123</v>
       </c>
       <c r="D83" t="s">
         <v>85</v>
@@ -2061,10 +2061,10 @@
     </row>
     <row r="84" spans="1:4">
       <c r="A84" s="2">
-        <v>46077</v>
+        <v>46101</v>
       </c>
       <c r="B84">
-        <v>6</v>
+        <v>20</v>
       </c>
       <c r="C84">
         <v>0</v>
@@ -2075,10 +2075,10 @@
     </row>
     <row r="85" spans="1:4">
       <c r="A85" s="2">
-        <v>46077</v>
+        <v>46101</v>
       </c>
       <c r="B85">
-        <v>7</v>
+        <v>21</v>
       </c>
       <c r="C85">
         <v>0</v>
@@ -2089,10 +2089,10 @@
     </row>
     <row r="86" spans="1:4">
       <c r="A86" s="2">
-        <v>46077</v>
+        <v>46101</v>
       </c>
       <c r="B86">
-        <v>8</v>
+        <v>22</v>
       </c>
       <c r="C86">
         <v>0</v>
@@ -2103,13 +2103,13 @@
     </row>
     <row r="87" spans="1:4">
       <c r="A87" s="2">
-        <v>46077</v>
+        <v>46101</v>
       </c>
       <c r="B87">
-        <v>9</v>
+        <v>23</v>
       </c>
       <c r="C87">
-        <v>0.015</v>
+        <v>0</v>
       </c>
       <c r="D87" t="s">
         <v>89</v>
@@ -2117,13 +2117,13 @@
     </row>
     <row r="88" spans="1:4">
       <c r="A88" s="2">
-        <v>46077</v>
+        <v>46101</v>
       </c>
       <c r="B88">
-        <v>10</v>
+        <v>24</v>
       </c>
       <c r="C88">
-        <v>0.166</v>
+        <v>0</v>
       </c>
       <c r="D88" t="s">
         <v>90</v>
@@ -2131,13 +2131,13 @@
     </row>
     <row r="89" spans="1:4">
       <c r="A89" s="2">
-        <v>46077</v>
+        <v>46102</v>
       </c>
       <c r="B89">
-        <v>11</v>
+        <v>1</v>
       </c>
       <c r="C89">
-        <v>0.482</v>
+        <v>0</v>
       </c>
       <c r="D89" t="s">
         <v>91</v>
@@ -2145,13 +2145,13 @@
     </row>
     <row r="90" spans="1:4">
       <c r="A90" s="2">
-        <v>46077</v>
+        <v>46102</v>
       </c>
       <c r="B90">
-        <v>12</v>
+        <v>2</v>
       </c>
       <c r="C90">
-        <v>0.709</v>
+        <v>0</v>
       </c>
       <c r="D90" t="s">
         <v>92</v>
@@ -2159,13 +2159,13 @@
     </row>
     <row r="91" spans="1:4">
       <c r="A91" s="2">
-        <v>46077</v>
+        <v>46102</v>
       </c>
       <c r="B91">
-        <v>13</v>
+        <v>3</v>
       </c>
       <c r="C91">
-        <v>0.6889999999999999</v>
+        <v>0</v>
       </c>
       <c r="D91" t="s">
         <v>93</v>
@@ -2173,13 +2173,13 @@
     </row>
     <row r="92" spans="1:4">
       <c r="A92" s="2">
-        <v>46077</v>
+        <v>46102</v>
       </c>
       <c r="B92">
-        <v>14</v>
+        <v>4</v>
       </c>
       <c r="C92">
-        <v>0.671</v>
+        <v>0</v>
       </c>
       <c r="D92" t="s">
         <v>94</v>
@@ -2187,13 +2187,13 @@
     </row>
     <row r="93" spans="1:4">
       <c r="A93" s="2">
-        <v>46077</v>
+        <v>46102</v>
       </c>
       <c r="B93">
-        <v>15</v>
+        <v>5</v>
       </c>
       <c r="C93">
-        <v>0.706</v>
+        <v>0</v>
       </c>
       <c r="D93" t="s">
         <v>95</v>
@@ -2201,13 +2201,13 @@
     </row>
     <row r="94" spans="1:4">
       <c r="A94" s="2">
-        <v>46077</v>
+        <v>46102</v>
       </c>
       <c r="B94">
-        <v>16</v>
+        <v>6</v>
       </c>
       <c r="C94">
-        <v>0.61</v>
+        <v>0</v>
       </c>
       <c r="D94" t="s">
         <v>96</v>
@@ -2215,13 +2215,13 @@
     </row>
     <row r="95" spans="1:4">
       <c r="A95" s="2">
-        <v>46077</v>
+        <v>46102</v>
       </c>
       <c r="B95">
-        <v>17</v>
+        <v>7</v>
       </c>
       <c r="C95">
-        <v>0.5610000000000001</v>
+        <v>0</v>
       </c>
       <c r="D95" t="s">
         <v>97</v>
@@ -2229,13 +2229,13 @@
     </row>
     <row r="96" spans="1:4">
       <c r="A96" s="2">
-        <v>46077</v>
+        <v>46102</v>
       </c>
       <c r="B96">
-        <v>18</v>
+        <v>8</v>
       </c>
       <c r="C96">
-        <v>0.255</v>
+        <v>0</v>
       </c>
       <c r="D96" t="s">
         <v>98</v>
@@ -2243,13 +2243,13 @@
     </row>
     <row r="97" spans="1:4">
       <c r="A97" s="2">
-        <v>46077</v>
+        <v>46102</v>
       </c>
       <c r="B97">
-        <v>19</v>
+        <v>9</v>
       </c>
       <c r="C97">
-        <v>0.046</v>
+        <v>0.299</v>
       </c>
       <c r="D97" t="s">
         <v>99</v>
@@ -2257,13 +2257,13 @@
     </row>
     <row r="98" spans="1:4">
       <c r="A98" s="2">
-        <v>46077</v>
+        <v>46102</v>
       </c>
       <c r="B98">
-        <v>20</v>
+        <v>10</v>
       </c>
       <c r="C98">
-        <v>0</v>
+        <v>0.928</v>
       </c>
       <c r="D98" t="s">
         <v>100</v>
@@ -2271,13 +2271,13 @@
     </row>
     <row r="99" spans="1:4">
       <c r="A99" s="2">
-        <v>46077</v>
+        <v>46102</v>
       </c>
       <c r="B99">
-        <v>21</v>
+        <v>11</v>
       </c>
       <c r="C99">
-        <v>0</v>
+        <v>1.485</v>
       </c>
       <c r="D99" t="s">
         <v>101</v>
@@ -2285,13 +2285,13 @@
     </row>
     <row r="100" spans="1:4">
       <c r="A100" s="2">
-        <v>46077</v>
+        <v>46102</v>
       </c>
       <c r="B100">
-        <v>22</v>
+        <v>12</v>
       </c>
       <c r="C100">
-        <v>0</v>
+        <v>1.937</v>
       </c>
       <c r="D100" t="s">
         <v>102</v>
@@ -2299,13 +2299,13 @@
     </row>
     <row r="101" spans="1:4">
       <c r="A101" s="2">
-        <v>46077</v>
+        <v>46102</v>
       </c>
       <c r="B101">
-        <v>23</v>
+        <v>13</v>
       </c>
       <c r="C101">
-        <v>0</v>
+        <v>2.054</v>
       </c>
       <c r="D101" t="s">
         <v>103</v>
@@ -2313,13 +2313,13 @@
     </row>
     <row r="102" spans="1:4">
       <c r="A102" s="2">
-        <v>46077</v>
+        <v>46102</v>
       </c>
       <c r="B102">
-        <v>24</v>
+        <v>14</v>
       </c>
       <c r="C102">
-        <v>0</v>
+        <v>2.038</v>
       </c>
       <c r="D102" t="s">
         <v>104</v>
@@ -2327,13 +2327,13 @@
     </row>
     <row r="103" spans="1:4">
       <c r="A103" s="2">
-        <v>46078</v>
+        <v>46102</v>
       </c>
       <c r="B103">
-        <v>1</v>
+        <v>15</v>
       </c>
       <c r="C103">
-        <v>0</v>
+        <v>1.949</v>
       </c>
       <c r="D103" t="s">
         <v>105</v>
@@ -2341,13 +2341,13 @@
     </row>
     <row r="104" spans="1:4">
       <c r="A104" s="2">
-        <v>46078</v>
+        <v>46102</v>
       </c>
       <c r="B104">
-        <v>2</v>
+        <v>16</v>
       </c>
       <c r="C104">
-        <v>0</v>
+        <v>1.771</v>
       </c>
       <c r="D104" t="s">
         <v>106</v>
@@ -2355,13 +2355,13 @@
     </row>
     <row r="105" spans="1:4">
       <c r="A105" s="2">
-        <v>46078</v>
+        <v>46102</v>
       </c>
       <c r="B105">
-        <v>3</v>
+        <v>17</v>
       </c>
       <c r="C105">
-        <v>0</v>
+        <v>1.508</v>
       </c>
       <c r="D105" t="s">
         <v>107</v>
@@ -2369,13 +2369,13 @@
     </row>
     <row r="106" spans="1:4">
       <c r="A106" s="2">
-        <v>46078</v>
+        <v>46102</v>
       </c>
       <c r="B106">
-        <v>4</v>
+        <v>18</v>
       </c>
       <c r="C106">
-        <v>0</v>
+        <v>0.927</v>
       </c>
       <c r="D106" t="s">
         <v>108</v>
@@ -2383,13 +2383,13 @@
     </row>
     <row r="107" spans="1:4">
       <c r="A107" s="2">
-        <v>46078</v>
+        <v>46102</v>
       </c>
       <c r="B107">
-        <v>5</v>
+        <v>19</v>
       </c>
       <c r="C107">
-        <v>0</v>
+        <v>0.289</v>
       </c>
       <c r="D107" t="s">
         <v>109</v>
@@ -2397,13 +2397,13 @@
     </row>
     <row r="108" spans="1:4">
       <c r="A108" s="2">
-        <v>46078</v>
+        <v>46102</v>
       </c>
       <c r="B108">
-        <v>6</v>
+        <v>20</v>
       </c>
       <c r="C108">
-        <v>0</v>
+        <v>0.017</v>
       </c>
       <c r="D108" t="s">
         <v>110</v>
@@ -2411,10 +2411,10 @@
     </row>
     <row r="109" spans="1:4">
       <c r="A109" s="2">
-        <v>46078</v>
+        <v>46102</v>
       </c>
       <c r="B109">
-        <v>7</v>
+        <v>21</v>
       </c>
       <c r="C109">
         <v>0</v>
@@ -2425,10 +2425,10 @@
     </row>
     <row r="110" spans="1:4">
       <c r="A110" s="2">
-        <v>46078</v>
+        <v>46102</v>
       </c>
       <c r="B110">
-        <v>8</v>
+        <v>22</v>
       </c>
       <c r="C110">
         <v>0</v>
@@ -2439,13 +2439,13 @@
     </row>
     <row r="111" spans="1:4">
       <c r="A111" s="2">
-        <v>46078</v>
+        <v>46102</v>
       </c>
       <c r="B111">
-        <v>9</v>
+        <v>23</v>
       </c>
       <c r="C111">
-        <v>0.028</v>
+        <v>0</v>
       </c>
       <c r="D111" t="s">
         <v>113</v>
@@ -2453,13 +2453,13 @@
     </row>
     <row r="112" spans="1:4">
       <c r="A112" s="2">
-        <v>46078</v>
+        <v>46102</v>
       </c>
       <c r="B112">
-        <v>10</v>
+        <v>24</v>
       </c>
       <c r="C112">
-        <v>0.419</v>
+        <v>0</v>
       </c>
       <c r="D112" t="s">
         <v>114</v>
@@ -2467,13 +2467,13 @@
     </row>
     <row r="113" spans="1:4">
       <c r="A113" s="2">
-        <v>46078</v>
+        <v>46103</v>
       </c>
       <c r="B113">
-        <v>11</v>
+        <v>1</v>
       </c>
       <c r="C113">
-        <v>1.085</v>
+        <v>0</v>
       </c>
       <c r="D113" t="s">
         <v>115</v>
@@ -2481,13 +2481,13 @@
     </row>
     <row r="114" spans="1:4">
       <c r="A114" s="2">
-        <v>46078</v>
+        <v>46103</v>
       </c>
       <c r="B114">
-        <v>12</v>
+        <v>2</v>
       </c>
       <c r="C114">
-        <v>1.733</v>
+        <v>0</v>
       </c>
       <c r="D114" t="s">
         <v>116</v>
@@ -2495,13 +2495,13 @@
     </row>
     <row r="115" spans="1:4">
       <c r="A115" s="2">
-        <v>46078</v>
+        <v>46103</v>
       </c>
       <c r="B115">
-        <v>13</v>
+        <v>3</v>
       </c>
       <c r="C115">
-        <v>2.334</v>
+        <v>0</v>
       </c>
       <c r="D115" t="s">
         <v>117</v>
@@ -2509,13 +2509,13 @@
     </row>
     <row r="116" spans="1:4">
       <c r="A116" s="2">
-        <v>46078</v>
+        <v>46103</v>
       </c>
       <c r="B116">
-        <v>14</v>
+        <v>4</v>
       </c>
       <c r="C116">
-        <v>2.394</v>
+        <v>0</v>
       </c>
       <c r="D116" t="s">
         <v>118</v>
@@ -2523,13 +2523,13 @@
     </row>
     <row r="117" spans="1:4">
       <c r="A117" s="2">
-        <v>46078</v>
+        <v>46103</v>
       </c>
       <c r="B117">
-        <v>15</v>
+        <v>5</v>
       </c>
       <c r="C117">
-        <v>2.472</v>
+        <v>0</v>
       </c>
       <c r="D117" t="s">
         <v>119</v>
@@ -2537,13 +2537,13 @@
     </row>
     <row r="118" spans="1:4">
       <c r="A118" s="2">
-        <v>46078</v>
+        <v>46103</v>
       </c>
       <c r="B118">
-        <v>16</v>
+        <v>6</v>
       </c>
       <c r="C118">
-        <v>2.069</v>
+        <v>0</v>
       </c>
       <c r="D118" t="s">
         <v>120</v>
@@ -2551,13 +2551,13 @@
     </row>
     <row r="119" spans="1:4">
       <c r="A119" s="2">
-        <v>46078</v>
+        <v>46103</v>
       </c>
       <c r="B119">
-        <v>17</v>
+        <v>7</v>
       </c>
       <c r="C119">
-        <v>1.426</v>
+        <v>0</v>
       </c>
       <c r="D119" t="s">
         <v>121</v>
@@ -2565,13 +2565,13 @@
     </row>
     <row r="120" spans="1:4">
       <c r="A120" s="2">
-        <v>46078</v>
+        <v>46103</v>
       </c>
       <c r="B120">
-        <v>18</v>
+        <v>8</v>
       </c>
       <c r="C120">
-        <v>0.548</v>
+        <v>0.012</v>
       </c>
       <c r="D120" t="s">
         <v>122</v>
@@ -2579,13 +2579,13 @@
     </row>
     <row r="121" spans="1:4">
       <c r="A121" s="2">
-        <v>46078</v>
+        <v>46103</v>
       </c>
       <c r="B121">
-        <v>19</v>
+        <v>9</v>
       </c>
       <c r="C121">
-        <v>0.057</v>
+        <v>0.306</v>
       </c>
       <c r="D121" t="s">
         <v>123</v>
@@ -2593,13 +2593,13 @@
     </row>
     <row r="122" spans="1:4">
       <c r="A122" s="2">
-        <v>46078</v>
+        <v>46103</v>
       </c>
       <c r="B122">
-        <v>20</v>
+        <v>10</v>
       </c>
       <c r="C122">
-        <v>0</v>
+        <v>0.918</v>
       </c>
       <c r="D122" t="s">
         <v>124</v>
@@ -2607,13 +2607,13 @@
     </row>
     <row r="123" spans="1:4">
       <c r="A123" s="2">
-        <v>46078</v>
+        <v>46103</v>
       </c>
       <c r="B123">
-        <v>21</v>
+        <v>11</v>
       </c>
       <c r="C123">
-        <v>0</v>
+        <v>1.318</v>
       </c>
       <c r="D123" t="s">
         <v>125</v>
@@ -2621,13 +2621,13 @@
     </row>
     <row r="124" spans="1:4">
       <c r="A124" s="2">
-        <v>46078</v>
+        <v>46103</v>
       </c>
       <c r="B124">
-        <v>22</v>
+        <v>12</v>
       </c>
       <c r="C124">
-        <v>0</v>
+        <v>1.712</v>
       </c>
       <c r="D124" t="s">
         <v>126</v>
@@ -2635,13 +2635,13 @@
     </row>
     <row r="125" spans="1:4">
       <c r="A125" s="2">
-        <v>46078</v>
+        <v>46103</v>
       </c>
       <c r="B125">
-        <v>23</v>
+        <v>13</v>
       </c>
       <c r="C125">
-        <v>0</v>
+        <v>1.945</v>
       </c>
       <c r="D125" t="s">
         <v>127</v>
@@ -2649,13 +2649,13 @@
     </row>
     <row r="126" spans="1:4">
       <c r="A126" s="2">
-        <v>46078</v>
+        <v>46103</v>
       </c>
       <c r="B126">
-        <v>24</v>
+        <v>14</v>
       </c>
       <c r="C126">
-        <v>0</v>
+        <v>1.996</v>
       </c>
       <c r="D126" t="s">
         <v>128</v>
@@ -2663,13 +2663,13 @@
     </row>
     <row r="127" spans="1:4">
       <c r="A127" s="2">
-        <v>46079</v>
+        <v>46103</v>
       </c>
       <c r="B127">
-        <v>1</v>
+        <v>15</v>
       </c>
       <c r="C127">
-        <v>0</v>
+        <v>1.906</v>
       </c>
       <c r="D127" t="s">
         <v>129</v>
@@ -2677,13 +2677,13 @@
     </row>
     <row r="128" spans="1:4">
       <c r="A128" s="2">
-        <v>46079</v>
+        <v>46103</v>
       </c>
       <c r="B128">
-        <v>2</v>
+        <v>16</v>
       </c>
       <c r="C128">
-        <v>0</v>
+        <v>1.646</v>
       </c>
       <c r="D128" t="s">
         <v>130</v>
@@ -2691,13 +2691,13 @@
     </row>
     <row r="129" spans="1:4">
       <c r="A129" s="2">
-        <v>46079</v>
+        <v>46103</v>
       </c>
       <c r="B129">
-        <v>3</v>
+        <v>17</v>
       </c>
       <c r="C129">
-        <v>0</v>
+        <v>1.134</v>
       </c>
       <c r="D129" t="s">
         <v>131</v>
@@ -2705,13 +2705,13 @@
     </row>
     <row r="130" spans="1:4">
       <c r="A130" s="2">
-        <v>46079</v>
+        <v>46103</v>
       </c>
       <c r="B130">
-        <v>4</v>
+        <v>18</v>
       </c>
       <c r="C130">
-        <v>0</v>
+        <v>0.595</v>
       </c>
       <c r="D130" t="s">
         <v>132</v>
@@ -2719,13 +2719,13 @@
     </row>
     <row r="131" spans="1:4">
       <c r="A131" s="2">
-        <v>46079</v>
+        <v>46103</v>
       </c>
       <c r="B131">
-        <v>5</v>
+        <v>19</v>
       </c>
       <c r="C131">
-        <v>0</v>
+        <v>0.139</v>
       </c>
       <c r="D131" t="s">
         <v>133</v>
@@ -2733,13 +2733,13 @@
     </row>
     <row r="132" spans="1:4">
       <c r="A132" s="2">
-        <v>46079</v>
+        <v>46103</v>
       </c>
       <c r="B132">
-        <v>6</v>
+        <v>20</v>
       </c>
       <c r="C132">
-        <v>0</v>
+        <v>0.012</v>
       </c>
       <c r="D132" t="s">
         <v>134</v>
@@ -2747,10 +2747,10 @@
     </row>
     <row r="133" spans="1:4">
       <c r="A133" s="2">
-        <v>46079</v>
+        <v>46103</v>
       </c>
       <c r="B133">
-        <v>7</v>
+        <v>21</v>
       </c>
       <c r="C133">
         <v>0</v>
@@ -2761,10 +2761,10 @@
     </row>
     <row r="134" spans="1:4">
       <c r="A134" s="2">
-        <v>46079</v>
+        <v>46103</v>
       </c>
       <c r="B134">
-        <v>8</v>
+        <v>22</v>
       </c>
       <c r="C134">
         <v>0</v>
@@ -2775,13 +2775,13 @@
     </row>
     <row r="135" spans="1:4">
       <c r="A135" s="2">
-        <v>46079</v>
+        <v>46103</v>
       </c>
       <c r="B135">
-        <v>9</v>
+        <v>23</v>
       </c>
       <c r="C135">
-        <v>0.03</v>
+        <v>0</v>
       </c>
       <c r="D135" t="s">
         <v>137</v>
@@ -2789,13 +2789,13 @@
     </row>
     <row r="136" spans="1:4">
       <c r="A136" s="2">
-        <v>46079</v>
+        <v>46103</v>
       </c>
       <c r="B136">
-        <v>10</v>
+        <v>24</v>
       </c>
       <c r="C136">
-        <v>0.437</v>
+        <v>0</v>
       </c>
       <c r="D136" t="s">
         <v>138</v>
@@ -2803,13 +2803,13 @@
     </row>
     <row r="137" spans="1:4">
       <c r="A137" s="2">
-        <v>46079</v>
+        <v>46104</v>
       </c>
       <c r="B137">
-        <v>11</v>
+        <v>1</v>
       </c>
       <c r="C137">
-        <v>1.009</v>
+        <v>0</v>
       </c>
       <c r="D137" t="s">
         <v>139</v>
@@ -2817,13 +2817,13 @@
     </row>
     <row r="138" spans="1:4">
       <c r="A138" s="2">
-        <v>46079</v>
+        <v>46104</v>
       </c>
       <c r="B138">
-        <v>12</v>
+        <v>2</v>
       </c>
       <c r="C138">
-        <v>1.787</v>
+        <v>0</v>
       </c>
       <c r="D138" t="s">
         <v>140</v>
@@ -2831,13 +2831,13 @@
     </row>
     <row r="139" spans="1:4">
       <c r="A139" s="2">
-        <v>46079</v>
+        <v>46104</v>
       </c>
       <c r="B139">
-        <v>13</v>
+        <v>3</v>
       </c>
       <c r="C139">
-        <v>2.299</v>
+        <v>0</v>
       </c>
       <c r="D139" t="s">
         <v>141</v>
@@ -2845,13 +2845,13 @@
     </row>
     <row r="140" spans="1:4">
       <c r="A140" s="2">
-        <v>46079</v>
+        <v>46104</v>
       </c>
       <c r="B140">
-        <v>14</v>
+        <v>4</v>
       </c>
       <c r="C140">
-        <v>2.47</v>
+        <v>0</v>
       </c>
       <c r="D140" t="s">
         <v>142</v>
@@ -2859,13 +2859,13 @@
     </row>
     <row r="141" spans="1:4">
       <c r="A141" s="2">
-        <v>46079</v>
+        <v>46104</v>
       </c>
       <c r="B141">
-        <v>15</v>
+        <v>5</v>
       </c>
       <c r="C141">
-        <v>2.351</v>
+        <v>0</v>
       </c>
       <c r="D141" t="s">
         <v>143</v>
@@ -2873,13 +2873,13 @@
     </row>
     <row r="142" spans="1:4">
       <c r="A142" s="2">
-        <v>46079</v>
+        <v>46104</v>
       </c>
       <c r="B142">
-        <v>16</v>
+        <v>6</v>
       </c>
       <c r="C142">
-        <v>2.074</v>
+        <v>0</v>
       </c>
       <c r="D142" t="s">
         <v>144</v>
@@ -2887,13 +2887,13 @@
     </row>
     <row r="143" spans="1:4">
       <c r="A143" s="2">
-        <v>46079</v>
+        <v>46104</v>
       </c>
       <c r="B143">
-        <v>17</v>
+        <v>7</v>
       </c>
       <c r="C143">
-        <v>1.577</v>
+        <v>0</v>
       </c>
       <c r="D143" t="s">
         <v>145</v>
@@ -2901,13 +2901,13 @@
     </row>
     <row r="144" spans="1:4">
       <c r="A144" s="2">
-        <v>46079</v>
+        <v>46104</v>
       </c>
       <c r="B144">
-        <v>18</v>
+        <v>8</v>
       </c>
       <c r="C144">
-        <v>0.695</v>
+        <v>0</v>
       </c>
       <c r="D144" t="s">
         <v>146</v>
@@ -2915,13 +2915,13 @@
     </row>
     <row r="145" spans="1:4">
       <c r="A145" s="2">
-        <v>46079</v>
+        <v>46104</v>
       </c>
       <c r="B145">
-        <v>19</v>
+        <v>9</v>
       </c>
       <c r="C145">
-        <v>0.08</v>
+        <v>0.226</v>
       </c>
       <c r="D145" t="s">
         <v>147</v>
@@ -2929,13 +2929,13 @@
     </row>
     <row r="146" spans="1:4">
       <c r="A146" s="2">
-        <v>46079</v>
+        <v>46104</v>
       </c>
       <c r="B146">
-        <v>20</v>
+        <v>10</v>
       </c>
       <c r="C146">
-        <v>0</v>
+        <v>0.753</v>
       </c>
       <c r="D146" t="s">
         <v>148</v>
@@ -2943,13 +2943,13 @@
     </row>
     <row r="147" spans="1:4">
       <c r="A147" s="2">
-        <v>46079</v>
+        <v>46104</v>
       </c>
       <c r="B147">
-        <v>21</v>
+        <v>11</v>
       </c>
       <c r="C147">
-        <v>0</v>
+        <v>1.097</v>
       </c>
       <c r="D147" t="s">
         <v>149</v>
@@ -2957,13 +2957,13 @@
     </row>
     <row r="148" spans="1:4">
       <c r="A148" s="2">
-        <v>46079</v>
+        <v>46104</v>
       </c>
       <c r="B148">
-        <v>22</v>
+        <v>12</v>
       </c>
       <c r="C148">
-        <v>0</v>
+        <v>1.587</v>
       </c>
       <c r="D148" t="s">
         <v>150</v>
@@ -2971,13 +2971,13 @@
     </row>
     <row r="149" spans="1:4">
       <c r="A149" s="2">
-        <v>46079</v>
+        <v>46104</v>
       </c>
       <c r="B149">
-        <v>23</v>
+        <v>13</v>
       </c>
       <c r="C149">
-        <v>0</v>
+        <v>1.893</v>
       </c>
       <c r="D149" t="s">
         <v>151</v>
@@ -2985,13 +2985,13 @@
     </row>
     <row r="150" spans="1:4">
       <c r="A150" s="2">
-        <v>46079</v>
+        <v>46104</v>
       </c>
       <c r="B150">
-        <v>24</v>
+        <v>14</v>
       </c>
       <c r="C150">
-        <v>0</v>
+        <v>1.962</v>
       </c>
       <c r="D150" t="s">
         <v>152</v>
@@ -2999,13 +2999,13 @@
     </row>
     <row r="151" spans="1:4">
       <c r="A151" s="2">
-        <v>46080</v>
+        <v>46104</v>
       </c>
       <c r="B151">
-        <v>1</v>
+        <v>15</v>
       </c>
       <c r="C151">
-        <v>0</v>
+        <v>1.96</v>
       </c>
       <c r="D151" t="s">
         <v>153</v>
@@ -3013,13 +3013,13 @@
     </row>
     <row r="152" spans="1:4">
       <c r="A152" s="2">
-        <v>46080</v>
+        <v>46104</v>
       </c>
       <c r="B152">
-        <v>2</v>
+        <v>16</v>
       </c>
       <c r="C152">
-        <v>0</v>
+        <v>1.774</v>
       </c>
       <c r="D152" t="s">
         <v>154</v>
@@ -3027,13 +3027,13 @@
     </row>
     <row r="153" spans="1:4">
       <c r="A153" s="2">
-        <v>46080</v>
+        <v>46104</v>
       </c>
       <c r="B153">
-        <v>3</v>
+        <v>17</v>
       </c>
       <c r="C153">
-        <v>0</v>
+        <v>1.313</v>
       </c>
       <c r="D153" t="s">
         <v>155</v>
@@ -3041,13 +3041,13 @@
     </row>
     <row r="154" spans="1:4">
       <c r="A154" s="2">
-        <v>46080</v>
+        <v>46104</v>
       </c>
       <c r="B154">
-        <v>4</v>
+        <v>18</v>
       </c>
       <c r="C154">
-        <v>0</v>
+        <v>0.705</v>
       </c>
       <c r="D154" t="s">
         <v>156</v>
@@ -3055,13 +3055,13 @@
     </row>
     <row r="155" spans="1:4">
       <c r="A155" s="2">
-        <v>46080</v>
+        <v>46104</v>
       </c>
       <c r="B155">
-        <v>5</v>
+        <v>19</v>
       </c>
       <c r="C155">
-        <v>0</v>
+        <v>0.205</v>
       </c>
       <c r="D155" t="s">
         <v>157</v>
@@ -3069,13 +3069,13 @@
     </row>
     <row r="156" spans="1:4">
       <c r="A156" s="2">
-        <v>46080</v>
+        <v>46104</v>
       </c>
       <c r="B156">
-        <v>6</v>
+        <v>20</v>
       </c>
       <c r="C156">
-        <v>0</v>
+        <v>0.013</v>
       </c>
       <c r="D156" t="s">
         <v>158</v>
@@ -3083,10 +3083,10 @@
     </row>
     <row r="157" spans="1:4">
       <c r="A157" s="2">
-        <v>46080</v>
+        <v>46104</v>
       </c>
       <c r="B157">
-        <v>7</v>
+        <v>21</v>
       </c>
       <c r="C157">
         <v>0</v>
@@ -3097,10 +3097,10 @@
     </row>
     <row r="158" spans="1:4">
       <c r="A158" s="2">
-        <v>46080</v>
+        <v>46104</v>
       </c>
       <c r="B158">
-        <v>8</v>
+        <v>22</v>
       </c>
       <c r="C158">
         <v>0</v>
@@ -3111,13 +3111,13 @@
     </row>
     <row r="159" spans="1:4">
       <c r="A159" s="2">
-        <v>46080</v>
+        <v>46104</v>
       </c>
       <c r="B159">
-        <v>9</v>
+        <v>23</v>
       </c>
       <c r="C159">
-        <v>0.027</v>
+        <v>0</v>
       </c>
       <c r="D159" t="s">
         <v>161</v>
@@ -3125,13 +3125,13 @@
     </row>
     <row r="160" spans="1:4">
       <c r="A160" s="2">
-        <v>46080</v>
+        <v>46104</v>
       </c>
       <c r="B160">
-        <v>10</v>
+        <v>24</v>
       </c>
       <c r="C160">
-        <v>0.349</v>
+        <v>0</v>
       </c>
       <c r="D160" t="s">
         <v>162</v>
@@ -3139,13 +3139,13 @@
     </row>
     <row r="161" spans="1:4">
       <c r="A161" s="2">
-        <v>46080</v>
+        <v>46105</v>
       </c>
       <c r="B161">
-        <v>11</v>
+        <v>1</v>
       </c>
       <c r="C161">
-        <v>0.844</v>
+        <v>0</v>
       </c>
       <c r="D161" t="s">
         <v>163</v>
@@ -3153,13 +3153,13 @@
     </row>
     <row r="162" spans="1:4">
       <c r="A162" s="2">
-        <v>46080</v>
+        <v>46105</v>
       </c>
       <c r="B162">
-        <v>12</v>
+        <v>2</v>
       </c>
       <c r="C162">
-        <v>1.538</v>
+        <v>0</v>
       </c>
       <c r="D162" t="s">
         <v>164</v>
@@ -3167,13 +3167,13 @@
     </row>
     <row r="163" spans="1:4">
       <c r="A163" s="2">
-        <v>46080</v>
+        <v>46105</v>
       </c>
       <c r="B163">
-        <v>13</v>
+        <v>3</v>
       </c>
       <c r="C163">
-        <v>1.87</v>
+        <v>0</v>
       </c>
       <c r="D163" t="s">
         <v>165</v>
@@ -3181,13 +3181,13 @@
     </row>
     <row r="164" spans="1:4">
       <c r="A164" s="2">
-        <v>46080</v>
+        <v>46105</v>
       </c>
       <c r="B164">
-        <v>14</v>
+        <v>4</v>
       </c>
       <c r="C164">
-        <v>2.077</v>
+        <v>0</v>
       </c>
       <c r="D164" t="s">
         <v>166</v>
@@ -3195,13 +3195,13 @@
     </row>
     <row r="165" spans="1:4">
       <c r="A165" s="2">
-        <v>46080</v>
+        <v>46105</v>
       </c>
       <c r="B165">
-        <v>15</v>
+        <v>5</v>
       </c>
       <c r="C165">
-        <v>2.02</v>
+        <v>0</v>
       </c>
       <c r="D165" t="s">
         <v>167</v>
@@ -3209,13 +3209,13 @@
     </row>
     <row r="166" spans="1:4">
       <c r="A166" s="2">
-        <v>46080</v>
+        <v>46105</v>
       </c>
       <c r="B166">
-        <v>16</v>
+        <v>6</v>
       </c>
       <c r="C166">
-        <v>1.723</v>
+        <v>0</v>
       </c>
       <c r="D166" t="s">
         <v>168</v>
@@ -3223,13 +3223,13 @@
     </row>
     <row r="167" spans="1:4">
       <c r="A167" s="2">
-        <v>46080</v>
+        <v>46105</v>
       </c>
       <c r="B167">
-        <v>17</v>
+        <v>7</v>
       </c>
       <c r="C167">
-        <v>1.084</v>
+        <v>0</v>
       </c>
       <c r="D167" t="s">
         <v>169</v>
@@ -3237,13 +3237,13 @@
     </row>
     <row r="168" spans="1:4">
       <c r="A168" s="2">
-        <v>46080</v>
+        <v>46105</v>
       </c>
       <c r="B168">
-        <v>18</v>
+        <v>8</v>
       </c>
       <c r="C168">
-        <v>0.419</v>
+        <v>0.016</v>
       </c>
       <c r="D168" t="s">
         <v>170</v>
@@ -3251,13 +3251,13 @@
     </row>
     <row r="169" spans="1:4">
       <c r="A169" s="2">
-        <v>46080</v>
+        <v>46105</v>
       </c>
       <c r="B169">
-        <v>19</v>
+        <v>9</v>
       </c>
       <c r="C169">
-        <v>0.061</v>
+        <v>0.361</v>
       </c>
       <c r="D169" t="s">
         <v>171</v>
@@ -3265,13 +3265,13 @@
     </row>
     <row r="170" spans="1:4">
       <c r="A170" s="2">
-        <v>46080</v>
+        <v>46105</v>
       </c>
       <c r="B170">
-        <v>20</v>
+        <v>10</v>
       </c>
       <c r="C170">
-        <v>0</v>
+        <v>0.914</v>
       </c>
       <c r="D170" t="s">
         <v>172</v>

</xml_diff>

<commit_message>
Switching to summer time
</commit_message>
<xml_diff>
--- a/Astro/Results_Production_Astro_xgb.xlsx
+++ b/Astro/Results_Production_Astro_xgb.xlsx
@@ -28,511 +28,511 @@
     <t>Lookup</t>
   </si>
   <si>
-    <t>17.03.202610</t>
-  </si>
-  <si>
-    <t>17.03.202611</t>
-  </si>
-  <si>
-    <t>17.03.202612</t>
-  </si>
-  <si>
-    <t>17.03.202613</t>
-  </si>
-  <si>
-    <t>17.03.202614</t>
-  </si>
-  <si>
-    <t>17.03.202615</t>
-  </si>
-  <si>
-    <t>17.03.202616</t>
-  </si>
-  <si>
-    <t>17.03.202617</t>
-  </si>
-  <si>
-    <t>17.03.202618</t>
-  </si>
-  <si>
-    <t>17.03.202619</t>
-  </si>
-  <si>
-    <t>17.03.202620</t>
-  </si>
-  <si>
-    <t>17.03.202621</t>
-  </si>
-  <si>
-    <t>17.03.202622</t>
-  </si>
-  <si>
-    <t>17.03.202623</t>
-  </si>
-  <si>
-    <t>17.03.202624</t>
-  </si>
-  <si>
-    <t>18.03.20261</t>
-  </si>
-  <si>
-    <t>18.03.20262</t>
-  </si>
-  <si>
-    <t>18.03.20263</t>
-  </si>
-  <si>
-    <t>18.03.20264</t>
-  </si>
-  <si>
-    <t>18.03.20265</t>
-  </si>
-  <si>
-    <t>18.03.20266</t>
-  </si>
-  <si>
-    <t>18.03.20267</t>
-  </si>
-  <si>
-    <t>18.03.20268</t>
-  </si>
-  <si>
-    <t>18.03.20269</t>
-  </si>
-  <si>
-    <t>18.03.202610</t>
-  </si>
-  <si>
-    <t>18.03.202611</t>
-  </si>
-  <si>
-    <t>18.03.202612</t>
-  </si>
-  <si>
-    <t>18.03.202613</t>
-  </si>
-  <si>
-    <t>18.03.202614</t>
-  </si>
-  <si>
-    <t>18.03.202615</t>
-  </si>
-  <si>
-    <t>18.03.202616</t>
-  </si>
-  <si>
-    <t>18.03.202617</t>
-  </si>
-  <si>
-    <t>18.03.202618</t>
-  </si>
-  <si>
-    <t>18.03.202619</t>
-  </si>
-  <si>
-    <t>18.03.202620</t>
-  </si>
-  <si>
-    <t>18.03.202621</t>
-  </si>
-  <si>
-    <t>18.03.202622</t>
-  </si>
-  <si>
-    <t>18.03.202623</t>
-  </si>
-  <si>
-    <t>18.03.202624</t>
-  </si>
-  <si>
-    <t>19.03.20261</t>
-  </si>
-  <si>
-    <t>19.03.20262</t>
-  </si>
-  <si>
-    <t>19.03.20263</t>
-  </si>
-  <si>
-    <t>19.03.20264</t>
-  </si>
-  <si>
-    <t>19.03.20265</t>
-  </si>
-  <si>
-    <t>19.03.20266</t>
-  </si>
-  <si>
-    <t>19.03.20267</t>
-  </si>
-  <si>
-    <t>19.03.20268</t>
-  </si>
-  <si>
-    <t>19.03.20269</t>
-  </si>
-  <si>
-    <t>19.03.202610</t>
-  </si>
-  <si>
-    <t>19.03.202611</t>
-  </si>
-  <si>
-    <t>19.03.202612</t>
-  </si>
-  <si>
-    <t>19.03.202613</t>
-  </si>
-  <si>
-    <t>19.03.202614</t>
-  </si>
-  <si>
-    <t>19.03.202615</t>
-  </si>
-  <si>
-    <t>19.03.202616</t>
-  </si>
-  <si>
-    <t>19.03.202617</t>
-  </si>
-  <si>
-    <t>19.03.202618</t>
-  </si>
-  <si>
-    <t>19.03.202619</t>
-  </si>
-  <si>
-    <t>19.03.202620</t>
-  </si>
-  <si>
-    <t>19.03.202621</t>
-  </si>
-  <si>
-    <t>19.03.202622</t>
-  </si>
-  <si>
-    <t>19.03.202623</t>
-  </si>
-  <si>
-    <t>19.03.202624</t>
-  </si>
-  <si>
-    <t>20.03.20261</t>
-  </si>
-  <si>
-    <t>20.03.20262</t>
-  </si>
-  <si>
-    <t>20.03.20263</t>
-  </si>
-  <si>
-    <t>20.03.20264</t>
-  </si>
-  <si>
-    <t>20.03.20265</t>
-  </si>
-  <si>
-    <t>20.03.20266</t>
-  </si>
-  <si>
-    <t>20.03.20267</t>
-  </si>
-  <si>
-    <t>20.03.20268</t>
-  </si>
-  <si>
-    <t>20.03.20269</t>
-  </si>
-  <si>
-    <t>20.03.202610</t>
-  </si>
-  <si>
-    <t>20.03.202611</t>
-  </si>
-  <si>
-    <t>20.03.202612</t>
-  </si>
-  <si>
-    <t>20.03.202613</t>
-  </si>
-  <si>
-    <t>20.03.202614</t>
-  </si>
-  <si>
-    <t>20.03.202615</t>
-  </si>
-  <si>
-    <t>20.03.202616</t>
-  </si>
-  <si>
-    <t>20.03.202617</t>
-  </si>
-  <si>
-    <t>20.03.202618</t>
-  </si>
-  <si>
-    <t>20.03.202619</t>
-  </si>
-  <si>
-    <t>20.03.202620</t>
-  </si>
-  <si>
-    <t>20.03.202621</t>
-  </si>
-  <si>
-    <t>20.03.202622</t>
-  </si>
-  <si>
-    <t>20.03.202623</t>
-  </si>
-  <si>
-    <t>20.03.202624</t>
-  </si>
-  <si>
-    <t>21.03.20261</t>
-  </si>
-  <si>
-    <t>21.03.20262</t>
-  </si>
-  <si>
-    <t>21.03.20263</t>
-  </si>
-  <si>
-    <t>21.03.20264</t>
-  </si>
-  <si>
-    <t>21.03.20265</t>
-  </si>
-  <si>
-    <t>21.03.20266</t>
-  </si>
-  <si>
-    <t>21.03.20267</t>
-  </si>
-  <si>
-    <t>21.03.20268</t>
-  </si>
-  <si>
-    <t>21.03.20269</t>
-  </si>
-  <si>
-    <t>21.03.202610</t>
-  </si>
-  <si>
-    <t>21.03.202611</t>
-  </si>
-  <si>
-    <t>21.03.202612</t>
-  </si>
-  <si>
-    <t>21.03.202613</t>
-  </si>
-  <si>
-    <t>21.03.202614</t>
-  </si>
-  <si>
-    <t>21.03.202615</t>
-  </si>
-  <si>
-    <t>21.03.202616</t>
-  </si>
-  <si>
-    <t>21.03.202617</t>
-  </si>
-  <si>
-    <t>21.03.202618</t>
-  </si>
-  <si>
-    <t>21.03.202619</t>
-  </si>
-  <si>
-    <t>21.03.202620</t>
-  </si>
-  <si>
-    <t>21.03.202621</t>
-  </si>
-  <si>
-    <t>21.03.202622</t>
-  </si>
-  <si>
-    <t>21.03.202623</t>
-  </si>
-  <si>
-    <t>21.03.202624</t>
-  </si>
-  <si>
-    <t>22.03.20261</t>
-  </si>
-  <si>
-    <t>22.03.20262</t>
-  </si>
-  <si>
-    <t>22.03.20263</t>
-  </si>
-  <si>
-    <t>22.03.20264</t>
-  </si>
-  <si>
-    <t>22.03.20265</t>
-  </si>
-  <si>
-    <t>22.03.20266</t>
-  </si>
-  <si>
-    <t>22.03.20267</t>
-  </si>
-  <si>
-    <t>22.03.20268</t>
-  </si>
-  <si>
-    <t>22.03.20269</t>
-  </si>
-  <si>
-    <t>22.03.202610</t>
-  </si>
-  <si>
-    <t>22.03.202611</t>
-  </si>
-  <si>
-    <t>22.03.202612</t>
-  </si>
-  <si>
-    <t>22.03.202613</t>
-  </si>
-  <si>
-    <t>22.03.202614</t>
-  </si>
-  <si>
-    <t>22.03.202615</t>
-  </si>
-  <si>
-    <t>22.03.202616</t>
-  </si>
-  <si>
-    <t>22.03.202617</t>
-  </si>
-  <si>
-    <t>22.03.202618</t>
-  </si>
-  <si>
-    <t>22.03.202619</t>
-  </si>
-  <si>
-    <t>22.03.202620</t>
-  </si>
-  <si>
-    <t>22.03.202621</t>
-  </si>
-  <si>
-    <t>22.03.202622</t>
-  </si>
-  <si>
-    <t>22.03.202623</t>
-  </si>
-  <si>
-    <t>22.03.202624</t>
-  </si>
-  <si>
-    <t>23.03.20261</t>
-  </si>
-  <si>
-    <t>23.03.20262</t>
-  </si>
-  <si>
-    <t>23.03.20263</t>
-  </si>
-  <si>
-    <t>23.03.20264</t>
-  </si>
-  <si>
-    <t>23.03.20265</t>
-  </si>
-  <si>
-    <t>23.03.20266</t>
-  </si>
-  <si>
-    <t>23.03.20267</t>
-  </si>
-  <si>
-    <t>23.03.20268</t>
-  </si>
-  <si>
-    <t>23.03.20269</t>
-  </si>
-  <si>
-    <t>23.03.202610</t>
-  </si>
-  <si>
-    <t>23.03.202611</t>
-  </si>
-  <si>
-    <t>23.03.202612</t>
-  </si>
-  <si>
-    <t>23.03.202613</t>
-  </si>
-  <si>
-    <t>23.03.202614</t>
-  </si>
-  <si>
-    <t>23.03.202615</t>
-  </si>
-  <si>
-    <t>23.03.202616</t>
-  </si>
-  <si>
-    <t>23.03.202617</t>
-  </si>
-  <si>
-    <t>23.03.202618</t>
-  </si>
-  <si>
-    <t>23.03.202619</t>
-  </si>
-  <si>
-    <t>23.03.202620</t>
-  </si>
-  <si>
-    <t>23.03.202621</t>
-  </si>
-  <si>
-    <t>23.03.202622</t>
-  </si>
-  <si>
-    <t>23.03.202623</t>
-  </si>
-  <si>
-    <t>23.03.202624</t>
-  </si>
-  <si>
-    <t>24.03.20261</t>
-  </si>
-  <si>
-    <t>24.03.20262</t>
-  </si>
-  <si>
-    <t>24.03.20263</t>
-  </si>
-  <si>
-    <t>24.03.20264</t>
-  </si>
-  <si>
-    <t>24.03.20265</t>
-  </si>
-  <si>
-    <t>24.03.20266</t>
-  </si>
-  <si>
-    <t>24.03.20267</t>
-  </si>
-  <si>
-    <t>24.03.20268</t>
-  </si>
-  <si>
-    <t>24.03.20269</t>
-  </si>
-  <si>
-    <t>24.03.202610</t>
+    <t>29.03.202611</t>
+  </si>
+  <si>
+    <t>29.03.202612</t>
+  </si>
+  <si>
+    <t>29.03.202613</t>
+  </si>
+  <si>
+    <t>29.03.202614</t>
+  </si>
+  <si>
+    <t>29.03.202615</t>
+  </si>
+  <si>
+    <t>29.03.202616</t>
+  </si>
+  <si>
+    <t>29.03.202617</t>
+  </si>
+  <si>
+    <t>29.03.202618</t>
+  </si>
+  <si>
+    <t>29.03.202619</t>
+  </si>
+  <si>
+    <t>29.03.202620</t>
+  </si>
+  <si>
+    <t>29.03.202621</t>
+  </si>
+  <si>
+    <t>29.03.202622</t>
+  </si>
+  <si>
+    <t>29.03.202623</t>
+  </si>
+  <si>
+    <t>29.03.202624</t>
+  </si>
+  <si>
+    <t>30.03.20261</t>
+  </si>
+  <si>
+    <t>30.03.20262</t>
+  </si>
+  <si>
+    <t>30.03.20263</t>
+  </si>
+  <si>
+    <t>30.03.20264</t>
+  </si>
+  <si>
+    <t>30.03.20265</t>
+  </si>
+  <si>
+    <t>30.03.20266</t>
+  </si>
+  <si>
+    <t>30.03.20267</t>
+  </si>
+  <si>
+    <t>30.03.20268</t>
+  </si>
+  <si>
+    <t>30.03.20269</t>
+  </si>
+  <si>
+    <t>30.03.202610</t>
+  </si>
+  <si>
+    <t>30.03.202611</t>
+  </si>
+  <si>
+    <t>30.03.202612</t>
+  </si>
+  <si>
+    <t>30.03.202613</t>
+  </si>
+  <si>
+    <t>30.03.202614</t>
+  </si>
+  <si>
+    <t>30.03.202615</t>
+  </si>
+  <si>
+    <t>30.03.202616</t>
+  </si>
+  <si>
+    <t>30.03.202617</t>
+  </si>
+  <si>
+    <t>30.03.202618</t>
+  </si>
+  <si>
+    <t>30.03.202619</t>
+  </si>
+  <si>
+    <t>30.03.202620</t>
+  </si>
+  <si>
+    <t>30.03.202621</t>
+  </si>
+  <si>
+    <t>30.03.202622</t>
+  </si>
+  <si>
+    <t>30.03.202623</t>
+  </si>
+  <si>
+    <t>30.03.202624</t>
+  </si>
+  <si>
+    <t>31.03.20261</t>
+  </si>
+  <si>
+    <t>31.03.20262</t>
+  </si>
+  <si>
+    <t>31.03.20263</t>
+  </si>
+  <si>
+    <t>31.03.20264</t>
+  </si>
+  <si>
+    <t>31.03.20265</t>
+  </si>
+  <si>
+    <t>31.03.20266</t>
+  </si>
+  <si>
+    <t>31.03.20267</t>
+  </si>
+  <si>
+    <t>31.03.20268</t>
+  </si>
+  <si>
+    <t>31.03.20269</t>
+  </si>
+  <si>
+    <t>31.03.202610</t>
+  </si>
+  <si>
+    <t>31.03.202611</t>
+  </si>
+  <si>
+    <t>31.03.202612</t>
+  </si>
+  <si>
+    <t>31.03.202613</t>
+  </si>
+  <si>
+    <t>31.03.202614</t>
+  </si>
+  <si>
+    <t>31.03.202615</t>
+  </si>
+  <si>
+    <t>31.03.202616</t>
+  </si>
+  <si>
+    <t>31.03.202617</t>
+  </si>
+  <si>
+    <t>31.03.202618</t>
+  </si>
+  <si>
+    <t>31.03.202619</t>
+  </si>
+  <si>
+    <t>31.03.202620</t>
+  </si>
+  <si>
+    <t>31.03.202621</t>
+  </si>
+  <si>
+    <t>31.03.202622</t>
+  </si>
+  <si>
+    <t>31.03.202623</t>
+  </si>
+  <si>
+    <t>31.03.202624</t>
+  </si>
+  <si>
+    <t>01.04.20261</t>
+  </si>
+  <si>
+    <t>01.04.20262</t>
+  </si>
+  <si>
+    <t>01.04.20263</t>
+  </si>
+  <si>
+    <t>01.04.20264</t>
+  </si>
+  <si>
+    <t>01.04.20265</t>
+  </si>
+  <si>
+    <t>01.04.20266</t>
+  </si>
+  <si>
+    <t>01.04.20267</t>
+  </si>
+  <si>
+    <t>01.04.20268</t>
+  </si>
+  <si>
+    <t>01.04.20269</t>
+  </si>
+  <si>
+    <t>01.04.202610</t>
+  </si>
+  <si>
+    <t>01.04.202611</t>
+  </si>
+  <si>
+    <t>01.04.202612</t>
+  </si>
+  <si>
+    <t>01.04.202613</t>
+  </si>
+  <si>
+    <t>01.04.202614</t>
+  </si>
+  <si>
+    <t>01.04.202615</t>
+  </si>
+  <si>
+    <t>01.04.202616</t>
+  </si>
+  <si>
+    <t>01.04.202617</t>
+  </si>
+  <si>
+    <t>01.04.202618</t>
+  </si>
+  <si>
+    <t>01.04.202619</t>
+  </si>
+  <si>
+    <t>01.04.202620</t>
+  </si>
+  <si>
+    <t>01.04.202621</t>
+  </si>
+  <si>
+    <t>01.04.202622</t>
+  </si>
+  <si>
+    <t>01.04.202623</t>
+  </si>
+  <si>
+    <t>01.04.202624</t>
+  </si>
+  <si>
+    <t>02.04.20261</t>
+  </si>
+  <si>
+    <t>02.04.20262</t>
+  </si>
+  <si>
+    <t>02.04.20263</t>
+  </si>
+  <si>
+    <t>02.04.20264</t>
+  </si>
+  <si>
+    <t>02.04.20265</t>
+  </si>
+  <si>
+    <t>02.04.20266</t>
+  </si>
+  <si>
+    <t>02.04.20267</t>
+  </si>
+  <si>
+    <t>02.04.20268</t>
+  </si>
+  <si>
+    <t>02.04.20269</t>
+  </si>
+  <si>
+    <t>02.04.202610</t>
+  </si>
+  <si>
+    <t>02.04.202611</t>
+  </si>
+  <si>
+    <t>02.04.202612</t>
+  </si>
+  <si>
+    <t>02.04.202613</t>
+  </si>
+  <si>
+    <t>02.04.202614</t>
+  </si>
+  <si>
+    <t>02.04.202615</t>
+  </si>
+  <si>
+    <t>02.04.202616</t>
+  </si>
+  <si>
+    <t>02.04.202617</t>
+  </si>
+  <si>
+    <t>02.04.202618</t>
+  </si>
+  <si>
+    <t>02.04.202619</t>
+  </si>
+  <si>
+    <t>02.04.202620</t>
+  </si>
+  <si>
+    <t>02.04.202621</t>
+  </si>
+  <si>
+    <t>02.04.202622</t>
+  </si>
+  <si>
+    <t>02.04.202623</t>
+  </si>
+  <si>
+    <t>02.04.202624</t>
+  </si>
+  <si>
+    <t>03.04.20261</t>
+  </si>
+  <si>
+    <t>03.04.20262</t>
+  </si>
+  <si>
+    <t>03.04.20263</t>
+  </si>
+  <si>
+    <t>03.04.20264</t>
+  </si>
+  <si>
+    <t>03.04.20265</t>
+  </si>
+  <si>
+    <t>03.04.20266</t>
+  </si>
+  <si>
+    <t>03.04.20267</t>
+  </si>
+  <si>
+    <t>03.04.20268</t>
+  </si>
+  <si>
+    <t>03.04.20269</t>
+  </si>
+  <si>
+    <t>03.04.202610</t>
+  </si>
+  <si>
+    <t>03.04.202611</t>
+  </si>
+  <si>
+    <t>03.04.202612</t>
+  </si>
+  <si>
+    <t>03.04.202613</t>
+  </si>
+  <si>
+    <t>03.04.202614</t>
+  </si>
+  <si>
+    <t>03.04.202615</t>
+  </si>
+  <si>
+    <t>03.04.202616</t>
+  </si>
+  <si>
+    <t>03.04.202617</t>
+  </si>
+  <si>
+    <t>03.04.202618</t>
+  </si>
+  <si>
+    <t>03.04.202619</t>
+  </si>
+  <si>
+    <t>03.04.202620</t>
+  </si>
+  <si>
+    <t>03.04.202621</t>
+  </si>
+  <si>
+    <t>03.04.202622</t>
+  </si>
+  <si>
+    <t>03.04.202623</t>
+  </si>
+  <si>
+    <t>03.04.202624</t>
+  </si>
+  <si>
+    <t>04.04.20261</t>
+  </si>
+  <si>
+    <t>04.04.20262</t>
+  </si>
+  <si>
+    <t>04.04.20263</t>
+  </si>
+  <si>
+    <t>04.04.20264</t>
+  </si>
+  <si>
+    <t>04.04.20265</t>
+  </si>
+  <si>
+    <t>04.04.20266</t>
+  </si>
+  <si>
+    <t>04.04.20267</t>
+  </si>
+  <si>
+    <t>04.04.20268</t>
+  </si>
+  <si>
+    <t>04.04.20269</t>
+  </si>
+  <si>
+    <t>04.04.202610</t>
+  </si>
+  <si>
+    <t>04.04.202611</t>
+  </si>
+  <si>
+    <t>04.04.202612</t>
+  </si>
+  <si>
+    <t>04.04.202613</t>
+  </si>
+  <si>
+    <t>04.04.202614</t>
+  </si>
+  <si>
+    <t>04.04.202615</t>
+  </si>
+  <si>
+    <t>04.04.202616</t>
+  </si>
+  <si>
+    <t>04.04.202617</t>
+  </si>
+  <si>
+    <t>04.04.202618</t>
+  </si>
+  <si>
+    <t>04.04.202619</t>
+  </si>
+  <si>
+    <t>04.04.202620</t>
+  </si>
+  <si>
+    <t>04.04.202621</t>
+  </si>
+  <si>
+    <t>04.04.202622</t>
+  </si>
+  <si>
+    <t>04.04.202623</t>
+  </si>
+  <si>
+    <t>04.04.202624</t>
+  </si>
+  <si>
+    <t>05.04.20261</t>
+  </si>
+  <si>
+    <t>05.04.20262</t>
+  </si>
+  <si>
+    <t>05.04.20263</t>
+  </si>
+  <si>
+    <t>05.04.20264</t>
+  </si>
+  <si>
+    <t>05.04.20265</t>
+  </si>
+  <si>
+    <t>05.04.20266</t>
+  </si>
+  <si>
+    <t>05.04.20267</t>
+  </si>
+  <si>
+    <t>05.04.20268</t>
+  </si>
+  <si>
+    <t>05.04.20269</t>
+  </si>
+  <si>
+    <t>05.04.202610</t>
+  </si>
+  <si>
+    <t>05.04.202611</t>
   </si>
 </sst>
 </file>
@@ -913,10 +913,10 @@
     </row>
     <row r="2" spans="1:4">
       <c r="A2" s="2">
-        <v>46098</v>
+        <v>46110</v>
       </c>
       <c r="B2">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="C2">
         <v>0</v>
@@ -927,10 +927,10 @@
     </row>
     <row r="3" spans="1:4">
       <c r="A3" s="2">
-        <v>46098</v>
+        <v>46110</v>
       </c>
       <c r="B3">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="C3">
         <v>0</v>
@@ -941,13 +941,13 @@
     </row>
     <row r="4" spans="1:4">
       <c r="A4" s="2">
-        <v>46098</v>
+        <v>46110</v>
       </c>
       <c r="B4">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="C4">
-        <v>2.792</v>
+        <v>1.259</v>
       </c>
       <c r="D4" t="s">
         <v>6</v>
@@ -955,13 +955,13 @@
     </row>
     <row r="5" spans="1:4">
       <c r="A5" s="2">
-        <v>46098</v>
+        <v>46110</v>
       </c>
       <c r="B5">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="C5">
-        <v>2.664</v>
+        <v>1.111</v>
       </c>
       <c r="D5" t="s">
         <v>7</v>
@@ -969,13 +969,13 @@
     </row>
     <row r="6" spans="1:4">
       <c r="A6" s="2">
-        <v>46098</v>
+        <v>46110</v>
       </c>
       <c r="B6">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="C6">
-        <v>2.792</v>
+        <v>0.904</v>
       </c>
       <c r="D6" t="s">
         <v>8</v>
@@ -983,13 +983,13 @@
     </row>
     <row r="7" spans="1:4">
       <c r="A7" s="2">
-        <v>46098</v>
+        <v>46110</v>
       </c>
       <c r="B7">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="C7">
-        <v>2.674</v>
+        <v>0.586</v>
       </c>
       <c r="D7" t="s">
         <v>9</v>
@@ -997,13 +997,13 @@
     </row>
     <row r="8" spans="1:4">
       <c r="A8" s="2">
-        <v>46098</v>
+        <v>46110</v>
       </c>
       <c r="B8">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="C8">
-        <v>2.399</v>
+        <v>0.465</v>
       </c>
       <c r="D8" t="s">
         <v>10</v>
@@ -1011,13 +1011,13 @@
     </row>
     <row r="9" spans="1:4">
       <c r="A9" s="2">
-        <v>46098</v>
+        <v>46110</v>
       </c>
       <c r="B9">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="C9">
-        <v>1.623</v>
+        <v>0.22</v>
       </c>
       <c r="D9" t="s">
         <v>11</v>
@@ -1025,13 +1025,13 @@
     </row>
     <row r="10" spans="1:4">
       <c r="A10" s="2">
-        <v>46098</v>
+        <v>46110</v>
       </c>
       <c r="B10">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="C10">
-        <v>0.927</v>
+        <v>0.08400000000000001</v>
       </c>
       <c r="D10" t="s">
         <v>12</v>
@@ -1039,13 +1039,13 @@
     </row>
     <row r="11" spans="1:4">
       <c r="A11" s="2">
-        <v>46098</v>
+        <v>46110</v>
       </c>
       <c r="B11">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="C11">
-        <v>0.185</v>
+        <v>0.011</v>
       </c>
       <c r="D11" t="s">
         <v>13</v>
@@ -1053,10 +1053,10 @@
     </row>
     <row r="12" spans="1:4">
       <c r="A12" s="2">
-        <v>46098</v>
+        <v>46110</v>
       </c>
       <c r="B12">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="C12">
         <v>0</v>
@@ -1067,10 +1067,10 @@
     </row>
     <row r="13" spans="1:4">
       <c r="A13" s="2">
-        <v>46098</v>
+        <v>46110</v>
       </c>
       <c r="B13">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="C13">
         <v>0</v>
@@ -1081,10 +1081,10 @@
     </row>
     <row r="14" spans="1:4">
       <c r="A14" s="2">
-        <v>46098</v>
+        <v>46110</v>
       </c>
       <c r="B14">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="C14">
         <v>0</v>
@@ -1095,10 +1095,10 @@
     </row>
     <row r="15" spans="1:4">
       <c r="A15" s="2">
-        <v>46098</v>
+        <v>46110</v>
       </c>
       <c r="B15">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="C15">
         <v>0</v>
@@ -1109,10 +1109,10 @@
     </row>
     <row r="16" spans="1:4">
       <c r="A16" s="2">
-        <v>46098</v>
+        <v>46111</v>
       </c>
       <c r="B16">
-        <v>24</v>
+        <v>1</v>
       </c>
       <c r="C16">
         <v>0</v>
@@ -1123,10 +1123,10 @@
     </row>
     <row r="17" spans="1:4">
       <c r="A17" s="2">
-        <v>46099</v>
+        <v>46111</v>
       </c>
       <c r="B17">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="C17">
         <v>0</v>
@@ -1137,10 +1137,10 @@
     </row>
     <row r="18" spans="1:4">
       <c r="A18" s="2">
-        <v>46099</v>
+        <v>46111</v>
       </c>
       <c r="B18">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="C18">
         <v>0</v>
@@ -1151,10 +1151,10 @@
     </row>
     <row r="19" spans="1:4">
       <c r="A19" s="2">
-        <v>46099</v>
+        <v>46111</v>
       </c>
       <c r="B19">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="C19">
         <v>0</v>
@@ -1165,10 +1165,10 @@
     </row>
     <row r="20" spans="1:4">
       <c r="A20" s="2">
-        <v>46099</v>
+        <v>46111</v>
       </c>
       <c r="B20">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="C20">
         <v>0</v>
@@ -1179,10 +1179,10 @@
     </row>
     <row r="21" spans="1:4">
       <c r="A21" s="2">
-        <v>46099</v>
+        <v>46111</v>
       </c>
       <c r="B21">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="C21">
         <v>0</v>
@@ -1193,10 +1193,10 @@
     </row>
     <row r="22" spans="1:4">
       <c r="A22" s="2">
-        <v>46099</v>
+        <v>46111</v>
       </c>
       <c r="B22">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="C22">
         <v>0</v>
@@ -1207,13 +1207,13 @@
     </row>
     <row r="23" spans="1:4">
       <c r="A23" s="2">
-        <v>46099</v>
+        <v>46111</v>
       </c>
       <c r="B23">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="C23">
-        <v>0</v>
+        <v>0.022</v>
       </c>
       <c r="D23" t="s">
         <v>25</v>
@@ -1221,13 +1221,13 @@
     </row>
     <row r="24" spans="1:4">
       <c r="A24" s="2">
-        <v>46099</v>
+        <v>46111</v>
       </c>
       <c r="B24">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="C24">
-        <v>0</v>
+        <v>0.287</v>
       </c>
       <c r="D24" t="s">
         <v>26</v>
@@ -1235,13 +1235,13 @@
     </row>
     <row r="25" spans="1:4">
       <c r="A25" s="2">
-        <v>46099</v>
+        <v>46111</v>
       </c>
       <c r="B25">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="C25">
-        <v>0.346</v>
+        <v>0.584</v>
       </c>
       <c r="D25" t="s">
         <v>27</v>
@@ -1249,13 +1249,13 @@
     </row>
     <row r="26" spans="1:4">
       <c r="A26" s="2">
-        <v>46099</v>
+        <v>46111</v>
       </c>
       <c r="B26">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="C26">
-        <v>1.107</v>
+        <v>0.895</v>
       </c>
       <c r="D26" t="s">
         <v>28</v>
@@ -1263,13 +1263,13 @@
     </row>
     <row r="27" spans="1:4">
       <c r="A27" s="2">
-        <v>46099</v>
+        <v>46111</v>
       </c>
       <c r="B27">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="C27">
-        <v>1.967</v>
+        <v>1.064</v>
       </c>
       <c r="D27" t="s">
         <v>29</v>
@@ -1277,13 +1277,13 @@
     </row>
     <row r="28" spans="1:4">
       <c r="A28" s="2">
-        <v>46099</v>
+        <v>46111</v>
       </c>
       <c r="B28">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="C28">
-        <v>2.674</v>
+        <v>1.105</v>
       </c>
       <c r="D28" t="s">
         <v>30</v>
@@ -1291,13 +1291,13 @@
     </row>
     <row r="29" spans="1:4">
       <c r="A29" s="2">
-        <v>46099</v>
+        <v>46111</v>
       </c>
       <c r="B29">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="C29">
-        <v>2.783</v>
+        <v>1.218</v>
       </c>
       <c r="D29" t="s">
         <v>31</v>
@@ -1305,13 +1305,13 @@
     </row>
     <row r="30" spans="1:4">
       <c r="A30" s="2">
-        <v>46099</v>
+        <v>46111</v>
       </c>
       <c r="B30">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="C30">
-        <v>2.878</v>
+        <v>1.322</v>
       </c>
       <c r="D30" t="s">
         <v>32</v>
@@ -1319,13 +1319,13 @@
     </row>
     <row r="31" spans="1:4">
       <c r="A31" s="2">
-        <v>46099</v>
+        <v>46111</v>
       </c>
       <c r="B31">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="C31">
-        <v>2.514</v>
+        <v>1.215</v>
       </c>
       <c r="D31" t="s">
         <v>33</v>
@@ -1333,13 +1333,13 @@
     </row>
     <row r="32" spans="1:4">
       <c r="A32" s="2">
-        <v>46099</v>
+        <v>46111</v>
       </c>
       <c r="B32">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="C32">
-        <v>2.297</v>
+        <v>1.011</v>
       </c>
       <c r="D32" t="s">
         <v>34</v>
@@ -1347,13 +1347,13 @@
     </row>
     <row r="33" spans="1:4">
       <c r="A33" s="2">
-        <v>46099</v>
+        <v>46111</v>
       </c>
       <c r="B33">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="C33">
-        <v>1.733</v>
+        <v>0.6</v>
       </c>
       <c r="D33" t="s">
         <v>35</v>
@@ -1361,13 +1361,13 @@
     </row>
     <row r="34" spans="1:4">
       <c r="A34" s="2">
-        <v>46099</v>
+        <v>46111</v>
       </c>
       <c r="B34">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="C34">
-        <v>1.129</v>
+        <v>0.151</v>
       </c>
       <c r="D34" t="s">
         <v>36</v>
@@ -1375,13 +1375,13 @@
     </row>
     <row r="35" spans="1:4">
       <c r="A35" s="2">
-        <v>46099</v>
+        <v>46111</v>
       </c>
       <c r="B35">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="C35">
-        <v>0.3</v>
+        <v>0.025</v>
       </c>
       <c r="D35" t="s">
         <v>37</v>
@@ -1389,13 +1389,13 @@
     </row>
     <row r="36" spans="1:4">
       <c r="A36" s="2">
-        <v>46099</v>
+        <v>46111</v>
       </c>
       <c r="B36">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="C36">
-        <v>0.015</v>
+        <v>0</v>
       </c>
       <c r="D36" t="s">
         <v>38</v>
@@ -1403,10 +1403,10 @@
     </row>
     <row r="37" spans="1:4">
       <c r="A37" s="2">
-        <v>46099</v>
+        <v>46111</v>
       </c>
       <c r="B37">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="C37">
         <v>0</v>
@@ -1417,10 +1417,10 @@
     </row>
     <row r="38" spans="1:4">
       <c r="A38" s="2">
-        <v>46099</v>
+        <v>46111</v>
       </c>
       <c r="B38">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="C38">
         <v>0</v>
@@ -1431,10 +1431,10 @@
     </row>
     <row r="39" spans="1:4">
       <c r="A39" s="2">
-        <v>46099</v>
+        <v>46111</v>
       </c>
       <c r="B39">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="C39">
         <v>0</v>
@@ -1445,10 +1445,10 @@
     </row>
     <row r="40" spans="1:4">
       <c r="A40" s="2">
-        <v>46099</v>
+        <v>46112</v>
       </c>
       <c r="B40">
-        <v>24</v>
+        <v>1</v>
       </c>
       <c r="C40">
         <v>0</v>
@@ -1459,10 +1459,10 @@
     </row>
     <row r="41" spans="1:4">
       <c r="A41" s="2">
-        <v>46100</v>
+        <v>46112</v>
       </c>
       <c r="B41">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="C41">
         <v>0</v>
@@ -1473,10 +1473,10 @@
     </row>
     <row r="42" spans="1:4">
       <c r="A42" s="2">
-        <v>46100</v>
+        <v>46112</v>
       </c>
       <c r="B42">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="C42">
         <v>0</v>
@@ -1487,10 +1487,10 @@
     </row>
     <row r="43" spans="1:4">
       <c r="A43" s="2">
-        <v>46100</v>
+        <v>46112</v>
       </c>
       <c r="B43">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="C43">
         <v>0</v>
@@ -1501,10 +1501,10 @@
     </row>
     <row r="44" spans="1:4">
       <c r="A44" s="2">
-        <v>46100</v>
+        <v>46112</v>
       </c>
       <c r="B44">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="C44">
         <v>0</v>
@@ -1515,10 +1515,10 @@
     </row>
     <row r="45" spans="1:4">
       <c r="A45" s="2">
-        <v>46100</v>
+        <v>46112</v>
       </c>
       <c r="B45">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="C45">
         <v>0</v>
@@ -1529,10 +1529,10 @@
     </row>
     <row r="46" spans="1:4">
       <c r="A46" s="2">
-        <v>46100</v>
+        <v>46112</v>
       </c>
       <c r="B46">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="C46">
         <v>0</v>
@@ -1543,13 +1543,13 @@
     </row>
     <row r="47" spans="1:4">
       <c r="A47" s="2">
-        <v>46100</v>
+        <v>46112</v>
       </c>
       <c r="B47">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="C47">
-        <v>0</v>
+        <v>0.017</v>
       </c>
       <c r="D47" t="s">
         <v>49</v>
@@ -1557,13 +1557,13 @@
     </row>
     <row r="48" spans="1:4">
       <c r="A48" s="2">
-        <v>46100</v>
+        <v>46112</v>
       </c>
       <c r="B48">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="C48">
-        <v>0</v>
+        <v>0.205</v>
       </c>
       <c r="D48" t="s">
         <v>50</v>
@@ -1571,13 +1571,13 @@
     </row>
     <row r="49" spans="1:4">
       <c r="A49" s="2">
-        <v>46100</v>
+        <v>46112</v>
       </c>
       <c r="B49">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="C49">
-        <v>0.312</v>
+        <v>0.383</v>
       </c>
       <c r="D49" t="s">
         <v>51</v>
@@ -1585,13 +1585,13 @@
     </row>
     <row r="50" spans="1:4">
       <c r="A50" s="2">
-        <v>46100</v>
+        <v>46112</v>
       </c>
       <c r="B50">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="C50">
-        <v>0.853</v>
+        <v>0.556</v>
       </c>
       <c r="D50" t="s">
         <v>52</v>
@@ -1599,13 +1599,13 @@
     </row>
     <row r="51" spans="1:4">
       <c r="A51" s="2">
-        <v>46100</v>
+        <v>46112</v>
       </c>
       <c r="B51">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="C51">
-        <v>1.469</v>
+        <v>0.638</v>
       </c>
       <c r="D51" t="s">
         <v>53</v>
@@ -1613,13 +1613,13 @@
     </row>
     <row r="52" spans="1:4">
       <c r="A52" s="2">
-        <v>46100</v>
+        <v>46112</v>
       </c>
       <c r="B52">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="C52">
-        <v>1.788</v>
+        <v>0.834</v>
       </c>
       <c r="D52" t="s">
         <v>54</v>
@@ -1627,13 +1627,13 @@
     </row>
     <row r="53" spans="1:4">
       <c r="A53" s="2">
-        <v>46100</v>
+        <v>46112</v>
       </c>
       <c r="B53">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="C53">
-        <v>1.987</v>
+        <v>0.873</v>
       </c>
       <c r="D53" t="s">
         <v>55</v>
@@ -1641,13 +1641,13 @@
     </row>
     <row r="54" spans="1:4">
       <c r="A54" s="2">
-        <v>46100</v>
+        <v>46112</v>
       </c>
       <c r="B54">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="C54">
-        <v>2.032</v>
+        <v>0.826</v>
       </c>
       <c r="D54" t="s">
         <v>56</v>
@@ -1655,13 +1655,13 @@
     </row>
     <row r="55" spans="1:4">
       <c r="A55" s="2">
-        <v>46100</v>
+        <v>46112</v>
       </c>
       <c r="B55">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="C55">
-        <v>1.982</v>
+        <v>0.706</v>
       </c>
       <c r="D55" t="s">
         <v>57</v>
@@ -1669,13 +1669,13 @@
     </row>
     <row r="56" spans="1:4">
       <c r="A56" s="2">
-        <v>46100</v>
+        <v>46112</v>
       </c>
       <c r="B56">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="C56">
-        <v>1.603</v>
+        <v>0.532</v>
       </c>
       <c r="D56" t="s">
         <v>58</v>
@@ -1683,13 +1683,13 @@
     </row>
     <row r="57" spans="1:4">
       <c r="A57" s="2">
-        <v>46100</v>
+        <v>46112</v>
       </c>
       <c r="B57">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="C57">
-        <v>1.224</v>
+        <v>0.316</v>
       </c>
       <c r="D57" t="s">
         <v>59</v>
@@ -1697,13 +1697,13 @@
     </row>
     <row r="58" spans="1:4">
       <c r="A58" s="2">
-        <v>46100</v>
+        <v>46112</v>
       </c>
       <c r="B58">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="C58">
-        <v>0.706</v>
+        <v>0.115</v>
       </c>
       <c r="D58" t="s">
         <v>60</v>
@@ -1711,13 +1711,13 @@
     </row>
     <row r="59" spans="1:4">
       <c r="A59" s="2">
-        <v>46100</v>
+        <v>46112</v>
       </c>
       <c r="B59">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="C59">
-        <v>0.19</v>
+        <v>0.012</v>
       </c>
       <c r="D59" t="s">
         <v>61</v>
@@ -1725,13 +1725,13 @@
     </row>
     <row r="60" spans="1:4">
       <c r="A60" s="2">
-        <v>46100</v>
+        <v>46112</v>
       </c>
       <c r="B60">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="C60">
-        <v>0.013</v>
+        <v>0</v>
       </c>
       <c r="D60" t="s">
         <v>62</v>
@@ -1739,10 +1739,10 @@
     </row>
     <row r="61" spans="1:4">
       <c r="A61" s="2">
-        <v>46100</v>
+        <v>46112</v>
       </c>
       <c r="B61">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="C61">
         <v>0</v>
@@ -1753,10 +1753,10 @@
     </row>
     <row r="62" spans="1:4">
       <c r="A62" s="2">
-        <v>46100</v>
+        <v>46112</v>
       </c>
       <c r="B62">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="C62">
         <v>0</v>
@@ -1767,10 +1767,10 @@
     </row>
     <row r="63" spans="1:4">
       <c r="A63" s="2">
-        <v>46100</v>
+        <v>46112</v>
       </c>
       <c r="B63">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="C63">
         <v>0</v>
@@ -1781,10 +1781,10 @@
     </row>
     <row r="64" spans="1:4">
       <c r="A64" s="2">
-        <v>46100</v>
+        <v>46113</v>
       </c>
       <c r="B64">
-        <v>24</v>
+        <v>1</v>
       </c>
       <c r="C64">
         <v>0</v>
@@ -1795,10 +1795,10 @@
     </row>
     <row r="65" spans="1:4">
       <c r="A65" s="2">
-        <v>46101</v>
+        <v>46113</v>
       </c>
       <c r="B65">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="C65">
         <v>0</v>
@@ -1809,10 +1809,10 @@
     </row>
     <row r="66" spans="1:4">
       <c r="A66" s="2">
-        <v>46101</v>
+        <v>46113</v>
       </c>
       <c r="B66">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="C66">
         <v>0</v>
@@ -1823,10 +1823,10 @@
     </row>
     <row r="67" spans="1:4">
       <c r="A67" s="2">
-        <v>46101</v>
+        <v>46113</v>
       </c>
       <c r="B67">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="C67">
         <v>0</v>
@@ -1837,10 +1837,10 @@
     </row>
     <row r="68" spans="1:4">
       <c r="A68" s="2">
-        <v>46101</v>
+        <v>46113</v>
       </c>
       <c r="B68">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="C68">
         <v>0</v>
@@ -1851,10 +1851,10 @@
     </row>
     <row r="69" spans="1:4">
       <c r="A69" s="2">
-        <v>46101</v>
+        <v>46113</v>
       </c>
       <c r="B69">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="C69">
         <v>0</v>
@@ -1865,10 +1865,10 @@
     </row>
     <row r="70" spans="1:4">
       <c r="A70" s="2">
-        <v>46101</v>
+        <v>46113</v>
       </c>
       <c r="B70">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="C70">
         <v>0</v>
@@ -1879,13 +1879,13 @@
     </row>
     <row r="71" spans="1:4">
       <c r="A71" s="2">
-        <v>46101</v>
+        <v>46113</v>
       </c>
       <c r="B71">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="C71">
-        <v>0</v>
+        <v>0.046</v>
       </c>
       <c r="D71" t="s">
         <v>73</v>
@@ -1893,13 +1893,13 @@
     </row>
     <row r="72" spans="1:4">
       <c r="A72" s="2">
-        <v>46101</v>
+        <v>46113</v>
       </c>
       <c r="B72">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="C72">
-        <v>0</v>
+        <v>0.529</v>
       </c>
       <c r="D72" t="s">
         <v>74</v>
@@ -1907,13 +1907,13 @@
     </row>
     <row r="73" spans="1:4">
       <c r="A73" s="2">
-        <v>46101</v>
+        <v>46113</v>
       </c>
       <c r="B73">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="C73">
-        <v>0.219</v>
+        <v>0.907</v>
       </c>
       <c r="D73" t="s">
         <v>75</v>
@@ -1921,13 +1921,13 @@
     </row>
     <row r="74" spans="1:4">
       <c r="A74" s="2">
-        <v>46101</v>
+        <v>46113</v>
       </c>
       <c r="B74">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="C74">
-        <v>0.678</v>
+        <v>1.499</v>
       </c>
       <c r="D74" t="s">
         <v>76</v>
@@ -1935,13 +1935,13 @@
     </row>
     <row r="75" spans="1:4">
       <c r="A75" s="2">
-        <v>46101</v>
+        <v>46113</v>
       </c>
       <c r="B75">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="C75">
-        <v>1.056</v>
+        <v>1.899</v>
       </c>
       <c r="D75" t="s">
         <v>77</v>
@@ -1949,13 +1949,13 @@
     </row>
     <row r="76" spans="1:4">
       <c r="A76" s="2">
-        <v>46101</v>
+        <v>46113</v>
       </c>
       <c r="B76">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="C76">
-        <v>1.524</v>
+        <v>1.953</v>
       </c>
       <c r="D76" t="s">
         <v>78</v>
@@ -1963,13 +1963,13 @@
     </row>
     <row r="77" spans="1:4">
       <c r="A77" s="2">
-        <v>46101</v>
+        <v>46113</v>
       </c>
       <c r="B77">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="C77">
-        <v>1.794</v>
+        <v>1.976</v>
       </c>
       <c r="D77" t="s">
         <v>79</v>
@@ -1977,13 +1977,13 @@
     </row>
     <row r="78" spans="1:4">
       <c r="A78" s="2">
-        <v>46101</v>
+        <v>46113</v>
       </c>
       <c r="B78">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="C78">
-        <v>1.794</v>
+        <v>1.94</v>
       </c>
       <c r="D78" t="s">
         <v>80</v>
@@ -1991,13 +1991,13 @@
     </row>
     <row r="79" spans="1:4">
       <c r="A79" s="2">
-        <v>46101</v>
+        <v>46113</v>
       </c>
       <c r="B79">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="C79">
-        <v>1.616</v>
+        <v>1.632</v>
       </c>
       <c r="D79" t="s">
         <v>81</v>
@@ -2005,13 +2005,13 @@
     </row>
     <row r="80" spans="1:4">
       <c r="A80" s="2">
-        <v>46101</v>
+        <v>46113</v>
       </c>
       <c r="B80">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="C80">
-        <v>1.35</v>
+        <v>1.179</v>
       </c>
       <c r="D80" t="s">
         <v>82</v>
@@ -2019,13 +2019,13 @@
     </row>
     <row r="81" spans="1:4">
       <c r="A81" s="2">
-        <v>46101</v>
+        <v>46113</v>
       </c>
       <c r="B81">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="C81">
-        <v>0.967</v>
+        <v>0.6889999999999999</v>
       </c>
       <c r="D81" t="s">
         <v>83</v>
@@ -2033,13 +2033,13 @@
     </row>
     <row r="82" spans="1:4">
       <c r="A82" s="2">
-        <v>46101</v>
+        <v>46113</v>
       </c>
       <c r="B82">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="C82">
-        <v>0.456</v>
+        <v>0.275</v>
       </c>
       <c r="D82" t="s">
         <v>84</v>
@@ -2047,13 +2047,13 @@
     </row>
     <row r="83" spans="1:4">
       <c r="A83" s="2">
-        <v>46101</v>
+        <v>46113</v>
       </c>
       <c r="B83">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="C83">
-        <v>0.123</v>
+        <v>0.024</v>
       </c>
       <c r="D83" t="s">
         <v>85</v>
@@ -2061,10 +2061,10 @@
     </row>
     <row r="84" spans="1:4">
       <c r="A84" s="2">
-        <v>46101</v>
+        <v>46113</v>
       </c>
       <c r="B84">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="C84">
         <v>0</v>
@@ -2075,10 +2075,10 @@
     </row>
     <row r="85" spans="1:4">
       <c r="A85" s="2">
-        <v>46101</v>
+        <v>46113</v>
       </c>
       <c r="B85">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="C85">
         <v>0</v>
@@ -2089,10 +2089,10 @@
     </row>
     <row r="86" spans="1:4">
       <c r="A86" s="2">
-        <v>46101</v>
+        <v>46113</v>
       </c>
       <c r="B86">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="C86">
         <v>0</v>
@@ -2103,10 +2103,10 @@
     </row>
     <row r="87" spans="1:4">
       <c r="A87" s="2">
-        <v>46101</v>
+        <v>46113</v>
       </c>
       <c r="B87">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="C87">
         <v>0</v>
@@ -2117,10 +2117,10 @@
     </row>
     <row r="88" spans="1:4">
       <c r="A88" s="2">
-        <v>46101</v>
+        <v>46114</v>
       </c>
       <c r="B88">
-        <v>24</v>
+        <v>1</v>
       </c>
       <c r="C88">
         <v>0</v>
@@ -2131,10 +2131,10 @@
     </row>
     <row r="89" spans="1:4">
       <c r="A89" s="2">
-        <v>46102</v>
+        <v>46114</v>
       </c>
       <c r="B89">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="C89">
         <v>0</v>
@@ -2145,10 +2145,10 @@
     </row>
     <row r="90" spans="1:4">
       <c r="A90" s="2">
-        <v>46102</v>
+        <v>46114</v>
       </c>
       <c r="B90">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="C90">
         <v>0</v>
@@ -2159,10 +2159,10 @@
     </row>
     <row r="91" spans="1:4">
       <c r="A91" s="2">
-        <v>46102</v>
+        <v>46114</v>
       </c>
       <c r="B91">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="C91">
         <v>0</v>
@@ -2173,10 +2173,10 @@
     </row>
     <row r="92" spans="1:4">
       <c r="A92" s="2">
-        <v>46102</v>
+        <v>46114</v>
       </c>
       <c r="B92">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="C92">
         <v>0</v>
@@ -2187,10 +2187,10 @@
     </row>
     <row r="93" spans="1:4">
       <c r="A93" s="2">
-        <v>46102</v>
+        <v>46114</v>
       </c>
       <c r="B93">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="C93">
         <v>0</v>
@@ -2201,10 +2201,10 @@
     </row>
     <row r="94" spans="1:4">
       <c r="A94" s="2">
-        <v>46102</v>
+        <v>46114</v>
       </c>
       <c r="B94">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="C94">
         <v>0</v>
@@ -2215,13 +2215,13 @@
     </row>
     <row r="95" spans="1:4">
       <c r="A95" s="2">
-        <v>46102</v>
+        <v>46114</v>
       </c>
       <c r="B95">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="C95">
-        <v>0</v>
+        <v>0.048</v>
       </c>
       <c r="D95" t="s">
         <v>97</v>
@@ -2229,13 +2229,13 @@
     </row>
     <row r="96" spans="1:4">
       <c r="A96" s="2">
-        <v>46102</v>
+        <v>46114</v>
       </c>
       <c r="B96">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="C96">
-        <v>0</v>
+        <v>0.538</v>
       </c>
       <c r="D96" t="s">
         <v>98</v>
@@ -2243,13 +2243,13 @@
     </row>
     <row r="97" spans="1:4">
       <c r="A97" s="2">
-        <v>46102</v>
+        <v>46114</v>
       </c>
       <c r="B97">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="C97">
-        <v>0.299</v>
+        <v>1.169</v>
       </c>
       <c r="D97" t="s">
         <v>99</v>
@@ -2257,13 +2257,13 @@
     </row>
     <row r="98" spans="1:4">
       <c r="A98" s="2">
-        <v>46102</v>
+        <v>46114</v>
       </c>
       <c r="B98">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="C98">
-        <v>0.928</v>
+        <v>1.935</v>
       </c>
       <c r="D98" t="s">
         <v>100</v>
@@ -2271,13 +2271,13 @@
     </row>
     <row r="99" spans="1:4">
       <c r="A99" s="2">
-        <v>46102</v>
+        <v>46114</v>
       </c>
       <c r="B99">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="C99">
-        <v>1.485</v>
+        <v>2.526</v>
       </c>
       <c r="D99" t="s">
         <v>101</v>
@@ -2285,13 +2285,13 @@
     </row>
     <row r="100" spans="1:4">
       <c r="A100" s="2">
-        <v>46102</v>
+        <v>46114</v>
       </c>
       <c r="B100">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="C100">
-        <v>1.937</v>
+        <v>2.525</v>
       </c>
       <c r="D100" t="s">
         <v>102</v>
@@ -2299,13 +2299,13 @@
     </row>
     <row r="101" spans="1:4">
       <c r="A101" s="2">
-        <v>46102</v>
+        <v>46114</v>
       </c>
       <c r="B101">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="C101">
-        <v>2.054</v>
+        <v>2.458</v>
       </c>
       <c r="D101" t="s">
         <v>103</v>
@@ -2313,13 +2313,13 @@
     </row>
     <row r="102" spans="1:4">
       <c r="A102" s="2">
-        <v>46102</v>
+        <v>46114</v>
       </c>
       <c r="B102">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="C102">
-        <v>2.038</v>
+        <v>2.194</v>
       </c>
       <c r="D102" t="s">
         <v>104</v>
@@ -2327,13 +2327,13 @@
     </row>
     <row r="103" spans="1:4">
       <c r="A103" s="2">
-        <v>46102</v>
+        <v>46114</v>
       </c>
       <c r="B103">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="C103">
-        <v>1.949</v>
+        <v>1.894</v>
       </c>
       <c r="D103" t="s">
         <v>105</v>
@@ -2341,13 +2341,13 @@
     </row>
     <row r="104" spans="1:4">
       <c r="A104" s="2">
-        <v>46102</v>
+        <v>46114</v>
       </c>
       <c r="B104">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="C104">
-        <v>1.771</v>
+        <v>1.479</v>
       </c>
       <c r="D104" t="s">
         <v>106</v>
@@ -2355,13 +2355,13 @@
     </row>
     <row r="105" spans="1:4">
       <c r="A105" s="2">
-        <v>46102</v>
+        <v>46114</v>
       </c>
       <c r="B105">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="C105">
-        <v>1.508</v>
+        <v>0.765</v>
       </c>
       <c r="D105" t="s">
         <v>107</v>
@@ -2369,13 +2369,13 @@
     </row>
     <row r="106" spans="1:4">
       <c r="A106" s="2">
-        <v>46102</v>
+        <v>46114</v>
       </c>
       <c r="B106">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="C106">
-        <v>0.927</v>
+        <v>0.278</v>
       </c>
       <c r="D106" t="s">
         <v>108</v>
@@ -2383,13 +2383,13 @@
     </row>
     <row r="107" spans="1:4">
       <c r="A107" s="2">
-        <v>46102</v>
+        <v>46114</v>
       </c>
       <c r="B107">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="C107">
-        <v>0.289</v>
+        <v>0.023</v>
       </c>
       <c r="D107" t="s">
         <v>109</v>
@@ -2397,13 +2397,13 @@
     </row>
     <row r="108" spans="1:4">
       <c r="A108" s="2">
-        <v>46102</v>
+        <v>46114</v>
       </c>
       <c r="B108">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="C108">
-        <v>0.017</v>
+        <v>0</v>
       </c>
       <c r="D108" t="s">
         <v>110</v>
@@ -2411,10 +2411,10 @@
     </row>
     <row r="109" spans="1:4">
       <c r="A109" s="2">
-        <v>46102</v>
+        <v>46114</v>
       </c>
       <c r="B109">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="C109">
         <v>0</v>
@@ -2425,10 +2425,10 @@
     </row>
     <row r="110" spans="1:4">
       <c r="A110" s="2">
-        <v>46102</v>
+        <v>46114</v>
       </c>
       <c r="B110">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="C110">
         <v>0</v>
@@ -2439,10 +2439,10 @@
     </row>
     <row r="111" spans="1:4">
       <c r="A111" s="2">
-        <v>46102</v>
+        <v>46114</v>
       </c>
       <c r="B111">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="C111">
         <v>0</v>
@@ -2453,10 +2453,10 @@
     </row>
     <row r="112" spans="1:4">
       <c r="A112" s="2">
-        <v>46102</v>
+        <v>46115</v>
       </c>
       <c r="B112">
-        <v>24</v>
+        <v>1</v>
       </c>
       <c r="C112">
         <v>0</v>
@@ -2467,10 +2467,10 @@
     </row>
     <row r="113" spans="1:4">
       <c r="A113" s="2">
-        <v>46103</v>
+        <v>46115</v>
       </c>
       <c r="B113">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="C113">
         <v>0</v>
@@ -2481,10 +2481,10 @@
     </row>
     <row r="114" spans="1:4">
       <c r="A114" s="2">
-        <v>46103</v>
+        <v>46115</v>
       </c>
       <c r="B114">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="C114">
         <v>0</v>
@@ -2495,10 +2495,10 @@
     </row>
     <row r="115" spans="1:4">
       <c r="A115" s="2">
-        <v>46103</v>
+        <v>46115</v>
       </c>
       <c r="B115">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="C115">
         <v>0</v>
@@ -2509,10 +2509,10 @@
     </row>
     <row r="116" spans="1:4">
       <c r="A116" s="2">
-        <v>46103</v>
+        <v>46115</v>
       </c>
       <c r="B116">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="C116">
         <v>0</v>
@@ -2523,10 +2523,10 @@
     </row>
     <row r="117" spans="1:4">
       <c r="A117" s="2">
-        <v>46103</v>
+        <v>46115</v>
       </c>
       <c r="B117">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="C117">
         <v>0</v>
@@ -2537,10 +2537,10 @@
     </row>
     <row r="118" spans="1:4">
       <c r="A118" s="2">
-        <v>46103</v>
+        <v>46115</v>
       </c>
       <c r="B118">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="C118">
         <v>0</v>
@@ -2551,13 +2551,13 @@
     </row>
     <row r="119" spans="1:4">
       <c r="A119" s="2">
-        <v>46103</v>
+        <v>46115</v>
       </c>
       <c r="B119">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="C119">
-        <v>0</v>
+        <v>0.032</v>
       </c>
       <c r="D119" t="s">
         <v>121</v>
@@ -2565,13 +2565,13 @@
     </row>
     <row r="120" spans="1:4">
       <c r="A120" s="2">
-        <v>46103</v>
+        <v>46115</v>
       </c>
       <c r="B120">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="C120">
-        <v>0.012</v>
+        <v>0.431</v>
       </c>
       <c r="D120" t="s">
         <v>122</v>
@@ -2579,13 +2579,13 @@
     </row>
     <row r="121" spans="1:4">
       <c r="A121" s="2">
-        <v>46103</v>
+        <v>46115</v>
       </c>
       <c r="B121">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="C121">
-        <v>0.306</v>
+        <v>0.89</v>
       </c>
       <c r="D121" t="s">
         <v>123</v>
@@ -2593,13 +2593,13 @@
     </row>
     <row r="122" spans="1:4">
       <c r="A122" s="2">
-        <v>46103</v>
+        <v>46115</v>
       </c>
       <c r="B122">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="C122">
-        <v>0.918</v>
+        <v>1.208</v>
       </c>
       <c r="D122" t="s">
         <v>124</v>
@@ -2607,13 +2607,13 @@
     </row>
     <row r="123" spans="1:4">
       <c r="A123" s="2">
-        <v>46103</v>
+        <v>46115</v>
       </c>
       <c r="B123">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="C123">
-        <v>1.318</v>
+        <v>1.685</v>
       </c>
       <c r="D123" t="s">
         <v>125</v>
@@ -2621,13 +2621,13 @@
     </row>
     <row r="124" spans="1:4">
       <c r="A124" s="2">
-        <v>46103</v>
+        <v>46115</v>
       </c>
       <c r="B124">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="C124">
-        <v>1.712</v>
+        <v>1.947</v>
       </c>
       <c r="D124" t="s">
         <v>126</v>
@@ -2635,13 +2635,13 @@
     </row>
     <row r="125" spans="1:4">
       <c r="A125" s="2">
-        <v>46103</v>
+        <v>46115</v>
       </c>
       <c r="B125">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="C125">
-        <v>1.945</v>
+        <v>1.922</v>
       </c>
       <c r="D125" t="s">
         <v>127</v>
@@ -2649,13 +2649,13 @@
     </row>
     <row r="126" spans="1:4">
       <c r="A126" s="2">
-        <v>46103</v>
+        <v>46115</v>
       </c>
       <c r="B126">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="C126">
-        <v>1.996</v>
+        <v>1.819</v>
       </c>
       <c r="D126" t="s">
         <v>128</v>
@@ -2663,13 +2663,13 @@
     </row>
     <row r="127" spans="1:4">
       <c r="A127" s="2">
-        <v>46103</v>
+        <v>46115</v>
       </c>
       <c r="B127">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="C127">
-        <v>1.906</v>
+        <v>1.566</v>
       </c>
       <c r="D127" t="s">
         <v>129</v>
@@ -2677,13 +2677,13 @@
     </row>
     <row r="128" spans="1:4">
       <c r="A128" s="2">
-        <v>46103</v>
+        <v>46115</v>
       </c>
       <c r="B128">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="C128">
-        <v>1.646</v>
+        <v>1.34</v>
       </c>
       <c r="D128" t="s">
         <v>130</v>
@@ -2691,13 +2691,13 @@
     </row>
     <row r="129" spans="1:4">
       <c r="A129" s="2">
-        <v>46103</v>
+        <v>46115</v>
       </c>
       <c r="B129">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="C129">
-        <v>1.134</v>
+        <v>0.788</v>
       </c>
       <c r="D129" t="s">
         <v>131</v>
@@ -2705,13 +2705,13 @@
     </row>
     <row r="130" spans="1:4">
       <c r="A130" s="2">
-        <v>46103</v>
+        <v>46115</v>
       </c>
       <c r="B130">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="C130">
-        <v>0.595</v>
+        <v>0.29</v>
       </c>
       <c r="D130" t="s">
         <v>132</v>
@@ -2719,13 +2719,13 @@
     </row>
     <row r="131" spans="1:4">
       <c r="A131" s="2">
-        <v>46103</v>
+        <v>46115</v>
       </c>
       <c r="B131">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="C131">
-        <v>0.139</v>
+        <v>0.026</v>
       </c>
       <c r="D131" t="s">
         <v>133</v>
@@ -2733,13 +2733,13 @@
     </row>
     <row r="132" spans="1:4">
       <c r="A132" s="2">
-        <v>46103</v>
+        <v>46115</v>
       </c>
       <c r="B132">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="C132">
-        <v>0.012</v>
+        <v>0</v>
       </c>
       <c r="D132" t="s">
         <v>134</v>
@@ -2747,10 +2747,10 @@
     </row>
     <row r="133" spans="1:4">
       <c r="A133" s="2">
-        <v>46103</v>
+        <v>46115</v>
       </c>
       <c r="B133">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="C133">
         <v>0</v>
@@ -2761,10 +2761,10 @@
     </row>
     <row r="134" spans="1:4">
       <c r="A134" s="2">
-        <v>46103</v>
+        <v>46115</v>
       </c>
       <c r="B134">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="C134">
         <v>0</v>
@@ -2775,10 +2775,10 @@
     </row>
     <row r="135" spans="1:4">
       <c r="A135" s="2">
-        <v>46103</v>
+        <v>46115</v>
       </c>
       <c r="B135">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="C135">
         <v>0</v>
@@ -2789,10 +2789,10 @@
     </row>
     <row r="136" spans="1:4">
       <c r="A136" s="2">
-        <v>46103</v>
+        <v>46116</v>
       </c>
       <c r="B136">
-        <v>24</v>
+        <v>1</v>
       </c>
       <c r="C136">
         <v>0</v>
@@ -2803,10 +2803,10 @@
     </row>
     <row r="137" spans="1:4">
       <c r="A137" s="2">
-        <v>46104</v>
+        <v>46116</v>
       </c>
       <c r="B137">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="C137">
         <v>0</v>
@@ -2817,10 +2817,10 @@
     </row>
     <row r="138" spans="1:4">
       <c r="A138" s="2">
-        <v>46104</v>
+        <v>46116</v>
       </c>
       <c r="B138">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="C138">
         <v>0</v>
@@ -2831,10 +2831,10 @@
     </row>
     <row r="139" spans="1:4">
       <c r="A139" s="2">
-        <v>46104</v>
+        <v>46116</v>
       </c>
       <c r="B139">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="C139">
         <v>0</v>
@@ -2845,10 +2845,10 @@
     </row>
     <row r="140" spans="1:4">
       <c r="A140" s="2">
-        <v>46104</v>
+        <v>46116</v>
       </c>
       <c r="B140">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="C140">
         <v>0</v>
@@ -2859,10 +2859,10 @@
     </row>
     <row r="141" spans="1:4">
       <c r="A141" s="2">
-        <v>46104</v>
+        <v>46116</v>
       </c>
       <c r="B141">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="C141">
         <v>0</v>
@@ -2873,10 +2873,10 @@
     </row>
     <row r="142" spans="1:4">
       <c r="A142" s="2">
-        <v>46104</v>
+        <v>46116</v>
       </c>
       <c r="B142">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="C142">
         <v>0</v>
@@ -2887,13 +2887,13 @@
     </row>
     <row r="143" spans="1:4">
       <c r="A143" s="2">
-        <v>46104</v>
+        <v>46116</v>
       </c>
       <c r="B143">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="C143">
-        <v>0</v>
+        <v>0.036</v>
       </c>
       <c r="D143" t="s">
         <v>145</v>
@@ -2901,13 +2901,13 @@
     </row>
     <row r="144" spans="1:4">
       <c r="A144" s="2">
-        <v>46104</v>
+        <v>46116</v>
       </c>
       <c r="B144">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="C144">
-        <v>0</v>
+        <v>0.468</v>
       </c>
       <c r="D144" t="s">
         <v>146</v>
@@ -2915,13 +2915,13 @@
     </row>
     <row r="145" spans="1:4">
       <c r="A145" s="2">
-        <v>46104</v>
+        <v>46116</v>
       </c>
       <c r="B145">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="C145">
-        <v>0.226</v>
+        <v>0.915</v>
       </c>
       <c r="D145" t="s">
         <v>147</v>
@@ -2929,13 +2929,13 @@
     </row>
     <row r="146" spans="1:4">
       <c r="A146" s="2">
-        <v>46104</v>
+        <v>46116</v>
       </c>
       <c r="B146">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="C146">
-        <v>0.753</v>
+        <v>1.451</v>
       </c>
       <c r="D146" t="s">
         <v>148</v>
@@ -2943,13 +2943,13 @@
     </row>
     <row r="147" spans="1:4">
       <c r="A147" s="2">
-        <v>46104</v>
+        <v>46116</v>
       </c>
       <c r="B147">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="C147">
-        <v>1.097</v>
+        <v>1.853</v>
       </c>
       <c r="D147" t="s">
         <v>149</v>
@@ -2957,13 +2957,13 @@
     </row>
     <row r="148" spans="1:4">
       <c r="A148" s="2">
-        <v>46104</v>
+        <v>46116</v>
       </c>
       <c r="B148">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="C148">
-        <v>1.587</v>
+        <v>1.975</v>
       </c>
       <c r="D148" t="s">
         <v>150</v>
@@ -2971,13 +2971,13 @@
     </row>
     <row r="149" spans="1:4">
       <c r="A149" s="2">
-        <v>46104</v>
+        <v>46116</v>
       </c>
       <c r="B149">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="C149">
-        <v>1.893</v>
+        <v>1.965</v>
       </c>
       <c r="D149" t="s">
         <v>151</v>
@@ -2985,13 +2985,13 @@
     </row>
     <row r="150" spans="1:4">
       <c r="A150" s="2">
-        <v>46104</v>
+        <v>46116</v>
       </c>
       <c r="B150">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="C150">
-        <v>1.962</v>
+        <v>1.961</v>
       </c>
       <c r="D150" t="s">
         <v>152</v>
@@ -2999,13 +2999,13 @@
     </row>
     <row r="151" spans="1:4">
       <c r="A151" s="2">
-        <v>46104</v>
+        <v>46116</v>
       </c>
       <c r="B151">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="C151">
-        <v>1.96</v>
+        <v>1.809</v>
       </c>
       <c r="D151" t="s">
         <v>153</v>
@@ -3013,13 +3013,13 @@
     </row>
     <row r="152" spans="1:4">
       <c r="A152" s="2">
-        <v>46104</v>
+        <v>46116</v>
       </c>
       <c r="B152">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="C152">
-        <v>1.774</v>
+        <v>1.395</v>
       </c>
       <c r="D152" t="s">
         <v>154</v>
@@ -3027,13 +3027,13 @@
     </row>
     <row r="153" spans="1:4">
       <c r="A153" s="2">
-        <v>46104</v>
+        <v>46116</v>
       </c>
       <c r="B153">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="C153">
-        <v>1.313</v>
+        <v>0.8159999999999999</v>
       </c>
       <c r="D153" t="s">
         <v>155</v>
@@ -3041,13 +3041,13 @@
     </row>
     <row r="154" spans="1:4">
       <c r="A154" s="2">
-        <v>46104</v>
+        <v>46116</v>
       </c>
       <c r="B154">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="C154">
-        <v>0.705</v>
+        <v>0.285</v>
       </c>
       <c r="D154" t="s">
         <v>156</v>
@@ -3055,13 +3055,13 @@
     </row>
     <row r="155" spans="1:4">
       <c r="A155" s="2">
-        <v>46104</v>
+        <v>46116</v>
       </c>
       <c r="B155">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="C155">
-        <v>0.205</v>
+        <v>0.025</v>
       </c>
       <c r="D155" t="s">
         <v>157</v>
@@ -3069,13 +3069,13 @@
     </row>
     <row r="156" spans="1:4">
       <c r="A156" s="2">
-        <v>46104</v>
+        <v>46116</v>
       </c>
       <c r="B156">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="C156">
-        <v>0.013</v>
+        <v>0</v>
       </c>
       <c r="D156" t="s">
         <v>158</v>
@@ -3083,10 +3083,10 @@
     </row>
     <row r="157" spans="1:4">
       <c r="A157" s="2">
-        <v>46104</v>
+        <v>46116</v>
       </c>
       <c r="B157">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="C157">
         <v>0</v>
@@ -3097,10 +3097,10 @@
     </row>
     <row r="158" spans="1:4">
       <c r="A158" s="2">
-        <v>46104</v>
+        <v>46116</v>
       </c>
       <c r="B158">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="C158">
         <v>0</v>
@@ -3111,10 +3111,10 @@
     </row>
     <row r="159" spans="1:4">
       <c r="A159" s="2">
-        <v>46104</v>
+        <v>46116</v>
       </c>
       <c r="B159">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="C159">
         <v>0</v>
@@ -3125,10 +3125,10 @@
     </row>
     <row r="160" spans="1:4">
       <c r="A160" s="2">
-        <v>46104</v>
+        <v>46117</v>
       </c>
       <c r="B160">
-        <v>24</v>
+        <v>1</v>
       </c>
       <c r="C160">
         <v>0</v>
@@ -3139,10 +3139,10 @@
     </row>
     <row r="161" spans="1:4">
       <c r="A161" s="2">
-        <v>46105</v>
+        <v>46117</v>
       </c>
       <c r="B161">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="C161">
         <v>0</v>
@@ -3153,10 +3153,10 @@
     </row>
     <row r="162" spans="1:4">
       <c r="A162" s="2">
-        <v>46105</v>
+        <v>46117</v>
       </c>
       <c r="B162">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="C162">
         <v>0</v>
@@ -3167,10 +3167,10 @@
     </row>
     <row r="163" spans="1:4">
       <c r="A163" s="2">
-        <v>46105</v>
+        <v>46117</v>
       </c>
       <c r="B163">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="C163">
         <v>0</v>
@@ -3181,10 +3181,10 @@
     </row>
     <row r="164" spans="1:4">
       <c r="A164" s="2">
-        <v>46105</v>
+        <v>46117</v>
       </c>
       <c r="B164">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="C164">
         <v>0</v>
@@ -3195,10 +3195,10 @@
     </row>
     <row r="165" spans="1:4">
       <c r="A165" s="2">
-        <v>46105</v>
+        <v>46117</v>
       </c>
       <c r="B165">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="C165">
         <v>0</v>
@@ -3209,10 +3209,10 @@
     </row>
     <row r="166" spans="1:4">
       <c r="A166" s="2">
-        <v>46105</v>
+        <v>46117</v>
       </c>
       <c r="B166">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="C166">
         <v>0</v>
@@ -3223,13 +3223,13 @@
     </row>
     <row r="167" spans="1:4">
       <c r="A167" s="2">
-        <v>46105</v>
+        <v>46117</v>
       </c>
       <c r="B167">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="C167">
-        <v>0</v>
+        <v>0.037</v>
       </c>
       <c r="D167" t="s">
         <v>169</v>
@@ -3237,13 +3237,13 @@
     </row>
     <row r="168" spans="1:4">
       <c r="A168" s="2">
-        <v>46105</v>
+        <v>46117</v>
       </c>
       <c r="B168">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="C168">
-        <v>0.016</v>
+        <v>0.375</v>
       </c>
       <c r="D168" t="s">
         <v>170</v>
@@ -3251,13 +3251,13 @@
     </row>
     <row r="169" spans="1:4">
       <c r="A169" s="2">
-        <v>46105</v>
+        <v>46117</v>
       </c>
       <c r="B169">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="C169">
-        <v>0.361</v>
+        <v>0.857</v>
       </c>
       <c r="D169" t="s">
         <v>171</v>
@@ -3265,13 +3265,13 @@
     </row>
     <row r="170" spans="1:4">
       <c r="A170" s="2">
-        <v>46105</v>
+        <v>46117</v>
       </c>
       <c r="B170">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="C170">
-        <v>0.914</v>
+        <v>1.012</v>
       </c>
       <c r="D170" t="s">
         <v>172</v>

</xml_diff>

<commit_message>
Adding Anto to the portfolio
</commit_message>
<xml_diff>
--- a/Astro/Results_Production_Astro_xgb.xlsx
+++ b/Astro/Results_Production_Astro_xgb.xlsx
@@ -28,108 +28,6 @@
     <t>Lookup</t>
   </si>
   <si>
-    <t>29.03.202611</t>
-  </si>
-  <si>
-    <t>29.03.202612</t>
-  </si>
-  <si>
-    <t>29.03.202613</t>
-  </si>
-  <si>
-    <t>29.03.202614</t>
-  </si>
-  <si>
-    <t>29.03.202615</t>
-  </si>
-  <si>
-    <t>29.03.202616</t>
-  </si>
-  <si>
-    <t>29.03.202617</t>
-  </si>
-  <si>
-    <t>29.03.202618</t>
-  </si>
-  <si>
-    <t>29.03.202619</t>
-  </si>
-  <si>
-    <t>29.03.202620</t>
-  </si>
-  <si>
-    <t>29.03.202621</t>
-  </si>
-  <si>
-    <t>29.03.202622</t>
-  </si>
-  <si>
-    <t>29.03.202623</t>
-  </si>
-  <si>
-    <t>29.03.202624</t>
-  </si>
-  <si>
-    <t>30.03.20261</t>
-  </si>
-  <si>
-    <t>30.03.20262</t>
-  </si>
-  <si>
-    <t>30.03.20263</t>
-  </si>
-  <si>
-    <t>30.03.20264</t>
-  </si>
-  <si>
-    <t>30.03.20265</t>
-  </si>
-  <si>
-    <t>30.03.20266</t>
-  </si>
-  <si>
-    <t>30.03.20267</t>
-  </si>
-  <si>
-    <t>30.03.20268</t>
-  </si>
-  <si>
-    <t>30.03.20269</t>
-  </si>
-  <si>
-    <t>30.03.202610</t>
-  </si>
-  <si>
-    <t>30.03.202611</t>
-  </si>
-  <si>
-    <t>30.03.202612</t>
-  </si>
-  <si>
-    <t>30.03.202613</t>
-  </si>
-  <si>
-    <t>30.03.202614</t>
-  </si>
-  <si>
-    <t>30.03.202615</t>
-  </si>
-  <si>
-    <t>30.03.202616</t>
-  </si>
-  <si>
-    <t>30.03.202617</t>
-  </si>
-  <si>
-    <t>30.03.202618</t>
-  </si>
-  <si>
-    <t>30.03.202619</t>
-  </si>
-  <si>
-    <t>30.03.202620</t>
-  </si>
-  <si>
     <t>30.03.202621</t>
   </si>
   <si>
@@ -533,6 +431,108 @@
   </si>
   <si>
     <t>05.04.202611</t>
+  </si>
+  <si>
+    <t>05.04.202612</t>
+  </si>
+  <si>
+    <t>05.04.202613</t>
+  </si>
+  <si>
+    <t>05.04.202614</t>
+  </si>
+  <si>
+    <t>05.04.202615</t>
+  </si>
+  <si>
+    <t>05.04.202616</t>
+  </si>
+  <si>
+    <t>05.04.202617</t>
+  </si>
+  <si>
+    <t>05.04.202618</t>
+  </si>
+  <si>
+    <t>05.04.202619</t>
+  </si>
+  <si>
+    <t>05.04.202620</t>
+  </si>
+  <si>
+    <t>05.04.202621</t>
+  </si>
+  <si>
+    <t>05.04.202622</t>
+  </si>
+  <si>
+    <t>05.04.202623</t>
+  </si>
+  <si>
+    <t>05.04.202624</t>
+  </si>
+  <si>
+    <t>06.04.20261</t>
+  </si>
+  <si>
+    <t>06.04.20262</t>
+  </si>
+  <si>
+    <t>06.04.20263</t>
+  </si>
+  <si>
+    <t>06.04.20264</t>
+  </si>
+  <si>
+    <t>06.04.20265</t>
+  </si>
+  <si>
+    <t>06.04.20266</t>
+  </si>
+  <si>
+    <t>06.04.20267</t>
+  </si>
+  <si>
+    <t>06.04.20268</t>
+  </si>
+  <si>
+    <t>06.04.20269</t>
+  </si>
+  <si>
+    <t>06.04.202610</t>
+  </si>
+  <si>
+    <t>06.04.202611</t>
+  </si>
+  <si>
+    <t>06.04.202612</t>
+  </si>
+  <si>
+    <t>06.04.202613</t>
+  </si>
+  <si>
+    <t>06.04.202614</t>
+  </si>
+  <si>
+    <t>06.04.202615</t>
+  </si>
+  <si>
+    <t>06.04.202616</t>
+  </si>
+  <si>
+    <t>06.04.202617</t>
+  </si>
+  <si>
+    <t>06.04.202618</t>
+  </si>
+  <si>
+    <t>06.04.202619</t>
+  </si>
+  <si>
+    <t>06.04.202620</t>
+  </si>
+  <si>
+    <t>06.04.202621</t>
   </si>
 </sst>
 </file>
@@ -913,10 +913,10 @@
     </row>
     <row r="2" spans="1:4">
       <c r="A2" s="2">
-        <v>46110</v>
+        <v>46111</v>
       </c>
       <c r="B2">
-        <v>11</v>
+        <v>21</v>
       </c>
       <c r="C2">
         <v>0</v>
@@ -927,10 +927,10 @@
     </row>
     <row r="3" spans="1:4">
       <c r="A3" s="2">
-        <v>46110</v>
+        <v>46111</v>
       </c>
       <c r="B3">
-        <v>12</v>
+        <v>22</v>
       </c>
       <c r="C3">
         <v>0</v>
@@ -941,13 +941,13 @@
     </row>
     <row r="4" spans="1:4">
       <c r="A4" s="2">
-        <v>46110</v>
+        <v>46111</v>
       </c>
       <c r="B4">
-        <v>13</v>
+        <v>23</v>
       </c>
       <c r="C4">
-        <v>1.259</v>
+        <v>0</v>
       </c>
       <c r="D4" t="s">
         <v>6</v>
@@ -955,13 +955,13 @@
     </row>
     <row r="5" spans="1:4">
       <c r="A5" s="2">
-        <v>46110</v>
+        <v>46111</v>
       </c>
       <c r="B5">
-        <v>14</v>
+        <v>24</v>
       </c>
       <c r="C5">
-        <v>1.111</v>
+        <v>0</v>
       </c>
       <c r="D5" t="s">
         <v>7</v>
@@ -969,13 +969,13 @@
     </row>
     <row r="6" spans="1:4">
       <c r="A6" s="2">
-        <v>46110</v>
+        <v>46112</v>
       </c>
       <c r="B6">
-        <v>15</v>
+        <v>1</v>
       </c>
       <c r="C6">
-        <v>0.904</v>
+        <v>0</v>
       </c>
       <c r="D6" t="s">
         <v>8</v>
@@ -983,13 +983,13 @@
     </row>
     <row r="7" spans="1:4">
       <c r="A7" s="2">
-        <v>46110</v>
+        <v>46112</v>
       </c>
       <c r="B7">
-        <v>16</v>
+        <v>2</v>
       </c>
       <c r="C7">
-        <v>0.586</v>
+        <v>0</v>
       </c>
       <c r="D7" t="s">
         <v>9</v>
@@ -997,13 +997,13 @@
     </row>
     <row r="8" spans="1:4">
       <c r="A8" s="2">
-        <v>46110</v>
+        <v>46112</v>
       </c>
       <c r="B8">
-        <v>17</v>
+        <v>3</v>
       </c>
       <c r="C8">
-        <v>0.465</v>
+        <v>0</v>
       </c>
       <c r="D8" t="s">
         <v>10</v>
@@ -1011,13 +1011,13 @@
     </row>
     <row r="9" spans="1:4">
       <c r="A9" s="2">
-        <v>46110</v>
+        <v>46112</v>
       </c>
       <c r="B9">
-        <v>18</v>
+        <v>4</v>
       </c>
       <c r="C9">
-        <v>0.22</v>
+        <v>0</v>
       </c>
       <c r="D9" t="s">
         <v>11</v>
@@ -1025,13 +1025,13 @@
     </row>
     <row r="10" spans="1:4">
       <c r="A10" s="2">
-        <v>46110</v>
+        <v>46112</v>
       </c>
       <c r="B10">
-        <v>19</v>
+        <v>5</v>
       </c>
       <c r="C10">
-        <v>0.08400000000000001</v>
+        <v>0</v>
       </c>
       <c r="D10" t="s">
         <v>12</v>
@@ -1039,13 +1039,13 @@
     </row>
     <row r="11" spans="1:4">
       <c r="A11" s="2">
-        <v>46110</v>
+        <v>46112</v>
       </c>
       <c r="B11">
-        <v>20</v>
+        <v>6</v>
       </c>
       <c r="C11">
-        <v>0.011</v>
+        <v>0</v>
       </c>
       <c r="D11" t="s">
         <v>13</v>
@@ -1053,10 +1053,10 @@
     </row>
     <row r="12" spans="1:4">
       <c r="A12" s="2">
-        <v>46110</v>
+        <v>46112</v>
       </c>
       <c r="B12">
-        <v>21</v>
+        <v>7</v>
       </c>
       <c r="C12">
         <v>0</v>
@@ -1067,13 +1067,13 @@
     </row>
     <row r="13" spans="1:4">
       <c r="A13" s="2">
-        <v>46110</v>
+        <v>46112</v>
       </c>
       <c r="B13">
-        <v>22</v>
+        <v>8</v>
       </c>
       <c r="C13">
-        <v>0</v>
+        <v>0.021</v>
       </c>
       <c r="D13" t="s">
         <v>15</v>
@@ -1081,13 +1081,13 @@
     </row>
     <row r="14" spans="1:4">
       <c r="A14" s="2">
-        <v>46110</v>
+        <v>46112</v>
       </c>
       <c r="B14">
-        <v>23</v>
+        <v>9</v>
       </c>
       <c r="C14">
-        <v>0</v>
+        <v>0.218</v>
       </c>
       <c r="D14" t="s">
         <v>16</v>
@@ -1095,13 +1095,13 @@
     </row>
     <row r="15" spans="1:4">
       <c r="A15" s="2">
-        <v>46110</v>
+        <v>46112</v>
       </c>
       <c r="B15">
-        <v>24</v>
+        <v>10</v>
       </c>
       <c r="C15">
-        <v>0</v>
+        <v>0.414</v>
       </c>
       <c r="D15" t="s">
         <v>17</v>
@@ -1109,13 +1109,13 @@
     </row>
     <row r="16" spans="1:4">
       <c r="A16" s="2">
-        <v>46111</v>
+        <v>46112</v>
       </c>
       <c r="B16">
-        <v>1</v>
+        <v>11</v>
       </c>
       <c r="C16">
-        <v>0</v>
+        <v>0.641</v>
       </c>
       <c r="D16" t="s">
         <v>18</v>
@@ -1123,13 +1123,13 @@
     </row>
     <row r="17" spans="1:4">
       <c r="A17" s="2">
-        <v>46111</v>
+        <v>46112</v>
       </c>
       <c r="B17">
-        <v>2</v>
+        <v>12</v>
       </c>
       <c r="C17">
-        <v>0</v>
+        <v>0.768</v>
       </c>
       <c r="D17" t="s">
         <v>19</v>
@@ -1137,13 +1137,13 @@
     </row>
     <row r="18" spans="1:4">
       <c r="A18" s="2">
-        <v>46111</v>
+        <v>46112</v>
       </c>
       <c r="B18">
-        <v>3</v>
+        <v>13</v>
       </c>
       <c r="C18">
-        <v>0</v>
+        <v>0.971</v>
       </c>
       <c r="D18" t="s">
         <v>20</v>
@@ -1151,13 +1151,13 @@
     </row>
     <row r="19" spans="1:4">
       <c r="A19" s="2">
-        <v>46111</v>
+        <v>46112</v>
       </c>
       <c r="B19">
-        <v>4</v>
+        <v>14</v>
       </c>
       <c r="C19">
-        <v>0</v>
+        <v>1.098</v>
       </c>
       <c r="D19" t="s">
         <v>21</v>
@@ -1165,13 +1165,13 @@
     </row>
     <row r="20" spans="1:4">
       <c r="A20" s="2">
-        <v>46111</v>
+        <v>46112</v>
       </c>
       <c r="B20">
-        <v>5</v>
+        <v>15</v>
       </c>
       <c r="C20">
-        <v>0</v>
+        <v>1.042</v>
       </c>
       <c r="D20" t="s">
         <v>22</v>
@@ -1179,13 +1179,13 @@
     </row>
     <row r="21" spans="1:4">
       <c r="A21" s="2">
-        <v>46111</v>
+        <v>46112</v>
       </c>
       <c r="B21">
-        <v>6</v>
+        <v>16</v>
       </c>
       <c r="C21">
-        <v>0</v>
+        <v>0.975</v>
       </c>
       <c r="D21" t="s">
         <v>23</v>
@@ -1193,13 +1193,13 @@
     </row>
     <row r="22" spans="1:4">
       <c r="A22" s="2">
-        <v>46111</v>
+        <v>46112</v>
       </c>
       <c r="B22">
-        <v>7</v>
+        <v>17</v>
       </c>
       <c r="C22">
-        <v>0</v>
+        <v>0.6830000000000001</v>
       </c>
       <c r="D22" t="s">
         <v>24</v>
@@ -1207,13 +1207,13 @@
     </row>
     <row r="23" spans="1:4">
       <c r="A23" s="2">
-        <v>46111</v>
+        <v>46112</v>
       </c>
       <c r="B23">
-        <v>8</v>
+        <v>18</v>
       </c>
       <c r="C23">
-        <v>0.022</v>
+        <v>0.352</v>
       </c>
       <c r="D23" t="s">
         <v>25</v>
@@ -1221,13 +1221,13 @@
     </row>
     <row r="24" spans="1:4">
       <c r="A24" s="2">
-        <v>46111</v>
+        <v>46112</v>
       </c>
       <c r="B24">
-        <v>9</v>
+        <v>19</v>
       </c>
       <c r="C24">
-        <v>0.287</v>
+        <v>0.146</v>
       </c>
       <c r="D24" t="s">
         <v>26</v>
@@ -1235,13 +1235,13 @@
     </row>
     <row r="25" spans="1:4">
       <c r="A25" s="2">
-        <v>46111</v>
+        <v>46112</v>
       </c>
       <c r="B25">
-        <v>10</v>
+        <v>20</v>
       </c>
       <c r="C25">
-        <v>0.584</v>
+        <v>0.012</v>
       </c>
       <c r="D25" t="s">
         <v>27</v>
@@ -1249,13 +1249,13 @@
     </row>
     <row r="26" spans="1:4">
       <c r="A26" s="2">
-        <v>46111</v>
+        <v>46112</v>
       </c>
       <c r="B26">
-        <v>11</v>
+        <v>21</v>
       </c>
       <c r="C26">
-        <v>0.895</v>
+        <v>0</v>
       </c>
       <c r="D26" t="s">
         <v>28</v>
@@ -1263,13 +1263,13 @@
     </row>
     <row r="27" spans="1:4">
       <c r="A27" s="2">
-        <v>46111</v>
+        <v>46112</v>
       </c>
       <c r="B27">
-        <v>12</v>
+        <v>22</v>
       </c>
       <c r="C27">
-        <v>1.064</v>
+        <v>0</v>
       </c>
       <c r="D27" t="s">
         <v>29</v>
@@ -1277,13 +1277,13 @@
     </row>
     <row r="28" spans="1:4">
       <c r="A28" s="2">
-        <v>46111</v>
+        <v>46112</v>
       </c>
       <c r="B28">
-        <v>13</v>
+        <v>23</v>
       </c>
       <c r="C28">
-        <v>1.105</v>
+        <v>0</v>
       </c>
       <c r="D28" t="s">
         <v>30</v>
@@ -1291,13 +1291,13 @@
     </row>
     <row r="29" spans="1:4">
       <c r="A29" s="2">
-        <v>46111</v>
+        <v>46112</v>
       </c>
       <c r="B29">
-        <v>14</v>
+        <v>24</v>
       </c>
       <c r="C29">
-        <v>1.218</v>
+        <v>0</v>
       </c>
       <c r="D29" t="s">
         <v>31</v>
@@ -1305,13 +1305,13 @@
     </row>
     <row r="30" spans="1:4">
       <c r="A30" s="2">
-        <v>46111</v>
+        <v>46113</v>
       </c>
       <c r="B30">
-        <v>15</v>
+        <v>1</v>
       </c>
       <c r="C30">
-        <v>1.322</v>
+        <v>0</v>
       </c>
       <c r="D30" t="s">
         <v>32</v>
@@ -1319,13 +1319,13 @@
     </row>
     <row r="31" spans="1:4">
       <c r="A31" s="2">
-        <v>46111</v>
+        <v>46113</v>
       </c>
       <c r="B31">
-        <v>16</v>
+        <v>2</v>
       </c>
       <c r="C31">
-        <v>1.215</v>
+        <v>0</v>
       </c>
       <c r="D31" t="s">
         <v>33</v>
@@ -1333,13 +1333,13 @@
     </row>
     <row r="32" spans="1:4">
       <c r="A32" s="2">
-        <v>46111</v>
+        <v>46113</v>
       </c>
       <c r="B32">
-        <v>17</v>
+        <v>3</v>
       </c>
       <c r="C32">
-        <v>1.011</v>
+        <v>0</v>
       </c>
       <c r="D32" t="s">
         <v>34</v>
@@ -1347,13 +1347,13 @@
     </row>
     <row r="33" spans="1:4">
       <c r="A33" s="2">
-        <v>46111</v>
+        <v>46113</v>
       </c>
       <c r="B33">
-        <v>18</v>
+        <v>4</v>
       </c>
       <c r="C33">
-        <v>0.6</v>
+        <v>0</v>
       </c>
       <c r="D33" t="s">
         <v>35</v>
@@ -1361,13 +1361,13 @@
     </row>
     <row r="34" spans="1:4">
       <c r="A34" s="2">
-        <v>46111</v>
+        <v>46113</v>
       </c>
       <c r="B34">
-        <v>19</v>
+        <v>5</v>
       </c>
       <c r="C34">
-        <v>0.151</v>
+        <v>0</v>
       </c>
       <c r="D34" t="s">
         <v>36</v>
@@ -1375,13 +1375,13 @@
     </row>
     <row r="35" spans="1:4">
       <c r="A35" s="2">
-        <v>46111</v>
+        <v>46113</v>
       </c>
       <c r="B35">
-        <v>20</v>
+        <v>6</v>
       </c>
       <c r="C35">
-        <v>0.025</v>
+        <v>0</v>
       </c>
       <c r="D35" t="s">
         <v>37</v>
@@ -1389,10 +1389,10 @@
     </row>
     <row r="36" spans="1:4">
       <c r="A36" s="2">
-        <v>46111</v>
+        <v>46113</v>
       </c>
       <c r="B36">
-        <v>21</v>
+        <v>7</v>
       </c>
       <c r="C36">
         <v>0</v>
@@ -1403,13 +1403,13 @@
     </row>
     <row r="37" spans="1:4">
       <c r="A37" s="2">
-        <v>46111</v>
+        <v>46113</v>
       </c>
       <c r="B37">
-        <v>22</v>
+        <v>8</v>
       </c>
       <c r="C37">
-        <v>0</v>
+        <v>0.045</v>
       </c>
       <c r="D37" t="s">
         <v>39</v>
@@ -1417,13 +1417,13 @@
     </row>
     <row r="38" spans="1:4">
       <c r="A38" s="2">
-        <v>46111</v>
+        <v>46113</v>
       </c>
       <c r="B38">
-        <v>23</v>
+        <v>9</v>
       </c>
       <c r="C38">
-        <v>0</v>
+        <v>0.523</v>
       </c>
       <c r="D38" t="s">
         <v>40</v>
@@ -1431,13 +1431,13 @@
     </row>
     <row r="39" spans="1:4">
       <c r="A39" s="2">
-        <v>46111</v>
+        <v>46113</v>
       </c>
       <c r="B39">
-        <v>24</v>
+        <v>10</v>
       </c>
       <c r="C39">
-        <v>0</v>
+        <v>0.903</v>
       </c>
       <c r="D39" t="s">
         <v>41</v>
@@ -1445,13 +1445,13 @@
     </row>
     <row r="40" spans="1:4">
       <c r="A40" s="2">
-        <v>46112</v>
+        <v>46113</v>
       </c>
       <c r="B40">
-        <v>1</v>
+        <v>11</v>
       </c>
       <c r="C40">
-        <v>0</v>
+        <v>1.642</v>
       </c>
       <c r="D40" t="s">
         <v>42</v>
@@ -1459,13 +1459,13 @@
     </row>
     <row r="41" spans="1:4">
       <c r="A41" s="2">
-        <v>46112</v>
+        <v>46113</v>
       </c>
       <c r="B41">
-        <v>2</v>
+        <v>12</v>
       </c>
       <c r="C41">
-        <v>0</v>
+        <v>2.034</v>
       </c>
       <c r="D41" t="s">
         <v>43</v>
@@ -1473,13 +1473,13 @@
     </row>
     <row r="42" spans="1:4">
       <c r="A42" s="2">
-        <v>46112</v>
+        <v>46113</v>
       </c>
       <c r="B42">
-        <v>3</v>
+        <v>13</v>
       </c>
       <c r="C42">
-        <v>0</v>
+        <v>2.206</v>
       </c>
       <c r="D42" t="s">
         <v>44</v>
@@ -1487,13 +1487,13 @@
     </row>
     <row r="43" spans="1:4">
       <c r="A43" s="2">
-        <v>46112</v>
+        <v>46113</v>
       </c>
       <c r="B43">
-        <v>4</v>
+        <v>14</v>
       </c>
       <c r="C43">
-        <v>0</v>
+        <v>2.314</v>
       </c>
       <c r="D43" t="s">
         <v>45</v>
@@ -1501,13 +1501,13 @@
     </row>
     <row r="44" spans="1:4">
       <c r="A44" s="2">
-        <v>46112</v>
+        <v>46113</v>
       </c>
       <c r="B44">
-        <v>5</v>
+        <v>15</v>
       </c>
       <c r="C44">
-        <v>0</v>
+        <v>2.153</v>
       </c>
       <c r="D44" t="s">
         <v>46</v>
@@ -1515,13 +1515,13 @@
     </row>
     <row r="45" spans="1:4">
       <c r="A45" s="2">
-        <v>46112</v>
+        <v>46113</v>
       </c>
       <c r="B45">
-        <v>6</v>
+        <v>16</v>
       </c>
       <c r="C45">
-        <v>0</v>
+        <v>1.691</v>
       </c>
       <c r="D45" t="s">
         <v>47</v>
@@ -1529,13 +1529,13 @@
     </row>
     <row r="46" spans="1:4">
       <c r="A46" s="2">
-        <v>46112</v>
+        <v>46113</v>
       </c>
       <c r="B46">
-        <v>7</v>
+        <v>17</v>
       </c>
       <c r="C46">
-        <v>0</v>
+        <v>1.179</v>
       </c>
       <c r="D46" t="s">
         <v>48</v>
@@ -1543,13 +1543,13 @@
     </row>
     <row r="47" spans="1:4">
       <c r="A47" s="2">
-        <v>46112</v>
+        <v>46113</v>
       </c>
       <c r="B47">
-        <v>8</v>
+        <v>18</v>
       </c>
       <c r="C47">
-        <v>0.017</v>
+        <v>0.774</v>
       </c>
       <c r="D47" t="s">
         <v>49</v>
@@ -1557,13 +1557,13 @@
     </row>
     <row r="48" spans="1:4">
       <c r="A48" s="2">
-        <v>46112</v>
+        <v>46113</v>
       </c>
       <c r="B48">
-        <v>9</v>
+        <v>19</v>
       </c>
       <c r="C48">
-        <v>0.205</v>
+        <v>0.292</v>
       </c>
       <c r="D48" t="s">
         <v>50</v>
@@ -1571,13 +1571,13 @@
     </row>
     <row r="49" spans="1:4">
       <c r="A49" s="2">
-        <v>46112</v>
+        <v>46113</v>
       </c>
       <c r="B49">
-        <v>10</v>
+        <v>20</v>
       </c>
       <c r="C49">
-        <v>0.383</v>
+        <v>0.026</v>
       </c>
       <c r="D49" t="s">
         <v>51</v>
@@ -1585,13 +1585,13 @@
     </row>
     <row r="50" spans="1:4">
       <c r="A50" s="2">
-        <v>46112</v>
+        <v>46113</v>
       </c>
       <c r="B50">
-        <v>11</v>
+        <v>21</v>
       </c>
       <c r="C50">
-        <v>0.556</v>
+        <v>0</v>
       </c>
       <c r="D50" t="s">
         <v>52</v>
@@ -1599,13 +1599,13 @@
     </row>
     <row r="51" spans="1:4">
       <c r="A51" s="2">
-        <v>46112</v>
+        <v>46113</v>
       </c>
       <c r="B51">
-        <v>12</v>
+        <v>22</v>
       </c>
       <c r="C51">
-        <v>0.638</v>
+        <v>0</v>
       </c>
       <c r="D51" t="s">
         <v>53</v>
@@ -1613,13 +1613,13 @@
     </row>
     <row r="52" spans="1:4">
       <c r="A52" s="2">
-        <v>46112</v>
+        <v>46113</v>
       </c>
       <c r="B52">
-        <v>13</v>
+        <v>23</v>
       </c>
       <c r="C52">
-        <v>0.834</v>
+        <v>0</v>
       </c>
       <c r="D52" t="s">
         <v>54</v>
@@ -1627,13 +1627,13 @@
     </row>
     <row r="53" spans="1:4">
       <c r="A53" s="2">
-        <v>46112</v>
+        <v>46113</v>
       </c>
       <c r="B53">
-        <v>14</v>
+        <v>24</v>
       </c>
       <c r="C53">
-        <v>0.873</v>
+        <v>0</v>
       </c>
       <c r="D53" t="s">
         <v>55</v>
@@ -1641,13 +1641,13 @@
     </row>
     <row r="54" spans="1:4">
       <c r="A54" s="2">
-        <v>46112</v>
+        <v>46114</v>
       </c>
       <c r="B54">
-        <v>15</v>
+        <v>1</v>
       </c>
       <c r="C54">
-        <v>0.826</v>
+        <v>0</v>
       </c>
       <c r="D54" t="s">
         <v>56</v>
@@ -1655,13 +1655,13 @@
     </row>
     <row r="55" spans="1:4">
       <c r="A55" s="2">
-        <v>46112</v>
+        <v>46114</v>
       </c>
       <c r="B55">
-        <v>16</v>
+        <v>2</v>
       </c>
       <c r="C55">
-        <v>0.706</v>
+        <v>0</v>
       </c>
       <c r="D55" t="s">
         <v>57</v>
@@ -1669,13 +1669,13 @@
     </row>
     <row r="56" spans="1:4">
       <c r="A56" s="2">
-        <v>46112</v>
+        <v>46114</v>
       </c>
       <c r="B56">
-        <v>17</v>
+        <v>3</v>
       </c>
       <c r="C56">
-        <v>0.532</v>
+        <v>0</v>
       </c>
       <c r="D56" t="s">
         <v>58</v>
@@ -1683,13 +1683,13 @@
     </row>
     <row r="57" spans="1:4">
       <c r="A57" s="2">
-        <v>46112</v>
+        <v>46114</v>
       </c>
       <c r="B57">
-        <v>18</v>
+        <v>4</v>
       </c>
       <c r="C57">
-        <v>0.316</v>
+        <v>0</v>
       </c>
       <c r="D57" t="s">
         <v>59</v>
@@ -1697,13 +1697,13 @@
     </row>
     <row r="58" spans="1:4">
       <c r="A58" s="2">
-        <v>46112</v>
+        <v>46114</v>
       </c>
       <c r="B58">
-        <v>19</v>
+        <v>5</v>
       </c>
       <c r="C58">
-        <v>0.115</v>
+        <v>0</v>
       </c>
       <c r="D58" t="s">
         <v>60</v>
@@ -1711,13 +1711,13 @@
     </row>
     <row r="59" spans="1:4">
       <c r="A59" s="2">
-        <v>46112</v>
+        <v>46114</v>
       </c>
       <c r="B59">
-        <v>20</v>
+        <v>6</v>
       </c>
       <c r="C59">
-        <v>0.012</v>
+        <v>0</v>
       </c>
       <c r="D59" t="s">
         <v>61</v>
@@ -1725,10 +1725,10 @@
     </row>
     <row r="60" spans="1:4">
       <c r="A60" s="2">
-        <v>46112</v>
+        <v>46114</v>
       </c>
       <c r="B60">
-        <v>21</v>
+        <v>7</v>
       </c>
       <c r="C60">
         <v>0</v>
@@ -1739,13 +1739,13 @@
     </row>
     <row r="61" spans="1:4">
       <c r="A61" s="2">
-        <v>46112</v>
+        <v>46114</v>
       </c>
       <c r="B61">
-        <v>22</v>
+        <v>8</v>
       </c>
       <c r="C61">
-        <v>0</v>
+        <v>0.066</v>
       </c>
       <c r="D61" t="s">
         <v>63</v>
@@ -1753,13 +1753,13 @@
     </row>
     <row r="62" spans="1:4">
       <c r="A62" s="2">
-        <v>46112</v>
+        <v>46114</v>
       </c>
       <c r="B62">
-        <v>23</v>
+        <v>9</v>
       </c>
       <c r="C62">
-        <v>0</v>
+        <v>0.646</v>
       </c>
       <c r="D62" t="s">
         <v>64</v>
@@ -1767,13 +1767,13 @@
     </row>
     <row r="63" spans="1:4">
       <c r="A63" s="2">
-        <v>46112</v>
+        <v>46114</v>
       </c>
       <c r="B63">
-        <v>24</v>
+        <v>10</v>
       </c>
       <c r="C63">
-        <v>0</v>
+        <v>1.402</v>
       </c>
       <c r="D63" t="s">
         <v>65</v>
@@ -1781,13 +1781,13 @@
     </row>
     <row r="64" spans="1:4">
       <c r="A64" s="2">
-        <v>46113</v>
+        <v>46114</v>
       </c>
       <c r="B64">
-        <v>1</v>
+        <v>11</v>
       </c>
       <c r="C64">
-        <v>0</v>
+        <v>1.99</v>
       </c>
       <c r="D64" t="s">
         <v>66</v>
@@ -1795,13 +1795,13 @@
     </row>
     <row r="65" spans="1:4">
       <c r="A65" s="2">
-        <v>46113</v>
+        <v>46114</v>
       </c>
       <c r="B65">
-        <v>2</v>
+        <v>12</v>
       </c>
       <c r="C65">
-        <v>0</v>
+        <v>2.3</v>
       </c>
       <c r="D65" t="s">
         <v>67</v>
@@ -1809,13 +1809,13 @@
     </row>
     <row r="66" spans="1:4">
       <c r="A66" s="2">
-        <v>46113</v>
+        <v>46114</v>
       </c>
       <c r="B66">
-        <v>3</v>
+        <v>13</v>
       </c>
       <c r="C66">
-        <v>0</v>
+        <v>2.26</v>
       </c>
       <c r="D66" t="s">
         <v>68</v>
@@ -1823,13 +1823,13 @@
     </row>
     <row r="67" spans="1:4">
       <c r="A67" s="2">
-        <v>46113</v>
+        <v>46114</v>
       </c>
       <c r="B67">
-        <v>4</v>
+        <v>14</v>
       </c>
       <c r="C67">
-        <v>0</v>
+        <v>2.127</v>
       </c>
       <c r="D67" t="s">
         <v>69</v>
@@ -1837,13 +1837,13 @@
     </row>
     <row r="68" spans="1:4">
       <c r="A68" s="2">
-        <v>46113</v>
+        <v>46114</v>
       </c>
       <c r="B68">
-        <v>5</v>
+        <v>15</v>
       </c>
       <c r="C68">
-        <v>0</v>
+        <v>2.022</v>
       </c>
       <c r="D68" t="s">
         <v>70</v>
@@ -1851,13 +1851,13 @@
     </row>
     <row r="69" spans="1:4">
       <c r="A69" s="2">
-        <v>46113</v>
+        <v>46114</v>
       </c>
       <c r="B69">
-        <v>6</v>
+        <v>16</v>
       </c>
       <c r="C69">
-        <v>0</v>
+        <v>1.766</v>
       </c>
       <c r="D69" t="s">
         <v>71</v>
@@ -1865,13 +1865,13 @@
     </row>
     <row r="70" spans="1:4">
       <c r="A70" s="2">
-        <v>46113</v>
+        <v>46114</v>
       </c>
       <c r="B70">
-        <v>7</v>
+        <v>17</v>
       </c>
       <c r="C70">
-        <v>0</v>
+        <v>1.241</v>
       </c>
       <c r="D70" t="s">
         <v>72</v>
@@ -1879,13 +1879,13 @@
     </row>
     <row r="71" spans="1:4">
       <c r="A71" s="2">
-        <v>46113</v>
+        <v>46114</v>
       </c>
       <c r="B71">
-        <v>8</v>
+        <v>18</v>
       </c>
       <c r="C71">
-        <v>0.046</v>
+        <v>0.73</v>
       </c>
       <c r="D71" t="s">
         <v>73</v>
@@ -1893,13 +1893,13 @@
     </row>
     <row r="72" spans="1:4">
       <c r="A72" s="2">
-        <v>46113</v>
+        <v>46114</v>
       </c>
       <c r="B72">
-        <v>9</v>
+        <v>19</v>
       </c>
       <c r="C72">
-        <v>0.529</v>
+        <v>0.273</v>
       </c>
       <c r="D72" t="s">
         <v>74</v>
@@ -1907,13 +1907,13 @@
     </row>
     <row r="73" spans="1:4">
       <c r="A73" s="2">
-        <v>46113</v>
+        <v>46114</v>
       </c>
       <c r="B73">
-        <v>10</v>
+        <v>20</v>
       </c>
       <c r="C73">
-        <v>0.907</v>
+        <v>0.02</v>
       </c>
       <c r="D73" t="s">
         <v>75</v>
@@ -1921,13 +1921,13 @@
     </row>
     <row r="74" spans="1:4">
       <c r="A74" s="2">
-        <v>46113</v>
+        <v>46114</v>
       </c>
       <c r="B74">
-        <v>11</v>
+        <v>21</v>
       </c>
       <c r="C74">
-        <v>1.499</v>
+        <v>0</v>
       </c>
       <c r="D74" t="s">
         <v>76</v>
@@ -1935,13 +1935,13 @@
     </row>
     <row r="75" spans="1:4">
       <c r="A75" s="2">
-        <v>46113</v>
+        <v>46114</v>
       </c>
       <c r="B75">
-        <v>12</v>
+        <v>22</v>
       </c>
       <c r="C75">
-        <v>1.899</v>
+        <v>0</v>
       </c>
       <c r="D75" t="s">
         <v>77</v>
@@ -1949,13 +1949,13 @@
     </row>
     <row r="76" spans="1:4">
       <c r="A76" s="2">
-        <v>46113</v>
+        <v>46114</v>
       </c>
       <c r="B76">
-        <v>13</v>
+        <v>23</v>
       </c>
       <c r="C76">
-        <v>1.953</v>
+        <v>0</v>
       </c>
       <c r="D76" t="s">
         <v>78</v>
@@ -1963,13 +1963,13 @@
     </row>
     <row r="77" spans="1:4">
       <c r="A77" s="2">
-        <v>46113</v>
+        <v>46114</v>
       </c>
       <c r="B77">
-        <v>14</v>
+        <v>24</v>
       </c>
       <c r="C77">
-        <v>1.976</v>
+        <v>0</v>
       </c>
       <c r="D77" t="s">
         <v>79</v>
@@ -1977,13 +1977,13 @@
     </row>
     <row r="78" spans="1:4">
       <c r="A78" s="2">
-        <v>46113</v>
+        <v>46115</v>
       </c>
       <c r="B78">
-        <v>15</v>
+        <v>1</v>
       </c>
       <c r="C78">
-        <v>1.94</v>
+        <v>0</v>
       </c>
       <c r="D78" t="s">
         <v>80</v>
@@ -1991,13 +1991,13 @@
     </row>
     <row r="79" spans="1:4">
       <c r="A79" s="2">
-        <v>46113</v>
+        <v>46115</v>
       </c>
       <c r="B79">
-        <v>16</v>
+        <v>2</v>
       </c>
       <c r="C79">
-        <v>1.632</v>
+        <v>0</v>
       </c>
       <c r="D79" t="s">
         <v>81</v>
@@ -2005,13 +2005,13 @@
     </row>
     <row r="80" spans="1:4">
       <c r="A80" s="2">
-        <v>46113</v>
+        <v>46115</v>
       </c>
       <c r="B80">
-        <v>17</v>
+        <v>3</v>
       </c>
       <c r="C80">
-        <v>1.179</v>
+        <v>0</v>
       </c>
       <c r="D80" t="s">
         <v>82</v>
@@ -2019,13 +2019,13 @@
     </row>
     <row r="81" spans="1:4">
       <c r="A81" s="2">
-        <v>46113</v>
+        <v>46115</v>
       </c>
       <c r="B81">
-        <v>18</v>
+        <v>4</v>
       </c>
       <c r="C81">
-        <v>0.6889999999999999</v>
+        <v>0</v>
       </c>
       <c r="D81" t="s">
         <v>83</v>
@@ -2033,13 +2033,13 @@
     </row>
     <row r="82" spans="1:4">
       <c r="A82" s="2">
-        <v>46113</v>
+        <v>46115</v>
       </c>
       <c r="B82">
-        <v>19</v>
+        <v>5</v>
       </c>
       <c r="C82">
-        <v>0.275</v>
+        <v>0</v>
       </c>
       <c r="D82" t="s">
         <v>84</v>
@@ -2047,13 +2047,13 @@
     </row>
     <row r="83" spans="1:4">
       <c r="A83" s="2">
-        <v>46113</v>
+        <v>46115</v>
       </c>
       <c r="B83">
-        <v>20</v>
+        <v>6</v>
       </c>
       <c r="C83">
-        <v>0.024</v>
+        <v>0</v>
       </c>
       <c r="D83" t="s">
         <v>85</v>
@@ -2061,10 +2061,10 @@
     </row>
     <row r="84" spans="1:4">
       <c r="A84" s="2">
-        <v>46113</v>
+        <v>46115</v>
       </c>
       <c r="B84">
-        <v>21</v>
+        <v>7</v>
       </c>
       <c r="C84">
         <v>0</v>
@@ -2075,13 +2075,13 @@
     </row>
     <row r="85" spans="1:4">
       <c r="A85" s="2">
-        <v>46113</v>
+        <v>46115</v>
       </c>
       <c r="B85">
-        <v>22</v>
+        <v>8</v>
       </c>
       <c r="C85">
-        <v>0</v>
+        <v>0.029</v>
       </c>
       <c r="D85" t="s">
         <v>87</v>
@@ -2089,13 +2089,13 @@
     </row>
     <row r="86" spans="1:4">
       <c r="A86" s="2">
-        <v>46113</v>
+        <v>46115</v>
       </c>
       <c r="B86">
-        <v>23</v>
+        <v>9</v>
       </c>
       <c r="C86">
-        <v>0</v>
+        <v>0.274</v>
       </c>
       <c r="D86" t="s">
         <v>88</v>
@@ -2103,13 +2103,13 @@
     </row>
     <row r="87" spans="1:4">
       <c r="A87" s="2">
-        <v>46113</v>
+        <v>46115</v>
       </c>
       <c r="B87">
-        <v>24</v>
+        <v>10</v>
       </c>
       <c r="C87">
-        <v>0</v>
+        <v>0.747</v>
       </c>
       <c r="D87" t="s">
         <v>89</v>
@@ -2117,13 +2117,13 @@
     </row>
     <row r="88" spans="1:4">
       <c r="A88" s="2">
-        <v>46114</v>
+        <v>46115</v>
       </c>
       <c r="B88">
-        <v>1</v>
+        <v>11</v>
       </c>
       <c r="C88">
-        <v>0</v>
+        <v>0.922</v>
       </c>
       <c r="D88" t="s">
         <v>90</v>
@@ -2131,13 +2131,13 @@
     </row>
     <row r="89" spans="1:4">
       <c r="A89" s="2">
-        <v>46114</v>
+        <v>46115</v>
       </c>
       <c r="B89">
-        <v>2</v>
+        <v>12</v>
       </c>
       <c r="C89">
-        <v>0</v>
+        <v>1.261</v>
       </c>
       <c r="D89" t="s">
         <v>91</v>
@@ -2145,13 +2145,13 @@
     </row>
     <row r="90" spans="1:4">
       <c r="A90" s="2">
-        <v>46114</v>
+        <v>46115</v>
       </c>
       <c r="B90">
-        <v>3</v>
+        <v>13</v>
       </c>
       <c r="C90">
-        <v>0</v>
+        <v>1.373</v>
       </c>
       <c r="D90" t="s">
         <v>92</v>
@@ -2159,13 +2159,13 @@
     </row>
     <row r="91" spans="1:4">
       <c r="A91" s="2">
-        <v>46114</v>
+        <v>46115</v>
       </c>
       <c r="B91">
-        <v>4</v>
+        <v>14</v>
       </c>
       <c r="C91">
-        <v>0</v>
+        <v>1.523</v>
       </c>
       <c r="D91" t="s">
         <v>93</v>
@@ -2173,13 +2173,13 @@
     </row>
     <row r="92" spans="1:4">
       <c r="A92" s="2">
-        <v>46114</v>
+        <v>46115</v>
       </c>
       <c r="B92">
-        <v>5</v>
+        <v>15</v>
       </c>
       <c r="C92">
-        <v>0</v>
+        <v>1.474</v>
       </c>
       <c r="D92" t="s">
         <v>94</v>
@@ -2187,13 +2187,13 @@
     </row>
     <row r="93" spans="1:4">
       <c r="A93" s="2">
-        <v>46114</v>
+        <v>46115</v>
       </c>
       <c r="B93">
-        <v>6</v>
+        <v>16</v>
       </c>
       <c r="C93">
-        <v>0</v>
+        <v>1.26</v>
       </c>
       <c r="D93" t="s">
         <v>95</v>
@@ -2201,13 +2201,13 @@
     </row>
     <row r="94" spans="1:4">
       <c r="A94" s="2">
-        <v>46114</v>
+        <v>46115</v>
       </c>
       <c r="B94">
-        <v>7</v>
+        <v>17</v>
       </c>
       <c r="C94">
-        <v>0</v>
+        <v>0.948</v>
       </c>
       <c r="D94" t="s">
         <v>96</v>
@@ -2215,13 +2215,13 @@
     </row>
     <row r="95" spans="1:4">
       <c r="A95" s="2">
-        <v>46114</v>
+        <v>46115</v>
       </c>
       <c r="B95">
-        <v>8</v>
+        <v>18</v>
       </c>
       <c r="C95">
-        <v>0.048</v>
+        <v>0.597</v>
       </c>
       <c r="D95" t="s">
         <v>97</v>
@@ -2229,13 +2229,13 @@
     </row>
     <row r="96" spans="1:4">
       <c r="A96" s="2">
-        <v>46114</v>
+        <v>46115</v>
       </c>
       <c r="B96">
-        <v>9</v>
+        <v>19</v>
       </c>
       <c r="C96">
-        <v>0.538</v>
+        <v>0.162</v>
       </c>
       <c r="D96" t="s">
         <v>98</v>
@@ -2243,13 +2243,13 @@
     </row>
     <row r="97" spans="1:4">
       <c r="A97" s="2">
-        <v>46114</v>
+        <v>46115</v>
       </c>
       <c r="B97">
-        <v>10</v>
+        <v>20</v>
       </c>
       <c r="C97">
-        <v>1.169</v>
+        <v>0.022</v>
       </c>
       <c r="D97" t="s">
         <v>99</v>
@@ -2257,13 +2257,13 @@
     </row>
     <row r="98" spans="1:4">
       <c r="A98" s="2">
-        <v>46114</v>
+        <v>46115</v>
       </c>
       <c r="B98">
-        <v>11</v>
+        <v>21</v>
       </c>
       <c r="C98">
-        <v>1.935</v>
+        <v>0</v>
       </c>
       <c r="D98" t="s">
         <v>100</v>
@@ -2271,13 +2271,13 @@
     </row>
     <row r="99" spans="1:4">
       <c r="A99" s="2">
-        <v>46114</v>
+        <v>46115</v>
       </c>
       <c r="B99">
-        <v>12</v>
+        <v>22</v>
       </c>
       <c r="C99">
-        <v>2.526</v>
+        <v>0</v>
       </c>
       <c r="D99" t="s">
         <v>101</v>
@@ -2285,13 +2285,13 @@
     </row>
     <row r="100" spans="1:4">
       <c r="A100" s="2">
-        <v>46114</v>
+        <v>46115</v>
       </c>
       <c r="B100">
-        <v>13</v>
+        <v>23</v>
       </c>
       <c r="C100">
-        <v>2.525</v>
+        <v>0</v>
       </c>
       <c r="D100" t="s">
         <v>102</v>
@@ -2299,13 +2299,13 @@
     </row>
     <row r="101" spans="1:4">
       <c r="A101" s="2">
-        <v>46114</v>
+        <v>46115</v>
       </c>
       <c r="B101">
-        <v>14</v>
+        <v>24</v>
       </c>
       <c r="C101">
-        <v>2.458</v>
+        <v>0</v>
       </c>
       <c r="D101" t="s">
         <v>103</v>
@@ -2313,13 +2313,13 @@
     </row>
     <row r="102" spans="1:4">
       <c r="A102" s="2">
-        <v>46114</v>
+        <v>46116</v>
       </c>
       <c r="B102">
-        <v>15</v>
+        <v>1</v>
       </c>
       <c r="C102">
-        <v>2.194</v>
+        <v>0</v>
       </c>
       <c r="D102" t="s">
         <v>104</v>
@@ -2327,13 +2327,13 @@
     </row>
     <row r="103" spans="1:4">
       <c r="A103" s="2">
-        <v>46114</v>
+        <v>46116</v>
       </c>
       <c r="B103">
-        <v>16</v>
+        <v>2</v>
       </c>
       <c r="C103">
-        <v>1.894</v>
+        <v>0</v>
       </c>
       <c r="D103" t="s">
         <v>105</v>
@@ -2341,13 +2341,13 @@
     </row>
     <row r="104" spans="1:4">
       <c r="A104" s="2">
-        <v>46114</v>
+        <v>46116</v>
       </c>
       <c r="B104">
-        <v>17</v>
+        <v>3</v>
       </c>
       <c r="C104">
-        <v>1.479</v>
+        <v>0</v>
       </c>
       <c r="D104" t="s">
         <v>106</v>
@@ -2355,13 +2355,13 @@
     </row>
     <row r="105" spans="1:4">
       <c r="A105" s="2">
-        <v>46114</v>
+        <v>46116</v>
       </c>
       <c r="B105">
-        <v>18</v>
+        <v>4</v>
       </c>
       <c r="C105">
-        <v>0.765</v>
+        <v>0</v>
       </c>
       <c r="D105" t="s">
         <v>107</v>
@@ -2369,13 +2369,13 @@
     </row>
     <row r="106" spans="1:4">
       <c r="A106" s="2">
-        <v>46114</v>
+        <v>46116</v>
       </c>
       <c r="B106">
-        <v>19</v>
+        <v>5</v>
       </c>
       <c r="C106">
-        <v>0.278</v>
+        <v>0</v>
       </c>
       <c r="D106" t="s">
         <v>108</v>
@@ -2383,13 +2383,13 @@
     </row>
     <row r="107" spans="1:4">
       <c r="A107" s="2">
-        <v>46114</v>
+        <v>46116</v>
       </c>
       <c r="B107">
-        <v>20</v>
+        <v>6</v>
       </c>
       <c r="C107">
-        <v>0.023</v>
+        <v>0</v>
       </c>
       <c r="D107" t="s">
         <v>109</v>
@@ -2397,10 +2397,10 @@
     </row>
     <row r="108" spans="1:4">
       <c r="A108" s="2">
-        <v>46114</v>
+        <v>46116</v>
       </c>
       <c r="B108">
-        <v>21</v>
+        <v>7</v>
       </c>
       <c r="C108">
         <v>0</v>
@@ -2411,13 +2411,13 @@
     </row>
     <row r="109" spans="1:4">
       <c r="A109" s="2">
-        <v>46114</v>
+        <v>46116</v>
       </c>
       <c r="B109">
-        <v>22</v>
+        <v>8</v>
       </c>
       <c r="C109">
-        <v>0</v>
+        <v>0.057</v>
       </c>
       <c r="D109" t="s">
         <v>111</v>
@@ -2425,13 +2425,13 @@
     </row>
     <row r="110" spans="1:4">
       <c r="A110" s="2">
-        <v>46114</v>
+        <v>46116</v>
       </c>
       <c r="B110">
-        <v>23</v>
+        <v>9</v>
       </c>
       <c r="C110">
-        <v>0</v>
+        <v>0.581</v>
       </c>
       <c r="D110" t="s">
         <v>112</v>
@@ -2439,13 +2439,13 @@
     </row>
     <row r="111" spans="1:4">
       <c r="A111" s="2">
-        <v>46114</v>
+        <v>46116</v>
       </c>
       <c r="B111">
-        <v>24</v>
+        <v>10</v>
       </c>
       <c r="C111">
-        <v>0</v>
+        <v>1.181</v>
       </c>
       <c r="D111" t="s">
         <v>113</v>
@@ -2453,13 +2453,13 @@
     </row>
     <row r="112" spans="1:4">
       <c r="A112" s="2">
-        <v>46115</v>
+        <v>46116</v>
       </c>
       <c r="B112">
-        <v>1</v>
+        <v>11</v>
       </c>
       <c r="C112">
-        <v>0</v>
+        <v>1.866</v>
       </c>
       <c r="D112" t="s">
         <v>114</v>
@@ -2467,13 +2467,13 @@
     </row>
     <row r="113" spans="1:4">
       <c r="A113" s="2">
-        <v>46115</v>
+        <v>46116</v>
       </c>
       <c r="B113">
-        <v>2</v>
+        <v>12</v>
       </c>
       <c r="C113">
-        <v>0</v>
+        <v>2.337</v>
       </c>
       <c r="D113" t="s">
         <v>115</v>
@@ -2481,13 +2481,13 @@
     </row>
     <row r="114" spans="1:4">
       <c r="A114" s="2">
-        <v>46115</v>
+        <v>46116</v>
       </c>
       <c r="B114">
-        <v>3</v>
+        <v>13</v>
       </c>
       <c r="C114">
-        <v>0</v>
+        <v>2.438</v>
       </c>
       <c r="D114" t="s">
         <v>116</v>
@@ -2495,13 +2495,13 @@
     </row>
     <row r="115" spans="1:4">
       <c r="A115" s="2">
-        <v>46115</v>
+        <v>46116</v>
       </c>
       <c r="B115">
-        <v>4</v>
+        <v>14</v>
       </c>
       <c r="C115">
-        <v>0</v>
+        <v>2.403</v>
       </c>
       <c r="D115" t="s">
         <v>117</v>
@@ -2509,13 +2509,13 @@
     </row>
     <row r="116" spans="1:4">
       <c r="A116" s="2">
-        <v>46115</v>
+        <v>46116</v>
       </c>
       <c r="B116">
-        <v>5</v>
+        <v>15</v>
       </c>
       <c r="C116">
-        <v>0</v>
+        <v>2.421</v>
       </c>
       <c r="D116" t="s">
         <v>118</v>
@@ -2523,13 +2523,13 @@
     </row>
     <row r="117" spans="1:4">
       <c r="A117" s="2">
-        <v>46115</v>
+        <v>46116</v>
       </c>
       <c r="B117">
-        <v>6</v>
+        <v>16</v>
       </c>
       <c r="C117">
-        <v>0</v>
+        <v>2.238</v>
       </c>
       <c r="D117" t="s">
         <v>119</v>
@@ -2537,13 +2537,13 @@
     </row>
     <row r="118" spans="1:4">
       <c r="A118" s="2">
-        <v>46115</v>
+        <v>46116</v>
       </c>
       <c r="B118">
-        <v>7</v>
+        <v>17</v>
       </c>
       <c r="C118">
-        <v>0</v>
+        <v>1.86</v>
       </c>
       <c r="D118" t="s">
         <v>120</v>
@@ -2551,13 +2551,13 @@
     </row>
     <row r="119" spans="1:4">
       <c r="A119" s="2">
-        <v>46115</v>
+        <v>46116</v>
       </c>
       <c r="B119">
-        <v>8</v>
+        <v>18</v>
       </c>
       <c r="C119">
-        <v>0.032</v>
+        <v>1.085</v>
       </c>
       <c r="D119" t="s">
         <v>121</v>
@@ -2565,13 +2565,13 @@
     </row>
     <row r="120" spans="1:4">
       <c r="A120" s="2">
-        <v>46115</v>
+        <v>46116</v>
       </c>
       <c r="B120">
-        <v>9</v>
+        <v>19</v>
       </c>
       <c r="C120">
-        <v>0.431</v>
+        <v>0.383</v>
       </c>
       <c r="D120" t="s">
         <v>122</v>
@@ -2579,13 +2579,13 @@
     </row>
     <row r="121" spans="1:4">
       <c r="A121" s="2">
-        <v>46115</v>
+        <v>46116</v>
       </c>
       <c r="B121">
-        <v>10</v>
+        <v>20</v>
       </c>
       <c r="C121">
-        <v>0.89</v>
+        <v>0.04</v>
       </c>
       <c r="D121" t="s">
         <v>123</v>
@@ -2593,13 +2593,13 @@
     </row>
     <row r="122" spans="1:4">
       <c r="A122" s="2">
-        <v>46115</v>
+        <v>46116</v>
       </c>
       <c r="B122">
-        <v>11</v>
+        <v>21</v>
       </c>
       <c r="C122">
-        <v>1.208</v>
+        <v>0</v>
       </c>
       <c r="D122" t="s">
         <v>124</v>
@@ -2607,13 +2607,13 @@
     </row>
     <row r="123" spans="1:4">
       <c r="A123" s="2">
-        <v>46115</v>
+        <v>46116</v>
       </c>
       <c r="B123">
-        <v>12</v>
+        <v>22</v>
       </c>
       <c r="C123">
-        <v>1.685</v>
+        <v>0</v>
       </c>
       <c r="D123" t="s">
         <v>125</v>
@@ -2621,13 +2621,13 @@
     </row>
     <row r="124" spans="1:4">
       <c r="A124" s="2">
-        <v>46115</v>
+        <v>46116</v>
       </c>
       <c r="B124">
-        <v>13</v>
+        <v>23</v>
       </c>
       <c r="C124">
-        <v>1.947</v>
+        <v>0</v>
       </c>
       <c r="D124" t="s">
         <v>126</v>
@@ -2635,13 +2635,13 @@
     </row>
     <row r="125" spans="1:4">
       <c r="A125" s="2">
-        <v>46115</v>
+        <v>46116</v>
       </c>
       <c r="B125">
-        <v>14</v>
+        <v>24</v>
       </c>
       <c r="C125">
-        <v>1.922</v>
+        <v>0</v>
       </c>
       <c r="D125" t="s">
         <v>127</v>
@@ -2649,13 +2649,13 @@
     </row>
     <row r="126" spans="1:4">
       <c r="A126" s="2">
-        <v>46115</v>
+        <v>46117</v>
       </c>
       <c r="B126">
-        <v>15</v>
+        <v>1</v>
       </c>
       <c r="C126">
-        <v>1.819</v>
+        <v>0</v>
       </c>
       <c r="D126" t="s">
         <v>128</v>
@@ -2663,13 +2663,13 @@
     </row>
     <row r="127" spans="1:4">
       <c r="A127" s="2">
-        <v>46115</v>
+        <v>46117</v>
       </c>
       <c r="B127">
-        <v>16</v>
+        <v>2</v>
       </c>
       <c r="C127">
-        <v>1.566</v>
+        <v>0</v>
       </c>
       <c r="D127" t="s">
         <v>129</v>
@@ -2677,13 +2677,13 @@
     </row>
     <row r="128" spans="1:4">
       <c r="A128" s="2">
-        <v>46115</v>
+        <v>46117</v>
       </c>
       <c r="B128">
-        <v>17</v>
+        <v>3</v>
       </c>
       <c r="C128">
-        <v>1.34</v>
+        <v>0</v>
       </c>
       <c r="D128" t="s">
         <v>130</v>
@@ -2691,13 +2691,13 @@
     </row>
     <row r="129" spans="1:4">
       <c r="A129" s="2">
-        <v>46115</v>
+        <v>46117</v>
       </c>
       <c r="B129">
-        <v>18</v>
+        <v>4</v>
       </c>
       <c r="C129">
-        <v>0.788</v>
+        <v>0</v>
       </c>
       <c r="D129" t="s">
         <v>131</v>
@@ -2705,13 +2705,13 @@
     </row>
     <row r="130" spans="1:4">
       <c r="A130" s="2">
-        <v>46115</v>
+        <v>46117</v>
       </c>
       <c r="B130">
-        <v>19</v>
+        <v>5</v>
       </c>
       <c r="C130">
-        <v>0.29</v>
+        <v>0</v>
       </c>
       <c r="D130" t="s">
         <v>132</v>
@@ -2719,13 +2719,13 @@
     </row>
     <row r="131" spans="1:4">
       <c r="A131" s="2">
-        <v>46115</v>
+        <v>46117</v>
       </c>
       <c r="B131">
-        <v>20</v>
+        <v>6</v>
       </c>
       <c r="C131">
-        <v>0.026</v>
+        <v>0</v>
       </c>
       <c r="D131" t="s">
         <v>133</v>
@@ -2733,10 +2733,10 @@
     </row>
     <row r="132" spans="1:4">
       <c r="A132" s="2">
-        <v>46115</v>
+        <v>46117</v>
       </c>
       <c r="B132">
-        <v>21</v>
+        <v>7</v>
       </c>
       <c r="C132">
         <v>0</v>
@@ -2747,13 +2747,13 @@
     </row>
     <row r="133" spans="1:4">
       <c r="A133" s="2">
-        <v>46115</v>
+        <v>46117</v>
       </c>
       <c r="B133">
-        <v>22</v>
+        <v>8</v>
       </c>
       <c r="C133">
-        <v>0</v>
+        <v>0.08500000000000001</v>
       </c>
       <c r="D133" t="s">
         <v>135</v>
@@ -2761,13 +2761,13 @@
     </row>
     <row r="134" spans="1:4">
       <c r="A134" s="2">
-        <v>46115</v>
+        <v>46117</v>
       </c>
       <c r="B134">
-        <v>23</v>
+        <v>9</v>
       </c>
       <c r="C134">
-        <v>0</v>
+        <v>0.638</v>
       </c>
       <c r="D134" t="s">
         <v>136</v>
@@ -2775,13 +2775,13 @@
     </row>
     <row r="135" spans="1:4">
       <c r="A135" s="2">
-        <v>46115</v>
+        <v>46117</v>
       </c>
       <c r="B135">
-        <v>24</v>
+        <v>10</v>
       </c>
       <c r="C135">
-        <v>0</v>
+        <v>1.474</v>
       </c>
       <c r="D135" t="s">
         <v>137</v>
@@ -2789,13 +2789,13 @@
     </row>
     <row r="136" spans="1:4">
       <c r="A136" s="2">
-        <v>46116</v>
+        <v>46117</v>
       </c>
       <c r="B136">
-        <v>1</v>
+        <v>11</v>
       </c>
       <c r="C136">
-        <v>0</v>
+        <v>2.134</v>
       </c>
       <c r="D136" t="s">
         <v>138</v>
@@ -2803,13 +2803,13 @@
     </row>
     <row r="137" spans="1:4">
       <c r="A137" s="2">
-        <v>46116</v>
+        <v>46117</v>
       </c>
       <c r="B137">
-        <v>2</v>
+        <v>12</v>
       </c>
       <c r="C137">
-        <v>0</v>
+        <v>2.629</v>
       </c>
       <c r="D137" t="s">
         <v>139</v>
@@ -2817,13 +2817,13 @@
     </row>
     <row r="138" spans="1:4">
       <c r="A138" s="2">
-        <v>46116</v>
+        <v>46117</v>
       </c>
       <c r="B138">
-        <v>3</v>
+        <v>13</v>
       </c>
       <c r="C138">
-        <v>0</v>
+        <v>2.931</v>
       </c>
       <c r="D138" t="s">
         <v>140</v>
@@ -2831,13 +2831,13 @@
     </row>
     <row r="139" spans="1:4">
       <c r="A139" s="2">
-        <v>46116</v>
+        <v>46117</v>
       </c>
       <c r="B139">
-        <v>4</v>
+        <v>14</v>
       </c>
       <c r="C139">
-        <v>0</v>
+        <v>2.921</v>
       </c>
       <c r="D139" t="s">
         <v>141</v>
@@ -2845,13 +2845,13 @@
     </row>
     <row r="140" spans="1:4">
       <c r="A140" s="2">
-        <v>46116</v>
+        <v>46117</v>
       </c>
       <c r="B140">
-        <v>5</v>
+        <v>15</v>
       </c>
       <c r="C140">
-        <v>0</v>
+        <v>2.895</v>
       </c>
       <c r="D140" t="s">
         <v>142</v>
@@ -2859,13 +2859,13 @@
     </row>
     <row r="141" spans="1:4">
       <c r="A141" s="2">
-        <v>46116</v>
+        <v>46117</v>
       </c>
       <c r="B141">
-        <v>6</v>
+        <v>16</v>
       </c>
       <c r="C141">
-        <v>0</v>
+        <v>2.503</v>
       </c>
       <c r="D141" t="s">
         <v>143</v>
@@ -2873,13 +2873,13 @@
     </row>
     <row r="142" spans="1:4">
       <c r="A142" s="2">
-        <v>46116</v>
+        <v>46117</v>
       </c>
       <c r="B142">
-        <v>7</v>
+        <v>17</v>
       </c>
       <c r="C142">
-        <v>0</v>
+        <v>2.042</v>
       </c>
       <c r="D142" t="s">
         <v>144</v>
@@ -2887,13 +2887,13 @@
     </row>
     <row r="143" spans="1:4">
       <c r="A143" s="2">
-        <v>46116</v>
+        <v>46117</v>
       </c>
       <c r="B143">
-        <v>8</v>
+        <v>18</v>
       </c>
       <c r="C143">
-        <v>0.036</v>
+        <v>1.304</v>
       </c>
       <c r="D143" t="s">
         <v>145</v>
@@ -2901,13 +2901,13 @@
     </row>
     <row r="144" spans="1:4">
       <c r="A144" s="2">
-        <v>46116</v>
+        <v>46117</v>
       </c>
       <c r="B144">
-        <v>9</v>
+        <v>19</v>
       </c>
       <c r="C144">
-        <v>0.468</v>
+        <v>0.458</v>
       </c>
       <c r="D144" t="s">
         <v>146</v>
@@ -2915,13 +2915,13 @@
     </row>
     <row r="145" spans="1:4">
       <c r="A145" s="2">
-        <v>46116</v>
+        <v>46117</v>
       </c>
       <c r="B145">
-        <v>10</v>
+        <v>20</v>
       </c>
       <c r="C145">
-        <v>0.915</v>
+        <v>0.049</v>
       </c>
       <c r="D145" t="s">
         <v>147</v>
@@ -2929,13 +2929,13 @@
     </row>
     <row r="146" spans="1:4">
       <c r="A146" s="2">
-        <v>46116</v>
+        <v>46117</v>
       </c>
       <c r="B146">
-        <v>11</v>
+        <v>21</v>
       </c>
       <c r="C146">
-        <v>1.451</v>
+        <v>0</v>
       </c>
       <c r="D146" t="s">
         <v>148</v>
@@ -2943,13 +2943,13 @@
     </row>
     <row r="147" spans="1:4">
       <c r="A147" s="2">
-        <v>46116</v>
+        <v>46117</v>
       </c>
       <c r="B147">
-        <v>12</v>
+        <v>22</v>
       </c>
       <c r="C147">
-        <v>1.853</v>
+        <v>0</v>
       </c>
       <c r="D147" t="s">
         <v>149</v>
@@ -2957,13 +2957,13 @@
     </row>
     <row r="148" spans="1:4">
       <c r="A148" s="2">
-        <v>46116</v>
+        <v>46117</v>
       </c>
       <c r="B148">
-        <v>13</v>
+        <v>23</v>
       </c>
       <c r="C148">
-        <v>1.975</v>
+        <v>0</v>
       </c>
       <c r="D148" t="s">
         <v>150</v>
@@ -2971,13 +2971,13 @@
     </row>
     <row r="149" spans="1:4">
       <c r="A149" s="2">
-        <v>46116</v>
+        <v>46117</v>
       </c>
       <c r="B149">
-        <v>14</v>
+        <v>24</v>
       </c>
       <c r="C149">
-        <v>1.965</v>
+        <v>0</v>
       </c>
       <c r="D149" t="s">
         <v>151</v>
@@ -2985,13 +2985,13 @@
     </row>
     <row r="150" spans="1:4">
       <c r="A150" s="2">
-        <v>46116</v>
+        <v>46118</v>
       </c>
       <c r="B150">
-        <v>15</v>
+        <v>1</v>
       </c>
       <c r="C150">
-        <v>1.961</v>
+        <v>0</v>
       </c>
       <c r="D150" t="s">
         <v>152</v>
@@ -2999,13 +2999,13 @@
     </row>
     <row r="151" spans="1:4">
       <c r="A151" s="2">
-        <v>46116</v>
+        <v>46118</v>
       </c>
       <c r="B151">
-        <v>16</v>
+        <v>2</v>
       </c>
       <c r="C151">
-        <v>1.809</v>
+        <v>0</v>
       </c>
       <c r="D151" t="s">
         <v>153</v>
@@ -3013,13 +3013,13 @@
     </row>
     <row r="152" spans="1:4">
       <c r="A152" s="2">
-        <v>46116</v>
+        <v>46118</v>
       </c>
       <c r="B152">
-        <v>17</v>
+        <v>3</v>
       </c>
       <c r="C152">
-        <v>1.395</v>
+        <v>0</v>
       </c>
       <c r="D152" t="s">
         <v>154</v>
@@ -3027,13 +3027,13 @@
     </row>
     <row r="153" spans="1:4">
       <c r="A153" s="2">
-        <v>46116</v>
+        <v>46118</v>
       </c>
       <c r="B153">
-        <v>18</v>
+        <v>4</v>
       </c>
       <c r="C153">
-        <v>0.8159999999999999</v>
+        <v>0</v>
       </c>
       <c r="D153" t="s">
         <v>155</v>
@@ -3041,13 +3041,13 @@
     </row>
     <row r="154" spans="1:4">
       <c r="A154" s="2">
-        <v>46116</v>
+        <v>46118</v>
       </c>
       <c r="B154">
-        <v>19</v>
+        <v>5</v>
       </c>
       <c r="C154">
-        <v>0.285</v>
+        <v>0</v>
       </c>
       <c r="D154" t="s">
         <v>156</v>
@@ -3055,13 +3055,13 @@
     </row>
     <row r="155" spans="1:4">
       <c r="A155" s="2">
-        <v>46116</v>
+        <v>46118</v>
       </c>
       <c r="B155">
-        <v>20</v>
+        <v>6</v>
       </c>
       <c r="C155">
-        <v>0.025</v>
+        <v>0</v>
       </c>
       <c r="D155" t="s">
         <v>157</v>
@@ -3069,10 +3069,10 @@
     </row>
     <row r="156" spans="1:4">
       <c r="A156" s="2">
-        <v>46116</v>
+        <v>46118</v>
       </c>
       <c r="B156">
-        <v>21</v>
+        <v>7</v>
       </c>
       <c r="C156">
         <v>0</v>
@@ -3083,13 +3083,13 @@
     </row>
     <row r="157" spans="1:4">
       <c r="A157" s="2">
-        <v>46116</v>
+        <v>46118</v>
       </c>
       <c r="B157">
-        <v>22</v>
+        <v>8</v>
       </c>
       <c r="C157">
-        <v>0</v>
+        <v>0.098</v>
       </c>
       <c r="D157" t="s">
         <v>159</v>
@@ -3097,13 +3097,13 @@
     </row>
     <row r="158" spans="1:4">
       <c r="A158" s="2">
-        <v>46116</v>
+        <v>46118</v>
       </c>
       <c r="B158">
-        <v>23</v>
+        <v>9</v>
       </c>
       <c r="C158">
-        <v>0</v>
+        <v>0.699</v>
       </c>
       <c r="D158" t="s">
         <v>160</v>
@@ -3111,13 +3111,13 @@
     </row>
     <row r="159" spans="1:4">
       <c r="A159" s="2">
-        <v>46116</v>
+        <v>46118</v>
       </c>
       <c r="B159">
-        <v>24</v>
+        <v>10</v>
       </c>
       <c r="C159">
-        <v>0</v>
+        <v>1.548</v>
       </c>
       <c r="D159" t="s">
         <v>161</v>
@@ -3125,13 +3125,13 @@
     </row>
     <row r="160" spans="1:4">
       <c r="A160" s="2">
-        <v>46117</v>
+        <v>46118</v>
       </c>
       <c r="B160">
-        <v>1</v>
+        <v>11</v>
       </c>
       <c r="C160">
-        <v>0</v>
+        <v>2.052</v>
       </c>
       <c r="D160" t="s">
         <v>162</v>
@@ -3139,13 +3139,13 @@
     </row>
     <row r="161" spans="1:4">
       <c r="A161" s="2">
-        <v>46117</v>
+        <v>46118</v>
       </c>
       <c r="B161">
-        <v>2</v>
+        <v>12</v>
       </c>
       <c r="C161">
-        <v>0</v>
+        <v>2.495</v>
       </c>
       <c r="D161" t="s">
         <v>163</v>
@@ -3153,13 +3153,13 @@
     </row>
     <row r="162" spans="1:4">
       <c r="A162" s="2">
-        <v>46117</v>
+        <v>46118</v>
       </c>
       <c r="B162">
-        <v>3</v>
+        <v>13</v>
       </c>
       <c r="C162">
-        <v>0</v>
+        <v>2.817</v>
       </c>
       <c r="D162" t="s">
         <v>164</v>
@@ -3167,13 +3167,13 @@
     </row>
     <row r="163" spans="1:4">
       <c r="A163" s="2">
-        <v>46117</v>
+        <v>46118</v>
       </c>
       <c r="B163">
-        <v>4</v>
+        <v>14</v>
       </c>
       <c r="C163">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="D163" t="s">
         <v>165</v>
@@ -3181,13 +3181,13 @@
     </row>
     <row r="164" spans="1:4">
       <c r="A164" s="2">
-        <v>46117</v>
+        <v>46118</v>
       </c>
       <c r="B164">
-        <v>5</v>
+        <v>15</v>
       </c>
       <c r="C164">
-        <v>0</v>
+        <v>2.955</v>
       </c>
       <c r="D164" t="s">
         <v>166</v>
@@ -3195,13 +3195,13 @@
     </row>
     <row r="165" spans="1:4">
       <c r="A165" s="2">
-        <v>46117</v>
+        <v>46118</v>
       </c>
       <c r="B165">
-        <v>6</v>
+        <v>16</v>
       </c>
       <c r="C165">
-        <v>0</v>
+        <v>2.512</v>
       </c>
       <c r="D165" t="s">
         <v>167</v>
@@ -3209,13 +3209,13 @@
     </row>
     <row r="166" spans="1:4">
       <c r="A166" s="2">
-        <v>46117</v>
+        <v>46118</v>
       </c>
       <c r="B166">
-        <v>7</v>
+        <v>17</v>
       </c>
       <c r="C166">
-        <v>0</v>
+        <v>1.998</v>
       </c>
       <c r="D166" t="s">
         <v>168</v>
@@ -3223,13 +3223,13 @@
     </row>
     <row r="167" spans="1:4">
       <c r="A167" s="2">
-        <v>46117</v>
+        <v>46118</v>
       </c>
       <c r="B167">
-        <v>8</v>
+        <v>18</v>
       </c>
       <c r="C167">
-        <v>0.037</v>
+        <v>1.223</v>
       </c>
       <c r="D167" t="s">
         <v>169</v>
@@ -3237,13 +3237,13 @@
     </row>
     <row r="168" spans="1:4">
       <c r="A168" s="2">
-        <v>46117</v>
+        <v>46118</v>
       </c>
       <c r="B168">
-        <v>9</v>
+        <v>19</v>
       </c>
       <c r="C168">
-        <v>0.375</v>
+        <v>0.433</v>
       </c>
       <c r="D168" t="s">
         <v>170</v>
@@ -3251,13 +3251,13 @@
     </row>
     <row r="169" spans="1:4">
       <c r="A169" s="2">
-        <v>46117</v>
+        <v>46118</v>
       </c>
       <c r="B169">
-        <v>10</v>
+        <v>20</v>
       </c>
       <c r="C169">
-        <v>0.857</v>
+        <v>0.047</v>
       </c>
       <c r="D169" t="s">
         <v>171</v>
@@ -3265,13 +3265,13 @@
     </row>
     <row r="170" spans="1:4">
       <c r="A170" s="2">
-        <v>46117</v>
+        <v>46118</v>
       </c>
       <c r="B170">
-        <v>11</v>
+        <v>21</v>
       </c>
       <c r="C170">
-        <v>1.012</v>
+        <v>0</v>
       </c>
       <c r="D170" t="s">
         <v>172</v>

</xml_diff>

<commit_message>
Retraining the models for Astro and Imerial with February real data
</commit_message>
<xml_diff>
--- a/Astro/Results_Production_Astro_xgb.xlsx
+++ b/Astro/Results_Production_Astro_xgb.xlsx
@@ -28,511 +28,511 @@
     <t>Lookup</t>
   </si>
   <si>
-    <t>30.03.202621</t>
-  </si>
-  <si>
-    <t>30.03.202622</t>
-  </si>
-  <si>
-    <t>30.03.202623</t>
-  </si>
-  <si>
-    <t>30.03.202624</t>
-  </si>
-  <si>
-    <t>31.03.20261</t>
-  </si>
-  <si>
-    <t>31.03.20262</t>
-  </si>
-  <si>
-    <t>31.03.20263</t>
-  </si>
-  <si>
-    <t>31.03.20264</t>
-  </si>
-  <si>
-    <t>31.03.20265</t>
-  </si>
-  <si>
-    <t>31.03.20266</t>
-  </si>
-  <si>
-    <t>31.03.20267</t>
-  </si>
-  <si>
-    <t>31.03.20268</t>
-  </si>
-  <si>
-    <t>31.03.20269</t>
-  </si>
-  <si>
-    <t>31.03.202610</t>
-  </si>
-  <si>
-    <t>31.03.202611</t>
-  </si>
-  <si>
-    <t>31.03.202612</t>
-  </si>
-  <si>
-    <t>31.03.202613</t>
-  </si>
-  <si>
-    <t>31.03.202614</t>
-  </si>
-  <si>
-    <t>31.03.202615</t>
-  </si>
-  <si>
-    <t>31.03.202616</t>
-  </si>
-  <si>
-    <t>31.03.202617</t>
-  </si>
-  <si>
-    <t>31.03.202618</t>
-  </si>
-  <si>
-    <t>31.03.202619</t>
-  </si>
-  <si>
-    <t>31.03.202620</t>
-  </si>
-  <si>
-    <t>31.03.202621</t>
-  </si>
-  <si>
-    <t>31.03.202622</t>
-  </si>
-  <si>
-    <t>31.03.202623</t>
-  </si>
-  <si>
-    <t>31.03.202624</t>
-  </si>
-  <si>
-    <t>01.04.20261</t>
-  </si>
-  <si>
-    <t>01.04.20262</t>
-  </si>
-  <si>
-    <t>01.04.20263</t>
-  </si>
-  <si>
-    <t>01.04.20264</t>
-  </si>
-  <si>
-    <t>01.04.20265</t>
-  </si>
-  <si>
-    <t>01.04.20266</t>
-  </si>
-  <si>
-    <t>01.04.20267</t>
-  </si>
-  <si>
-    <t>01.04.20268</t>
-  </si>
-  <si>
-    <t>01.04.20269</t>
-  </si>
-  <si>
-    <t>01.04.202610</t>
-  </si>
-  <si>
-    <t>01.04.202611</t>
-  </si>
-  <si>
-    <t>01.04.202612</t>
-  </si>
-  <si>
-    <t>01.04.202613</t>
-  </si>
-  <si>
-    <t>01.04.202614</t>
-  </si>
-  <si>
-    <t>01.04.202615</t>
-  </si>
-  <si>
-    <t>01.04.202616</t>
-  </si>
-  <si>
-    <t>01.04.202617</t>
-  </si>
-  <si>
-    <t>01.04.202618</t>
-  </si>
-  <si>
-    <t>01.04.202619</t>
-  </si>
-  <si>
-    <t>01.04.202620</t>
-  </si>
-  <si>
-    <t>01.04.202621</t>
-  </si>
-  <si>
-    <t>01.04.202622</t>
-  </si>
-  <si>
-    <t>01.04.202623</t>
-  </si>
-  <si>
-    <t>01.04.202624</t>
-  </si>
-  <si>
-    <t>02.04.20261</t>
-  </si>
-  <si>
-    <t>02.04.20262</t>
-  </si>
-  <si>
-    <t>02.04.20263</t>
-  </si>
-  <si>
-    <t>02.04.20264</t>
-  </si>
-  <si>
-    <t>02.04.20265</t>
-  </si>
-  <si>
-    <t>02.04.20266</t>
-  </si>
-  <si>
-    <t>02.04.20267</t>
-  </si>
-  <si>
-    <t>02.04.20268</t>
-  </si>
-  <si>
-    <t>02.04.20269</t>
-  </si>
-  <si>
-    <t>02.04.202610</t>
-  </si>
-  <si>
-    <t>02.04.202611</t>
-  </si>
-  <si>
-    <t>02.04.202612</t>
-  </si>
-  <si>
-    <t>02.04.202613</t>
-  </si>
-  <si>
-    <t>02.04.202614</t>
-  </si>
-  <si>
-    <t>02.04.202615</t>
-  </si>
-  <si>
-    <t>02.04.202616</t>
-  </si>
-  <si>
-    <t>02.04.202617</t>
-  </si>
-  <si>
-    <t>02.04.202618</t>
-  </si>
-  <si>
-    <t>02.04.202619</t>
-  </si>
-  <si>
-    <t>02.04.202620</t>
-  </si>
-  <si>
-    <t>02.04.202621</t>
-  </si>
-  <si>
-    <t>02.04.202622</t>
-  </si>
-  <si>
-    <t>02.04.202623</t>
-  </si>
-  <si>
-    <t>02.04.202624</t>
-  </si>
-  <si>
-    <t>03.04.20261</t>
-  </si>
-  <si>
-    <t>03.04.20262</t>
-  </si>
-  <si>
-    <t>03.04.20263</t>
-  </si>
-  <si>
-    <t>03.04.20264</t>
-  </si>
-  <si>
-    <t>03.04.20265</t>
-  </si>
-  <si>
-    <t>03.04.20266</t>
-  </si>
-  <si>
-    <t>03.04.20267</t>
-  </si>
-  <si>
-    <t>03.04.20268</t>
-  </si>
-  <si>
-    <t>03.04.20269</t>
-  </si>
-  <si>
-    <t>03.04.202610</t>
-  </si>
-  <si>
-    <t>03.04.202611</t>
-  </si>
-  <si>
-    <t>03.04.202612</t>
-  </si>
-  <si>
-    <t>03.04.202613</t>
-  </si>
-  <si>
-    <t>03.04.202614</t>
-  </si>
-  <si>
-    <t>03.04.202615</t>
-  </si>
-  <si>
-    <t>03.04.202616</t>
-  </si>
-  <si>
-    <t>03.04.202617</t>
-  </si>
-  <si>
-    <t>03.04.202618</t>
-  </si>
-  <si>
-    <t>03.04.202619</t>
-  </si>
-  <si>
-    <t>03.04.202620</t>
-  </si>
-  <si>
-    <t>03.04.202621</t>
-  </si>
-  <si>
-    <t>03.04.202622</t>
-  </si>
-  <si>
-    <t>03.04.202623</t>
-  </si>
-  <si>
-    <t>03.04.202624</t>
-  </si>
-  <si>
-    <t>04.04.20261</t>
-  </si>
-  <si>
-    <t>04.04.20262</t>
-  </si>
-  <si>
-    <t>04.04.20263</t>
-  </si>
-  <si>
-    <t>04.04.20264</t>
-  </si>
-  <si>
-    <t>04.04.20265</t>
-  </si>
-  <si>
-    <t>04.04.20266</t>
-  </si>
-  <si>
-    <t>04.04.20267</t>
-  </si>
-  <si>
-    <t>04.04.20268</t>
-  </si>
-  <si>
-    <t>04.04.20269</t>
-  </si>
-  <si>
-    <t>04.04.202610</t>
-  </si>
-  <si>
-    <t>04.04.202611</t>
-  </si>
-  <si>
-    <t>04.04.202612</t>
-  </si>
-  <si>
-    <t>04.04.202613</t>
-  </si>
-  <si>
-    <t>04.04.202614</t>
-  </si>
-  <si>
-    <t>04.04.202615</t>
-  </si>
-  <si>
-    <t>04.04.202616</t>
-  </si>
-  <si>
-    <t>04.04.202617</t>
-  </si>
-  <si>
-    <t>04.04.202618</t>
-  </si>
-  <si>
-    <t>04.04.202619</t>
-  </si>
-  <si>
-    <t>04.04.202620</t>
-  </si>
-  <si>
-    <t>04.04.202621</t>
-  </si>
-  <si>
-    <t>04.04.202622</t>
-  </si>
-  <si>
-    <t>04.04.202623</t>
-  </si>
-  <si>
-    <t>04.04.202624</t>
-  </si>
-  <si>
-    <t>05.04.20261</t>
-  </si>
-  <si>
-    <t>05.04.20262</t>
-  </si>
-  <si>
-    <t>05.04.20263</t>
-  </si>
-  <si>
-    <t>05.04.20264</t>
-  </si>
-  <si>
-    <t>05.04.20265</t>
-  </si>
-  <si>
-    <t>05.04.20266</t>
-  </si>
-  <si>
-    <t>05.04.20267</t>
-  </si>
-  <si>
-    <t>05.04.20268</t>
-  </si>
-  <si>
-    <t>05.04.20269</t>
-  </si>
-  <si>
-    <t>05.04.202610</t>
-  </si>
-  <si>
-    <t>05.04.202611</t>
-  </si>
-  <si>
-    <t>05.04.202612</t>
-  </si>
-  <si>
-    <t>05.04.202613</t>
-  </si>
-  <si>
-    <t>05.04.202614</t>
-  </si>
-  <si>
-    <t>05.04.202615</t>
-  </si>
-  <si>
-    <t>05.04.202616</t>
-  </si>
-  <si>
-    <t>05.04.202617</t>
-  </si>
-  <si>
-    <t>05.04.202618</t>
-  </si>
-  <si>
-    <t>05.04.202619</t>
-  </si>
-  <si>
-    <t>05.04.202620</t>
-  </si>
-  <si>
-    <t>05.04.202621</t>
-  </si>
-  <si>
-    <t>05.04.202622</t>
-  </si>
-  <si>
-    <t>05.04.202623</t>
-  </si>
-  <si>
-    <t>05.04.202624</t>
-  </si>
-  <si>
-    <t>06.04.20261</t>
-  </si>
-  <si>
-    <t>06.04.20262</t>
-  </si>
-  <si>
-    <t>06.04.20263</t>
-  </si>
-  <si>
-    <t>06.04.20264</t>
-  </si>
-  <si>
-    <t>06.04.20265</t>
-  </si>
-  <si>
-    <t>06.04.20266</t>
-  </si>
-  <si>
-    <t>06.04.20267</t>
-  </si>
-  <si>
-    <t>06.04.20268</t>
-  </si>
-  <si>
-    <t>06.04.20269</t>
-  </si>
-  <si>
-    <t>06.04.202610</t>
-  </si>
-  <si>
-    <t>06.04.202611</t>
-  </si>
-  <si>
-    <t>06.04.202612</t>
-  </si>
-  <si>
-    <t>06.04.202613</t>
-  </si>
-  <si>
-    <t>06.04.202614</t>
-  </si>
-  <si>
-    <t>06.04.202615</t>
-  </si>
-  <si>
-    <t>06.04.202616</t>
-  </si>
-  <si>
-    <t>06.04.202617</t>
-  </si>
-  <si>
-    <t>06.04.202618</t>
-  </si>
-  <si>
-    <t>06.04.202619</t>
-  </si>
-  <si>
-    <t>06.04.202620</t>
-  </si>
-  <si>
-    <t>06.04.202621</t>
+    <t>10.04.202610</t>
+  </si>
+  <si>
+    <t>10.04.202611</t>
+  </si>
+  <si>
+    <t>10.04.202612</t>
+  </si>
+  <si>
+    <t>10.04.202613</t>
+  </si>
+  <si>
+    <t>10.04.202614</t>
+  </si>
+  <si>
+    <t>10.04.202615</t>
+  </si>
+  <si>
+    <t>10.04.202616</t>
+  </si>
+  <si>
+    <t>10.04.202617</t>
+  </si>
+  <si>
+    <t>10.04.202618</t>
+  </si>
+  <si>
+    <t>10.04.202619</t>
+  </si>
+  <si>
+    <t>10.04.202620</t>
+  </si>
+  <si>
+    <t>10.04.202621</t>
+  </si>
+  <si>
+    <t>10.04.202622</t>
+  </si>
+  <si>
+    <t>10.04.202623</t>
+  </si>
+  <si>
+    <t>10.04.202624</t>
+  </si>
+  <si>
+    <t>11.04.20261</t>
+  </si>
+  <si>
+    <t>11.04.20262</t>
+  </si>
+  <si>
+    <t>11.04.20263</t>
+  </si>
+  <si>
+    <t>11.04.20264</t>
+  </si>
+  <si>
+    <t>11.04.20265</t>
+  </si>
+  <si>
+    <t>11.04.20266</t>
+  </si>
+  <si>
+    <t>11.04.20267</t>
+  </si>
+  <si>
+    <t>11.04.20268</t>
+  </si>
+  <si>
+    <t>11.04.20269</t>
+  </si>
+  <si>
+    <t>11.04.202610</t>
+  </si>
+  <si>
+    <t>11.04.202611</t>
+  </si>
+  <si>
+    <t>11.04.202612</t>
+  </si>
+  <si>
+    <t>11.04.202613</t>
+  </si>
+  <si>
+    <t>11.04.202614</t>
+  </si>
+  <si>
+    <t>11.04.202615</t>
+  </si>
+  <si>
+    <t>11.04.202616</t>
+  </si>
+  <si>
+    <t>11.04.202617</t>
+  </si>
+  <si>
+    <t>11.04.202618</t>
+  </si>
+  <si>
+    <t>11.04.202619</t>
+  </si>
+  <si>
+    <t>11.04.202620</t>
+  </si>
+  <si>
+    <t>11.04.202621</t>
+  </si>
+  <si>
+    <t>11.04.202622</t>
+  </si>
+  <si>
+    <t>11.04.202623</t>
+  </si>
+  <si>
+    <t>11.04.202624</t>
+  </si>
+  <si>
+    <t>12.04.20261</t>
+  </si>
+  <si>
+    <t>12.04.20262</t>
+  </si>
+  <si>
+    <t>12.04.20263</t>
+  </si>
+  <si>
+    <t>12.04.20264</t>
+  </si>
+  <si>
+    <t>12.04.20265</t>
+  </si>
+  <si>
+    <t>12.04.20266</t>
+  </si>
+  <si>
+    <t>12.04.20267</t>
+  </si>
+  <si>
+    <t>12.04.20268</t>
+  </si>
+  <si>
+    <t>12.04.20269</t>
+  </si>
+  <si>
+    <t>12.04.202610</t>
+  </si>
+  <si>
+    <t>12.04.202611</t>
+  </si>
+  <si>
+    <t>12.04.202612</t>
+  </si>
+  <si>
+    <t>12.04.202613</t>
+  </si>
+  <si>
+    <t>12.04.202614</t>
+  </si>
+  <si>
+    <t>12.04.202615</t>
+  </si>
+  <si>
+    <t>12.04.202616</t>
+  </si>
+  <si>
+    <t>12.04.202617</t>
+  </si>
+  <si>
+    <t>12.04.202618</t>
+  </si>
+  <si>
+    <t>12.04.202619</t>
+  </si>
+  <si>
+    <t>12.04.202620</t>
+  </si>
+  <si>
+    <t>12.04.202621</t>
+  </si>
+  <si>
+    <t>12.04.202622</t>
+  </si>
+  <si>
+    <t>12.04.202623</t>
+  </si>
+  <si>
+    <t>12.04.202624</t>
+  </si>
+  <si>
+    <t>13.04.20261</t>
+  </si>
+  <si>
+    <t>13.04.20262</t>
+  </si>
+  <si>
+    <t>13.04.20263</t>
+  </si>
+  <si>
+    <t>13.04.20264</t>
+  </si>
+  <si>
+    <t>13.04.20265</t>
+  </si>
+  <si>
+    <t>13.04.20266</t>
+  </si>
+  <si>
+    <t>13.04.20267</t>
+  </si>
+  <si>
+    <t>13.04.20268</t>
+  </si>
+  <si>
+    <t>13.04.20269</t>
+  </si>
+  <si>
+    <t>13.04.202610</t>
+  </si>
+  <si>
+    <t>13.04.202611</t>
+  </si>
+  <si>
+    <t>13.04.202612</t>
+  </si>
+  <si>
+    <t>13.04.202613</t>
+  </si>
+  <si>
+    <t>13.04.202614</t>
+  </si>
+  <si>
+    <t>13.04.202615</t>
+  </si>
+  <si>
+    <t>13.04.202616</t>
+  </si>
+  <si>
+    <t>13.04.202617</t>
+  </si>
+  <si>
+    <t>13.04.202618</t>
+  </si>
+  <si>
+    <t>13.04.202619</t>
+  </si>
+  <si>
+    <t>13.04.202620</t>
+  </si>
+  <si>
+    <t>13.04.202621</t>
+  </si>
+  <si>
+    <t>13.04.202622</t>
+  </si>
+  <si>
+    <t>13.04.202623</t>
+  </si>
+  <si>
+    <t>13.04.202624</t>
+  </si>
+  <si>
+    <t>14.04.20261</t>
+  </si>
+  <si>
+    <t>14.04.20262</t>
+  </si>
+  <si>
+    <t>14.04.20263</t>
+  </si>
+  <si>
+    <t>14.04.20264</t>
+  </si>
+  <si>
+    <t>14.04.20265</t>
+  </si>
+  <si>
+    <t>14.04.20266</t>
+  </si>
+  <si>
+    <t>14.04.20267</t>
+  </si>
+  <si>
+    <t>14.04.20268</t>
+  </si>
+  <si>
+    <t>14.04.20269</t>
+  </si>
+  <si>
+    <t>14.04.202610</t>
+  </si>
+  <si>
+    <t>14.04.202611</t>
+  </si>
+  <si>
+    <t>14.04.202612</t>
+  </si>
+  <si>
+    <t>14.04.202613</t>
+  </si>
+  <si>
+    <t>14.04.202614</t>
+  </si>
+  <si>
+    <t>14.04.202615</t>
+  </si>
+  <si>
+    <t>14.04.202616</t>
+  </si>
+  <si>
+    <t>14.04.202617</t>
+  </si>
+  <si>
+    <t>14.04.202618</t>
+  </si>
+  <si>
+    <t>14.04.202619</t>
+  </si>
+  <si>
+    <t>14.04.202620</t>
+  </si>
+  <si>
+    <t>14.04.202621</t>
+  </si>
+  <si>
+    <t>14.04.202622</t>
+  </si>
+  <si>
+    <t>14.04.202623</t>
+  </si>
+  <si>
+    <t>14.04.202624</t>
+  </si>
+  <si>
+    <t>15.04.20261</t>
+  </si>
+  <si>
+    <t>15.04.20262</t>
+  </si>
+  <si>
+    <t>15.04.20263</t>
+  </si>
+  <si>
+    <t>15.04.20264</t>
+  </si>
+  <si>
+    <t>15.04.20265</t>
+  </si>
+  <si>
+    <t>15.04.20266</t>
+  </si>
+  <si>
+    <t>15.04.20267</t>
+  </si>
+  <si>
+    <t>15.04.20268</t>
+  </si>
+  <si>
+    <t>15.04.20269</t>
+  </si>
+  <si>
+    <t>15.04.202610</t>
+  </si>
+  <si>
+    <t>15.04.202611</t>
+  </si>
+  <si>
+    <t>15.04.202612</t>
+  </si>
+  <si>
+    <t>15.04.202613</t>
+  </si>
+  <si>
+    <t>15.04.202614</t>
+  </si>
+  <si>
+    <t>15.04.202615</t>
+  </si>
+  <si>
+    <t>15.04.202616</t>
+  </si>
+  <si>
+    <t>15.04.202617</t>
+  </si>
+  <si>
+    <t>15.04.202618</t>
+  </si>
+  <si>
+    <t>15.04.202619</t>
+  </si>
+  <si>
+    <t>15.04.202620</t>
+  </si>
+  <si>
+    <t>15.04.202621</t>
+  </si>
+  <si>
+    <t>15.04.202622</t>
+  </si>
+  <si>
+    <t>15.04.202623</t>
+  </si>
+  <si>
+    <t>15.04.202624</t>
+  </si>
+  <si>
+    <t>16.04.20261</t>
+  </si>
+  <si>
+    <t>16.04.20262</t>
+  </si>
+  <si>
+    <t>16.04.20263</t>
+  </si>
+  <si>
+    <t>16.04.20264</t>
+  </si>
+  <si>
+    <t>16.04.20265</t>
+  </si>
+  <si>
+    <t>16.04.20266</t>
+  </si>
+  <si>
+    <t>16.04.20267</t>
+  </si>
+  <si>
+    <t>16.04.20268</t>
+  </si>
+  <si>
+    <t>16.04.20269</t>
+  </si>
+  <si>
+    <t>16.04.202610</t>
+  </si>
+  <si>
+    <t>16.04.202611</t>
+  </si>
+  <si>
+    <t>16.04.202612</t>
+  </si>
+  <si>
+    <t>16.04.202613</t>
+  </si>
+  <si>
+    <t>16.04.202614</t>
+  </si>
+  <si>
+    <t>16.04.202615</t>
+  </si>
+  <si>
+    <t>16.04.202616</t>
+  </si>
+  <si>
+    <t>16.04.202617</t>
+  </si>
+  <si>
+    <t>16.04.202618</t>
+  </si>
+  <si>
+    <t>16.04.202619</t>
+  </si>
+  <si>
+    <t>16.04.202620</t>
+  </si>
+  <si>
+    <t>16.04.202621</t>
+  </si>
+  <si>
+    <t>16.04.202622</t>
+  </si>
+  <si>
+    <t>16.04.202623</t>
+  </si>
+  <si>
+    <t>16.04.202624</t>
+  </si>
+  <si>
+    <t>17.04.20261</t>
+  </si>
+  <si>
+    <t>17.04.20262</t>
+  </si>
+  <si>
+    <t>17.04.20263</t>
+  </si>
+  <si>
+    <t>17.04.20264</t>
+  </si>
+  <si>
+    <t>17.04.20265</t>
+  </si>
+  <si>
+    <t>17.04.20266</t>
+  </si>
+  <si>
+    <t>17.04.20267</t>
+  </si>
+  <si>
+    <t>17.04.20268</t>
+  </si>
+  <si>
+    <t>17.04.20269</t>
+  </si>
+  <si>
+    <t>17.04.202610</t>
   </si>
 </sst>
 </file>
@@ -913,10 +913,10 @@
     </row>
     <row r="2" spans="1:4">
       <c r="A2" s="2">
-        <v>46111</v>
+        <v>46122</v>
       </c>
       <c r="B2">
-        <v>21</v>
+        <v>10</v>
       </c>
       <c r="C2">
         <v>0</v>
@@ -927,10 +927,10 @@
     </row>
     <row r="3" spans="1:4">
       <c r="A3" s="2">
-        <v>46111</v>
+        <v>46122</v>
       </c>
       <c r="B3">
-        <v>22</v>
+        <v>11</v>
       </c>
       <c r="C3">
         <v>0</v>
@@ -941,13 +941,13 @@
     </row>
     <row r="4" spans="1:4">
       <c r="A4" s="2">
-        <v>46111</v>
+        <v>46122</v>
       </c>
       <c r="B4">
-        <v>23</v>
+        <v>12</v>
       </c>
       <c r="C4">
-        <v>0</v>
+        <v>3.238</v>
       </c>
       <c r="D4" t="s">
         <v>6</v>
@@ -955,13 +955,13 @@
     </row>
     <row r="5" spans="1:4">
       <c r="A5" s="2">
-        <v>46111</v>
+        <v>46122</v>
       </c>
       <c r="B5">
-        <v>24</v>
+        <v>13</v>
       </c>
       <c r="C5">
-        <v>0</v>
+        <v>2.961</v>
       </c>
       <c r="D5" t="s">
         <v>7</v>
@@ -969,13 +969,13 @@
     </row>
     <row r="6" spans="1:4">
       <c r="A6" s="2">
-        <v>46112</v>
+        <v>46122</v>
       </c>
       <c r="B6">
-        <v>1</v>
+        <v>14</v>
       </c>
       <c r="C6">
-        <v>0</v>
+        <v>2.632</v>
       </c>
       <c r="D6" t="s">
         <v>8</v>
@@ -983,13 +983,13 @@
     </row>
     <row r="7" spans="1:4">
       <c r="A7" s="2">
-        <v>46112</v>
+        <v>46122</v>
       </c>
       <c r="B7">
-        <v>2</v>
+        <v>15</v>
       </c>
       <c r="C7">
-        <v>0</v>
+        <v>2.421</v>
       </c>
       <c r="D7" t="s">
         <v>9</v>
@@ -997,13 +997,13 @@
     </row>
     <row r="8" spans="1:4">
       <c r="A8" s="2">
-        <v>46112</v>
+        <v>46122</v>
       </c>
       <c r="B8">
-        <v>3</v>
+        <v>16</v>
       </c>
       <c r="C8">
-        <v>0</v>
+        <v>1.856</v>
       </c>
       <c r="D8" t="s">
         <v>10</v>
@@ -1011,13 +1011,13 @@
     </row>
     <row r="9" spans="1:4">
       <c r="A9" s="2">
-        <v>46112</v>
+        <v>46122</v>
       </c>
       <c r="B9">
-        <v>4</v>
+        <v>17</v>
       </c>
       <c r="C9">
-        <v>0</v>
+        <v>1.687</v>
       </c>
       <c r="D9" t="s">
         <v>11</v>
@@ -1025,13 +1025,13 @@
     </row>
     <row r="10" spans="1:4">
       <c r="A10" s="2">
-        <v>46112</v>
+        <v>46122</v>
       </c>
       <c r="B10">
-        <v>5</v>
+        <v>18</v>
       </c>
       <c r="C10">
-        <v>0</v>
+        <v>1.091</v>
       </c>
       <c r="D10" t="s">
         <v>12</v>
@@ -1039,13 +1039,13 @@
     </row>
     <row r="11" spans="1:4">
       <c r="A11" s="2">
-        <v>46112</v>
+        <v>46122</v>
       </c>
       <c r="B11">
-        <v>6</v>
+        <v>19</v>
       </c>
       <c r="C11">
-        <v>0</v>
+        <v>0.438</v>
       </c>
       <c r="D11" t="s">
         <v>13</v>
@@ -1053,13 +1053,13 @@
     </row>
     <row r="12" spans="1:4">
       <c r="A12" s="2">
-        <v>46112</v>
+        <v>46122</v>
       </c>
       <c r="B12">
-        <v>7</v>
+        <v>20</v>
       </c>
       <c r="C12">
-        <v>0</v>
+        <v>0.06900000000000001</v>
       </c>
       <c r="D12" t="s">
         <v>14</v>
@@ -1067,13 +1067,13 @@
     </row>
     <row r="13" spans="1:4">
       <c r="A13" s="2">
-        <v>46112</v>
+        <v>46122</v>
       </c>
       <c r="B13">
-        <v>8</v>
+        <v>21</v>
       </c>
       <c r="C13">
-        <v>0.021</v>
+        <v>0</v>
       </c>
       <c r="D13" t="s">
         <v>15</v>
@@ -1081,13 +1081,13 @@
     </row>
     <row r="14" spans="1:4">
       <c r="A14" s="2">
-        <v>46112</v>
+        <v>46122</v>
       </c>
       <c r="B14">
-        <v>9</v>
+        <v>22</v>
       </c>
       <c r="C14">
-        <v>0.218</v>
+        <v>0</v>
       </c>
       <c r="D14" t="s">
         <v>16</v>
@@ -1095,13 +1095,13 @@
     </row>
     <row r="15" spans="1:4">
       <c r="A15" s="2">
-        <v>46112</v>
+        <v>46122</v>
       </c>
       <c r="B15">
-        <v>10</v>
+        <v>23</v>
       </c>
       <c r="C15">
-        <v>0.414</v>
+        <v>0</v>
       </c>
       <c r="D15" t="s">
         <v>17</v>
@@ -1109,13 +1109,13 @@
     </row>
     <row r="16" spans="1:4">
       <c r="A16" s="2">
-        <v>46112</v>
+        <v>46122</v>
       </c>
       <c r="B16">
-        <v>11</v>
+        <v>24</v>
       </c>
       <c r="C16">
-        <v>0.641</v>
+        <v>0</v>
       </c>
       <c r="D16" t="s">
         <v>18</v>
@@ -1123,13 +1123,13 @@
     </row>
     <row r="17" spans="1:4">
       <c r="A17" s="2">
-        <v>46112</v>
+        <v>46123</v>
       </c>
       <c r="B17">
-        <v>12</v>
+        <v>1</v>
       </c>
       <c r="C17">
-        <v>0.768</v>
+        <v>0</v>
       </c>
       <c r="D17" t="s">
         <v>19</v>
@@ -1137,13 +1137,13 @@
     </row>
     <row r="18" spans="1:4">
       <c r="A18" s="2">
-        <v>46112</v>
+        <v>46123</v>
       </c>
       <c r="B18">
-        <v>13</v>
+        <v>2</v>
       </c>
       <c r="C18">
-        <v>0.971</v>
+        <v>0</v>
       </c>
       <c r="D18" t="s">
         <v>20</v>
@@ -1151,13 +1151,13 @@
     </row>
     <row r="19" spans="1:4">
       <c r="A19" s="2">
-        <v>46112</v>
+        <v>46123</v>
       </c>
       <c r="B19">
-        <v>14</v>
+        <v>3</v>
       </c>
       <c r="C19">
-        <v>1.098</v>
+        <v>0</v>
       </c>
       <c r="D19" t="s">
         <v>21</v>
@@ -1165,13 +1165,13 @@
     </row>
     <row r="20" spans="1:4">
       <c r="A20" s="2">
-        <v>46112</v>
+        <v>46123</v>
       </c>
       <c r="B20">
-        <v>15</v>
+        <v>4</v>
       </c>
       <c r="C20">
-        <v>1.042</v>
+        <v>0</v>
       </c>
       <c r="D20" t="s">
         <v>22</v>
@@ -1179,13 +1179,13 @@
     </row>
     <row r="21" spans="1:4">
       <c r="A21" s="2">
-        <v>46112</v>
+        <v>46123</v>
       </c>
       <c r="B21">
-        <v>16</v>
+        <v>5</v>
       </c>
       <c r="C21">
-        <v>0.975</v>
+        <v>0</v>
       </c>
       <c r="D21" t="s">
         <v>23</v>
@@ -1193,13 +1193,13 @@
     </row>
     <row r="22" spans="1:4">
       <c r="A22" s="2">
-        <v>46112</v>
+        <v>46123</v>
       </c>
       <c r="B22">
-        <v>17</v>
+        <v>6</v>
       </c>
       <c r="C22">
-        <v>0.6830000000000001</v>
+        <v>0</v>
       </c>
       <c r="D22" t="s">
         <v>24</v>
@@ -1207,13 +1207,13 @@
     </row>
     <row r="23" spans="1:4">
       <c r="A23" s="2">
-        <v>46112</v>
+        <v>46123</v>
       </c>
       <c r="B23">
-        <v>18</v>
+        <v>7</v>
       </c>
       <c r="C23">
-        <v>0.352</v>
+        <v>0</v>
       </c>
       <c r="D23" t="s">
         <v>25</v>
@@ -1221,13 +1221,13 @@
     </row>
     <row r="24" spans="1:4">
       <c r="A24" s="2">
-        <v>46112</v>
+        <v>46123</v>
       </c>
       <c r="B24">
-        <v>19</v>
+        <v>8</v>
       </c>
       <c r="C24">
-        <v>0.146</v>
+        <v>0.154</v>
       </c>
       <c r="D24" t="s">
         <v>26</v>
@@ -1235,13 +1235,13 @@
     </row>
     <row r="25" spans="1:4">
       <c r="A25" s="2">
-        <v>46112</v>
+        <v>46123</v>
       </c>
       <c r="B25">
-        <v>20</v>
+        <v>9</v>
       </c>
       <c r="C25">
-        <v>0.012</v>
+        <v>0.6909999999999999</v>
       </c>
       <c r="D25" t="s">
         <v>27</v>
@@ -1249,13 +1249,13 @@
     </row>
     <row r="26" spans="1:4">
       <c r="A26" s="2">
-        <v>46112</v>
+        <v>46123</v>
       </c>
       <c r="B26">
-        <v>21</v>
+        <v>10</v>
       </c>
       <c r="C26">
-        <v>0</v>
+        <v>1.175</v>
       </c>
       <c r="D26" t="s">
         <v>28</v>
@@ -1263,13 +1263,13 @@
     </row>
     <row r="27" spans="1:4">
       <c r="A27" s="2">
-        <v>46112</v>
+        <v>46123</v>
       </c>
       <c r="B27">
-        <v>22</v>
+        <v>11</v>
       </c>
       <c r="C27">
-        <v>0</v>
+        <v>1.871</v>
       </c>
       <c r="D27" t="s">
         <v>29</v>
@@ -1277,13 +1277,13 @@
     </row>
     <row r="28" spans="1:4">
       <c r="A28" s="2">
-        <v>46112</v>
+        <v>46123</v>
       </c>
       <c r="B28">
-        <v>23</v>
+        <v>12</v>
       </c>
       <c r="C28">
-        <v>0</v>
+        <v>2.031</v>
       </c>
       <c r="D28" t="s">
         <v>30</v>
@@ -1291,13 +1291,13 @@
     </row>
     <row r="29" spans="1:4">
       <c r="A29" s="2">
-        <v>46112</v>
+        <v>46123</v>
       </c>
       <c r="B29">
-        <v>24</v>
+        <v>13</v>
       </c>
       <c r="C29">
-        <v>0</v>
+        <v>2.02</v>
       </c>
       <c r="D29" t="s">
         <v>31</v>
@@ -1305,13 +1305,13 @@
     </row>
     <row r="30" spans="1:4">
       <c r="A30" s="2">
-        <v>46113</v>
+        <v>46123</v>
       </c>
       <c r="B30">
-        <v>1</v>
+        <v>14</v>
       </c>
       <c r="C30">
-        <v>0</v>
+        <v>2.062</v>
       </c>
       <c r="D30" t="s">
         <v>32</v>
@@ -1319,13 +1319,13 @@
     </row>
     <row r="31" spans="1:4">
       <c r="A31" s="2">
-        <v>46113</v>
+        <v>46123</v>
       </c>
       <c r="B31">
-        <v>2</v>
+        <v>15</v>
       </c>
       <c r="C31">
-        <v>0</v>
+        <v>1.985</v>
       </c>
       <c r="D31" t="s">
         <v>33</v>
@@ -1333,13 +1333,13 @@
     </row>
     <row r="32" spans="1:4">
       <c r="A32" s="2">
-        <v>46113</v>
+        <v>46123</v>
       </c>
       <c r="B32">
-        <v>3</v>
+        <v>16</v>
       </c>
       <c r="C32">
-        <v>0</v>
+        <v>1.934</v>
       </c>
       <c r="D32" t="s">
         <v>34</v>
@@ -1347,13 +1347,13 @@
     </row>
     <row r="33" spans="1:4">
       <c r="A33" s="2">
-        <v>46113</v>
+        <v>46123</v>
       </c>
       <c r="B33">
-        <v>4</v>
+        <v>17</v>
       </c>
       <c r="C33">
-        <v>0</v>
+        <v>1.532</v>
       </c>
       <c r="D33" t="s">
         <v>35</v>
@@ -1361,13 +1361,13 @@
     </row>
     <row r="34" spans="1:4">
       <c r="A34" s="2">
-        <v>46113</v>
+        <v>46123</v>
       </c>
       <c r="B34">
-        <v>5</v>
+        <v>18</v>
       </c>
       <c r="C34">
-        <v>0</v>
+        <v>0.901</v>
       </c>
       <c r="D34" t="s">
         <v>36</v>
@@ -1375,13 +1375,13 @@
     </row>
     <row r="35" spans="1:4">
       <c r="A35" s="2">
-        <v>46113</v>
+        <v>46123</v>
       </c>
       <c r="B35">
-        <v>6</v>
+        <v>19</v>
       </c>
       <c r="C35">
-        <v>0</v>
+        <v>0.395</v>
       </c>
       <c r="D35" t="s">
         <v>37</v>
@@ -1389,13 +1389,13 @@
     </row>
     <row r="36" spans="1:4">
       <c r="A36" s="2">
-        <v>46113</v>
+        <v>46123</v>
       </c>
       <c r="B36">
-        <v>7</v>
+        <v>20</v>
       </c>
       <c r="C36">
-        <v>0</v>
+        <v>0.061</v>
       </c>
       <c r="D36" t="s">
         <v>38</v>
@@ -1403,13 +1403,13 @@
     </row>
     <row r="37" spans="1:4">
       <c r="A37" s="2">
-        <v>46113</v>
+        <v>46123</v>
       </c>
       <c r="B37">
-        <v>8</v>
+        <v>21</v>
       </c>
       <c r="C37">
-        <v>0.045</v>
+        <v>0</v>
       </c>
       <c r="D37" t="s">
         <v>39</v>
@@ -1417,13 +1417,13 @@
     </row>
     <row r="38" spans="1:4">
       <c r="A38" s="2">
-        <v>46113</v>
+        <v>46123</v>
       </c>
       <c r="B38">
-        <v>9</v>
+        <v>22</v>
       </c>
       <c r="C38">
-        <v>0.523</v>
+        <v>0</v>
       </c>
       <c r="D38" t="s">
         <v>40</v>
@@ -1431,13 +1431,13 @@
     </row>
     <row r="39" spans="1:4">
       <c r="A39" s="2">
-        <v>46113</v>
+        <v>46123</v>
       </c>
       <c r="B39">
-        <v>10</v>
+        <v>23</v>
       </c>
       <c r="C39">
-        <v>0.903</v>
+        <v>0</v>
       </c>
       <c r="D39" t="s">
         <v>41</v>
@@ -1445,13 +1445,13 @@
     </row>
     <row r="40" spans="1:4">
       <c r="A40" s="2">
-        <v>46113</v>
+        <v>46123</v>
       </c>
       <c r="B40">
-        <v>11</v>
+        <v>24</v>
       </c>
       <c r="C40">
-        <v>1.642</v>
+        <v>0</v>
       </c>
       <c r="D40" t="s">
         <v>42</v>
@@ -1459,13 +1459,13 @@
     </row>
     <row r="41" spans="1:4">
       <c r="A41" s="2">
-        <v>46113</v>
+        <v>46124</v>
       </c>
       <c r="B41">
-        <v>12</v>
+        <v>1</v>
       </c>
       <c r="C41">
-        <v>2.034</v>
+        <v>0</v>
       </c>
       <c r="D41" t="s">
         <v>43</v>
@@ -1473,13 +1473,13 @@
     </row>
     <row r="42" spans="1:4">
       <c r="A42" s="2">
-        <v>46113</v>
+        <v>46124</v>
       </c>
       <c r="B42">
-        <v>13</v>
+        <v>2</v>
       </c>
       <c r="C42">
-        <v>2.206</v>
+        <v>0</v>
       </c>
       <c r="D42" t="s">
         <v>44</v>
@@ -1487,13 +1487,13 @@
     </row>
     <row r="43" spans="1:4">
       <c r="A43" s="2">
-        <v>46113</v>
+        <v>46124</v>
       </c>
       <c r="B43">
-        <v>14</v>
+        <v>3</v>
       </c>
       <c r="C43">
-        <v>2.314</v>
+        <v>0</v>
       </c>
       <c r="D43" t="s">
         <v>45</v>
@@ -1501,13 +1501,13 @@
     </row>
     <row r="44" spans="1:4">
       <c r="A44" s="2">
-        <v>46113</v>
+        <v>46124</v>
       </c>
       <c r="B44">
-        <v>15</v>
+        <v>4</v>
       </c>
       <c r="C44">
-        <v>2.153</v>
+        <v>0</v>
       </c>
       <c r="D44" t="s">
         <v>46</v>
@@ -1515,13 +1515,13 @@
     </row>
     <row r="45" spans="1:4">
       <c r="A45" s="2">
-        <v>46113</v>
+        <v>46124</v>
       </c>
       <c r="B45">
-        <v>16</v>
+        <v>5</v>
       </c>
       <c r="C45">
-        <v>1.691</v>
+        <v>0</v>
       </c>
       <c r="D45" t="s">
         <v>47</v>
@@ -1529,13 +1529,13 @@
     </row>
     <row r="46" spans="1:4">
       <c r="A46" s="2">
-        <v>46113</v>
+        <v>46124</v>
       </c>
       <c r="B46">
-        <v>17</v>
+        <v>6</v>
       </c>
       <c r="C46">
-        <v>1.179</v>
+        <v>0</v>
       </c>
       <c r="D46" t="s">
         <v>48</v>
@@ -1543,13 +1543,13 @@
     </row>
     <row r="47" spans="1:4">
       <c r="A47" s="2">
-        <v>46113</v>
+        <v>46124</v>
       </c>
       <c r="B47">
-        <v>18</v>
+        <v>7</v>
       </c>
       <c r="C47">
-        <v>0.774</v>
+        <v>0</v>
       </c>
       <c r="D47" t="s">
         <v>49</v>
@@ -1557,13 +1557,13 @@
     </row>
     <row r="48" spans="1:4">
       <c r="A48" s="2">
-        <v>46113</v>
+        <v>46124</v>
       </c>
       <c r="B48">
-        <v>19</v>
+        <v>8</v>
       </c>
       <c r="C48">
-        <v>0.292</v>
+        <v>0.19</v>
       </c>
       <c r="D48" t="s">
         <v>50</v>
@@ -1571,13 +1571,13 @@
     </row>
     <row r="49" spans="1:4">
       <c r="A49" s="2">
-        <v>46113</v>
+        <v>46124</v>
       </c>
       <c r="B49">
-        <v>20</v>
+        <v>9</v>
       </c>
       <c r="C49">
-        <v>0.026</v>
+        <v>0.9330000000000001</v>
       </c>
       <c r="D49" t="s">
         <v>51</v>
@@ -1585,13 +1585,13 @@
     </row>
     <row r="50" spans="1:4">
       <c r="A50" s="2">
-        <v>46113</v>
+        <v>46124</v>
       </c>
       <c r="B50">
-        <v>21</v>
+        <v>10</v>
       </c>
       <c r="C50">
-        <v>0</v>
+        <v>1.932</v>
       </c>
       <c r="D50" t="s">
         <v>52</v>
@@ -1599,13 +1599,13 @@
     </row>
     <row r="51" spans="1:4">
       <c r="A51" s="2">
-        <v>46113</v>
+        <v>46124</v>
       </c>
       <c r="B51">
-        <v>22</v>
+        <v>11</v>
       </c>
       <c r="C51">
-        <v>0</v>
+        <v>2.694</v>
       </c>
       <c r="D51" t="s">
         <v>53</v>
@@ -1613,13 +1613,13 @@
     </row>
     <row r="52" spans="1:4">
       <c r="A52" s="2">
-        <v>46113</v>
+        <v>46124</v>
       </c>
       <c r="B52">
-        <v>23</v>
+        <v>12</v>
       </c>
       <c r="C52">
-        <v>0</v>
+        <v>3.077</v>
       </c>
       <c r="D52" t="s">
         <v>54</v>
@@ -1627,13 +1627,13 @@
     </row>
     <row r="53" spans="1:4">
       <c r="A53" s="2">
-        <v>46113</v>
+        <v>46124</v>
       </c>
       <c r="B53">
-        <v>24</v>
+        <v>13</v>
       </c>
       <c r="C53">
-        <v>0</v>
+        <v>3.132</v>
       </c>
       <c r="D53" t="s">
         <v>55</v>
@@ -1641,13 +1641,13 @@
     </row>
     <row r="54" spans="1:4">
       <c r="A54" s="2">
-        <v>46114</v>
+        <v>46124</v>
       </c>
       <c r="B54">
-        <v>1</v>
+        <v>14</v>
       </c>
       <c r="C54">
-        <v>0</v>
+        <v>3.161</v>
       </c>
       <c r="D54" t="s">
         <v>56</v>
@@ -1655,13 +1655,13 @@
     </row>
     <row r="55" spans="1:4">
       <c r="A55" s="2">
-        <v>46114</v>
+        <v>46124</v>
       </c>
       <c r="B55">
-        <v>2</v>
+        <v>15</v>
       </c>
       <c r="C55">
-        <v>0</v>
+        <v>3.048</v>
       </c>
       <c r="D55" t="s">
         <v>57</v>
@@ -1669,13 +1669,13 @@
     </row>
     <row r="56" spans="1:4">
       <c r="A56" s="2">
-        <v>46114</v>
+        <v>46124</v>
       </c>
       <c r="B56">
-        <v>3</v>
+        <v>16</v>
       </c>
       <c r="C56">
-        <v>0</v>
+        <v>2.632</v>
       </c>
       <c r="D56" t="s">
         <v>58</v>
@@ -1683,13 +1683,13 @@
     </row>
     <row r="57" spans="1:4">
       <c r="A57" s="2">
-        <v>46114</v>
+        <v>46124</v>
       </c>
       <c r="B57">
-        <v>4</v>
+        <v>17</v>
       </c>
       <c r="C57">
-        <v>0</v>
+        <v>2.25</v>
       </c>
       <c r="D57" t="s">
         <v>59</v>
@@ -1697,13 +1697,13 @@
     </row>
     <row r="58" spans="1:4">
       <c r="A58" s="2">
-        <v>46114</v>
+        <v>46124</v>
       </c>
       <c r="B58">
-        <v>5</v>
+        <v>18</v>
       </c>
       <c r="C58">
-        <v>0</v>
+        <v>1.471</v>
       </c>
       <c r="D58" t="s">
         <v>60</v>
@@ -1711,13 +1711,13 @@
     </row>
     <row r="59" spans="1:4">
       <c r="A59" s="2">
-        <v>46114</v>
+        <v>46124</v>
       </c>
       <c r="B59">
-        <v>6</v>
+        <v>19</v>
       </c>
       <c r="C59">
-        <v>0</v>
+        <v>0.523</v>
       </c>
       <c r="D59" t="s">
         <v>61</v>
@@ -1725,13 +1725,13 @@
     </row>
     <row r="60" spans="1:4">
       <c r="A60" s="2">
-        <v>46114</v>
+        <v>46124</v>
       </c>
       <c r="B60">
-        <v>7</v>
+        <v>20</v>
       </c>
       <c r="C60">
-        <v>0</v>
+        <v>0.066</v>
       </c>
       <c r="D60" t="s">
         <v>62</v>
@@ -1739,13 +1739,13 @@
     </row>
     <row r="61" spans="1:4">
       <c r="A61" s="2">
-        <v>46114</v>
+        <v>46124</v>
       </c>
       <c r="B61">
-        <v>8</v>
+        <v>21</v>
       </c>
       <c r="C61">
-        <v>0.066</v>
+        <v>0</v>
       </c>
       <c r="D61" t="s">
         <v>63</v>
@@ -1753,13 +1753,13 @@
     </row>
     <row r="62" spans="1:4">
       <c r="A62" s="2">
-        <v>46114</v>
+        <v>46124</v>
       </c>
       <c r="B62">
-        <v>9</v>
+        <v>22</v>
       </c>
       <c r="C62">
-        <v>0.646</v>
+        <v>0</v>
       </c>
       <c r="D62" t="s">
         <v>64</v>
@@ -1767,13 +1767,13 @@
     </row>
     <row r="63" spans="1:4">
       <c r="A63" s="2">
-        <v>46114</v>
+        <v>46124</v>
       </c>
       <c r="B63">
-        <v>10</v>
+        <v>23</v>
       </c>
       <c r="C63">
-        <v>1.402</v>
+        <v>0</v>
       </c>
       <c r="D63" t="s">
         <v>65</v>
@@ -1781,13 +1781,13 @@
     </row>
     <row r="64" spans="1:4">
       <c r="A64" s="2">
-        <v>46114</v>
+        <v>46124</v>
       </c>
       <c r="B64">
-        <v>11</v>
+        <v>24</v>
       </c>
       <c r="C64">
-        <v>1.99</v>
+        <v>0</v>
       </c>
       <c r="D64" t="s">
         <v>66</v>
@@ -1795,13 +1795,13 @@
     </row>
     <row r="65" spans="1:4">
       <c r="A65" s="2">
-        <v>46114</v>
+        <v>46125</v>
       </c>
       <c r="B65">
-        <v>12</v>
+        <v>1</v>
       </c>
       <c r="C65">
-        <v>2.3</v>
+        <v>0</v>
       </c>
       <c r="D65" t="s">
         <v>67</v>
@@ -1809,13 +1809,13 @@
     </row>
     <row r="66" spans="1:4">
       <c r="A66" s="2">
-        <v>46114</v>
+        <v>46125</v>
       </c>
       <c r="B66">
-        <v>13</v>
+        <v>2</v>
       </c>
       <c r="C66">
-        <v>2.26</v>
+        <v>0</v>
       </c>
       <c r="D66" t="s">
         <v>68</v>
@@ -1823,13 +1823,13 @@
     </row>
     <row r="67" spans="1:4">
       <c r="A67" s="2">
-        <v>46114</v>
+        <v>46125</v>
       </c>
       <c r="B67">
-        <v>14</v>
+        <v>3</v>
       </c>
       <c r="C67">
-        <v>2.127</v>
+        <v>0</v>
       </c>
       <c r="D67" t="s">
         <v>69</v>
@@ -1837,13 +1837,13 @@
     </row>
     <row r="68" spans="1:4">
       <c r="A68" s="2">
-        <v>46114</v>
+        <v>46125</v>
       </c>
       <c r="B68">
-        <v>15</v>
+        <v>4</v>
       </c>
       <c r="C68">
-        <v>2.022</v>
+        <v>0</v>
       </c>
       <c r="D68" t="s">
         <v>70</v>
@@ -1851,13 +1851,13 @@
     </row>
     <row r="69" spans="1:4">
       <c r="A69" s="2">
-        <v>46114</v>
+        <v>46125</v>
       </c>
       <c r="B69">
-        <v>16</v>
+        <v>5</v>
       </c>
       <c r="C69">
-        <v>1.766</v>
+        <v>0</v>
       </c>
       <c r="D69" t="s">
         <v>71</v>
@@ -1865,13 +1865,13 @@
     </row>
     <row r="70" spans="1:4">
       <c r="A70" s="2">
-        <v>46114</v>
+        <v>46125</v>
       </c>
       <c r="B70">
-        <v>17</v>
+        <v>6</v>
       </c>
       <c r="C70">
-        <v>1.241</v>
+        <v>0</v>
       </c>
       <c r="D70" t="s">
         <v>72</v>
@@ -1879,13 +1879,13 @@
     </row>
     <row r="71" spans="1:4">
       <c r="A71" s="2">
-        <v>46114</v>
+        <v>46125</v>
       </c>
       <c r="B71">
-        <v>18</v>
+        <v>7</v>
       </c>
       <c r="C71">
-        <v>0.73</v>
+        <v>0</v>
       </c>
       <c r="D71" t="s">
         <v>73</v>
@@ -1893,13 +1893,13 @@
     </row>
     <row r="72" spans="1:4">
       <c r="A72" s="2">
-        <v>46114</v>
+        <v>46125</v>
       </c>
       <c r="B72">
-        <v>19</v>
+        <v>8</v>
       </c>
       <c r="C72">
-        <v>0.273</v>
+        <v>0.179</v>
       </c>
       <c r="D72" t="s">
         <v>74</v>
@@ -1907,13 +1907,13 @@
     </row>
     <row r="73" spans="1:4">
       <c r="A73" s="2">
-        <v>46114</v>
+        <v>46125</v>
       </c>
       <c r="B73">
-        <v>20</v>
+        <v>9</v>
       </c>
       <c r="C73">
-        <v>0.02</v>
+        <v>0.893</v>
       </c>
       <c r="D73" t="s">
         <v>75</v>
@@ -1921,13 +1921,13 @@
     </row>
     <row r="74" spans="1:4">
       <c r="A74" s="2">
-        <v>46114</v>
+        <v>46125</v>
       </c>
       <c r="B74">
-        <v>21</v>
+        <v>10</v>
       </c>
       <c r="C74">
-        <v>0</v>
+        <v>1.904</v>
       </c>
       <c r="D74" t="s">
         <v>76</v>
@@ -1935,13 +1935,13 @@
     </row>
     <row r="75" spans="1:4">
       <c r="A75" s="2">
-        <v>46114</v>
+        <v>46125</v>
       </c>
       <c r="B75">
-        <v>22</v>
+        <v>11</v>
       </c>
       <c r="C75">
-        <v>0</v>
+        <v>2.608</v>
       </c>
       <c r="D75" t="s">
         <v>77</v>
@@ -1949,13 +1949,13 @@
     </row>
     <row r="76" spans="1:4">
       <c r="A76" s="2">
-        <v>46114</v>
+        <v>46125</v>
       </c>
       <c r="B76">
-        <v>23</v>
+        <v>12</v>
       </c>
       <c r="C76">
-        <v>0</v>
+        <v>3.088</v>
       </c>
       <c r="D76" t="s">
         <v>78</v>
@@ -1963,13 +1963,13 @@
     </row>
     <row r="77" spans="1:4">
       <c r="A77" s="2">
-        <v>46114</v>
+        <v>46125</v>
       </c>
       <c r="B77">
-        <v>24</v>
+        <v>13</v>
       </c>
       <c r="C77">
-        <v>0</v>
+        <v>3.065</v>
       </c>
       <c r="D77" t="s">
         <v>79</v>
@@ -1977,13 +1977,13 @@
     </row>
     <row r="78" spans="1:4">
       <c r="A78" s="2">
-        <v>46115</v>
+        <v>46125</v>
       </c>
       <c r="B78">
-        <v>1</v>
+        <v>14</v>
       </c>
       <c r="C78">
-        <v>0</v>
+        <v>2.974</v>
       </c>
       <c r="D78" t="s">
         <v>80</v>
@@ -1991,13 +1991,13 @@
     </row>
     <row r="79" spans="1:4">
       <c r="A79" s="2">
-        <v>46115</v>
+        <v>46125</v>
       </c>
       <c r="B79">
-        <v>2</v>
+        <v>15</v>
       </c>
       <c r="C79">
-        <v>0</v>
+        <v>2.902</v>
       </c>
       <c r="D79" t="s">
         <v>81</v>
@@ -2005,13 +2005,13 @@
     </row>
     <row r="80" spans="1:4">
       <c r="A80" s="2">
-        <v>46115</v>
+        <v>46125</v>
       </c>
       <c r="B80">
-        <v>3</v>
+        <v>16</v>
       </c>
       <c r="C80">
-        <v>0</v>
+        <v>2.393</v>
       </c>
       <c r="D80" t="s">
         <v>82</v>
@@ -2019,13 +2019,13 @@
     </row>
     <row r="81" spans="1:4">
       <c r="A81" s="2">
-        <v>46115</v>
+        <v>46125</v>
       </c>
       <c r="B81">
-        <v>4</v>
+        <v>17</v>
       </c>
       <c r="C81">
-        <v>0</v>
+        <v>1.987</v>
       </c>
       <c r="D81" t="s">
         <v>83</v>
@@ -2033,13 +2033,13 @@
     </row>
     <row r="82" spans="1:4">
       <c r="A82" s="2">
-        <v>46115</v>
+        <v>46125</v>
       </c>
       <c r="B82">
-        <v>5</v>
+        <v>18</v>
       </c>
       <c r="C82">
-        <v>0</v>
+        <v>1.224</v>
       </c>
       <c r="D82" t="s">
         <v>84</v>
@@ -2047,13 +2047,13 @@
     </row>
     <row r="83" spans="1:4">
       <c r="A83" s="2">
-        <v>46115</v>
+        <v>46125</v>
       </c>
       <c r="B83">
-        <v>6</v>
+        <v>19</v>
       </c>
       <c r="C83">
-        <v>0</v>
+        <v>0.457</v>
       </c>
       <c r="D83" t="s">
         <v>85</v>
@@ -2061,13 +2061,13 @@
     </row>
     <row r="84" spans="1:4">
       <c r="A84" s="2">
-        <v>46115</v>
+        <v>46125</v>
       </c>
       <c r="B84">
-        <v>7</v>
+        <v>20</v>
       </c>
       <c r="C84">
-        <v>0</v>
+        <v>0.067</v>
       </c>
       <c r="D84" t="s">
         <v>86</v>
@@ -2075,13 +2075,13 @@
     </row>
     <row r="85" spans="1:4">
       <c r="A85" s="2">
-        <v>46115</v>
+        <v>46125</v>
       </c>
       <c r="B85">
-        <v>8</v>
+        <v>21</v>
       </c>
       <c r="C85">
-        <v>0.029</v>
+        <v>0</v>
       </c>
       <c r="D85" t="s">
         <v>87</v>
@@ -2089,13 +2089,13 @@
     </row>
     <row r="86" spans="1:4">
       <c r="A86" s="2">
-        <v>46115</v>
+        <v>46125</v>
       </c>
       <c r="B86">
-        <v>9</v>
+        <v>22</v>
       </c>
       <c r="C86">
-        <v>0.274</v>
+        <v>0</v>
       </c>
       <c r="D86" t="s">
         <v>88</v>
@@ -2103,13 +2103,13 @@
     </row>
     <row r="87" spans="1:4">
       <c r="A87" s="2">
-        <v>46115</v>
+        <v>46125</v>
       </c>
       <c r="B87">
-        <v>10</v>
+        <v>23</v>
       </c>
       <c r="C87">
-        <v>0.747</v>
+        <v>0</v>
       </c>
       <c r="D87" t="s">
         <v>89</v>
@@ -2117,13 +2117,13 @@
     </row>
     <row r="88" spans="1:4">
       <c r="A88" s="2">
-        <v>46115</v>
+        <v>46125</v>
       </c>
       <c r="B88">
-        <v>11</v>
+        <v>24</v>
       </c>
       <c r="C88">
-        <v>0.922</v>
+        <v>0</v>
       </c>
       <c r="D88" t="s">
         <v>90</v>
@@ -2131,13 +2131,13 @@
     </row>
     <row r="89" spans="1:4">
       <c r="A89" s="2">
-        <v>46115</v>
+        <v>46126</v>
       </c>
       <c r="B89">
-        <v>12</v>
+        <v>1</v>
       </c>
       <c r="C89">
-        <v>1.261</v>
+        <v>0</v>
       </c>
       <c r="D89" t="s">
         <v>91</v>
@@ -2145,13 +2145,13 @@
     </row>
     <row r="90" spans="1:4">
       <c r="A90" s="2">
-        <v>46115</v>
+        <v>46126</v>
       </c>
       <c r="B90">
-        <v>13</v>
+        <v>2</v>
       </c>
       <c r="C90">
-        <v>1.373</v>
+        <v>0</v>
       </c>
       <c r="D90" t="s">
         <v>92</v>
@@ -2159,13 +2159,13 @@
     </row>
     <row r="91" spans="1:4">
       <c r="A91" s="2">
-        <v>46115</v>
+        <v>46126</v>
       </c>
       <c r="B91">
-        <v>14</v>
+        <v>3</v>
       </c>
       <c r="C91">
-        <v>1.523</v>
+        <v>0</v>
       </c>
       <c r="D91" t="s">
         <v>93</v>
@@ -2173,13 +2173,13 @@
     </row>
     <row r="92" spans="1:4">
       <c r="A92" s="2">
-        <v>46115</v>
+        <v>46126</v>
       </c>
       <c r="B92">
-        <v>15</v>
+        <v>4</v>
       </c>
       <c r="C92">
-        <v>1.474</v>
+        <v>0</v>
       </c>
       <c r="D92" t="s">
         <v>94</v>
@@ -2187,13 +2187,13 @@
     </row>
     <row r="93" spans="1:4">
       <c r="A93" s="2">
-        <v>46115</v>
+        <v>46126</v>
       </c>
       <c r="B93">
-        <v>16</v>
+        <v>5</v>
       </c>
       <c r="C93">
-        <v>1.26</v>
+        <v>0</v>
       </c>
       <c r="D93" t="s">
         <v>95</v>
@@ -2201,13 +2201,13 @@
     </row>
     <row r="94" spans="1:4">
       <c r="A94" s="2">
-        <v>46115</v>
+        <v>46126</v>
       </c>
       <c r="B94">
-        <v>17</v>
+        <v>6</v>
       </c>
       <c r="C94">
-        <v>0.948</v>
+        <v>0</v>
       </c>
       <c r="D94" t="s">
         <v>96</v>
@@ -2215,13 +2215,13 @@
     </row>
     <row r="95" spans="1:4">
       <c r="A95" s="2">
-        <v>46115</v>
+        <v>46126</v>
       </c>
       <c r="B95">
-        <v>18</v>
+        <v>7</v>
       </c>
       <c r="C95">
-        <v>0.597</v>
+        <v>0</v>
       </c>
       <c r="D95" t="s">
         <v>97</v>
@@ -2229,13 +2229,13 @@
     </row>
     <row r="96" spans="1:4">
       <c r="A96" s="2">
-        <v>46115</v>
+        <v>46126</v>
       </c>
       <c r="B96">
-        <v>19</v>
+        <v>8</v>
       </c>
       <c r="C96">
-        <v>0.162</v>
+        <v>0.179</v>
       </c>
       <c r="D96" t="s">
         <v>98</v>
@@ -2243,13 +2243,13 @@
     </row>
     <row r="97" spans="1:4">
       <c r="A97" s="2">
-        <v>46115</v>
+        <v>46126</v>
       </c>
       <c r="B97">
-        <v>20</v>
+        <v>9</v>
       </c>
       <c r="C97">
-        <v>0.022</v>
+        <v>0.773</v>
       </c>
       <c r="D97" t="s">
         <v>99</v>
@@ -2257,13 +2257,13 @@
     </row>
     <row r="98" spans="1:4">
       <c r="A98" s="2">
-        <v>46115</v>
+        <v>46126</v>
       </c>
       <c r="B98">
-        <v>21</v>
+        <v>10</v>
       </c>
       <c r="C98">
-        <v>0</v>
+        <v>1.553</v>
       </c>
       <c r="D98" t="s">
         <v>100</v>
@@ -2271,13 +2271,13 @@
     </row>
     <row r="99" spans="1:4">
       <c r="A99" s="2">
-        <v>46115</v>
+        <v>46126</v>
       </c>
       <c r="B99">
-        <v>22</v>
+        <v>11</v>
       </c>
       <c r="C99">
-        <v>0</v>
+        <v>1.885</v>
       </c>
       <c r="D99" t="s">
         <v>101</v>
@@ -2285,13 +2285,13 @@
     </row>
     <row r="100" spans="1:4">
       <c r="A100" s="2">
-        <v>46115</v>
+        <v>46126</v>
       </c>
       <c r="B100">
-        <v>23</v>
+        <v>12</v>
       </c>
       <c r="C100">
-        <v>0</v>
+        <v>2.004</v>
       </c>
       <c r="D100" t="s">
         <v>102</v>
@@ -2299,13 +2299,13 @@
     </row>
     <row r="101" spans="1:4">
       <c r="A101" s="2">
-        <v>46115</v>
+        <v>46126</v>
       </c>
       <c r="B101">
-        <v>24</v>
+        <v>13</v>
       </c>
       <c r="C101">
-        <v>0</v>
+        <v>1.98</v>
       </c>
       <c r="D101" t="s">
         <v>103</v>
@@ -2313,13 +2313,13 @@
     </row>
     <row r="102" spans="1:4">
       <c r="A102" s="2">
-        <v>46116</v>
+        <v>46126</v>
       </c>
       <c r="B102">
-        <v>1</v>
+        <v>14</v>
       </c>
       <c r="C102">
-        <v>0</v>
+        <v>2.016</v>
       </c>
       <c r="D102" t="s">
         <v>104</v>
@@ -2327,13 +2327,13 @@
     </row>
     <row r="103" spans="1:4">
       <c r="A103" s="2">
-        <v>46116</v>
+        <v>46126</v>
       </c>
       <c r="B103">
-        <v>2</v>
+        <v>15</v>
       </c>
       <c r="C103">
-        <v>0</v>
+        <v>2.049</v>
       </c>
       <c r="D103" t="s">
         <v>105</v>
@@ -2341,13 +2341,13 @@
     </row>
     <row r="104" spans="1:4">
       <c r="A104" s="2">
-        <v>46116</v>
+        <v>46126</v>
       </c>
       <c r="B104">
-        <v>3</v>
+        <v>16</v>
       </c>
       <c r="C104">
-        <v>0</v>
+        <v>1.994</v>
       </c>
       <c r="D104" t="s">
         <v>106</v>
@@ -2355,13 +2355,13 @@
     </row>
     <row r="105" spans="1:4">
       <c r="A105" s="2">
-        <v>46116</v>
+        <v>46126</v>
       </c>
       <c r="B105">
-        <v>4</v>
+        <v>17</v>
       </c>
       <c r="C105">
-        <v>0</v>
+        <v>1.825</v>
       </c>
       <c r="D105" t="s">
         <v>107</v>
@@ -2369,13 +2369,13 @@
     </row>
     <row r="106" spans="1:4">
       <c r="A106" s="2">
-        <v>46116</v>
+        <v>46126</v>
       </c>
       <c r="B106">
-        <v>5</v>
+        <v>18</v>
       </c>
       <c r="C106">
-        <v>0</v>
+        <v>1.135</v>
       </c>
       <c r="D106" t="s">
         <v>108</v>
@@ -2383,13 +2383,13 @@
     </row>
     <row r="107" spans="1:4">
       <c r="A107" s="2">
-        <v>46116</v>
+        <v>46126</v>
       </c>
       <c r="B107">
-        <v>6</v>
+        <v>19</v>
       </c>
       <c r="C107">
-        <v>0</v>
+        <v>0.462</v>
       </c>
       <c r="D107" t="s">
         <v>109</v>
@@ -2397,13 +2397,13 @@
     </row>
     <row r="108" spans="1:4">
       <c r="A108" s="2">
-        <v>46116</v>
+        <v>46126</v>
       </c>
       <c r="B108">
-        <v>7</v>
+        <v>20</v>
       </c>
       <c r="C108">
-        <v>0</v>
+        <v>0.07099999999999999</v>
       </c>
       <c r="D108" t="s">
         <v>110</v>
@@ -2411,13 +2411,13 @@
     </row>
     <row r="109" spans="1:4">
       <c r="A109" s="2">
-        <v>46116</v>
+        <v>46126</v>
       </c>
       <c r="B109">
-        <v>8</v>
+        <v>21</v>
       </c>
       <c r="C109">
-        <v>0.057</v>
+        <v>0</v>
       </c>
       <c r="D109" t="s">
         <v>111</v>
@@ -2425,13 +2425,13 @@
     </row>
     <row r="110" spans="1:4">
       <c r="A110" s="2">
-        <v>46116</v>
+        <v>46126</v>
       </c>
       <c r="B110">
-        <v>9</v>
+        <v>22</v>
       </c>
       <c r="C110">
-        <v>0.581</v>
+        <v>0</v>
       </c>
       <c r="D110" t="s">
         <v>112</v>
@@ -2439,13 +2439,13 @@
     </row>
     <row r="111" spans="1:4">
       <c r="A111" s="2">
-        <v>46116</v>
+        <v>46126</v>
       </c>
       <c r="B111">
-        <v>10</v>
+        <v>23</v>
       </c>
       <c r="C111">
-        <v>1.181</v>
+        <v>0</v>
       </c>
       <c r="D111" t="s">
         <v>113</v>
@@ -2453,13 +2453,13 @@
     </row>
     <row r="112" spans="1:4">
       <c r="A112" s="2">
-        <v>46116</v>
+        <v>46126</v>
       </c>
       <c r="B112">
-        <v>11</v>
+        <v>24</v>
       </c>
       <c r="C112">
-        <v>1.866</v>
+        <v>0</v>
       </c>
       <c r="D112" t="s">
         <v>114</v>
@@ -2467,13 +2467,13 @@
     </row>
     <row r="113" spans="1:4">
       <c r="A113" s="2">
-        <v>46116</v>
+        <v>46127</v>
       </c>
       <c r="B113">
-        <v>12</v>
+        <v>1</v>
       </c>
       <c r="C113">
-        <v>2.337</v>
+        <v>0</v>
       </c>
       <c r="D113" t="s">
         <v>115</v>
@@ -2481,13 +2481,13 @@
     </row>
     <row r="114" spans="1:4">
       <c r="A114" s="2">
-        <v>46116</v>
+        <v>46127</v>
       </c>
       <c r="B114">
-        <v>13</v>
+        <v>2</v>
       </c>
       <c r="C114">
-        <v>2.438</v>
+        <v>0</v>
       </c>
       <c r="D114" t="s">
         <v>116</v>
@@ -2495,13 +2495,13 @@
     </row>
     <row r="115" spans="1:4">
       <c r="A115" s="2">
-        <v>46116</v>
+        <v>46127</v>
       </c>
       <c r="B115">
-        <v>14</v>
+        <v>3</v>
       </c>
       <c r="C115">
-        <v>2.403</v>
+        <v>0</v>
       </c>
       <c r="D115" t="s">
         <v>117</v>
@@ -2509,13 +2509,13 @@
     </row>
     <row r="116" spans="1:4">
       <c r="A116" s="2">
-        <v>46116</v>
+        <v>46127</v>
       </c>
       <c r="B116">
-        <v>15</v>
+        <v>4</v>
       </c>
       <c r="C116">
-        <v>2.421</v>
+        <v>0</v>
       </c>
       <c r="D116" t="s">
         <v>118</v>
@@ -2523,13 +2523,13 @@
     </row>
     <row r="117" spans="1:4">
       <c r="A117" s="2">
-        <v>46116</v>
+        <v>46127</v>
       </c>
       <c r="B117">
-        <v>16</v>
+        <v>5</v>
       </c>
       <c r="C117">
-        <v>2.238</v>
+        <v>0</v>
       </c>
       <c r="D117" t="s">
         <v>119</v>
@@ -2537,13 +2537,13 @@
     </row>
     <row r="118" spans="1:4">
       <c r="A118" s="2">
-        <v>46116</v>
+        <v>46127</v>
       </c>
       <c r="B118">
-        <v>17</v>
+        <v>6</v>
       </c>
       <c r="C118">
-        <v>1.86</v>
+        <v>0</v>
       </c>
       <c r="D118" t="s">
         <v>120</v>
@@ -2551,13 +2551,13 @@
     </row>
     <row r="119" spans="1:4">
       <c r="A119" s="2">
-        <v>46116</v>
+        <v>46127</v>
       </c>
       <c r="B119">
-        <v>18</v>
+        <v>7</v>
       </c>
       <c r="C119">
-        <v>1.085</v>
+        <v>0</v>
       </c>
       <c r="D119" t="s">
         <v>121</v>
@@ -2565,13 +2565,13 @@
     </row>
     <row r="120" spans="1:4">
       <c r="A120" s="2">
-        <v>46116</v>
+        <v>46127</v>
       </c>
       <c r="B120">
-        <v>19</v>
+        <v>8</v>
       </c>
       <c r="C120">
-        <v>0.383</v>
+        <v>0.228</v>
       </c>
       <c r="D120" t="s">
         <v>122</v>
@@ -2579,13 +2579,13 @@
     </row>
     <row r="121" spans="1:4">
       <c r="A121" s="2">
-        <v>46116</v>
+        <v>46127</v>
       </c>
       <c r="B121">
-        <v>20</v>
+        <v>9</v>
       </c>
       <c r="C121">
-        <v>0.04</v>
+        <v>0.914</v>
       </c>
       <c r="D121" t="s">
         <v>123</v>
@@ -2593,13 +2593,13 @@
     </row>
     <row r="122" spans="1:4">
       <c r="A122" s="2">
-        <v>46116</v>
+        <v>46127</v>
       </c>
       <c r="B122">
-        <v>21</v>
+        <v>10</v>
       </c>
       <c r="C122">
-        <v>0</v>
+        <v>1.899</v>
       </c>
       <c r="D122" t="s">
         <v>124</v>
@@ -2607,13 +2607,13 @@
     </row>
     <row r="123" spans="1:4">
       <c r="A123" s="2">
-        <v>46116</v>
+        <v>46127</v>
       </c>
       <c r="B123">
-        <v>22</v>
+        <v>11</v>
       </c>
       <c r="C123">
-        <v>0</v>
+        <v>2.567</v>
       </c>
       <c r="D123" t="s">
         <v>125</v>
@@ -2621,13 +2621,13 @@
     </row>
     <row r="124" spans="1:4">
       <c r="A124" s="2">
-        <v>46116</v>
+        <v>46127</v>
       </c>
       <c r="B124">
-        <v>23</v>
+        <v>12</v>
       </c>
       <c r="C124">
-        <v>0</v>
+        <v>3.049</v>
       </c>
       <c r="D124" t="s">
         <v>126</v>
@@ -2635,13 +2635,13 @@
     </row>
     <row r="125" spans="1:4">
       <c r="A125" s="2">
-        <v>46116</v>
+        <v>46127</v>
       </c>
       <c r="B125">
-        <v>24</v>
+        <v>13</v>
       </c>
       <c r="C125">
-        <v>0</v>
+        <v>3.26</v>
       </c>
       <c r="D125" t="s">
         <v>127</v>
@@ -2649,13 +2649,13 @@
     </row>
     <row r="126" spans="1:4">
       <c r="A126" s="2">
-        <v>46117</v>
+        <v>46127</v>
       </c>
       <c r="B126">
-        <v>1</v>
+        <v>14</v>
       </c>
       <c r="C126">
-        <v>0</v>
+        <v>3.203</v>
       </c>
       <c r="D126" t="s">
         <v>128</v>
@@ -2663,13 +2663,13 @@
     </row>
     <row r="127" spans="1:4">
       <c r="A127" s="2">
-        <v>46117</v>
+        <v>46127</v>
       </c>
       <c r="B127">
-        <v>2</v>
+        <v>15</v>
       </c>
       <c r="C127">
-        <v>0</v>
+        <v>2.992</v>
       </c>
       <c r="D127" t="s">
         <v>129</v>
@@ -2677,13 +2677,13 @@
     </row>
     <row r="128" spans="1:4">
       <c r="A128" s="2">
-        <v>46117</v>
+        <v>46127</v>
       </c>
       <c r="B128">
-        <v>3</v>
+        <v>16</v>
       </c>
       <c r="C128">
-        <v>0</v>
+        <v>2.588</v>
       </c>
       <c r="D128" t="s">
         <v>130</v>
@@ -2691,13 +2691,13 @@
     </row>
     <row r="129" spans="1:4">
       <c r="A129" s="2">
-        <v>46117</v>
+        <v>46127</v>
       </c>
       <c r="B129">
-        <v>4</v>
+        <v>17</v>
       </c>
       <c r="C129">
-        <v>0</v>
+        <v>2.107</v>
       </c>
       <c r="D129" t="s">
         <v>131</v>
@@ -2705,13 +2705,13 @@
     </row>
     <row r="130" spans="1:4">
       <c r="A130" s="2">
-        <v>46117</v>
+        <v>46127</v>
       </c>
       <c r="B130">
-        <v>5</v>
+        <v>18</v>
       </c>
       <c r="C130">
-        <v>0</v>
+        <v>1.27</v>
       </c>
       <c r="D130" t="s">
         <v>132</v>
@@ -2719,13 +2719,13 @@
     </row>
     <row r="131" spans="1:4">
       <c r="A131" s="2">
-        <v>46117</v>
+        <v>46127</v>
       </c>
       <c r="B131">
-        <v>6</v>
+        <v>19</v>
       </c>
       <c r="C131">
-        <v>0</v>
+        <v>0.496</v>
       </c>
       <c r="D131" t="s">
         <v>133</v>
@@ -2733,13 +2733,13 @@
     </row>
     <row r="132" spans="1:4">
       <c r="A132" s="2">
-        <v>46117</v>
+        <v>46127</v>
       </c>
       <c r="B132">
-        <v>7</v>
+        <v>20</v>
       </c>
       <c r="C132">
-        <v>0</v>
+        <v>0.077</v>
       </c>
       <c r="D132" t="s">
         <v>134</v>
@@ -2747,13 +2747,13 @@
     </row>
     <row r="133" spans="1:4">
       <c r="A133" s="2">
-        <v>46117</v>
+        <v>46127</v>
       </c>
       <c r="B133">
-        <v>8</v>
+        <v>21</v>
       </c>
       <c r="C133">
-        <v>0.08500000000000001</v>
+        <v>0</v>
       </c>
       <c r="D133" t="s">
         <v>135</v>
@@ -2761,13 +2761,13 @@
     </row>
     <row r="134" spans="1:4">
       <c r="A134" s="2">
-        <v>46117</v>
+        <v>46127</v>
       </c>
       <c r="B134">
-        <v>9</v>
+        <v>22</v>
       </c>
       <c r="C134">
-        <v>0.638</v>
+        <v>0</v>
       </c>
       <c r="D134" t="s">
         <v>136</v>
@@ -2775,13 +2775,13 @@
     </row>
     <row r="135" spans="1:4">
       <c r="A135" s="2">
-        <v>46117</v>
+        <v>46127</v>
       </c>
       <c r="B135">
-        <v>10</v>
+        <v>23</v>
       </c>
       <c r="C135">
-        <v>1.474</v>
+        <v>0</v>
       </c>
       <c r="D135" t="s">
         <v>137</v>
@@ -2789,13 +2789,13 @@
     </row>
     <row r="136" spans="1:4">
       <c r="A136" s="2">
-        <v>46117</v>
+        <v>46127</v>
       </c>
       <c r="B136">
-        <v>11</v>
+        <v>24</v>
       </c>
       <c r="C136">
-        <v>2.134</v>
+        <v>0</v>
       </c>
       <c r="D136" t="s">
         <v>138</v>
@@ -2803,13 +2803,13 @@
     </row>
     <row r="137" spans="1:4">
       <c r="A137" s="2">
-        <v>46117</v>
+        <v>46128</v>
       </c>
       <c r="B137">
-        <v>12</v>
+        <v>1</v>
       </c>
       <c r="C137">
-        <v>2.629</v>
+        <v>0</v>
       </c>
       <c r="D137" t="s">
         <v>139</v>
@@ -2817,13 +2817,13 @@
     </row>
     <row r="138" spans="1:4">
       <c r="A138" s="2">
-        <v>46117</v>
+        <v>46128</v>
       </c>
       <c r="B138">
-        <v>13</v>
+        <v>2</v>
       </c>
       <c r="C138">
-        <v>2.931</v>
+        <v>0</v>
       </c>
       <c r="D138" t="s">
         <v>140</v>
@@ -2831,13 +2831,13 @@
     </row>
     <row r="139" spans="1:4">
       <c r="A139" s="2">
-        <v>46117</v>
+        <v>46128</v>
       </c>
       <c r="B139">
-        <v>14</v>
+        <v>3</v>
       </c>
       <c r="C139">
-        <v>2.921</v>
+        <v>0</v>
       </c>
       <c r="D139" t="s">
         <v>141</v>
@@ -2845,13 +2845,13 @@
     </row>
     <row r="140" spans="1:4">
       <c r="A140" s="2">
-        <v>46117</v>
+        <v>46128</v>
       </c>
       <c r="B140">
-        <v>15</v>
+        <v>4</v>
       </c>
       <c r="C140">
-        <v>2.895</v>
+        <v>0</v>
       </c>
       <c r="D140" t="s">
         <v>142</v>
@@ -2859,13 +2859,13 @@
     </row>
     <row r="141" spans="1:4">
       <c r="A141" s="2">
-        <v>46117</v>
+        <v>46128</v>
       </c>
       <c r="B141">
-        <v>16</v>
+        <v>5</v>
       </c>
       <c r="C141">
-        <v>2.503</v>
+        <v>0</v>
       </c>
       <c r="D141" t="s">
         <v>143</v>
@@ -2873,13 +2873,13 @@
     </row>
     <row r="142" spans="1:4">
       <c r="A142" s="2">
-        <v>46117</v>
+        <v>46128</v>
       </c>
       <c r="B142">
-        <v>17</v>
+        <v>6</v>
       </c>
       <c r="C142">
-        <v>2.042</v>
+        <v>0</v>
       </c>
       <c r="D142" t="s">
         <v>144</v>
@@ -2887,13 +2887,13 @@
     </row>
     <row r="143" spans="1:4">
       <c r="A143" s="2">
-        <v>46117</v>
+        <v>46128</v>
       </c>
       <c r="B143">
-        <v>18</v>
+        <v>7</v>
       </c>
       <c r="C143">
-        <v>1.304</v>
+        <v>0</v>
       </c>
       <c r="D143" t="s">
         <v>145</v>
@@ -2901,13 +2901,13 @@
     </row>
     <row r="144" spans="1:4">
       <c r="A144" s="2">
-        <v>46117</v>
+        <v>46128</v>
       </c>
       <c r="B144">
-        <v>19</v>
+        <v>8</v>
       </c>
       <c r="C144">
-        <v>0.458</v>
+        <v>0.229</v>
       </c>
       <c r="D144" t="s">
         <v>146</v>
@@ -2915,13 +2915,13 @@
     </row>
     <row r="145" spans="1:4">
       <c r="A145" s="2">
-        <v>46117</v>
+        <v>46128</v>
       </c>
       <c r="B145">
-        <v>20</v>
+        <v>9</v>
       </c>
       <c r="C145">
-        <v>0.049</v>
+        <v>0.929</v>
       </c>
       <c r="D145" t="s">
         <v>147</v>
@@ -2929,13 +2929,13 @@
     </row>
     <row r="146" spans="1:4">
       <c r="A146" s="2">
-        <v>46117</v>
+        <v>46128</v>
       </c>
       <c r="B146">
-        <v>21</v>
+        <v>10</v>
       </c>
       <c r="C146">
-        <v>0</v>
+        <v>1.936</v>
       </c>
       <c r="D146" t="s">
         <v>148</v>
@@ -2943,13 +2943,13 @@
     </row>
     <row r="147" spans="1:4">
       <c r="A147" s="2">
-        <v>46117</v>
+        <v>46128</v>
       </c>
       <c r="B147">
-        <v>22</v>
+        <v>11</v>
       </c>
       <c r="C147">
-        <v>0</v>
+        <v>2.48</v>
       </c>
       <c r="D147" t="s">
         <v>149</v>
@@ -2957,13 +2957,13 @@
     </row>
     <row r="148" spans="1:4">
       <c r="A148" s="2">
-        <v>46117</v>
+        <v>46128</v>
       </c>
       <c r="B148">
-        <v>23</v>
+        <v>12</v>
       </c>
       <c r="C148">
-        <v>0</v>
+        <v>2.848</v>
       </c>
       <c r="D148" t="s">
         <v>150</v>
@@ -2971,13 +2971,13 @@
     </row>
     <row r="149" spans="1:4">
       <c r="A149" s="2">
-        <v>46117</v>
+        <v>46128</v>
       </c>
       <c r="B149">
-        <v>24</v>
+        <v>13</v>
       </c>
       <c r="C149">
-        <v>0</v>
+        <v>2.995</v>
       </c>
       <c r="D149" t="s">
         <v>151</v>
@@ -2985,13 +2985,13 @@
     </row>
     <row r="150" spans="1:4">
       <c r="A150" s="2">
-        <v>46118</v>
+        <v>46128</v>
       </c>
       <c r="B150">
-        <v>1</v>
+        <v>14</v>
       </c>
       <c r="C150">
-        <v>0</v>
+        <v>2.965</v>
       </c>
       <c r="D150" t="s">
         <v>152</v>
@@ -2999,13 +2999,13 @@
     </row>
     <row r="151" spans="1:4">
       <c r="A151" s="2">
-        <v>46118</v>
+        <v>46128</v>
       </c>
       <c r="B151">
-        <v>2</v>
+        <v>15</v>
       </c>
       <c r="C151">
-        <v>0</v>
+        <v>2.645</v>
       </c>
       <c r="D151" t="s">
         <v>153</v>
@@ -3013,13 +3013,13 @@
     </row>
     <row r="152" spans="1:4">
       <c r="A152" s="2">
-        <v>46118</v>
+        <v>46128</v>
       </c>
       <c r="B152">
-        <v>3</v>
+        <v>16</v>
       </c>
       <c r="C152">
-        <v>0</v>
+        <v>2.361</v>
       </c>
       <c r="D152" t="s">
         <v>154</v>
@@ -3027,13 +3027,13 @@
     </row>
     <row r="153" spans="1:4">
       <c r="A153" s="2">
-        <v>46118</v>
+        <v>46128</v>
       </c>
       <c r="B153">
-        <v>4</v>
+        <v>17</v>
       </c>
       <c r="C153">
-        <v>0</v>
+        <v>1.913</v>
       </c>
       <c r="D153" t="s">
         <v>155</v>
@@ -3041,13 +3041,13 @@
     </row>
     <row r="154" spans="1:4">
       <c r="A154" s="2">
-        <v>46118</v>
+        <v>46128</v>
       </c>
       <c r="B154">
-        <v>5</v>
+        <v>18</v>
       </c>
       <c r="C154">
-        <v>0</v>
+        <v>1.226</v>
       </c>
       <c r="D154" t="s">
         <v>156</v>
@@ -3055,13 +3055,13 @@
     </row>
     <row r="155" spans="1:4">
       <c r="A155" s="2">
-        <v>46118</v>
+        <v>46128</v>
       </c>
       <c r="B155">
-        <v>6</v>
+        <v>19</v>
       </c>
       <c r="C155">
-        <v>0</v>
+        <v>0.499</v>
       </c>
       <c r="D155" t="s">
         <v>157</v>
@@ -3069,13 +3069,13 @@
     </row>
     <row r="156" spans="1:4">
       <c r="A156" s="2">
-        <v>46118</v>
+        <v>46128</v>
       </c>
       <c r="B156">
-        <v>7</v>
+        <v>20</v>
       </c>
       <c r="C156">
-        <v>0</v>
+        <v>0.09</v>
       </c>
       <c r="D156" t="s">
         <v>158</v>
@@ -3083,13 +3083,13 @@
     </row>
     <row r="157" spans="1:4">
       <c r="A157" s="2">
-        <v>46118</v>
+        <v>46128</v>
       </c>
       <c r="B157">
-        <v>8</v>
+        <v>21</v>
       </c>
       <c r="C157">
-        <v>0.098</v>
+        <v>0</v>
       </c>
       <c r="D157" t="s">
         <v>159</v>
@@ -3097,13 +3097,13 @@
     </row>
     <row r="158" spans="1:4">
       <c r="A158" s="2">
-        <v>46118</v>
+        <v>46128</v>
       </c>
       <c r="B158">
-        <v>9</v>
+        <v>22</v>
       </c>
       <c r="C158">
-        <v>0.699</v>
+        <v>0</v>
       </c>
       <c r="D158" t="s">
         <v>160</v>
@@ -3111,13 +3111,13 @@
     </row>
     <row r="159" spans="1:4">
       <c r="A159" s="2">
-        <v>46118</v>
+        <v>46128</v>
       </c>
       <c r="B159">
-        <v>10</v>
+        <v>23</v>
       </c>
       <c r="C159">
-        <v>1.548</v>
+        <v>0</v>
       </c>
       <c r="D159" t="s">
         <v>161</v>
@@ -3125,13 +3125,13 @@
     </row>
     <row r="160" spans="1:4">
       <c r="A160" s="2">
-        <v>46118</v>
+        <v>46128</v>
       </c>
       <c r="B160">
-        <v>11</v>
+        <v>24</v>
       </c>
       <c r="C160">
-        <v>2.052</v>
+        <v>0</v>
       </c>
       <c r="D160" t="s">
         <v>162</v>
@@ -3139,13 +3139,13 @@
     </row>
     <row r="161" spans="1:4">
       <c r="A161" s="2">
-        <v>46118</v>
+        <v>46129</v>
       </c>
       <c r="B161">
-        <v>12</v>
+        <v>1</v>
       </c>
       <c r="C161">
-        <v>2.495</v>
+        <v>0</v>
       </c>
       <c r="D161" t="s">
         <v>163</v>
@@ -3153,13 +3153,13 @@
     </row>
     <row r="162" spans="1:4">
       <c r="A162" s="2">
-        <v>46118</v>
+        <v>46129</v>
       </c>
       <c r="B162">
-        <v>13</v>
+        <v>2</v>
       </c>
       <c r="C162">
-        <v>2.817</v>
+        <v>0</v>
       </c>
       <c r="D162" t="s">
         <v>164</v>
@@ -3167,13 +3167,13 @@
     </row>
     <row r="163" spans="1:4">
       <c r="A163" s="2">
-        <v>46118</v>
+        <v>46129</v>
       </c>
       <c r="B163">
-        <v>14</v>
+        <v>3</v>
       </c>
       <c r="C163">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="D163" t="s">
         <v>165</v>
@@ -3181,13 +3181,13 @@
     </row>
     <row r="164" spans="1:4">
       <c r="A164" s="2">
-        <v>46118</v>
+        <v>46129</v>
       </c>
       <c r="B164">
-        <v>15</v>
+        <v>4</v>
       </c>
       <c r="C164">
-        <v>2.955</v>
+        <v>0</v>
       </c>
       <c r="D164" t="s">
         <v>166</v>
@@ -3195,13 +3195,13 @@
     </row>
     <row r="165" spans="1:4">
       <c r="A165" s="2">
-        <v>46118</v>
+        <v>46129</v>
       </c>
       <c r="B165">
-        <v>16</v>
+        <v>5</v>
       </c>
       <c r="C165">
-        <v>2.512</v>
+        <v>0</v>
       </c>
       <c r="D165" t="s">
         <v>167</v>
@@ -3209,13 +3209,13 @@
     </row>
     <row r="166" spans="1:4">
       <c r="A166" s="2">
-        <v>46118</v>
+        <v>46129</v>
       </c>
       <c r="B166">
-        <v>17</v>
+        <v>6</v>
       </c>
       <c r="C166">
-        <v>1.998</v>
+        <v>0</v>
       </c>
       <c r="D166" t="s">
         <v>168</v>
@@ -3223,13 +3223,13 @@
     </row>
     <row r="167" spans="1:4">
       <c r="A167" s="2">
-        <v>46118</v>
+        <v>46129</v>
       </c>
       <c r="B167">
-        <v>18</v>
+        <v>7</v>
       </c>
       <c r="C167">
-        <v>1.223</v>
+        <v>0</v>
       </c>
       <c r="D167" t="s">
         <v>169</v>
@@ -3237,13 +3237,13 @@
     </row>
     <row r="168" spans="1:4">
       <c r="A168" s="2">
-        <v>46118</v>
+        <v>46129</v>
       </c>
       <c r="B168">
-        <v>19</v>
+        <v>8</v>
       </c>
       <c r="C168">
-        <v>0.433</v>
+        <v>0.216</v>
       </c>
       <c r="D168" t="s">
         <v>170</v>
@@ -3251,13 +3251,13 @@
     </row>
     <row r="169" spans="1:4">
       <c r="A169" s="2">
-        <v>46118</v>
+        <v>46129</v>
       </c>
       <c r="B169">
-        <v>20</v>
+        <v>9</v>
       </c>
       <c r="C169">
-        <v>0.047</v>
+        <v>0.739</v>
       </c>
       <c r="D169" t="s">
         <v>171</v>
@@ -3265,13 +3265,13 @@
     </row>
     <row r="170" spans="1:4">
       <c r="A170" s="2">
-        <v>46118</v>
+        <v>46129</v>
       </c>
       <c r="B170">
-        <v>21</v>
+        <v>10</v>
       </c>
       <c r="C170">
-        <v>0</v>
+        <v>1.201</v>
       </c>
       <c r="D170" t="s">
         <v>172</v>

</xml_diff>

<commit_message>
Retraining the model for Elnet
</commit_message>
<xml_diff>
--- a/Astro/Results_Production_Astro_xgb.xlsx
+++ b/Astro/Results_Production_Astro_xgb.xlsx
@@ -28,511 +28,511 @@
     <t>Lookup</t>
   </si>
   <si>
-    <t>10.04.202610</t>
-  </si>
-  <si>
-    <t>10.04.202611</t>
-  </si>
-  <si>
-    <t>10.04.202612</t>
-  </si>
-  <si>
-    <t>10.04.202613</t>
-  </si>
-  <si>
-    <t>10.04.202614</t>
-  </si>
-  <si>
-    <t>10.04.202615</t>
-  </si>
-  <si>
-    <t>10.04.202616</t>
-  </si>
-  <si>
-    <t>10.04.202617</t>
-  </si>
-  <si>
-    <t>10.04.202618</t>
-  </si>
-  <si>
-    <t>10.04.202619</t>
-  </si>
-  <si>
-    <t>10.04.202620</t>
-  </si>
-  <si>
-    <t>10.04.202621</t>
-  </si>
-  <si>
-    <t>10.04.202622</t>
-  </si>
-  <si>
-    <t>10.04.202623</t>
-  </si>
-  <si>
-    <t>10.04.202624</t>
-  </si>
-  <si>
-    <t>11.04.20261</t>
-  </si>
-  <si>
-    <t>11.04.20262</t>
-  </si>
-  <si>
-    <t>11.04.20263</t>
-  </si>
-  <si>
-    <t>11.04.20264</t>
-  </si>
-  <si>
-    <t>11.04.20265</t>
-  </si>
-  <si>
-    <t>11.04.20266</t>
-  </si>
-  <si>
-    <t>11.04.20267</t>
-  </si>
-  <si>
-    <t>11.04.20268</t>
-  </si>
-  <si>
-    <t>11.04.20269</t>
-  </si>
-  <si>
-    <t>11.04.202610</t>
-  </si>
-  <si>
-    <t>11.04.202611</t>
-  </si>
-  <si>
-    <t>11.04.202612</t>
-  </si>
-  <si>
-    <t>11.04.202613</t>
-  </si>
-  <si>
-    <t>11.04.202614</t>
-  </si>
-  <si>
-    <t>11.04.202615</t>
-  </si>
-  <si>
-    <t>11.04.202616</t>
-  </si>
-  <si>
-    <t>11.04.202617</t>
-  </si>
-  <si>
-    <t>11.04.202618</t>
-  </si>
-  <si>
-    <t>11.04.202619</t>
-  </si>
-  <si>
-    <t>11.04.202620</t>
-  </si>
-  <si>
-    <t>11.04.202621</t>
-  </si>
-  <si>
-    <t>11.04.202622</t>
-  </si>
-  <si>
-    <t>11.04.202623</t>
-  </si>
-  <si>
-    <t>11.04.202624</t>
-  </si>
-  <si>
-    <t>12.04.20261</t>
-  </si>
-  <si>
-    <t>12.04.20262</t>
-  </si>
-  <si>
-    <t>12.04.20263</t>
-  </si>
-  <si>
-    <t>12.04.20264</t>
-  </si>
-  <si>
-    <t>12.04.20265</t>
-  </si>
-  <si>
-    <t>12.04.20266</t>
-  </si>
-  <si>
-    <t>12.04.20267</t>
-  </si>
-  <si>
-    <t>12.04.20268</t>
-  </si>
-  <si>
-    <t>12.04.20269</t>
-  </si>
-  <si>
-    <t>12.04.202610</t>
-  </si>
-  <si>
-    <t>12.04.202611</t>
-  </si>
-  <si>
-    <t>12.04.202612</t>
-  </si>
-  <si>
-    <t>12.04.202613</t>
-  </si>
-  <si>
-    <t>12.04.202614</t>
-  </si>
-  <si>
-    <t>12.04.202615</t>
-  </si>
-  <si>
-    <t>12.04.202616</t>
-  </si>
-  <si>
-    <t>12.04.202617</t>
-  </si>
-  <si>
-    <t>12.04.202618</t>
-  </si>
-  <si>
-    <t>12.04.202619</t>
-  </si>
-  <si>
-    <t>12.04.202620</t>
-  </si>
-  <si>
-    <t>12.04.202621</t>
-  </si>
-  <si>
-    <t>12.04.202622</t>
-  </si>
-  <si>
-    <t>12.04.202623</t>
-  </si>
-  <si>
-    <t>12.04.202624</t>
-  </si>
-  <si>
-    <t>13.04.20261</t>
-  </si>
-  <si>
-    <t>13.04.20262</t>
-  </si>
-  <si>
-    <t>13.04.20263</t>
-  </si>
-  <si>
-    <t>13.04.20264</t>
-  </si>
-  <si>
-    <t>13.04.20265</t>
-  </si>
-  <si>
-    <t>13.04.20266</t>
-  </si>
-  <si>
-    <t>13.04.20267</t>
-  </si>
-  <si>
-    <t>13.04.20268</t>
-  </si>
-  <si>
-    <t>13.04.20269</t>
-  </si>
-  <si>
-    <t>13.04.202610</t>
-  </si>
-  <si>
-    <t>13.04.202611</t>
-  </si>
-  <si>
-    <t>13.04.202612</t>
-  </si>
-  <si>
-    <t>13.04.202613</t>
-  </si>
-  <si>
-    <t>13.04.202614</t>
-  </si>
-  <si>
-    <t>13.04.202615</t>
-  </si>
-  <si>
-    <t>13.04.202616</t>
-  </si>
-  <si>
-    <t>13.04.202617</t>
-  </si>
-  <si>
-    <t>13.04.202618</t>
-  </si>
-  <si>
-    <t>13.04.202619</t>
-  </si>
-  <si>
-    <t>13.04.202620</t>
-  </si>
-  <si>
-    <t>13.04.202621</t>
-  </si>
-  <si>
-    <t>13.04.202622</t>
-  </si>
-  <si>
-    <t>13.04.202623</t>
-  </si>
-  <si>
-    <t>13.04.202624</t>
-  </si>
-  <si>
-    <t>14.04.20261</t>
-  </si>
-  <si>
-    <t>14.04.20262</t>
-  </si>
-  <si>
-    <t>14.04.20263</t>
-  </si>
-  <si>
-    <t>14.04.20264</t>
-  </si>
-  <si>
-    <t>14.04.20265</t>
-  </si>
-  <si>
-    <t>14.04.20266</t>
-  </si>
-  <si>
-    <t>14.04.20267</t>
-  </si>
-  <si>
-    <t>14.04.20268</t>
-  </si>
-  <si>
-    <t>14.04.20269</t>
-  </si>
-  <si>
-    <t>14.04.202610</t>
-  </si>
-  <si>
-    <t>14.04.202611</t>
-  </si>
-  <si>
-    <t>14.04.202612</t>
-  </si>
-  <si>
-    <t>14.04.202613</t>
-  </si>
-  <si>
-    <t>14.04.202614</t>
-  </si>
-  <si>
-    <t>14.04.202615</t>
-  </si>
-  <si>
-    <t>14.04.202616</t>
-  </si>
-  <si>
-    <t>14.04.202617</t>
-  </si>
-  <si>
-    <t>14.04.202618</t>
-  </si>
-  <si>
-    <t>14.04.202619</t>
-  </si>
-  <si>
-    <t>14.04.202620</t>
-  </si>
-  <si>
-    <t>14.04.202621</t>
-  </si>
-  <si>
-    <t>14.04.202622</t>
-  </si>
-  <si>
-    <t>14.04.202623</t>
-  </si>
-  <si>
-    <t>14.04.202624</t>
-  </si>
-  <si>
-    <t>15.04.20261</t>
-  </si>
-  <si>
-    <t>15.04.20262</t>
-  </si>
-  <si>
-    <t>15.04.20263</t>
-  </si>
-  <si>
-    <t>15.04.20264</t>
-  </si>
-  <si>
-    <t>15.04.20265</t>
-  </si>
-  <si>
-    <t>15.04.20266</t>
-  </si>
-  <si>
-    <t>15.04.20267</t>
-  </si>
-  <si>
-    <t>15.04.20268</t>
-  </si>
-  <si>
-    <t>15.04.20269</t>
-  </si>
-  <si>
-    <t>15.04.202610</t>
-  </si>
-  <si>
-    <t>15.04.202611</t>
-  </si>
-  <si>
-    <t>15.04.202612</t>
-  </si>
-  <si>
-    <t>15.04.202613</t>
-  </si>
-  <si>
-    <t>15.04.202614</t>
-  </si>
-  <si>
-    <t>15.04.202615</t>
-  </si>
-  <si>
-    <t>15.04.202616</t>
-  </si>
-  <si>
-    <t>15.04.202617</t>
-  </si>
-  <si>
-    <t>15.04.202618</t>
-  </si>
-  <si>
-    <t>15.04.202619</t>
-  </si>
-  <si>
-    <t>15.04.202620</t>
-  </si>
-  <si>
-    <t>15.04.202621</t>
-  </si>
-  <si>
-    <t>15.04.202622</t>
-  </si>
-  <si>
-    <t>15.04.202623</t>
-  </si>
-  <si>
-    <t>15.04.202624</t>
-  </si>
-  <si>
-    <t>16.04.20261</t>
-  </si>
-  <si>
-    <t>16.04.20262</t>
-  </si>
-  <si>
-    <t>16.04.20263</t>
-  </si>
-  <si>
-    <t>16.04.20264</t>
-  </si>
-  <si>
-    <t>16.04.20265</t>
-  </si>
-  <si>
-    <t>16.04.20266</t>
-  </si>
-  <si>
-    <t>16.04.20267</t>
-  </si>
-  <si>
-    <t>16.04.20268</t>
-  </si>
-  <si>
-    <t>16.04.20269</t>
-  </si>
-  <si>
-    <t>16.04.202610</t>
-  </si>
-  <si>
-    <t>16.04.202611</t>
-  </si>
-  <si>
-    <t>16.04.202612</t>
-  </si>
-  <si>
-    <t>16.04.202613</t>
-  </si>
-  <si>
-    <t>16.04.202614</t>
-  </si>
-  <si>
-    <t>16.04.202615</t>
-  </si>
-  <si>
-    <t>16.04.202616</t>
-  </si>
-  <si>
-    <t>16.04.202617</t>
-  </si>
-  <si>
-    <t>16.04.202618</t>
-  </si>
-  <si>
-    <t>16.04.202619</t>
-  </si>
-  <si>
-    <t>16.04.202620</t>
-  </si>
-  <si>
-    <t>16.04.202621</t>
-  </si>
-  <si>
-    <t>16.04.202622</t>
-  </si>
-  <si>
-    <t>16.04.202623</t>
-  </si>
-  <si>
-    <t>16.04.202624</t>
-  </si>
-  <si>
-    <t>17.04.20261</t>
-  </si>
-  <si>
-    <t>17.04.20262</t>
-  </si>
-  <si>
-    <t>17.04.20263</t>
-  </si>
-  <si>
-    <t>17.04.20264</t>
-  </si>
-  <si>
-    <t>17.04.20265</t>
-  </si>
-  <si>
-    <t>17.04.20266</t>
-  </si>
-  <si>
-    <t>17.04.20267</t>
-  </si>
-  <si>
-    <t>17.04.20268</t>
-  </si>
-  <si>
-    <t>17.04.20269</t>
-  </si>
-  <si>
-    <t>17.04.202610</t>
+    <t>21.04.202610</t>
+  </si>
+  <si>
+    <t>21.04.202611</t>
+  </si>
+  <si>
+    <t>21.04.202612</t>
+  </si>
+  <si>
+    <t>21.04.202613</t>
+  </si>
+  <si>
+    <t>21.04.202614</t>
+  </si>
+  <si>
+    <t>21.04.202615</t>
+  </si>
+  <si>
+    <t>21.04.202616</t>
+  </si>
+  <si>
+    <t>21.04.202617</t>
+  </si>
+  <si>
+    <t>21.04.202618</t>
+  </si>
+  <si>
+    <t>21.04.202619</t>
+  </si>
+  <si>
+    <t>21.04.202620</t>
+  </si>
+  <si>
+    <t>21.04.202621</t>
+  </si>
+  <si>
+    <t>21.04.202622</t>
+  </si>
+  <si>
+    <t>21.04.202623</t>
+  </si>
+  <si>
+    <t>21.04.202624</t>
+  </si>
+  <si>
+    <t>22.04.20261</t>
+  </si>
+  <si>
+    <t>22.04.20262</t>
+  </si>
+  <si>
+    <t>22.04.20263</t>
+  </si>
+  <si>
+    <t>22.04.20264</t>
+  </si>
+  <si>
+    <t>22.04.20265</t>
+  </si>
+  <si>
+    <t>22.04.20266</t>
+  </si>
+  <si>
+    <t>22.04.20267</t>
+  </si>
+  <si>
+    <t>22.04.20268</t>
+  </si>
+  <si>
+    <t>22.04.20269</t>
+  </si>
+  <si>
+    <t>22.04.202610</t>
+  </si>
+  <si>
+    <t>22.04.202611</t>
+  </si>
+  <si>
+    <t>22.04.202612</t>
+  </si>
+  <si>
+    <t>22.04.202613</t>
+  </si>
+  <si>
+    <t>22.04.202614</t>
+  </si>
+  <si>
+    <t>22.04.202615</t>
+  </si>
+  <si>
+    <t>22.04.202616</t>
+  </si>
+  <si>
+    <t>22.04.202617</t>
+  </si>
+  <si>
+    <t>22.04.202618</t>
+  </si>
+  <si>
+    <t>22.04.202619</t>
+  </si>
+  <si>
+    <t>22.04.202620</t>
+  </si>
+  <si>
+    <t>22.04.202621</t>
+  </si>
+  <si>
+    <t>22.04.202622</t>
+  </si>
+  <si>
+    <t>22.04.202623</t>
+  </si>
+  <si>
+    <t>22.04.202624</t>
+  </si>
+  <si>
+    <t>23.04.20261</t>
+  </si>
+  <si>
+    <t>23.04.20262</t>
+  </si>
+  <si>
+    <t>23.04.20263</t>
+  </si>
+  <si>
+    <t>23.04.20264</t>
+  </si>
+  <si>
+    <t>23.04.20265</t>
+  </si>
+  <si>
+    <t>23.04.20266</t>
+  </si>
+  <si>
+    <t>23.04.20267</t>
+  </si>
+  <si>
+    <t>23.04.20268</t>
+  </si>
+  <si>
+    <t>23.04.20269</t>
+  </si>
+  <si>
+    <t>23.04.202610</t>
+  </si>
+  <si>
+    <t>23.04.202611</t>
+  </si>
+  <si>
+    <t>23.04.202612</t>
+  </si>
+  <si>
+    <t>23.04.202613</t>
+  </si>
+  <si>
+    <t>23.04.202614</t>
+  </si>
+  <si>
+    <t>23.04.202615</t>
+  </si>
+  <si>
+    <t>23.04.202616</t>
+  </si>
+  <si>
+    <t>23.04.202617</t>
+  </si>
+  <si>
+    <t>23.04.202618</t>
+  </si>
+  <si>
+    <t>23.04.202619</t>
+  </si>
+  <si>
+    <t>23.04.202620</t>
+  </si>
+  <si>
+    <t>23.04.202621</t>
+  </si>
+  <si>
+    <t>23.04.202622</t>
+  </si>
+  <si>
+    <t>23.04.202623</t>
+  </si>
+  <si>
+    <t>23.04.202624</t>
+  </si>
+  <si>
+    <t>24.04.20261</t>
+  </si>
+  <si>
+    <t>24.04.20262</t>
+  </si>
+  <si>
+    <t>24.04.20263</t>
+  </si>
+  <si>
+    <t>24.04.20264</t>
+  </si>
+  <si>
+    <t>24.04.20265</t>
+  </si>
+  <si>
+    <t>24.04.20266</t>
+  </si>
+  <si>
+    <t>24.04.20267</t>
+  </si>
+  <si>
+    <t>24.04.20268</t>
+  </si>
+  <si>
+    <t>24.04.20269</t>
+  </si>
+  <si>
+    <t>24.04.202610</t>
+  </si>
+  <si>
+    <t>24.04.202611</t>
+  </si>
+  <si>
+    <t>24.04.202612</t>
+  </si>
+  <si>
+    <t>24.04.202613</t>
+  </si>
+  <si>
+    <t>24.04.202614</t>
+  </si>
+  <si>
+    <t>24.04.202615</t>
+  </si>
+  <si>
+    <t>24.04.202616</t>
+  </si>
+  <si>
+    <t>24.04.202617</t>
+  </si>
+  <si>
+    <t>24.04.202618</t>
+  </si>
+  <si>
+    <t>24.04.202619</t>
+  </si>
+  <si>
+    <t>24.04.202620</t>
+  </si>
+  <si>
+    <t>24.04.202621</t>
+  </si>
+  <si>
+    <t>24.04.202622</t>
+  </si>
+  <si>
+    <t>24.04.202623</t>
+  </si>
+  <si>
+    <t>24.04.202624</t>
+  </si>
+  <si>
+    <t>25.04.20261</t>
+  </si>
+  <si>
+    <t>25.04.20262</t>
+  </si>
+  <si>
+    <t>25.04.20263</t>
+  </si>
+  <si>
+    <t>25.04.20264</t>
+  </si>
+  <si>
+    <t>25.04.20265</t>
+  </si>
+  <si>
+    <t>25.04.20266</t>
+  </si>
+  <si>
+    <t>25.04.20267</t>
+  </si>
+  <si>
+    <t>25.04.20268</t>
+  </si>
+  <si>
+    <t>25.04.20269</t>
+  </si>
+  <si>
+    <t>25.04.202610</t>
+  </si>
+  <si>
+    <t>25.04.202611</t>
+  </si>
+  <si>
+    <t>25.04.202612</t>
+  </si>
+  <si>
+    <t>25.04.202613</t>
+  </si>
+  <si>
+    <t>25.04.202614</t>
+  </si>
+  <si>
+    <t>25.04.202615</t>
+  </si>
+  <si>
+    <t>25.04.202616</t>
+  </si>
+  <si>
+    <t>25.04.202617</t>
+  </si>
+  <si>
+    <t>25.04.202618</t>
+  </si>
+  <si>
+    <t>25.04.202619</t>
+  </si>
+  <si>
+    <t>25.04.202620</t>
+  </si>
+  <si>
+    <t>25.04.202621</t>
+  </si>
+  <si>
+    <t>25.04.202622</t>
+  </si>
+  <si>
+    <t>25.04.202623</t>
+  </si>
+  <si>
+    <t>25.04.202624</t>
+  </si>
+  <si>
+    <t>26.04.20261</t>
+  </si>
+  <si>
+    <t>26.04.20262</t>
+  </si>
+  <si>
+    <t>26.04.20263</t>
+  </si>
+  <si>
+    <t>26.04.20264</t>
+  </si>
+  <si>
+    <t>26.04.20265</t>
+  </si>
+  <si>
+    <t>26.04.20266</t>
+  </si>
+  <si>
+    <t>26.04.20267</t>
+  </si>
+  <si>
+    <t>26.04.20268</t>
+  </si>
+  <si>
+    <t>26.04.20269</t>
+  </si>
+  <si>
+    <t>26.04.202610</t>
+  </si>
+  <si>
+    <t>26.04.202611</t>
+  </si>
+  <si>
+    <t>26.04.202612</t>
+  </si>
+  <si>
+    <t>26.04.202613</t>
+  </si>
+  <si>
+    <t>26.04.202614</t>
+  </si>
+  <si>
+    <t>26.04.202615</t>
+  </si>
+  <si>
+    <t>26.04.202616</t>
+  </si>
+  <si>
+    <t>26.04.202617</t>
+  </si>
+  <si>
+    <t>26.04.202618</t>
+  </si>
+  <si>
+    <t>26.04.202619</t>
+  </si>
+  <si>
+    <t>26.04.202620</t>
+  </si>
+  <si>
+    <t>26.04.202621</t>
+  </si>
+  <si>
+    <t>26.04.202622</t>
+  </si>
+  <si>
+    <t>26.04.202623</t>
+  </si>
+  <si>
+    <t>26.04.202624</t>
+  </si>
+  <si>
+    <t>27.04.20261</t>
+  </si>
+  <si>
+    <t>27.04.20262</t>
+  </si>
+  <si>
+    <t>27.04.20263</t>
+  </si>
+  <si>
+    <t>27.04.20264</t>
+  </si>
+  <si>
+    <t>27.04.20265</t>
+  </si>
+  <si>
+    <t>27.04.20266</t>
+  </si>
+  <si>
+    <t>27.04.20267</t>
+  </si>
+  <si>
+    <t>27.04.20268</t>
+  </si>
+  <si>
+    <t>27.04.20269</t>
+  </si>
+  <si>
+    <t>27.04.202610</t>
+  </si>
+  <si>
+    <t>27.04.202611</t>
+  </si>
+  <si>
+    <t>27.04.202612</t>
+  </si>
+  <si>
+    <t>27.04.202613</t>
+  </si>
+  <si>
+    <t>27.04.202614</t>
+  </si>
+  <si>
+    <t>27.04.202615</t>
+  </si>
+  <si>
+    <t>27.04.202616</t>
+  </si>
+  <si>
+    <t>27.04.202617</t>
+  </si>
+  <si>
+    <t>27.04.202618</t>
+  </si>
+  <si>
+    <t>27.04.202619</t>
+  </si>
+  <si>
+    <t>27.04.202620</t>
+  </si>
+  <si>
+    <t>27.04.202621</t>
+  </si>
+  <si>
+    <t>27.04.202622</t>
+  </si>
+  <si>
+    <t>27.04.202623</t>
+  </si>
+  <si>
+    <t>27.04.202624</t>
+  </si>
+  <si>
+    <t>28.04.20261</t>
+  </si>
+  <si>
+    <t>28.04.20262</t>
+  </si>
+  <si>
+    <t>28.04.20263</t>
+  </si>
+  <si>
+    <t>28.04.20264</t>
+  </si>
+  <si>
+    <t>28.04.20265</t>
+  </si>
+  <si>
+    <t>28.04.20266</t>
+  </si>
+  <si>
+    <t>28.04.20267</t>
+  </si>
+  <si>
+    <t>28.04.20268</t>
+  </si>
+  <si>
+    <t>28.04.20269</t>
+  </si>
+  <si>
+    <t>28.04.202610</t>
   </si>
 </sst>
 </file>
@@ -913,7 +913,7 @@
     </row>
     <row r="2" spans="1:4">
       <c r="A2" s="2">
-        <v>46122</v>
+        <v>46133</v>
       </c>
       <c r="B2">
         <v>10</v>
@@ -927,7 +927,7 @@
     </row>
     <row r="3" spans="1:4">
       <c r="A3" s="2">
-        <v>46122</v>
+        <v>46133</v>
       </c>
       <c r="B3">
         <v>11</v>
@@ -941,13 +941,13 @@
     </row>
     <row r="4" spans="1:4">
       <c r="A4" s="2">
-        <v>46122</v>
+        <v>46133</v>
       </c>
       <c r="B4">
         <v>12</v>
       </c>
       <c r="C4">
-        <v>3.238</v>
+        <v>2.224</v>
       </c>
       <c r="D4" t="s">
         <v>6</v>
@@ -955,13 +955,13 @@
     </row>
     <row r="5" spans="1:4">
       <c r="A5" s="2">
-        <v>46122</v>
+        <v>46133</v>
       </c>
       <c r="B5">
         <v>13</v>
       </c>
       <c r="C5">
-        <v>2.961</v>
+        <v>1.968</v>
       </c>
       <c r="D5" t="s">
         <v>7</v>
@@ -969,13 +969,13 @@
     </row>
     <row r="6" spans="1:4">
       <c r="A6" s="2">
-        <v>46122</v>
+        <v>46133</v>
       </c>
       <c r="B6">
         <v>14</v>
       </c>
       <c r="C6">
-        <v>2.632</v>
+        <v>2.07</v>
       </c>
       <c r="D6" t="s">
         <v>8</v>
@@ -983,13 +983,13 @@
     </row>
     <row r="7" spans="1:4">
       <c r="A7" s="2">
-        <v>46122</v>
+        <v>46133</v>
       </c>
       <c r="B7">
         <v>15</v>
       </c>
       <c r="C7">
-        <v>2.421</v>
+        <v>1.987</v>
       </c>
       <c r="D7" t="s">
         <v>9</v>
@@ -997,13 +997,13 @@
     </row>
     <row r="8" spans="1:4">
       <c r="A8" s="2">
-        <v>46122</v>
+        <v>46133</v>
       </c>
       <c r="B8">
         <v>16</v>
       </c>
       <c r="C8">
-        <v>1.856</v>
+        <v>1.894</v>
       </c>
       <c r="D8" t="s">
         <v>10</v>
@@ -1011,13 +1011,13 @@
     </row>
     <row r="9" spans="1:4">
       <c r="A9" s="2">
-        <v>46122</v>
+        <v>46133</v>
       </c>
       <c r="B9">
         <v>17</v>
       </c>
       <c r="C9">
-        <v>1.687</v>
+        <v>1.587</v>
       </c>
       <c r="D9" t="s">
         <v>11</v>
@@ -1025,13 +1025,13 @@
     </row>
     <row r="10" spans="1:4">
       <c r="A10" s="2">
-        <v>46122</v>
+        <v>46133</v>
       </c>
       <c r="B10">
         <v>18</v>
       </c>
       <c r="C10">
-        <v>1.091</v>
+        <v>0.88</v>
       </c>
       <c r="D10" t="s">
         <v>12</v>
@@ -1039,13 +1039,13 @@
     </row>
     <row r="11" spans="1:4">
       <c r="A11" s="2">
-        <v>46122</v>
+        <v>46133</v>
       </c>
       <c r="B11">
         <v>19</v>
       </c>
       <c r="C11">
-        <v>0.438</v>
+        <v>0.426</v>
       </c>
       <c r="D11" t="s">
         <v>13</v>
@@ -1053,13 +1053,13 @@
     </row>
     <row r="12" spans="1:4">
       <c r="A12" s="2">
-        <v>46122</v>
+        <v>46133</v>
       </c>
       <c r="B12">
         <v>20</v>
       </c>
       <c r="C12">
-        <v>0.06900000000000001</v>
+        <v>0.08400000000000001</v>
       </c>
       <c r="D12" t="s">
         <v>14</v>
@@ -1067,7 +1067,7 @@
     </row>
     <row r="13" spans="1:4">
       <c r="A13" s="2">
-        <v>46122</v>
+        <v>46133</v>
       </c>
       <c r="B13">
         <v>21</v>
@@ -1081,7 +1081,7 @@
     </row>
     <row r="14" spans="1:4">
       <c r="A14" s="2">
-        <v>46122</v>
+        <v>46133</v>
       </c>
       <c r="B14">
         <v>22</v>
@@ -1095,7 +1095,7 @@
     </row>
     <row r="15" spans="1:4">
       <c r="A15" s="2">
-        <v>46122</v>
+        <v>46133</v>
       </c>
       <c r="B15">
         <v>23</v>
@@ -1109,7 +1109,7 @@
     </row>
     <row r="16" spans="1:4">
       <c r="A16" s="2">
-        <v>46122</v>
+        <v>46133</v>
       </c>
       <c r="B16">
         <v>24</v>
@@ -1123,7 +1123,7 @@
     </row>
     <row r="17" spans="1:4">
       <c r="A17" s="2">
-        <v>46123</v>
+        <v>46134</v>
       </c>
       <c r="B17">
         <v>1</v>
@@ -1137,7 +1137,7 @@
     </row>
     <row r="18" spans="1:4">
       <c r="A18" s="2">
-        <v>46123</v>
+        <v>46134</v>
       </c>
       <c r="B18">
         <v>2</v>
@@ -1151,7 +1151,7 @@
     </row>
     <row r="19" spans="1:4">
       <c r="A19" s="2">
-        <v>46123</v>
+        <v>46134</v>
       </c>
       <c r="B19">
         <v>3</v>
@@ -1165,7 +1165,7 @@
     </row>
     <row r="20" spans="1:4">
       <c r="A20" s="2">
-        <v>46123</v>
+        <v>46134</v>
       </c>
       <c r="B20">
         <v>4</v>
@@ -1179,7 +1179,7 @@
     </row>
     <row r="21" spans="1:4">
       <c r="A21" s="2">
-        <v>46123</v>
+        <v>46134</v>
       </c>
       <c r="B21">
         <v>5</v>
@@ -1193,7 +1193,7 @@
     </row>
     <row r="22" spans="1:4">
       <c r="A22" s="2">
-        <v>46123</v>
+        <v>46134</v>
       </c>
       <c r="B22">
         <v>6</v>
@@ -1207,13 +1207,13 @@
     </row>
     <row r="23" spans="1:4">
       <c r="A23" s="2">
-        <v>46123</v>
+        <v>46134</v>
       </c>
       <c r="B23">
         <v>7</v>
       </c>
       <c r="C23">
-        <v>0</v>
+        <v>0.013</v>
       </c>
       <c r="D23" t="s">
         <v>25</v>
@@ -1221,13 +1221,13 @@
     </row>
     <row r="24" spans="1:4">
       <c r="A24" s="2">
-        <v>46123</v>
+        <v>46134</v>
       </c>
       <c r="B24">
         <v>8</v>
       </c>
       <c r="C24">
-        <v>0.154</v>
+        <v>0.242</v>
       </c>
       <c r="D24" t="s">
         <v>26</v>
@@ -1235,13 +1235,13 @@
     </row>
     <row r="25" spans="1:4">
       <c r="A25" s="2">
-        <v>46123</v>
+        <v>46134</v>
       </c>
       <c r="B25">
         <v>9</v>
       </c>
       <c r="C25">
-        <v>0.6909999999999999</v>
+        <v>0.772</v>
       </c>
       <c r="D25" t="s">
         <v>27</v>
@@ -1249,13 +1249,13 @@
     </row>
     <row r="26" spans="1:4">
       <c r="A26" s="2">
-        <v>46123</v>
+        <v>46134</v>
       </c>
       <c r="B26">
         <v>10</v>
       </c>
       <c r="C26">
-        <v>1.175</v>
+        <v>1.524</v>
       </c>
       <c r="D26" t="s">
         <v>28</v>
@@ -1263,13 +1263,13 @@
     </row>
     <row r="27" spans="1:4">
       <c r="A27" s="2">
-        <v>46123</v>
+        <v>46134</v>
       </c>
       <c r="B27">
         <v>11</v>
       </c>
       <c r="C27">
-        <v>1.871</v>
+        <v>2.111</v>
       </c>
       <c r="D27" t="s">
         <v>29</v>
@@ -1277,13 +1277,13 @@
     </row>
     <row r="28" spans="1:4">
       <c r="A28" s="2">
-        <v>46123</v>
+        <v>46134</v>
       </c>
       <c r="B28">
         <v>12</v>
       </c>
       <c r="C28">
-        <v>2.031</v>
+        <v>2.502</v>
       </c>
       <c r="D28" t="s">
         <v>30</v>
@@ -1291,13 +1291,13 @@
     </row>
     <row r="29" spans="1:4">
       <c r="A29" s="2">
-        <v>46123</v>
+        <v>46134</v>
       </c>
       <c r="B29">
         <v>13</v>
       </c>
       <c r="C29">
-        <v>2.02</v>
+        <v>2.611</v>
       </c>
       <c r="D29" t="s">
         <v>31</v>
@@ -1305,13 +1305,13 @@
     </row>
     <row r="30" spans="1:4">
       <c r="A30" s="2">
-        <v>46123</v>
+        <v>46134</v>
       </c>
       <c r="B30">
         <v>14</v>
       </c>
       <c r="C30">
-        <v>2.062</v>
+        <v>2.417</v>
       </c>
       <c r="D30" t="s">
         <v>32</v>
@@ -1319,13 +1319,13 @@
     </row>
     <row r="31" spans="1:4">
       <c r="A31" s="2">
-        <v>46123</v>
+        <v>46134</v>
       </c>
       <c r="B31">
         <v>15</v>
       </c>
       <c r="C31">
-        <v>1.985</v>
+        <v>2.118</v>
       </c>
       <c r="D31" t="s">
         <v>33</v>
@@ -1333,13 +1333,13 @@
     </row>
     <row r="32" spans="1:4">
       <c r="A32" s="2">
-        <v>46123</v>
+        <v>46134</v>
       </c>
       <c r="B32">
         <v>16</v>
       </c>
       <c r="C32">
-        <v>1.934</v>
+        <v>1.922</v>
       </c>
       <c r="D32" t="s">
         <v>34</v>
@@ -1347,13 +1347,13 @@
     </row>
     <row r="33" spans="1:4">
       <c r="A33" s="2">
-        <v>46123</v>
+        <v>46134</v>
       </c>
       <c r="B33">
         <v>17</v>
       </c>
       <c r="C33">
-        <v>1.532</v>
+        <v>1.893</v>
       </c>
       <c r="D33" t="s">
         <v>35</v>
@@ -1361,13 +1361,13 @@
     </row>
     <row r="34" spans="1:4">
       <c r="A34" s="2">
-        <v>46123</v>
+        <v>46134</v>
       </c>
       <c r="B34">
         <v>18</v>
       </c>
       <c r="C34">
-        <v>0.901</v>
+        <v>1.341</v>
       </c>
       <c r="D34" t="s">
         <v>36</v>
@@ -1375,13 +1375,13 @@
     </row>
     <row r="35" spans="1:4">
       <c r="A35" s="2">
-        <v>46123</v>
+        <v>46134</v>
       </c>
       <c r="B35">
         <v>19</v>
       </c>
       <c r="C35">
-        <v>0.395</v>
+        <v>0.615</v>
       </c>
       <c r="D35" t="s">
         <v>37</v>
@@ -1389,13 +1389,13 @@
     </row>
     <row r="36" spans="1:4">
       <c r="A36" s="2">
-        <v>46123</v>
+        <v>46134</v>
       </c>
       <c r="B36">
         <v>20</v>
       </c>
       <c r="C36">
-        <v>0.061</v>
+        <v>0.122</v>
       </c>
       <c r="D36" t="s">
         <v>38</v>
@@ -1403,7 +1403,7 @@
     </row>
     <row r="37" spans="1:4">
       <c r="A37" s="2">
-        <v>46123</v>
+        <v>46134</v>
       </c>
       <c r="B37">
         <v>21</v>
@@ -1417,7 +1417,7 @@
     </row>
     <row r="38" spans="1:4">
       <c r="A38" s="2">
-        <v>46123</v>
+        <v>46134</v>
       </c>
       <c r="B38">
         <v>22</v>
@@ -1431,7 +1431,7 @@
     </row>
     <row r="39" spans="1:4">
       <c r="A39" s="2">
-        <v>46123</v>
+        <v>46134</v>
       </c>
       <c r="B39">
         <v>23</v>
@@ -1445,7 +1445,7 @@
     </row>
     <row r="40" spans="1:4">
       <c r="A40" s="2">
-        <v>46123</v>
+        <v>46134</v>
       </c>
       <c r="B40">
         <v>24</v>
@@ -1459,7 +1459,7 @@
     </row>
     <row r="41" spans="1:4">
       <c r="A41" s="2">
-        <v>46124</v>
+        <v>46135</v>
       </c>
       <c r="B41">
         <v>1</v>
@@ -1473,7 +1473,7 @@
     </row>
     <row r="42" spans="1:4">
       <c r="A42" s="2">
-        <v>46124</v>
+        <v>46135</v>
       </c>
       <c r="B42">
         <v>2</v>
@@ -1487,7 +1487,7 @@
     </row>
     <row r="43" spans="1:4">
       <c r="A43" s="2">
-        <v>46124</v>
+        <v>46135</v>
       </c>
       <c r="B43">
         <v>3</v>
@@ -1501,7 +1501,7 @@
     </row>
     <row r="44" spans="1:4">
       <c r="A44" s="2">
-        <v>46124</v>
+        <v>46135</v>
       </c>
       <c r="B44">
         <v>4</v>
@@ -1515,7 +1515,7 @@
     </row>
     <row r="45" spans="1:4">
       <c r="A45" s="2">
-        <v>46124</v>
+        <v>46135</v>
       </c>
       <c r="B45">
         <v>5</v>
@@ -1529,7 +1529,7 @@
     </row>
     <row r="46" spans="1:4">
       <c r="A46" s="2">
-        <v>46124</v>
+        <v>46135</v>
       </c>
       <c r="B46">
         <v>6</v>
@@ -1543,13 +1543,13 @@
     </row>
     <row r="47" spans="1:4">
       <c r="A47" s="2">
-        <v>46124</v>
+        <v>46135</v>
       </c>
       <c r="B47">
         <v>7</v>
       </c>
       <c r="C47">
-        <v>0</v>
+        <v>0.014</v>
       </c>
       <c r="D47" t="s">
         <v>49</v>
@@ -1557,13 +1557,13 @@
     </row>
     <row r="48" spans="1:4">
       <c r="A48" s="2">
-        <v>46124</v>
+        <v>46135</v>
       </c>
       <c r="B48">
         <v>8</v>
       </c>
       <c r="C48">
-        <v>0.19</v>
+        <v>0.321</v>
       </c>
       <c r="D48" t="s">
         <v>50</v>
@@ -1571,13 +1571,13 @@
     </row>
     <row r="49" spans="1:4">
       <c r="A49" s="2">
-        <v>46124</v>
+        <v>46135</v>
       </c>
       <c r="B49">
         <v>9</v>
       </c>
       <c r="C49">
-        <v>0.9330000000000001</v>
+        <v>0.791</v>
       </c>
       <c r="D49" t="s">
         <v>51</v>
@@ -1585,13 +1585,13 @@
     </row>
     <row r="50" spans="1:4">
       <c r="A50" s="2">
-        <v>46124</v>
+        <v>46135</v>
       </c>
       <c r="B50">
         <v>10</v>
       </c>
       <c r="C50">
-        <v>1.932</v>
+        <v>1.197</v>
       </c>
       <c r="D50" t="s">
         <v>52</v>
@@ -1599,13 +1599,13 @@
     </row>
     <row r="51" spans="1:4">
       <c r="A51" s="2">
-        <v>46124</v>
+        <v>46135</v>
       </c>
       <c r="B51">
         <v>11</v>
       </c>
       <c r="C51">
-        <v>2.694</v>
+        <v>1.558</v>
       </c>
       <c r="D51" t="s">
         <v>53</v>
@@ -1613,13 +1613,13 @@
     </row>
     <row r="52" spans="1:4">
       <c r="A52" s="2">
-        <v>46124</v>
+        <v>46135</v>
       </c>
       <c r="B52">
         <v>12</v>
       </c>
       <c r="C52">
-        <v>3.077</v>
+        <v>1.894</v>
       </c>
       <c r="D52" t="s">
         <v>54</v>
@@ -1627,13 +1627,13 @@
     </row>
     <row r="53" spans="1:4">
       <c r="A53" s="2">
-        <v>46124</v>
+        <v>46135</v>
       </c>
       <c r="B53">
         <v>13</v>
       </c>
       <c r="C53">
-        <v>3.132</v>
+        <v>1.99</v>
       </c>
       <c r="D53" t="s">
         <v>55</v>
@@ -1641,13 +1641,13 @@
     </row>
     <row r="54" spans="1:4">
       <c r="A54" s="2">
-        <v>46124</v>
+        <v>46135</v>
       </c>
       <c r="B54">
         <v>14</v>
       </c>
       <c r="C54">
-        <v>3.161</v>
+        <v>2.029</v>
       </c>
       <c r="D54" t="s">
         <v>56</v>
@@ -1655,13 +1655,13 @@
     </row>
     <row r="55" spans="1:4">
       <c r="A55" s="2">
-        <v>46124</v>
+        <v>46135</v>
       </c>
       <c r="B55">
         <v>15</v>
       </c>
       <c r="C55">
-        <v>3.048</v>
+        <v>2</v>
       </c>
       <c r="D55" t="s">
         <v>57</v>
@@ -1669,13 +1669,13 @@
     </row>
     <row r="56" spans="1:4">
       <c r="A56" s="2">
-        <v>46124</v>
+        <v>46135</v>
       </c>
       <c r="B56">
         <v>16</v>
       </c>
       <c r="C56">
-        <v>2.632</v>
+        <v>1.859</v>
       </c>
       <c r="D56" t="s">
         <v>58</v>
@@ -1683,13 +1683,13 @@
     </row>
     <row r="57" spans="1:4">
       <c r="A57" s="2">
-        <v>46124</v>
+        <v>46135</v>
       </c>
       <c r="B57">
         <v>17</v>
       </c>
       <c r="C57">
-        <v>2.25</v>
+        <v>1.337</v>
       </c>
       <c r="D57" t="s">
         <v>59</v>
@@ -1697,13 +1697,13 @@
     </row>
     <row r="58" spans="1:4">
       <c r="A58" s="2">
-        <v>46124</v>
+        <v>46135</v>
       </c>
       <c r="B58">
         <v>18</v>
       </c>
       <c r="C58">
-        <v>1.471</v>
+        <v>0.766</v>
       </c>
       <c r="D58" t="s">
         <v>60</v>
@@ -1711,13 +1711,13 @@
     </row>
     <row r="59" spans="1:4">
       <c r="A59" s="2">
-        <v>46124</v>
+        <v>46135</v>
       </c>
       <c r="B59">
         <v>19</v>
       </c>
       <c r="C59">
-        <v>0.523</v>
+        <v>0.387</v>
       </c>
       <c r="D59" t="s">
         <v>61</v>
@@ -1725,13 +1725,13 @@
     </row>
     <row r="60" spans="1:4">
       <c r="A60" s="2">
-        <v>46124</v>
+        <v>46135</v>
       </c>
       <c r="B60">
         <v>20</v>
       </c>
       <c r="C60">
-        <v>0.066</v>
+        <v>0.067</v>
       </c>
       <c r="D60" t="s">
         <v>62</v>
@@ -1739,7 +1739,7 @@
     </row>
     <row r="61" spans="1:4">
       <c r="A61" s="2">
-        <v>46124</v>
+        <v>46135</v>
       </c>
       <c r="B61">
         <v>21</v>
@@ -1753,7 +1753,7 @@
     </row>
     <row r="62" spans="1:4">
       <c r="A62" s="2">
-        <v>46124</v>
+        <v>46135</v>
       </c>
       <c r="B62">
         <v>22</v>
@@ -1767,7 +1767,7 @@
     </row>
     <row r="63" spans="1:4">
       <c r="A63" s="2">
-        <v>46124</v>
+        <v>46135</v>
       </c>
       <c r="B63">
         <v>23</v>
@@ -1781,7 +1781,7 @@
     </row>
     <row r="64" spans="1:4">
       <c r="A64" s="2">
-        <v>46124</v>
+        <v>46135</v>
       </c>
       <c r="B64">
         <v>24</v>
@@ -1795,7 +1795,7 @@
     </row>
     <row r="65" spans="1:4">
       <c r="A65" s="2">
-        <v>46125</v>
+        <v>46136</v>
       </c>
       <c r="B65">
         <v>1</v>
@@ -1809,7 +1809,7 @@
     </row>
     <row r="66" spans="1:4">
       <c r="A66" s="2">
-        <v>46125</v>
+        <v>46136</v>
       </c>
       <c r="B66">
         <v>2</v>
@@ -1823,7 +1823,7 @@
     </row>
     <row r="67" spans="1:4">
       <c r="A67" s="2">
-        <v>46125</v>
+        <v>46136</v>
       </c>
       <c r="B67">
         <v>3</v>
@@ -1837,7 +1837,7 @@
     </row>
     <row r="68" spans="1:4">
       <c r="A68" s="2">
-        <v>46125</v>
+        <v>46136</v>
       </c>
       <c r="B68">
         <v>4</v>
@@ -1851,7 +1851,7 @@
     </row>
     <row r="69" spans="1:4">
       <c r="A69" s="2">
-        <v>46125</v>
+        <v>46136</v>
       </c>
       <c r="B69">
         <v>5</v>
@@ -1865,7 +1865,7 @@
     </row>
     <row r="70" spans="1:4">
       <c r="A70" s="2">
-        <v>46125</v>
+        <v>46136</v>
       </c>
       <c r="B70">
         <v>6</v>
@@ -1879,13 +1879,13 @@
     </row>
     <row r="71" spans="1:4">
       <c r="A71" s="2">
-        <v>46125</v>
+        <v>46136</v>
       </c>
       <c r="B71">
         <v>7</v>
       </c>
       <c r="C71">
-        <v>0</v>
+        <v>0.028</v>
       </c>
       <c r="D71" t="s">
         <v>73</v>
@@ -1893,13 +1893,13 @@
     </row>
     <row r="72" spans="1:4">
       <c r="A72" s="2">
-        <v>46125</v>
+        <v>46136</v>
       </c>
       <c r="B72">
         <v>8</v>
       </c>
       <c r="C72">
-        <v>0.179</v>
+        <v>0.404</v>
       </c>
       <c r="D72" t="s">
         <v>74</v>
@@ -1907,13 +1907,13 @@
     </row>
     <row r="73" spans="1:4">
       <c r="A73" s="2">
-        <v>46125</v>
+        <v>46136</v>
       </c>
       <c r="B73">
         <v>9</v>
       </c>
       <c r="C73">
-        <v>0.893</v>
+        <v>1.082</v>
       </c>
       <c r="D73" t="s">
         <v>75</v>
@@ -1921,13 +1921,13 @@
     </row>
     <row r="74" spans="1:4">
       <c r="A74" s="2">
-        <v>46125</v>
+        <v>46136</v>
       </c>
       <c r="B74">
         <v>10</v>
       </c>
       <c r="C74">
-        <v>1.904</v>
+        <v>1.867</v>
       </c>
       <c r="D74" t="s">
         <v>76</v>
@@ -1935,13 +1935,13 @@
     </row>
     <row r="75" spans="1:4">
       <c r="A75" s="2">
-        <v>46125</v>
+        <v>46136</v>
       </c>
       <c r="B75">
         <v>11</v>
       </c>
       <c r="C75">
-        <v>2.608</v>
+        <v>2.068</v>
       </c>
       <c r="D75" t="s">
         <v>77</v>
@@ -1949,13 +1949,13 @@
     </row>
     <row r="76" spans="1:4">
       <c r="A76" s="2">
-        <v>46125</v>
+        <v>46136</v>
       </c>
       <c r="B76">
         <v>12</v>
       </c>
       <c r="C76">
-        <v>3.088</v>
+        <v>1.991</v>
       </c>
       <c r="D76" t="s">
         <v>78</v>
@@ -1963,13 +1963,13 @@
     </row>
     <row r="77" spans="1:4">
       <c r="A77" s="2">
-        <v>46125</v>
+        <v>46136</v>
       </c>
       <c r="B77">
         <v>13</v>
       </c>
       <c r="C77">
-        <v>3.065</v>
+        <v>1.887</v>
       </c>
       <c r="D77" t="s">
         <v>79</v>
@@ -1977,13 +1977,13 @@
     </row>
     <row r="78" spans="1:4">
       <c r="A78" s="2">
-        <v>46125</v>
+        <v>46136</v>
       </c>
       <c r="B78">
         <v>14</v>
       </c>
       <c r="C78">
-        <v>2.974</v>
+        <v>1.863</v>
       </c>
       <c r="D78" t="s">
         <v>80</v>
@@ -1991,13 +1991,13 @@
     </row>
     <row r="79" spans="1:4">
       <c r="A79" s="2">
-        <v>46125</v>
+        <v>46136</v>
       </c>
       <c r="B79">
         <v>15</v>
       </c>
       <c r="C79">
-        <v>2.902</v>
+        <v>1.904</v>
       </c>
       <c r="D79" t="s">
         <v>81</v>
@@ -2005,13 +2005,13 @@
     </row>
     <row r="80" spans="1:4">
       <c r="A80" s="2">
-        <v>46125</v>
+        <v>46136</v>
       </c>
       <c r="B80">
         <v>16</v>
       </c>
       <c r="C80">
-        <v>2.393</v>
+        <v>1.729</v>
       </c>
       <c r="D80" t="s">
         <v>82</v>
@@ -2019,13 +2019,13 @@
     </row>
     <row r="81" spans="1:4">
       <c r="A81" s="2">
-        <v>46125</v>
+        <v>46136</v>
       </c>
       <c r="B81">
         <v>17</v>
       </c>
       <c r="C81">
-        <v>1.987</v>
+        <v>1.516</v>
       </c>
       <c r="D81" t="s">
         <v>83</v>
@@ -2033,13 +2033,13 @@
     </row>
     <row r="82" spans="1:4">
       <c r="A82" s="2">
-        <v>46125</v>
+        <v>46136</v>
       </c>
       <c r="B82">
         <v>18</v>
       </c>
       <c r="C82">
-        <v>1.224</v>
+        <v>1.061</v>
       </c>
       <c r="D82" t="s">
         <v>84</v>
@@ -2047,13 +2047,13 @@
     </row>
     <row r="83" spans="1:4">
       <c r="A83" s="2">
-        <v>46125</v>
+        <v>46136</v>
       </c>
       <c r="B83">
         <v>19</v>
       </c>
       <c r="C83">
-        <v>0.457</v>
+        <v>0.454</v>
       </c>
       <c r="D83" t="s">
         <v>85</v>
@@ -2061,13 +2061,13 @@
     </row>
     <row r="84" spans="1:4">
       <c r="A84" s="2">
-        <v>46125</v>
+        <v>46136</v>
       </c>
       <c r="B84">
         <v>20</v>
       </c>
       <c r="C84">
-        <v>0.067</v>
+        <v>0.098</v>
       </c>
       <c r="D84" t="s">
         <v>86</v>
@@ -2075,7 +2075,7 @@
     </row>
     <row r="85" spans="1:4">
       <c r="A85" s="2">
-        <v>46125</v>
+        <v>46136</v>
       </c>
       <c r="B85">
         <v>21</v>
@@ -2089,7 +2089,7 @@
     </row>
     <row r="86" spans="1:4">
       <c r="A86" s="2">
-        <v>46125</v>
+        <v>46136</v>
       </c>
       <c r="B86">
         <v>22</v>
@@ -2103,7 +2103,7 @@
     </row>
     <row r="87" spans="1:4">
       <c r="A87" s="2">
-        <v>46125</v>
+        <v>46136</v>
       </c>
       <c r="B87">
         <v>23</v>
@@ -2117,7 +2117,7 @@
     </row>
     <row r="88" spans="1:4">
       <c r="A88" s="2">
-        <v>46125</v>
+        <v>46136</v>
       </c>
       <c r="B88">
         <v>24</v>
@@ -2131,7 +2131,7 @@
     </row>
     <row r="89" spans="1:4">
       <c r="A89" s="2">
-        <v>46126</v>
+        <v>46137</v>
       </c>
       <c r="B89">
         <v>1</v>
@@ -2145,7 +2145,7 @@
     </row>
     <row r="90" spans="1:4">
       <c r="A90" s="2">
-        <v>46126</v>
+        <v>46137</v>
       </c>
       <c r="B90">
         <v>2</v>
@@ -2159,7 +2159,7 @@
     </row>
     <row r="91" spans="1:4">
       <c r="A91" s="2">
-        <v>46126</v>
+        <v>46137</v>
       </c>
       <c r="B91">
         <v>3</v>
@@ -2173,7 +2173,7 @@
     </row>
     <row r="92" spans="1:4">
       <c r="A92" s="2">
-        <v>46126</v>
+        <v>46137</v>
       </c>
       <c r="B92">
         <v>4</v>
@@ -2187,7 +2187,7 @@
     </row>
     <row r="93" spans="1:4">
       <c r="A93" s="2">
-        <v>46126</v>
+        <v>46137</v>
       </c>
       <c r="B93">
         <v>5</v>
@@ -2201,7 +2201,7 @@
     </row>
     <row r="94" spans="1:4">
       <c r="A94" s="2">
-        <v>46126</v>
+        <v>46137</v>
       </c>
       <c r="B94">
         <v>6</v>
@@ -2215,13 +2215,13 @@
     </row>
     <row r="95" spans="1:4">
       <c r="A95" s="2">
-        <v>46126</v>
+        <v>46137</v>
       </c>
       <c r="B95">
         <v>7</v>
       </c>
       <c r="C95">
-        <v>0</v>
+        <v>0.015</v>
       </c>
       <c r="D95" t="s">
         <v>97</v>
@@ -2229,13 +2229,13 @@
     </row>
     <row r="96" spans="1:4">
       <c r="A96" s="2">
-        <v>46126</v>
+        <v>46137</v>
       </c>
       <c r="B96">
         <v>8</v>
       </c>
       <c r="C96">
-        <v>0.179</v>
+        <v>0.314</v>
       </c>
       <c r="D96" t="s">
         <v>98</v>
@@ -2243,13 +2243,13 @@
     </row>
     <row r="97" spans="1:4">
       <c r="A97" s="2">
-        <v>46126</v>
+        <v>46137</v>
       </c>
       <c r="B97">
         <v>9</v>
       </c>
       <c r="C97">
-        <v>0.773</v>
+        <v>0.882</v>
       </c>
       <c r="D97" t="s">
         <v>99</v>
@@ -2257,13 +2257,13 @@
     </row>
     <row r="98" spans="1:4">
       <c r="A98" s="2">
-        <v>46126</v>
+        <v>46137</v>
       </c>
       <c r="B98">
         <v>10</v>
       </c>
       <c r="C98">
-        <v>1.553</v>
+        <v>1.406</v>
       </c>
       <c r="D98" t="s">
         <v>100</v>
@@ -2271,13 +2271,13 @@
     </row>
     <row r="99" spans="1:4">
       <c r="A99" s="2">
-        <v>46126</v>
+        <v>46137</v>
       </c>
       <c r="B99">
         <v>11</v>
       </c>
       <c r="C99">
-        <v>1.885</v>
+        <v>1.84</v>
       </c>
       <c r="D99" t="s">
         <v>101</v>
@@ -2285,13 +2285,13 @@
     </row>
     <row r="100" spans="1:4">
       <c r="A100" s="2">
-        <v>46126</v>
+        <v>46137</v>
       </c>
       <c r="B100">
         <v>12</v>
       </c>
       <c r="C100">
-        <v>2.004</v>
+        <v>1.978</v>
       </c>
       <c r="D100" t="s">
         <v>102</v>
@@ -2299,13 +2299,13 @@
     </row>
     <row r="101" spans="1:4">
       <c r="A101" s="2">
-        <v>46126</v>
+        <v>46137</v>
       </c>
       <c r="B101">
         <v>13</v>
       </c>
       <c r="C101">
-        <v>1.98</v>
+        <v>1.958</v>
       </c>
       <c r="D101" t="s">
         <v>103</v>
@@ -2313,13 +2313,13 @@
     </row>
     <row r="102" spans="1:4">
       <c r="A102" s="2">
-        <v>46126</v>
+        <v>46137</v>
       </c>
       <c r="B102">
         <v>14</v>
       </c>
       <c r="C102">
-        <v>2.016</v>
+        <v>1.931</v>
       </c>
       <c r="D102" t="s">
         <v>104</v>
@@ -2327,13 +2327,13 @@
     </row>
     <row r="103" spans="1:4">
       <c r="A103" s="2">
-        <v>46126</v>
+        <v>46137</v>
       </c>
       <c r="B103">
         <v>15</v>
       </c>
       <c r="C103">
-        <v>2.049</v>
+        <v>1.939</v>
       </c>
       <c r="D103" t="s">
         <v>105</v>
@@ -2341,13 +2341,13 @@
     </row>
     <row r="104" spans="1:4">
       <c r="A104" s="2">
-        <v>46126</v>
+        <v>46137</v>
       </c>
       <c r="B104">
         <v>16</v>
       </c>
       <c r="C104">
-        <v>1.994</v>
+        <v>1.619</v>
       </c>
       <c r="D104" t="s">
         <v>106</v>
@@ -2355,13 +2355,13 @@
     </row>
     <row r="105" spans="1:4">
       <c r="A105" s="2">
-        <v>46126</v>
+        <v>46137</v>
       </c>
       <c r="B105">
         <v>17</v>
       </c>
       <c r="C105">
-        <v>1.825</v>
+        <v>1.317</v>
       </c>
       <c r="D105" t="s">
         <v>107</v>
@@ -2369,13 +2369,13 @@
     </row>
     <row r="106" spans="1:4">
       <c r="A106" s="2">
-        <v>46126</v>
+        <v>46137</v>
       </c>
       <c r="B106">
         <v>18</v>
       </c>
       <c r="C106">
-        <v>1.135</v>
+        <v>0.857</v>
       </c>
       <c r="D106" t="s">
         <v>108</v>
@@ -2383,13 +2383,13 @@
     </row>
     <row r="107" spans="1:4">
       <c r="A107" s="2">
-        <v>46126</v>
+        <v>46137</v>
       </c>
       <c r="B107">
         <v>19</v>
       </c>
       <c r="C107">
-        <v>0.462</v>
+        <v>0.424</v>
       </c>
       <c r="D107" t="s">
         <v>109</v>
@@ -2397,13 +2397,13 @@
     </row>
     <row r="108" spans="1:4">
       <c r="A108" s="2">
-        <v>46126</v>
+        <v>46137</v>
       </c>
       <c r="B108">
         <v>20</v>
       </c>
       <c r="C108">
-        <v>0.07099999999999999</v>
+        <v>0.06900000000000001</v>
       </c>
       <c r="D108" t="s">
         <v>110</v>
@@ -2411,7 +2411,7 @@
     </row>
     <row r="109" spans="1:4">
       <c r="A109" s="2">
-        <v>46126</v>
+        <v>46137</v>
       </c>
       <c r="B109">
         <v>21</v>
@@ -2425,7 +2425,7 @@
     </row>
     <row r="110" spans="1:4">
       <c r="A110" s="2">
-        <v>46126</v>
+        <v>46137</v>
       </c>
       <c r="B110">
         <v>22</v>
@@ -2439,7 +2439,7 @@
     </row>
     <row r="111" spans="1:4">
       <c r="A111" s="2">
-        <v>46126</v>
+        <v>46137</v>
       </c>
       <c r="B111">
         <v>23</v>
@@ -2453,7 +2453,7 @@
     </row>
     <row r="112" spans="1:4">
       <c r="A112" s="2">
-        <v>46126</v>
+        <v>46137</v>
       </c>
       <c r="B112">
         <v>24</v>
@@ -2467,7 +2467,7 @@
     </row>
     <row r="113" spans="1:4">
       <c r="A113" s="2">
-        <v>46127</v>
+        <v>46138</v>
       </c>
       <c r="B113">
         <v>1</v>
@@ -2481,7 +2481,7 @@
     </row>
     <row r="114" spans="1:4">
       <c r="A114" s="2">
-        <v>46127</v>
+        <v>46138</v>
       </c>
       <c r="B114">
         <v>2</v>
@@ -2495,7 +2495,7 @@
     </row>
     <row r="115" spans="1:4">
       <c r="A115" s="2">
-        <v>46127</v>
+        <v>46138</v>
       </c>
       <c r="B115">
         <v>3</v>
@@ -2509,7 +2509,7 @@
     </row>
     <row r="116" spans="1:4">
       <c r="A116" s="2">
-        <v>46127</v>
+        <v>46138</v>
       </c>
       <c r="B116">
         <v>4</v>
@@ -2523,7 +2523,7 @@
     </row>
     <row r="117" spans="1:4">
       <c r="A117" s="2">
-        <v>46127</v>
+        <v>46138</v>
       </c>
       <c r="B117">
         <v>5</v>
@@ -2537,7 +2537,7 @@
     </row>
     <row r="118" spans="1:4">
       <c r="A118" s="2">
-        <v>46127</v>
+        <v>46138</v>
       </c>
       <c r="B118">
         <v>6</v>
@@ -2551,13 +2551,13 @@
     </row>
     <row r="119" spans="1:4">
       <c r="A119" s="2">
-        <v>46127</v>
+        <v>46138</v>
       </c>
       <c r="B119">
         <v>7</v>
       </c>
       <c r="C119">
-        <v>0</v>
+        <v>0.029</v>
       </c>
       <c r="D119" t="s">
         <v>121</v>
@@ -2565,13 +2565,13 @@
     </row>
     <row r="120" spans="1:4">
       <c r="A120" s="2">
-        <v>46127</v>
+        <v>46138</v>
       </c>
       <c r="B120">
         <v>8</v>
       </c>
       <c r="C120">
-        <v>0.228</v>
+        <v>0.37</v>
       </c>
       <c r="D120" t="s">
         <v>122</v>
@@ -2579,13 +2579,13 @@
     </row>
     <row r="121" spans="1:4">
       <c r="A121" s="2">
-        <v>46127</v>
+        <v>46138</v>
       </c>
       <c r="B121">
         <v>9</v>
       </c>
       <c r="C121">
-        <v>0.914</v>
+        <v>1.048</v>
       </c>
       <c r="D121" t="s">
         <v>123</v>
@@ -2593,13 +2593,13 @@
     </row>
     <row r="122" spans="1:4">
       <c r="A122" s="2">
-        <v>46127</v>
+        <v>46138</v>
       </c>
       <c r="B122">
         <v>10</v>
       </c>
       <c r="C122">
-        <v>1.899</v>
+        <v>1.783</v>
       </c>
       <c r="D122" t="s">
         <v>124</v>
@@ -2607,13 +2607,13 @@
     </row>
     <row r="123" spans="1:4">
       <c r="A123" s="2">
-        <v>46127</v>
+        <v>46138</v>
       </c>
       <c r="B123">
         <v>11</v>
       </c>
       <c r="C123">
-        <v>2.567</v>
+        <v>2.024</v>
       </c>
       <c r="D123" t="s">
         <v>125</v>
@@ -2621,13 +2621,13 @@
     </row>
     <row r="124" spans="1:4">
       <c r="A124" s="2">
-        <v>46127</v>
+        <v>46138</v>
       </c>
       <c r="B124">
         <v>12</v>
       </c>
       <c r="C124">
-        <v>3.049</v>
+        <v>1.998</v>
       </c>
       <c r="D124" t="s">
         <v>126</v>
@@ -2635,13 +2635,13 @@
     </row>
     <row r="125" spans="1:4">
       <c r="A125" s="2">
-        <v>46127</v>
+        <v>46138</v>
       </c>
       <c r="B125">
         <v>13</v>
       </c>
       <c r="C125">
-        <v>3.26</v>
+        <v>1.963</v>
       </c>
       <c r="D125" t="s">
         <v>127</v>
@@ -2649,13 +2649,13 @@
     </row>
     <row r="126" spans="1:4">
       <c r="A126" s="2">
-        <v>46127</v>
+        <v>46138</v>
       </c>
       <c r="B126">
         <v>14</v>
       </c>
       <c r="C126">
-        <v>3.203</v>
+        <v>1.939</v>
       </c>
       <c r="D126" t="s">
         <v>128</v>
@@ -2663,13 +2663,13 @@
     </row>
     <row r="127" spans="1:4">
       <c r="A127" s="2">
-        <v>46127</v>
+        <v>46138</v>
       </c>
       <c r="B127">
         <v>15</v>
       </c>
       <c r="C127">
-        <v>2.992</v>
+        <v>1.977</v>
       </c>
       <c r="D127" t="s">
         <v>129</v>
@@ -2677,13 +2677,13 @@
     </row>
     <row r="128" spans="1:4">
       <c r="A128" s="2">
-        <v>46127</v>
+        <v>46138</v>
       </c>
       <c r="B128">
         <v>16</v>
       </c>
       <c r="C128">
-        <v>2.588</v>
+        <v>1.942</v>
       </c>
       <c r="D128" t="s">
         <v>130</v>
@@ -2691,13 +2691,13 @@
     </row>
     <row r="129" spans="1:4">
       <c r="A129" s="2">
-        <v>46127</v>
+        <v>46138</v>
       </c>
       <c r="B129">
         <v>17</v>
       </c>
       <c r="C129">
-        <v>2.107</v>
+        <v>1.588</v>
       </c>
       <c r="D129" t="s">
         <v>131</v>
@@ -2705,13 +2705,13 @@
     </row>
     <row r="130" spans="1:4">
       <c r="A130" s="2">
-        <v>46127</v>
+        <v>46138</v>
       </c>
       <c r="B130">
         <v>18</v>
       </c>
       <c r="C130">
-        <v>1.27</v>
+        <v>1.197</v>
       </c>
       <c r="D130" t="s">
         <v>132</v>
@@ -2719,13 +2719,13 @@
     </row>
     <row r="131" spans="1:4">
       <c r="A131" s="2">
-        <v>46127</v>
+        <v>46138</v>
       </c>
       <c r="B131">
         <v>19</v>
       </c>
       <c r="C131">
-        <v>0.496</v>
+        <v>0.465</v>
       </c>
       <c r="D131" t="s">
         <v>133</v>
@@ -2733,13 +2733,13 @@
     </row>
     <row r="132" spans="1:4">
       <c r="A132" s="2">
-        <v>46127</v>
+        <v>46138</v>
       </c>
       <c r="B132">
         <v>20</v>
       </c>
       <c r="C132">
-        <v>0.077</v>
+        <v>0.106</v>
       </c>
       <c r="D132" t="s">
         <v>134</v>
@@ -2747,7 +2747,7 @@
     </row>
     <row r="133" spans="1:4">
       <c r="A133" s="2">
-        <v>46127</v>
+        <v>46138</v>
       </c>
       <c r="B133">
         <v>21</v>
@@ -2761,7 +2761,7 @@
     </row>
     <row r="134" spans="1:4">
       <c r="A134" s="2">
-        <v>46127</v>
+        <v>46138</v>
       </c>
       <c r="B134">
         <v>22</v>
@@ -2775,7 +2775,7 @@
     </row>
     <row r="135" spans="1:4">
       <c r="A135" s="2">
-        <v>46127</v>
+        <v>46138</v>
       </c>
       <c r="B135">
         <v>23</v>
@@ -2789,7 +2789,7 @@
     </row>
     <row r="136" spans="1:4">
       <c r="A136" s="2">
-        <v>46127</v>
+        <v>46138</v>
       </c>
       <c r="B136">
         <v>24</v>
@@ -2803,7 +2803,7 @@
     </row>
     <row r="137" spans="1:4">
       <c r="A137" s="2">
-        <v>46128</v>
+        <v>46139</v>
       </c>
       <c r="B137">
         <v>1</v>
@@ -2817,7 +2817,7 @@
     </row>
     <row r="138" spans="1:4">
       <c r="A138" s="2">
-        <v>46128</v>
+        <v>46139</v>
       </c>
       <c r="B138">
         <v>2</v>
@@ -2831,7 +2831,7 @@
     </row>
     <row r="139" spans="1:4">
       <c r="A139" s="2">
-        <v>46128</v>
+        <v>46139</v>
       </c>
       <c r="B139">
         <v>3</v>
@@ -2845,7 +2845,7 @@
     </row>
     <row r="140" spans="1:4">
       <c r="A140" s="2">
-        <v>46128</v>
+        <v>46139</v>
       </c>
       <c r="B140">
         <v>4</v>
@@ -2859,7 +2859,7 @@
     </row>
     <row r="141" spans="1:4">
       <c r="A141" s="2">
-        <v>46128</v>
+        <v>46139</v>
       </c>
       <c r="B141">
         <v>5</v>
@@ -2873,7 +2873,7 @@
     </row>
     <row r="142" spans="1:4">
       <c r="A142" s="2">
-        <v>46128</v>
+        <v>46139</v>
       </c>
       <c r="B142">
         <v>6</v>
@@ -2887,13 +2887,13 @@
     </row>
     <row r="143" spans="1:4">
       <c r="A143" s="2">
-        <v>46128</v>
+        <v>46139</v>
       </c>
       <c r="B143">
         <v>7</v>
       </c>
       <c r="C143">
-        <v>0</v>
+        <v>0.03</v>
       </c>
       <c r="D143" t="s">
         <v>145</v>
@@ -2901,13 +2901,13 @@
     </row>
     <row r="144" spans="1:4">
       <c r="A144" s="2">
-        <v>46128</v>
+        <v>46139</v>
       </c>
       <c r="B144">
         <v>8</v>
       </c>
       <c r="C144">
-        <v>0.229</v>
+        <v>0.455</v>
       </c>
       <c r="D144" t="s">
         <v>146</v>
@@ -2915,13 +2915,13 @@
     </row>
     <row r="145" spans="1:4">
       <c r="A145" s="2">
-        <v>46128</v>
+        <v>46139</v>
       </c>
       <c r="B145">
         <v>9</v>
       </c>
       <c r="C145">
-        <v>0.929</v>
+        <v>1.222</v>
       </c>
       <c r="D145" t="s">
         <v>147</v>
@@ -2929,13 +2929,13 @@
     </row>
     <row r="146" spans="1:4">
       <c r="A146" s="2">
-        <v>46128</v>
+        <v>46139</v>
       </c>
       <c r="B146">
         <v>10</v>
       </c>
       <c r="C146">
-        <v>1.936</v>
+        <v>2.16</v>
       </c>
       <c r="D146" t="s">
         <v>148</v>
@@ -2943,13 +2943,13 @@
     </row>
     <row r="147" spans="1:4">
       <c r="A147" s="2">
-        <v>46128</v>
+        <v>46139</v>
       </c>
       <c r="B147">
         <v>11</v>
       </c>
       <c r="C147">
-        <v>2.48</v>
+        <v>2.899</v>
       </c>
       <c r="D147" t="s">
         <v>149</v>
@@ -2957,13 +2957,13 @@
     </row>
     <row r="148" spans="1:4">
       <c r="A148" s="2">
-        <v>46128</v>
+        <v>46139</v>
       </c>
       <c r="B148">
         <v>12</v>
       </c>
       <c r="C148">
-        <v>2.848</v>
+        <v>3.232</v>
       </c>
       <c r="D148" t="s">
         <v>150</v>
@@ -2971,13 +2971,13 @@
     </row>
     <row r="149" spans="1:4">
       <c r="A149" s="2">
-        <v>46128</v>
+        <v>46139</v>
       </c>
       <c r="B149">
         <v>13</v>
       </c>
       <c r="C149">
-        <v>2.995</v>
+        <v>3.232</v>
       </c>
       <c r="D149" t="s">
         <v>151</v>
@@ -2985,13 +2985,13 @@
     </row>
     <row r="150" spans="1:4">
       <c r="A150" s="2">
-        <v>46128</v>
+        <v>46139</v>
       </c>
       <c r="B150">
         <v>14</v>
       </c>
       <c r="C150">
-        <v>2.965</v>
+        <v>3.158</v>
       </c>
       <c r="D150" t="s">
         <v>152</v>
@@ -2999,13 +2999,13 @@
     </row>
     <row r="151" spans="1:4">
       <c r="A151" s="2">
-        <v>46128</v>
+        <v>46139</v>
       </c>
       <c r="B151">
         <v>15</v>
       </c>
       <c r="C151">
-        <v>2.645</v>
+        <v>3.133</v>
       </c>
       <c r="D151" t="s">
         <v>153</v>
@@ -3013,13 +3013,13 @@
     </row>
     <row r="152" spans="1:4">
       <c r="A152" s="2">
-        <v>46128</v>
+        <v>46139</v>
       </c>
       <c r="B152">
         <v>16</v>
       </c>
       <c r="C152">
-        <v>2.361</v>
+        <v>2.778</v>
       </c>
       <c r="D152" t="s">
         <v>154</v>
@@ -3027,13 +3027,13 @@
     </row>
     <row r="153" spans="1:4">
       <c r="A153" s="2">
-        <v>46128</v>
+        <v>46139</v>
       </c>
       <c r="B153">
         <v>17</v>
       </c>
       <c r="C153">
-        <v>1.913</v>
+        <v>2.192</v>
       </c>
       <c r="D153" t="s">
         <v>155</v>
@@ -3041,13 +3041,13 @@
     </row>
     <row r="154" spans="1:4">
       <c r="A154" s="2">
-        <v>46128</v>
+        <v>46139</v>
       </c>
       <c r="B154">
         <v>18</v>
       </c>
       <c r="C154">
-        <v>1.226</v>
+        <v>1.444</v>
       </c>
       <c r="D154" t="s">
         <v>156</v>
@@ -3055,13 +3055,13 @@
     </row>
     <row r="155" spans="1:4">
       <c r="A155" s="2">
-        <v>46128</v>
+        <v>46139</v>
       </c>
       <c r="B155">
         <v>19</v>
       </c>
       <c r="C155">
-        <v>0.499</v>
+        <v>0.621</v>
       </c>
       <c r="D155" t="s">
         <v>157</v>
@@ -3069,13 +3069,13 @@
     </row>
     <row r="156" spans="1:4">
       <c r="A156" s="2">
-        <v>46128</v>
+        <v>46139</v>
       </c>
       <c r="B156">
         <v>20</v>
       </c>
       <c r="C156">
-        <v>0.09</v>
+        <v>0.136</v>
       </c>
       <c r="D156" t="s">
         <v>158</v>
@@ -3083,7 +3083,7 @@
     </row>
     <row r="157" spans="1:4">
       <c r="A157" s="2">
-        <v>46128</v>
+        <v>46139</v>
       </c>
       <c r="B157">
         <v>21</v>
@@ -3097,7 +3097,7 @@
     </row>
     <row r="158" spans="1:4">
       <c r="A158" s="2">
-        <v>46128</v>
+        <v>46139</v>
       </c>
       <c r="B158">
         <v>22</v>
@@ -3111,7 +3111,7 @@
     </row>
     <row r="159" spans="1:4">
       <c r="A159" s="2">
-        <v>46128</v>
+        <v>46139</v>
       </c>
       <c r="B159">
         <v>23</v>
@@ -3125,7 +3125,7 @@
     </row>
     <row r="160" spans="1:4">
       <c r="A160" s="2">
-        <v>46128</v>
+        <v>46139</v>
       </c>
       <c r="B160">
         <v>24</v>
@@ -3139,7 +3139,7 @@
     </row>
     <row r="161" spans="1:4">
       <c r="A161" s="2">
-        <v>46129</v>
+        <v>46140</v>
       </c>
       <c r="B161">
         <v>1</v>
@@ -3153,7 +3153,7 @@
     </row>
     <row r="162" spans="1:4">
       <c r="A162" s="2">
-        <v>46129</v>
+        <v>46140</v>
       </c>
       <c r="B162">
         <v>2</v>
@@ -3167,7 +3167,7 @@
     </row>
     <row r="163" spans="1:4">
       <c r="A163" s="2">
-        <v>46129</v>
+        <v>46140</v>
       </c>
       <c r="B163">
         <v>3</v>
@@ -3181,7 +3181,7 @@
     </row>
     <row r="164" spans="1:4">
       <c r="A164" s="2">
-        <v>46129</v>
+        <v>46140</v>
       </c>
       <c r="B164">
         <v>4</v>
@@ -3195,7 +3195,7 @@
     </row>
     <row r="165" spans="1:4">
       <c r="A165" s="2">
-        <v>46129</v>
+        <v>46140</v>
       </c>
       <c r="B165">
         <v>5</v>
@@ -3209,7 +3209,7 @@
     </row>
     <row r="166" spans="1:4">
       <c r="A166" s="2">
-        <v>46129</v>
+        <v>46140</v>
       </c>
       <c r="B166">
         <v>6</v>
@@ -3223,13 +3223,13 @@
     </row>
     <row r="167" spans="1:4">
       <c r="A167" s="2">
-        <v>46129</v>
+        <v>46140</v>
       </c>
       <c r="B167">
         <v>7</v>
       </c>
       <c r="C167">
-        <v>0</v>
+        <v>0.028</v>
       </c>
       <c r="D167" t="s">
         <v>169</v>
@@ -3237,13 +3237,13 @@
     </row>
     <row r="168" spans="1:4">
       <c r="A168" s="2">
-        <v>46129</v>
+        <v>46140</v>
       </c>
       <c r="B168">
         <v>8</v>
       </c>
       <c r="C168">
-        <v>0.216</v>
+        <v>0.42</v>
       </c>
       <c r="D168" t="s">
         <v>170</v>
@@ -3251,13 +3251,13 @@
     </row>
     <row r="169" spans="1:4">
       <c r="A169" s="2">
-        <v>46129</v>
+        <v>46140</v>
       </c>
       <c r="B169">
         <v>9</v>
       </c>
       <c r="C169">
-        <v>0.739</v>
+        <v>1.064</v>
       </c>
       <c r="D169" t="s">
         <v>171</v>
@@ -3265,13 +3265,13 @@
     </row>
     <row r="170" spans="1:4">
       <c r="A170" s="2">
-        <v>46129</v>
+        <v>46140</v>
       </c>
       <c r="B170">
         <v>10</v>
       </c>
       <c r="C170">
-        <v>1.201</v>
+        <v>2.105</v>
       </c>
       <c r="D170" t="s">
         <v>172</v>

</xml_diff>

<commit_message>
Adding Ferma Frumusica to the portfolio
</commit_message>
<xml_diff>
--- a/Astro/Results_Production_Astro_xgb.xlsx
+++ b/Astro/Results_Production_Astro_xgb.xlsx
@@ -28,511 +28,511 @@
     <t>Lookup</t>
   </si>
   <si>
-    <t>21.04.202610</t>
-  </si>
-  <si>
-    <t>21.04.202611</t>
-  </si>
-  <si>
-    <t>21.04.202612</t>
-  </si>
-  <si>
-    <t>21.04.202613</t>
-  </si>
-  <si>
-    <t>21.04.202614</t>
-  </si>
-  <si>
-    <t>21.04.202615</t>
-  </si>
-  <si>
-    <t>21.04.202616</t>
-  </si>
-  <si>
-    <t>21.04.202617</t>
-  </si>
-  <si>
-    <t>21.04.202618</t>
-  </si>
-  <si>
-    <t>21.04.202619</t>
-  </si>
-  <si>
-    <t>21.04.202620</t>
-  </si>
-  <si>
-    <t>21.04.202621</t>
-  </si>
-  <si>
-    <t>21.04.202622</t>
-  </si>
-  <si>
-    <t>21.04.202623</t>
-  </si>
-  <si>
-    <t>21.04.202624</t>
-  </si>
-  <si>
-    <t>22.04.20261</t>
-  </si>
-  <si>
-    <t>22.04.20262</t>
-  </si>
-  <si>
-    <t>22.04.20263</t>
-  </si>
-  <si>
-    <t>22.04.20264</t>
-  </si>
-  <si>
-    <t>22.04.20265</t>
-  </si>
-  <si>
-    <t>22.04.20266</t>
-  </si>
-  <si>
-    <t>22.04.20267</t>
-  </si>
-  <si>
-    <t>22.04.20268</t>
-  </si>
-  <si>
-    <t>22.04.20269</t>
-  </si>
-  <si>
-    <t>22.04.202610</t>
-  </si>
-  <si>
-    <t>22.04.202611</t>
-  </si>
-  <si>
-    <t>22.04.202612</t>
-  </si>
-  <si>
-    <t>22.04.202613</t>
-  </si>
-  <si>
-    <t>22.04.202614</t>
-  </si>
-  <si>
-    <t>22.04.202615</t>
-  </si>
-  <si>
-    <t>22.04.202616</t>
-  </si>
-  <si>
-    <t>22.04.202617</t>
-  </si>
-  <si>
-    <t>22.04.202618</t>
-  </si>
-  <si>
-    <t>22.04.202619</t>
-  </si>
-  <si>
-    <t>22.04.202620</t>
-  </si>
-  <si>
-    <t>22.04.202621</t>
-  </si>
-  <si>
-    <t>22.04.202622</t>
-  </si>
-  <si>
-    <t>22.04.202623</t>
-  </si>
-  <si>
-    <t>22.04.202624</t>
-  </si>
-  <si>
-    <t>23.04.20261</t>
-  </si>
-  <si>
-    <t>23.04.20262</t>
-  </si>
-  <si>
-    <t>23.04.20263</t>
-  </si>
-  <si>
-    <t>23.04.20264</t>
-  </si>
-  <si>
-    <t>23.04.20265</t>
-  </si>
-  <si>
-    <t>23.04.20266</t>
-  </si>
-  <si>
-    <t>23.04.20267</t>
-  </si>
-  <si>
-    <t>23.04.20268</t>
-  </si>
-  <si>
-    <t>23.04.20269</t>
-  </si>
-  <si>
-    <t>23.04.202610</t>
-  </si>
-  <si>
-    <t>23.04.202611</t>
-  </si>
-  <si>
-    <t>23.04.202612</t>
-  </si>
-  <si>
-    <t>23.04.202613</t>
-  </si>
-  <si>
-    <t>23.04.202614</t>
-  </si>
-  <si>
-    <t>23.04.202615</t>
-  </si>
-  <si>
-    <t>23.04.202616</t>
-  </si>
-  <si>
-    <t>23.04.202617</t>
-  </si>
-  <si>
-    <t>23.04.202618</t>
-  </si>
-  <si>
-    <t>23.04.202619</t>
-  </si>
-  <si>
-    <t>23.04.202620</t>
-  </si>
-  <si>
-    <t>23.04.202621</t>
-  </si>
-  <si>
-    <t>23.04.202622</t>
-  </si>
-  <si>
-    <t>23.04.202623</t>
-  </si>
-  <si>
-    <t>23.04.202624</t>
-  </si>
-  <si>
-    <t>24.04.20261</t>
-  </si>
-  <si>
-    <t>24.04.20262</t>
-  </si>
-  <si>
-    <t>24.04.20263</t>
-  </si>
-  <si>
-    <t>24.04.20264</t>
-  </si>
-  <si>
-    <t>24.04.20265</t>
-  </si>
-  <si>
-    <t>24.04.20266</t>
-  </si>
-  <si>
-    <t>24.04.20267</t>
-  </si>
-  <si>
-    <t>24.04.20268</t>
-  </si>
-  <si>
-    <t>24.04.20269</t>
-  </si>
-  <si>
-    <t>24.04.202610</t>
-  </si>
-  <si>
-    <t>24.04.202611</t>
-  </si>
-  <si>
-    <t>24.04.202612</t>
-  </si>
-  <si>
-    <t>24.04.202613</t>
-  </si>
-  <si>
-    <t>24.04.202614</t>
-  </si>
-  <si>
-    <t>24.04.202615</t>
-  </si>
-  <si>
-    <t>24.04.202616</t>
-  </si>
-  <si>
-    <t>24.04.202617</t>
-  </si>
-  <si>
-    <t>24.04.202618</t>
-  </si>
-  <si>
-    <t>24.04.202619</t>
-  </si>
-  <si>
-    <t>24.04.202620</t>
-  </si>
-  <si>
-    <t>24.04.202621</t>
-  </si>
-  <si>
-    <t>24.04.202622</t>
-  </si>
-  <si>
-    <t>24.04.202623</t>
-  </si>
-  <si>
-    <t>24.04.202624</t>
-  </si>
-  <si>
-    <t>25.04.20261</t>
-  </si>
-  <si>
-    <t>25.04.20262</t>
-  </si>
-  <si>
-    <t>25.04.20263</t>
-  </si>
-  <si>
-    <t>25.04.20264</t>
-  </si>
-  <si>
-    <t>25.04.20265</t>
-  </si>
-  <si>
-    <t>25.04.20266</t>
-  </si>
-  <si>
-    <t>25.04.20267</t>
-  </si>
-  <si>
-    <t>25.04.20268</t>
-  </si>
-  <si>
-    <t>25.04.20269</t>
-  </si>
-  <si>
-    <t>25.04.202610</t>
-  </si>
-  <si>
-    <t>25.04.202611</t>
-  </si>
-  <si>
-    <t>25.04.202612</t>
-  </si>
-  <si>
-    <t>25.04.202613</t>
-  </si>
-  <si>
-    <t>25.04.202614</t>
-  </si>
-  <si>
-    <t>25.04.202615</t>
-  </si>
-  <si>
-    <t>25.04.202616</t>
-  </si>
-  <si>
-    <t>25.04.202617</t>
-  </si>
-  <si>
-    <t>25.04.202618</t>
-  </si>
-  <si>
-    <t>25.04.202619</t>
-  </si>
-  <si>
-    <t>25.04.202620</t>
-  </si>
-  <si>
-    <t>25.04.202621</t>
-  </si>
-  <si>
-    <t>25.04.202622</t>
-  </si>
-  <si>
-    <t>25.04.202623</t>
-  </si>
-  <si>
-    <t>25.04.202624</t>
-  </si>
-  <si>
-    <t>26.04.20261</t>
-  </si>
-  <si>
-    <t>26.04.20262</t>
-  </si>
-  <si>
-    <t>26.04.20263</t>
-  </si>
-  <si>
-    <t>26.04.20264</t>
-  </si>
-  <si>
-    <t>26.04.20265</t>
-  </si>
-  <si>
-    <t>26.04.20266</t>
-  </si>
-  <si>
-    <t>26.04.20267</t>
-  </si>
-  <si>
-    <t>26.04.20268</t>
-  </si>
-  <si>
-    <t>26.04.20269</t>
-  </si>
-  <si>
-    <t>26.04.202610</t>
-  </si>
-  <si>
-    <t>26.04.202611</t>
-  </si>
-  <si>
-    <t>26.04.202612</t>
-  </si>
-  <si>
-    <t>26.04.202613</t>
-  </si>
-  <si>
-    <t>26.04.202614</t>
-  </si>
-  <si>
-    <t>26.04.202615</t>
-  </si>
-  <si>
-    <t>26.04.202616</t>
-  </si>
-  <si>
-    <t>26.04.202617</t>
-  </si>
-  <si>
-    <t>26.04.202618</t>
-  </si>
-  <si>
-    <t>26.04.202619</t>
-  </si>
-  <si>
-    <t>26.04.202620</t>
-  </si>
-  <si>
-    <t>26.04.202621</t>
-  </si>
-  <si>
-    <t>26.04.202622</t>
-  </si>
-  <si>
-    <t>26.04.202623</t>
-  </si>
-  <si>
-    <t>26.04.202624</t>
-  </si>
-  <si>
-    <t>27.04.20261</t>
-  </si>
-  <si>
-    <t>27.04.20262</t>
-  </si>
-  <si>
-    <t>27.04.20263</t>
-  </si>
-  <si>
-    <t>27.04.20264</t>
-  </si>
-  <si>
-    <t>27.04.20265</t>
-  </si>
-  <si>
-    <t>27.04.20266</t>
-  </si>
-  <si>
-    <t>27.04.20267</t>
-  </si>
-  <si>
-    <t>27.04.20268</t>
-  </si>
-  <si>
-    <t>27.04.20269</t>
-  </si>
-  <si>
-    <t>27.04.202610</t>
-  </si>
-  <si>
-    <t>27.04.202611</t>
-  </si>
-  <si>
-    <t>27.04.202612</t>
-  </si>
-  <si>
-    <t>27.04.202613</t>
-  </si>
-  <si>
-    <t>27.04.202614</t>
-  </si>
-  <si>
-    <t>27.04.202615</t>
-  </si>
-  <si>
-    <t>27.04.202616</t>
-  </si>
-  <si>
-    <t>27.04.202617</t>
-  </si>
-  <si>
-    <t>27.04.202618</t>
-  </si>
-  <si>
-    <t>27.04.202619</t>
-  </si>
-  <si>
-    <t>27.04.202620</t>
-  </si>
-  <si>
-    <t>27.04.202621</t>
-  </si>
-  <si>
-    <t>27.04.202622</t>
-  </si>
-  <si>
-    <t>27.04.202623</t>
-  </si>
-  <si>
-    <t>27.04.202624</t>
-  </si>
-  <si>
-    <t>28.04.20261</t>
-  </si>
-  <si>
-    <t>28.04.20262</t>
-  </si>
-  <si>
-    <t>28.04.20263</t>
-  </si>
-  <si>
-    <t>28.04.20264</t>
-  </si>
-  <si>
-    <t>28.04.20265</t>
-  </si>
-  <si>
-    <t>28.04.20266</t>
-  </si>
-  <si>
-    <t>28.04.20267</t>
-  </si>
-  <si>
-    <t>28.04.20268</t>
-  </si>
-  <si>
-    <t>28.04.20269</t>
-  </si>
-  <si>
-    <t>28.04.202610</t>
+    <t>31.05.202610</t>
+  </si>
+  <si>
+    <t>31.05.202611</t>
+  </si>
+  <si>
+    <t>31.05.202612</t>
+  </si>
+  <si>
+    <t>31.05.202613</t>
+  </si>
+  <si>
+    <t>31.05.202614</t>
+  </si>
+  <si>
+    <t>31.05.202615</t>
+  </si>
+  <si>
+    <t>31.05.202616</t>
+  </si>
+  <si>
+    <t>31.05.202617</t>
+  </si>
+  <si>
+    <t>31.05.202618</t>
+  </si>
+  <si>
+    <t>31.05.202619</t>
+  </si>
+  <si>
+    <t>31.05.202620</t>
+  </si>
+  <si>
+    <t>31.05.202621</t>
+  </si>
+  <si>
+    <t>31.05.202622</t>
+  </si>
+  <si>
+    <t>31.05.202623</t>
+  </si>
+  <si>
+    <t>31.05.202624</t>
+  </si>
+  <si>
+    <t>01.06.20261</t>
+  </si>
+  <si>
+    <t>01.06.20262</t>
+  </si>
+  <si>
+    <t>01.06.20263</t>
+  </si>
+  <si>
+    <t>01.06.20264</t>
+  </si>
+  <si>
+    <t>01.06.20265</t>
+  </si>
+  <si>
+    <t>01.06.20266</t>
+  </si>
+  <si>
+    <t>01.06.20267</t>
+  </si>
+  <si>
+    <t>01.06.20268</t>
+  </si>
+  <si>
+    <t>01.06.20269</t>
+  </si>
+  <si>
+    <t>01.06.202610</t>
+  </si>
+  <si>
+    <t>01.06.202611</t>
+  </si>
+  <si>
+    <t>01.06.202612</t>
+  </si>
+  <si>
+    <t>01.06.202613</t>
+  </si>
+  <si>
+    <t>01.06.202614</t>
+  </si>
+  <si>
+    <t>01.06.202615</t>
+  </si>
+  <si>
+    <t>01.06.202616</t>
+  </si>
+  <si>
+    <t>01.06.202617</t>
+  </si>
+  <si>
+    <t>01.06.202618</t>
+  </si>
+  <si>
+    <t>01.06.202619</t>
+  </si>
+  <si>
+    <t>01.06.202620</t>
+  </si>
+  <si>
+    <t>01.06.202621</t>
+  </si>
+  <si>
+    <t>01.06.202622</t>
+  </si>
+  <si>
+    <t>01.06.202623</t>
+  </si>
+  <si>
+    <t>01.06.202624</t>
+  </si>
+  <si>
+    <t>02.06.20261</t>
+  </si>
+  <si>
+    <t>02.06.20262</t>
+  </si>
+  <si>
+    <t>02.06.20263</t>
+  </si>
+  <si>
+    <t>02.06.20264</t>
+  </si>
+  <si>
+    <t>02.06.20265</t>
+  </si>
+  <si>
+    <t>02.06.20266</t>
+  </si>
+  <si>
+    <t>02.06.20267</t>
+  </si>
+  <si>
+    <t>02.06.20268</t>
+  </si>
+  <si>
+    <t>02.06.20269</t>
+  </si>
+  <si>
+    <t>02.06.202610</t>
+  </si>
+  <si>
+    <t>02.06.202611</t>
+  </si>
+  <si>
+    <t>02.06.202612</t>
+  </si>
+  <si>
+    <t>02.06.202613</t>
+  </si>
+  <si>
+    <t>02.06.202614</t>
+  </si>
+  <si>
+    <t>02.06.202615</t>
+  </si>
+  <si>
+    <t>02.06.202616</t>
+  </si>
+  <si>
+    <t>02.06.202617</t>
+  </si>
+  <si>
+    <t>02.06.202618</t>
+  </si>
+  <si>
+    <t>02.06.202619</t>
+  </si>
+  <si>
+    <t>02.06.202620</t>
+  </si>
+  <si>
+    <t>02.06.202621</t>
+  </si>
+  <si>
+    <t>02.06.202622</t>
+  </si>
+  <si>
+    <t>02.06.202623</t>
+  </si>
+  <si>
+    <t>02.06.202624</t>
+  </si>
+  <si>
+    <t>03.06.20261</t>
+  </si>
+  <si>
+    <t>03.06.20262</t>
+  </si>
+  <si>
+    <t>03.06.20263</t>
+  </si>
+  <si>
+    <t>03.06.20264</t>
+  </si>
+  <si>
+    <t>03.06.20265</t>
+  </si>
+  <si>
+    <t>03.06.20266</t>
+  </si>
+  <si>
+    <t>03.06.20267</t>
+  </si>
+  <si>
+    <t>03.06.20268</t>
+  </si>
+  <si>
+    <t>03.06.20269</t>
+  </si>
+  <si>
+    <t>03.06.202610</t>
+  </si>
+  <si>
+    <t>03.06.202611</t>
+  </si>
+  <si>
+    <t>03.06.202612</t>
+  </si>
+  <si>
+    <t>03.06.202613</t>
+  </si>
+  <si>
+    <t>03.06.202614</t>
+  </si>
+  <si>
+    <t>03.06.202615</t>
+  </si>
+  <si>
+    <t>03.06.202616</t>
+  </si>
+  <si>
+    <t>03.06.202617</t>
+  </si>
+  <si>
+    <t>03.06.202618</t>
+  </si>
+  <si>
+    <t>03.06.202619</t>
+  </si>
+  <si>
+    <t>03.06.202620</t>
+  </si>
+  <si>
+    <t>03.06.202621</t>
+  </si>
+  <si>
+    <t>03.06.202622</t>
+  </si>
+  <si>
+    <t>03.06.202623</t>
+  </si>
+  <si>
+    <t>03.06.202624</t>
+  </si>
+  <si>
+    <t>04.06.20261</t>
+  </si>
+  <si>
+    <t>04.06.20262</t>
+  </si>
+  <si>
+    <t>04.06.20263</t>
+  </si>
+  <si>
+    <t>04.06.20264</t>
+  </si>
+  <si>
+    <t>04.06.20265</t>
+  </si>
+  <si>
+    <t>04.06.20266</t>
+  </si>
+  <si>
+    <t>04.06.20267</t>
+  </si>
+  <si>
+    <t>04.06.20268</t>
+  </si>
+  <si>
+    <t>04.06.20269</t>
+  </si>
+  <si>
+    <t>04.06.202610</t>
+  </si>
+  <si>
+    <t>04.06.202611</t>
+  </si>
+  <si>
+    <t>04.06.202612</t>
+  </si>
+  <si>
+    <t>04.06.202613</t>
+  </si>
+  <si>
+    <t>04.06.202614</t>
+  </si>
+  <si>
+    <t>04.06.202615</t>
+  </si>
+  <si>
+    <t>04.06.202616</t>
+  </si>
+  <si>
+    <t>04.06.202617</t>
+  </si>
+  <si>
+    <t>04.06.202618</t>
+  </si>
+  <si>
+    <t>04.06.202619</t>
+  </si>
+  <si>
+    <t>04.06.202620</t>
+  </si>
+  <si>
+    <t>04.06.202621</t>
+  </si>
+  <si>
+    <t>04.06.202622</t>
+  </si>
+  <si>
+    <t>04.06.202623</t>
+  </si>
+  <si>
+    <t>04.06.202624</t>
+  </si>
+  <si>
+    <t>05.06.20261</t>
+  </si>
+  <si>
+    <t>05.06.20262</t>
+  </si>
+  <si>
+    <t>05.06.20263</t>
+  </si>
+  <si>
+    <t>05.06.20264</t>
+  </si>
+  <si>
+    <t>05.06.20265</t>
+  </si>
+  <si>
+    <t>05.06.20266</t>
+  </si>
+  <si>
+    <t>05.06.20267</t>
+  </si>
+  <si>
+    <t>05.06.20268</t>
+  </si>
+  <si>
+    <t>05.06.20269</t>
+  </si>
+  <si>
+    <t>05.06.202610</t>
+  </si>
+  <si>
+    <t>05.06.202611</t>
+  </si>
+  <si>
+    <t>05.06.202612</t>
+  </si>
+  <si>
+    <t>05.06.202613</t>
+  </si>
+  <si>
+    <t>05.06.202614</t>
+  </si>
+  <si>
+    <t>05.06.202615</t>
+  </si>
+  <si>
+    <t>05.06.202616</t>
+  </si>
+  <si>
+    <t>05.06.202617</t>
+  </si>
+  <si>
+    <t>05.06.202618</t>
+  </si>
+  <si>
+    <t>05.06.202619</t>
+  </si>
+  <si>
+    <t>05.06.202620</t>
+  </si>
+  <si>
+    <t>05.06.202621</t>
+  </si>
+  <si>
+    <t>05.06.202622</t>
+  </si>
+  <si>
+    <t>05.06.202623</t>
+  </si>
+  <si>
+    <t>05.06.202624</t>
+  </si>
+  <si>
+    <t>06.06.20261</t>
+  </si>
+  <si>
+    <t>06.06.20262</t>
+  </si>
+  <si>
+    <t>06.06.20263</t>
+  </si>
+  <si>
+    <t>06.06.20264</t>
+  </si>
+  <si>
+    <t>06.06.20265</t>
+  </si>
+  <si>
+    <t>06.06.20266</t>
+  </si>
+  <si>
+    <t>06.06.20267</t>
+  </si>
+  <si>
+    <t>06.06.20268</t>
+  </si>
+  <si>
+    <t>06.06.20269</t>
+  </si>
+  <si>
+    <t>06.06.202610</t>
+  </si>
+  <si>
+    <t>06.06.202611</t>
+  </si>
+  <si>
+    <t>06.06.202612</t>
+  </si>
+  <si>
+    <t>06.06.202613</t>
+  </si>
+  <si>
+    <t>06.06.202614</t>
+  </si>
+  <si>
+    <t>06.06.202615</t>
+  </si>
+  <si>
+    <t>06.06.202616</t>
+  </si>
+  <si>
+    <t>06.06.202617</t>
+  </si>
+  <si>
+    <t>06.06.202618</t>
+  </si>
+  <si>
+    <t>06.06.202619</t>
+  </si>
+  <si>
+    <t>06.06.202620</t>
+  </si>
+  <si>
+    <t>06.06.202621</t>
+  </si>
+  <si>
+    <t>06.06.202622</t>
+  </si>
+  <si>
+    <t>06.06.202623</t>
+  </si>
+  <si>
+    <t>06.06.202624</t>
+  </si>
+  <si>
+    <t>07.06.20261</t>
+  </si>
+  <si>
+    <t>07.06.20262</t>
+  </si>
+  <si>
+    <t>07.06.20263</t>
+  </si>
+  <si>
+    <t>07.06.20264</t>
+  </si>
+  <si>
+    <t>07.06.20265</t>
+  </si>
+  <si>
+    <t>07.06.20266</t>
+  </si>
+  <si>
+    <t>07.06.20267</t>
+  </si>
+  <si>
+    <t>07.06.20268</t>
+  </si>
+  <si>
+    <t>07.06.20269</t>
+  </si>
+  <si>
+    <t>07.06.202610</t>
   </si>
 </sst>
 </file>
@@ -913,7 +913,7 @@
     </row>
     <row r="2" spans="1:4">
       <c r="A2" s="2">
-        <v>46133</v>
+        <v>46173</v>
       </c>
       <c r="B2">
         <v>10</v>
@@ -927,7 +927,7 @@
     </row>
     <row r="3" spans="1:4">
       <c r="A3" s="2">
-        <v>46133</v>
+        <v>46173</v>
       </c>
       <c r="B3">
         <v>11</v>
@@ -941,13 +941,13 @@
     </row>
     <row r="4" spans="1:4">
       <c r="A4" s="2">
-        <v>46133</v>
+        <v>46173</v>
       </c>
       <c r="B4">
         <v>12</v>
       </c>
       <c r="C4">
-        <v>2.224</v>
+        <v>2.055</v>
       </c>
       <c r="D4" t="s">
         <v>6</v>
@@ -955,13 +955,13 @@
     </row>
     <row r="5" spans="1:4">
       <c r="A5" s="2">
-        <v>46133</v>
+        <v>46173</v>
       </c>
       <c r="B5">
         <v>13</v>
       </c>
       <c r="C5">
-        <v>1.968</v>
+        <v>2.39</v>
       </c>
       <c r="D5" t="s">
         <v>7</v>
@@ -969,13 +969,13 @@
     </row>
     <row r="6" spans="1:4">
       <c r="A6" s="2">
-        <v>46133</v>
+        <v>46173</v>
       </c>
       <c r="B6">
         <v>14</v>
       </c>
       <c r="C6">
-        <v>2.07</v>
+        <v>2.833</v>
       </c>
       <c r="D6" t="s">
         <v>8</v>
@@ -983,13 +983,13 @@
     </row>
     <row r="7" spans="1:4">
       <c r="A7" s="2">
-        <v>46133</v>
+        <v>46173</v>
       </c>
       <c r="B7">
         <v>15</v>
       </c>
       <c r="C7">
-        <v>1.987</v>
+        <v>2.705</v>
       </c>
       <c r="D7" t="s">
         <v>9</v>
@@ -997,13 +997,13 @@
     </row>
     <row r="8" spans="1:4">
       <c r="A8" s="2">
-        <v>46133</v>
+        <v>46173</v>
       </c>
       <c r="B8">
         <v>16</v>
       </c>
       <c r="C8">
-        <v>1.894</v>
+        <v>2.305</v>
       </c>
       <c r="D8" t="s">
         <v>10</v>
@@ -1011,13 +1011,13 @@
     </row>
     <row r="9" spans="1:4">
       <c r="A9" s="2">
-        <v>46133</v>
+        <v>46173</v>
       </c>
       <c r="B9">
         <v>17</v>
       </c>
       <c r="C9">
-        <v>1.587</v>
+        <v>1.945</v>
       </c>
       <c r="D9" t="s">
         <v>11</v>
@@ -1025,13 +1025,13 @@
     </row>
     <row r="10" spans="1:4">
       <c r="A10" s="2">
-        <v>46133</v>
+        <v>46173</v>
       </c>
       <c r="B10">
         <v>18</v>
       </c>
       <c r="C10">
-        <v>0.88</v>
+        <v>1.419</v>
       </c>
       <c r="D10" t="s">
         <v>12</v>
@@ -1039,13 +1039,13 @@
     </row>
     <row r="11" spans="1:4">
       <c r="A11" s="2">
-        <v>46133</v>
+        <v>46173</v>
       </c>
       <c r="B11">
         <v>19</v>
       </c>
       <c r="C11">
-        <v>0.426</v>
+        <v>0.8159999999999999</v>
       </c>
       <c r="D11" t="s">
         <v>13</v>
@@ -1053,13 +1053,13 @@
     </row>
     <row r="12" spans="1:4">
       <c r="A12" s="2">
-        <v>46133</v>
+        <v>46173</v>
       </c>
       <c r="B12">
         <v>20</v>
       </c>
       <c r="C12">
-        <v>0.08400000000000001</v>
+        <v>0.282</v>
       </c>
       <c r="D12" t="s">
         <v>14</v>
@@ -1067,13 +1067,13 @@
     </row>
     <row r="13" spans="1:4">
       <c r="A13" s="2">
-        <v>46133</v>
+        <v>46173</v>
       </c>
       <c r="B13">
         <v>21</v>
       </c>
       <c r="C13">
-        <v>0</v>
+        <v>0.057</v>
       </c>
       <c r="D13" t="s">
         <v>15</v>
@@ -1081,7 +1081,7 @@
     </row>
     <row r="14" spans="1:4">
       <c r="A14" s="2">
-        <v>46133</v>
+        <v>46173</v>
       </c>
       <c r="B14">
         <v>22</v>
@@ -1095,7 +1095,7 @@
     </row>
     <row r="15" spans="1:4">
       <c r="A15" s="2">
-        <v>46133</v>
+        <v>46173</v>
       </c>
       <c r="B15">
         <v>23</v>
@@ -1109,7 +1109,7 @@
     </row>
     <row r="16" spans="1:4">
       <c r="A16" s="2">
-        <v>46133</v>
+        <v>46173</v>
       </c>
       <c r="B16">
         <v>24</v>
@@ -1123,7 +1123,7 @@
     </row>
     <row r="17" spans="1:4">
       <c r="A17" s="2">
-        <v>46134</v>
+        <v>46174</v>
       </c>
       <c r="B17">
         <v>1</v>
@@ -1137,7 +1137,7 @@
     </row>
     <row r="18" spans="1:4">
       <c r="A18" s="2">
-        <v>46134</v>
+        <v>46174</v>
       </c>
       <c r="B18">
         <v>2</v>
@@ -1151,7 +1151,7 @@
     </row>
     <row r="19" spans="1:4">
       <c r="A19" s="2">
-        <v>46134</v>
+        <v>46174</v>
       </c>
       <c r="B19">
         <v>3</v>
@@ -1165,7 +1165,7 @@
     </row>
     <row r="20" spans="1:4">
       <c r="A20" s="2">
-        <v>46134</v>
+        <v>46174</v>
       </c>
       <c r="B20">
         <v>4</v>
@@ -1179,7 +1179,7 @@
     </row>
     <row r="21" spans="1:4">
       <c r="A21" s="2">
-        <v>46134</v>
+        <v>46174</v>
       </c>
       <c r="B21">
         <v>5</v>
@@ -1193,7 +1193,7 @@
     </row>
     <row r="22" spans="1:4">
       <c r="A22" s="2">
-        <v>46134</v>
+        <v>46174</v>
       </c>
       <c r="B22">
         <v>6</v>
@@ -1207,13 +1207,13 @@
     </row>
     <row r="23" spans="1:4">
       <c r="A23" s="2">
-        <v>46134</v>
+        <v>46174</v>
       </c>
       <c r="B23">
         <v>7</v>
       </c>
       <c r="C23">
-        <v>0.013</v>
+        <v>0.068</v>
       </c>
       <c r="D23" t="s">
         <v>25</v>
@@ -1221,13 +1221,13 @@
     </row>
     <row r="24" spans="1:4">
       <c r="A24" s="2">
-        <v>46134</v>
+        <v>46174</v>
       </c>
       <c r="B24">
         <v>8</v>
       </c>
       <c r="C24">
-        <v>0.242</v>
+        <v>0.283</v>
       </c>
       <c r="D24" t="s">
         <v>26</v>
@@ -1235,13 +1235,13 @@
     </row>
     <row r="25" spans="1:4">
       <c r="A25" s="2">
-        <v>46134</v>
+        <v>46174</v>
       </c>
       <c r="B25">
         <v>9</v>
       </c>
       <c r="C25">
-        <v>0.772</v>
+        <v>0.642</v>
       </c>
       <c r="D25" t="s">
         <v>27</v>
@@ -1249,13 +1249,13 @@
     </row>
     <row r="26" spans="1:4">
       <c r="A26" s="2">
-        <v>46134</v>
+        <v>46174</v>
       </c>
       <c r="B26">
         <v>10</v>
       </c>
       <c r="C26">
-        <v>1.524</v>
+        <v>0.744</v>
       </c>
       <c r="D26" t="s">
         <v>28</v>
@@ -1263,13 +1263,13 @@
     </row>
     <row r="27" spans="1:4">
       <c r="A27" s="2">
-        <v>46134</v>
+        <v>46174</v>
       </c>
       <c r="B27">
         <v>11</v>
       </c>
       <c r="C27">
-        <v>2.111</v>
+        <v>0.853</v>
       </c>
       <c r="D27" t="s">
         <v>29</v>
@@ -1277,13 +1277,13 @@
     </row>
     <row r="28" spans="1:4">
       <c r="A28" s="2">
-        <v>46134</v>
+        <v>46174</v>
       </c>
       <c r="B28">
         <v>12</v>
       </c>
       <c r="C28">
-        <v>2.502</v>
+        <v>0.792</v>
       </c>
       <c r="D28" t="s">
         <v>30</v>
@@ -1291,13 +1291,13 @@
     </row>
     <row r="29" spans="1:4">
       <c r="A29" s="2">
-        <v>46134</v>
+        <v>46174</v>
       </c>
       <c r="B29">
         <v>13</v>
       </c>
       <c r="C29">
-        <v>2.611</v>
+        <v>0.742</v>
       </c>
       <c r="D29" t="s">
         <v>31</v>
@@ -1305,13 +1305,13 @@
     </row>
     <row r="30" spans="1:4">
       <c r="A30" s="2">
-        <v>46134</v>
+        <v>46174</v>
       </c>
       <c r="B30">
         <v>14</v>
       </c>
       <c r="C30">
-        <v>2.417</v>
+        <v>0.705</v>
       </c>
       <c r="D30" t="s">
         <v>32</v>
@@ -1319,13 +1319,13 @@
     </row>
     <row r="31" spans="1:4">
       <c r="A31" s="2">
-        <v>46134</v>
+        <v>46174</v>
       </c>
       <c r="B31">
         <v>15</v>
       </c>
       <c r="C31">
-        <v>2.118</v>
+        <v>0.673</v>
       </c>
       <c r="D31" t="s">
         <v>33</v>
@@ -1333,13 +1333,13 @@
     </row>
     <row r="32" spans="1:4">
       <c r="A32" s="2">
-        <v>46134</v>
+        <v>46174</v>
       </c>
       <c r="B32">
         <v>16</v>
       </c>
       <c r="C32">
-        <v>1.922</v>
+        <v>0.5600000000000001</v>
       </c>
       <c r="D32" t="s">
         <v>34</v>
@@ -1347,13 +1347,13 @@
     </row>
     <row r="33" spans="1:4">
       <c r="A33" s="2">
-        <v>46134</v>
+        <v>46174</v>
       </c>
       <c r="B33">
         <v>17</v>
       </c>
       <c r="C33">
-        <v>1.893</v>
+        <v>0.466</v>
       </c>
       <c r="D33" t="s">
         <v>35</v>
@@ -1361,13 +1361,13 @@
     </row>
     <row r="34" spans="1:4">
       <c r="A34" s="2">
-        <v>46134</v>
+        <v>46174</v>
       </c>
       <c r="B34">
         <v>18</v>
       </c>
       <c r="C34">
-        <v>1.341</v>
+        <v>0.348</v>
       </c>
       <c r="D34" t="s">
         <v>36</v>
@@ -1375,13 +1375,13 @@
     </row>
     <row r="35" spans="1:4">
       <c r="A35" s="2">
-        <v>46134</v>
+        <v>46174</v>
       </c>
       <c r="B35">
         <v>19</v>
       </c>
       <c r="C35">
-        <v>0.615</v>
+        <v>0.152</v>
       </c>
       <c r="D35" t="s">
         <v>37</v>
@@ -1389,13 +1389,13 @@
     </row>
     <row r="36" spans="1:4">
       <c r="A36" s="2">
-        <v>46134</v>
+        <v>46174</v>
       </c>
       <c r="B36">
         <v>20</v>
       </c>
       <c r="C36">
-        <v>0.122</v>
+        <v>0.063</v>
       </c>
       <c r="D36" t="s">
         <v>38</v>
@@ -1403,7 +1403,7 @@
     </row>
     <row r="37" spans="1:4">
       <c r="A37" s="2">
-        <v>46134</v>
+        <v>46174</v>
       </c>
       <c r="B37">
         <v>21</v>
@@ -1417,7 +1417,7 @@
     </row>
     <row r="38" spans="1:4">
       <c r="A38" s="2">
-        <v>46134</v>
+        <v>46174</v>
       </c>
       <c r="B38">
         <v>22</v>
@@ -1431,7 +1431,7 @@
     </row>
     <row r="39" spans="1:4">
       <c r="A39" s="2">
-        <v>46134</v>
+        <v>46174</v>
       </c>
       <c r="B39">
         <v>23</v>
@@ -1445,7 +1445,7 @@
     </row>
     <row r="40" spans="1:4">
       <c r="A40" s="2">
-        <v>46134</v>
+        <v>46174</v>
       </c>
       <c r="B40">
         <v>24</v>
@@ -1459,7 +1459,7 @@
     </row>
     <row r="41" spans="1:4">
       <c r="A41" s="2">
-        <v>46135</v>
+        <v>46175</v>
       </c>
       <c r="B41">
         <v>1</v>
@@ -1473,7 +1473,7 @@
     </row>
     <row r="42" spans="1:4">
       <c r="A42" s="2">
-        <v>46135</v>
+        <v>46175</v>
       </c>
       <c r="B42">
         <v>2</v>
@@ -1487,7 +1487,7 @@
     </row>
     <row r="43" spans="1:4">
       <c r="A43" s="2">
-        <v>46135</v>
+        <v>46175</v>
       </c>
       <c r="B43">
         <v>3</v>
@@ -1501,7 +1501,7 @@
     </row>
     <row r="44" spans="1:4">
       <c r="A44" s="2">
-        <v>46135</v>
+        <v>46175</v>
       </c>
       <c r="B44">
         <v>4</v>
@@ -1515,7 +1515,7 @@
     </row>
     <row r="45" spans="1:4">
       <c r="A45" s="2">
-        <v>46135</v>
+        <v>46175</v>
       </c>
       <c r="B45">
         <v>5</v>
@@ -1529,7 +1529,7 @@
     </row>
     <row r="46" spans="1:4">
       <c r="A46" s="2">
-        <v>46135</v>
+        <v>46175</v>
       </c>
       <c r="B46">
         <v>6</v>
@@ -1543,13 +1543,13 @@
     </row>
     <row r="47" spans="1:4">
       <c r="A47" s="2">
-        <v>46135</v>
+        <v>46175</v>
       </c>
       <c r="B47">
         <v>7</v>
       </c>
       <c r="C47">
-        <v>0.014</v>
+        <v>0.05</v>
       </c>
       <c r="D47" t="s">
         <v>49</v>
@@ -1557,13 +1557,13 @@
     </row>
     <row r="48" spans="1:4">
       <c r="A48" s="2">
-        <v>46135</v>
+        <v>46175</v>
       </c>
       <c r="B48">
         <v>8</v>
       </c>
       <c r="C48">
-        <v>0.321</v>
+        <v>0.19</v>
       </c>
       <c r="D48" t="s">
         <v>50</v>
@@ -1571,13 +1571,13 @@
     </row>
     <row r="49" spans="1:4">
       <c r="A49" s="2">
-        <v>46135</v>
+        <v>46175</v>
       </c>
       <c r="B49">
         <v>9</v>
       </c>
       <c r="C49">
-        <v>0.791</v>
+        <v>0.386</v>
       </c>
       <c r="D49" t="s">
         <v>51</v>
@@ -1585,13 +1585,13 @@
     </row>
     <row r="50" spans="1:4">
       <c r="A50" s="2">
-        <v>46135</v>
+        <v>46175</v>
       </c>
       <c r="B50">
         <v>10</v>
       </c>
       <c r="C50">
-        <v>1.197</v>
+        <v>0.732</v>
       </c>
       <c r="D50" t="s">
         <v>52</v>
@@ -1599,13 +1599,13 @@
     </row>
     <row r="51" spans="1:4">
       <c r="A51" s="2">
-        <v>46135</v>
+        <v>46175</v>
       </c>
       <c r="B51">
         <v>11</v>
       </c>
       <c r="C51">
-        <v>1.558</v>
+        <v>1.102</v>
       </c>
       <c r="D51" t="s">
         <v>53</v>
@@ -1613,13 +1613,13 @@
     </row>
     <row r="52" spans="1:4">
       <c r="A52" s="2">
-        <v>46135</v>
+        <v>46175</v>
       </c>
       <c r="B52">
         <v>12</v>
       </c>
       <c r="C52">
-        <v>1.894</v>
+        <v>1.205</v>
       </c>
       <c r="D52" t="s">
         <v>54</v>
@@ -1627,13 +1627,13 @@
     </row>
     <row r="53" spans="1:4">
       <c r="A53" s="2">
-        <v>46135</v>
+        <v>46175</v>
       </c>
       <c r="B53">
         <v>13</v>
       </c>
       <c r="C53">
-        <v>1.99</v>
+        <v>1.319</v>
       </c>
       <c r="D53" t="s">
         <v>55</v>
@@ -1641,13 +1641,13 @@
     </row>
     <row r="54" spans="1:4">
       <c r="A54" s="2">
-        <v>46135</v>
+        <v>46175</v>
       </c>
       <c r="B54">
         <v>14</v>
       </c>
       <c r="C54">
-        <v>2.029</v>
+        <v>1.291</v>
       </c>
       <c r="D54" t="s">
         <v>56</v>
@@ -1655,13 +1655,13 @@
     </row>
     <row r="55" spans="1:4">
       <c r="A55" s="2">
-        <v>46135</v>
+        <v>46175</v>
       </c>
       <c r="B55">
         <v>15</v>
       </c>
       <c r="C55">
-        <v>2</v>
+        <v>1.193</v>
       </c>
       <c r="D55" t="s">
         <v>57</v>
@@ -1669,13 +1669,13 @@
     </row>
     <row r="56" spans="1:4">
       <c r="A56" s="2">
-        <v>46135</v>
+        <v>46175</v>
       </c>
       <c r="B56">
         <v>16</v>
       </c>
       <c r="C56">
-        <v>1.859</v>
+        <v>0.913</v>
       </c>
       <c r="D56" t="s">
         <v>58</v>
@@ -1683,13 +1683,13 @@
     </row>
     <row r="57" spans="1:4">
       <c r="A57" s="2">
-        <v>46135</v>
+        <v>46175</v>
       </c>
       <c r="B57">
         <v>17</v>
       </c>
       <c r="C57">
-        <v>1.337</v>
+        <v>1.028</v>
       </c>
       <c r="D57" t="s">
         <v>59</v>
@@ -1697,13 +1697,13 @@
     </row>
     <row r="58" spans="1:4">
       <c r="A58" s="2">
-        <v>46135</v>
+        <v>46175</v>
       </c>
       <c r="B58">
         <v>18</v>
       </c>
       <c r="C58">
-        <v>0.766</v>
+        <v>0.8110000000000001</v>
       </c>
       <c r="D58" t="s">
         <v>60</v>
@@ -1711,13 +1711,13 @@
     </row>
     <row r="59" spans="1:4">
       <c r="A59" s="2">
-        <v>46135</v>
+        <v>46175</v>
       </c>
       <c r="B59">
         <v>19</v>
       </c>
       <c r="C59">
-        <v>0.387</v>
+        <v>0.421</v>
       </c>
       <c r="D59" t="s">
         <v>61</v>
@@ -1725,13 +1725,13 @@
     </row>
     <row r="60" spans="1:4">
       <c r="A60" s="2">
-        <v>46135</v>
+        <v>46175</v>
       </c>
       <c r="B60">
         <v>20</v>
       </c>
       <c r="C60">
-        <v>0.067</v>
+        <v>0.224</v>
       </c>
       <c r="D60" t="s">
         <v>62</v>
@@ -1739,13 +1739,13 @@
     </row>
     <row r="61" spans="1:4">
       <c r="A61" s="2">
-        <v>46135</v>
+        <v>46175</v>
       </c>
       <c r="B61">
         <v>21</v>
       </c>
       <c r="C61">
-        <v>0</v>
+        <v>0.043</v>
       </c>
       <c r="D61" t="s">
         <v>63</v>
@@ -1753,7 +1753,7 @@
     </row>
     <row r="62" spans="1:4">
       <c r="A62" s="2">
-        <v>46135</v>
+        <v>46175</v>
       </c>
       <c r="B62">
         <v>22</v>
@@ -1767,7 +1767,7 @@
     </row>
     <row r="63" spans="1:4">
       <c r="A63" s="2">
-        <v>46135</v>
+        <v>46175</v>
       </c>
       <c r="B63">
         <v>23</v>
@@ -1781,7 +1781,7 @@
     </row>
     <row r="64" spans="1:4">
       <c r="A64" s="2">
-        <v>46135</v>
+        <v>46175</v>
       </c>
       <c r="B64">
         <v>24</v>
@@ -1795,7 +1795,7 @@
     </row>
     <row r="65" spans="1:4">
       <c r="A65" s="2">
-        <v>46136</v>
+        <v>46176</v>
       </c>
       <c r="B65">
         <v>1</v>
@@ -1809,7 +1809,7 @@
     </row>
     <row r="66" spans="1:4">
       <c r="A66" s="2">
-        <v>46136</v>
+        <v>46176</v>
       </c>
       <c r="B66">
         <v>2</v>
@@ -1823,7 +1823,7 @@
     </row>
     <row r="67" spans="1:4">
       <c r="A67" s="2">
-        <v>46136</v>
+        <v>46176</v>
       </c>
       <c r="B67">
         <v>3</v>
@@ -1837,7 +1837,7 @@
     </row>
     <row r="68" spans="1:4">
       <c r="A68" s="2">
-        <v>46136</v>
+        <v>46176</v>
       </c>
       <c r="B68">
         <v>4</v>
@@ -1851,7 +1851,7 @@
     </row>
     <row r="69" spans="1:4">
       <c r="A69" s="2">
-        <v>46136</v>
+        <v>46176</v>
       </c>
       <c r="B69">
         <v>5</v>
@@ -1865,7 +1865,7 @@
     </row>
     <row r="70" spans="1:4">
       <c r="A70" s="2">
-        <v>46136</v>
+        <v>46176</v>
       </c>
       <c r="B70">
         <v>6</v>
@@ -1879,13 +1879,13 @@
     </row>
     <row r="71" spans="1:4">
       <c r="A71" s="2">
-        <v>46136</v>
+        <v>46176</v>
       </c>
       <c r="B71">
         <v>7</v>
       </c>
       <c r="C71">
-        <v>0.028</v>
+        <v>0.091</v>
       </c>
       <c r="D71" t="s">
         <v>73</v>
@@ -1893,13 +1893,13 @@
     </row>
     <row r="72" spans="1:4">
       <c r="A72" s="2">
-        <v>46136</v>
+        <v>46176</v>
       </c>
       <c r="B72">
         <v>8</v>
       </c>
       <c r="C72">
-        <v>0.404</v>
+        <v>0.405</v>
       </c>
       <c r="D72" t="s">
         <v>74</v>
@@ -1907,13 +1907,13 @@
     </row>
     <row r="73" spans="1:4">
       <c r="A73" s="2">
-        <v>46136</v>
+        <v>46176</v>
       </c>
       <c r="B73">
         <v>9</v>
       </c>
       <c r="C73">
-        <v>1.082</v>
+        <v>0.98</v>
       </c>
       <c r="D73" t="s">
         <v>75</v>
@@ -1921,13 +1921,13 @@
     </row>
     <row r="74" spans="1:4">
       <c r="A74" s="2">
-        <v>46136</v>
+        <v>46176</v>
       </c>
       <c r="B74">
         <v>10</v>
       </c>
       <c r="C74">
-        <v>1.867</v>
+        <v>1.532</v>
       </c>
       <c r="D74" t="s">
         <v>76</v>
@@ -1935,13 +1935,13 @@
     </row>
     <row r="75" spans="1:4">
       <c r="A75" s="2">
-        <v>46136</v>
+        <v>46176</v>
       </c>
       <c r="B75">
         <v>11</v>
       </c>
       <c r="C75">
-        <v>2.068</v>
+        <v>2.061</v>
       </c>
       <c r="D75" t="s">
         <v>77</v>
@@ -1949,13 +1949,13 @@
     </row>
     <row r="76" spans="1:4">
       <c r="A76" s="2">
-        <v>46136</v>
+        <v>46176</v>
       </c>
       <c r="B76">
         <v>12</v>
       </c>
       <c r="C76">
-        <v>1.991</v>
+        <v>2.462</v>
       </c>
       <c r="D76" t="s">
         <v>78</v>
@@ -1963,13 +1963,13 @@
     </row>
     <row r="77" spans="1:4">
       <c r="A77" s="2">
-        <v>46136</v>
+        <v>46176</v>
       </c>
       <c r="B77">
         <v>13</v>
       </c>
       <c r="C77">
-        <v>1.887</v>
+        <v>2.819</v>
       </c>
       <c r="D77" t="s">
         <v>79</v>
@@ -1977,13 +1977,13 @@
     </row>
     <row r="78" spans="1:4">
       <c r="A78" s="2">
-        <v>46136</v>
+        <v>46176</v>
       </c>
       <c r="B78">
         <v>14</v>
       </c>
       <c r="C78">
-        <v>1.863</v>
+        <v>2.875</v>
       </c>
       <c r="D78" t="s">
         <v>80</v>
@@ -1991,13 +1991,13 @@
     </row>
     <row r="79" spans="1:4">
       <c r="A79" s="2">
-        <v>46136</v>
+        <v>46176</v>
       </c>
       <c r="B79">
         <v>15</v>
       </c>
       <c r="C79">
-        <v>1.904</v>
+        <v>2.691</v>
       </c>
       <c r="D79" t="s">
         <v>81</v>
@@ -2005,13 +2005,13 @@
     </row>
     <row r="80" spans="1:4">
       <c r="A80" s="2">
-        <v>46136</v>
+        <v>46176</v>
       </c>
       <c r="B80">
         <v>16</v>
       </c>
       <c r="C80">
-        <v>1.729</v>
+        <v>2.326</v>
       </c>
       <c r="D80" t="s">
         <v>82</v>
@@ -2019,13 +2019,13 @@
     </row>
     <row r="81" spans="1:4">
       <c r="A81" s="2">
-        <v>46136</v>
+        <v>46176</v>
       </c>
       <c r="B81">
         <v>17</v>
       </c>
       <c r="C81">
-        <v>1.516</v>
+        <v>1.916</v>
       </c>
       <c r="D81" t="s">
         <v>83</v>
@@ -2033,13 +2033,13 @@
     </row>
     <row r="82" spans="1:4">
       <c r="A82" s="2">
-        <v>46136</v>
+        <v>46176</v>
       </c>
       <c r="B82">
         <v>18</v>
       </c>
       <c r="C82">
-        <v>1.061</v>
+        <v>1.398</v>
       </c>
       <c r="D82" t="s">
         <v>84</v>
@@ -2047,13 +2047,13 @@
     </row>
     <row r="83" spans="1:4">
       <c r="A83" s="2">
-        <v>46136</v>
+        <v>46176</v>
       </c>
       <c r="B83">
         <v>19</v>
       </c>
       <c r="C83">
-        <v>0.454</v>
+        <v>0.822</v>
       </c>
       <c r="D83" t="s">
         <v>85</v>
@@ -2061,13 +2061,13 @@
     </row>
     <row r="84" spans="1:4">
       <c r="A84" s="2">
-        <v>46136</v>
+        <v>46176</v>
       </c>
       <c r="B84">
         <v>20</v>
       </c>
       <c r="C84">
-        <v>0.098</v>
+        <v>0.344</v>
       </c>
       <c r="D84" t="s">
         <v>86</v>
@@ -2075,13 +2075,13 @@
     </row>
     <row r="85" spans="1:4">
       <c r="A85" s="2">
-        <v>46136</v>
+        <v>46176</v>
       </c>
       <c r="B85">
         <v>21</v>
       </c>
       <c r="C85">
-        <v>0</v>
+        <v>0.056</v>
       </c>
       <c r="D85" t="s">
         <v>87</v>
@@ -2089,7 +2089,7 @@
     </row>
     <row r="86" spans="1:4">
       <c r="A86" s="2">
-        <v>46136</v>
+        <v>46176</v>
       </c>
       <c r="B86">
         <v>22</v>
@@ -2103,7 +2103,7 @@
     </row>
     <row r="87" spans="1:4">
       <c r="A87" s="2">
-        <v>46136</v>
+        <v>46176</v>
       </c>
       <c r="B87">
         <v>23</v>
@@ -2117,7 +2117,7 @@
     </row>
     <row r="88" spans="1:4">
       <c r="A88" s="2">
-        <v>46136</v>
+        <v>46176</v>
       </c>
       <c r="B88">
         <v>24</v>
@@ -2131,7 +2131,7 @@
     </row>
     <row r="89" spans="1:4">
       <c r="A89" s="2">
-        <v>46137</v>
+        <v>46177</v>
       </c>
       <c r="B89">
         <v>1</v>
@@ -2145,7 +2145,7 @@
     </row>
     <row r="90" spans="1:4">
       <c r="A90" s="2">
-        <v>46137</v>
+        <v>46177</v>
       </c>
       <c r="B90">
         <v>2</v>
@@ -2159,7 +2159,7 @@
     </row>
     <row r="91" spans="1:4">
       <c r="A91" s="2">
-        <v>46137</v>
+        <v>46177</v>
       </c>
       <c r="B91">
         <v>3</v>
@@ -2173,7 +2173,7 @@
     </row>
     <row r="92" spans="1:4">
       <c r="A92" s="2">
-        <v>46137</v>
+        <v>46177</v>
       </c>
       <c r="B92">
         <v>4</v>
@@ -2187,7 +2187,7 @@
     </row>
     <row r="93" spans="1:4">
       <c r="A93" s="2">
-        <v>46137</v>
+        <v>46177</v>
       </c>
       <c r="B93">
         <v>5</v>
@@ -2201,7 +2201,7 @@
     </row>
     <row r="94" spans="1:4">
       <c r="A94" s="2">
-        <v>46137</v>
+        <v>46177</v>
       </c>
       <c r="B94">
         <v>6</v>
@@ -2215,13 +2215,13 @@
     </row>
     <row r="95" spans="1:4">
       <c r="A95" s="2">
-        <v>46137</v>
+        <v>46177</v>
       </c>
       <c r="B95">
         <v>7</v>
       </c>
       <c r="C95">
-        <v>0.015</v>
+        <v>0.105</v>
       </c>
       <c r="D95" t="s">
         <v>97</v>
@@ -2229,13 +2229,13 @@
     </row>
     <row r="96" spans="1:4">
       <c r="A96" s="2">
-        <v>46137</v>
+        <v>46177</v>
       </c>
       <c r="B96">
         <v>8</v>
       </c>
       <c r="C96">
-        <v>0.314</v>
+        <v>0.417</v>
       </c>
       <c r="D96" t="s">
         <v>98</v>
@@ -2243,13 +2243,13 @@
     </row>
     <row r="97" spans="1:4">
       <c r="A97" s="2">
-        <v>46137</v>
+        <v>46177</v>
       </c>
       <c r="B97">
         <v>9</v>
       </c>
       <c r="C97">
-        <v>0.882</v>
+        <v>0.928</v>
       </c>
       <c r="D97" t="s">
         <v>99</v>
@@ -2257,13 +2257,13 @@
     </row>
     <row r="98" spans="1:4">
       <c r="A98" s="2">
-        <v>46137</v>
+        <v>46177</v>
       </c>
       <c r="B98">
         <v>10</v>
       </c>
       <c r="C98">
-        <v>1.406</v>
+        <v>1.543</v>
       </c>
       <c r="D98" t="s">
         <v>100</v>
@@ -2271,13 +2271,13 @@
     </row>
     <row r="99" spans="1:4">
       <c r="A99" s="2">
-        <v>46137</v>
+        <v>46177</v>
       </c>
       <c r="B99">
         <v>11</v>
       </c>
       <c r="C99">
-        <v>1.84</v>
+        <v>2.028</v>
       </c>
       <c r="D99" t="s">
         <v>101</v>
@@ -2285,13 +2285,13 @@
     </row>
     <row r="100" spans="1:4">
       <c r="A100" s="2">
-        <v>46137</v>
+        <v>46177</v>
       </c>
       <c r="B100">
         <v>12</v>
       </c>
       <c r="C100">
-        <v>1.978</v>
+        <v>2.455</v>
       </c>
       <c r="D100" t="s">
         <v>102</v>
@@ -2299,13 +2299,13 @@
     </row>
     <row r="101" spans="1:4">
       <c r="A101" s="2">
-        <v>46137</v>
+        <v>46177</v>
       </c>
       <c r="B101">
         <v>13</v>
       </c>
       <c r="C101">
-        <v>1.958</v>
+        <v>2.47</v>
       </c>
       <c r="D101" t="s">
         <v>103</v>
@@ -2313,13 +2313,13 @@
     </row>
     <row r="102" spans="1:4">
       <c r="A102" s="2">
-        <v>46137</v>
+        <v>46177</v>
       </c>
       <c r="B102">
         <v>14</v>
       </c>
       <c r="C102">
-        <v>1.931</v>
+        <v>2.442</v>
       </c>
       <c r="D102" t="s">
         <v>104</v>
@@ -2327,13 +2327,13 @@
     </row>
     <row r="103" spans="1:4">
       <c r="A103" s="2">
-        <v>46137</v>
+        <v>46177</v>
       </c>
       <c r="B103">
         <v>15</v>
       </c>
       <c r="C103">
-        <v>1.939</v>
+        <v>2.15</v>
       </c>
       <c r="D103" t="s">
         <v>105</v>
@@ -2341,13 +2341,13 @@
     </row>
     <row r="104" spans="1:4">
       <c r="A104" s="2">
-        <v>46137</v>
+        <v>46177</v>
       </c>
       <c r="B104">
         <v>16</v>
       </c>
       <c r="C104">
-        <v>1.619</v>
+        <v>1.809</v>
       </c>
       <c r="D104" t="s">
         <v>106</v>
@@ -2355,13 +2355,13 @@
     </row>
     <row r="105" spans="1:4">
       <c r="A105" s="2">
-        <v>46137</v>
+        <v>46177</v>
       </c>
       <c r="B105">
         <v>17</v>
       </c>
       <c r="C105">
-        <v>1.317</v>
+        <v>1.677</v>
       </c>
       <c r="D105" t="s">
         <v>107</v>
@@ -2369,13 +2369,13 @@
     </row>
     <row r="106" spans="1:4">
       <c r="A106" s="2">
-        <v>46137</v>
+        <v>46177</v>
       </c>
       <c r="B106">
         <v>18</v>
       </c>
       <c r="C106">
-        <v>0.857</v>
+        <v>1.124</v>
       </c>
       <c r="D106" t="s">
         <v>108</v>
@@ -2383,13 +2383,13 @@
     </row>
     <row r="107" spans="1:4">
       <c r="A107" s="2">
-        <v>46137</v>
+        <v>46177</v>
       </c>
       <c r="B107">
         <v>19</v>
       </c>
       <c r="C107">
-        <v>0.424</v>
+        <v>0.635</v>
       </c>
       <c r="D107" t="s">
         <v>109</v>
@@ -2397,13 +2397,13 @@
     </row>
     <row r="108" spans="1:4">
       <c r="A108" s="2">
-        <v>46137</v>
+        <v>46177</v>
       </c>
       <c r="B108">
         <v>20</v>
       </c>
       <c r="C108">
-        <v>0.06900000000000001</v>
+        <v>0.272</v>
       </c>
       <c r="D108" t="s">
         <v>110</v>
@@ -2411,13 +2411,13 @@
     </row>
     <row r="109" spans="1:4">
       <c r="A109" s="2">
-        <v>46137</v>
+        <v>46177</v>
       </c>
       <c r="B109">
         <v>21</v>
       </c>
       <c r="C109">
-        <v>0</v>
+        <v>0.046</v>
       </c>
       <c r="D109" t="s">
         <v>111</v>
@@ -2425,7 +2425,7 @@
     </row>
     <row r="110" spans="1:4">
       <c r="A110" s="2">
-        <v>46137</v>
+        <v>46177</v>
       </c>
       <c r="B110">
         <v>22</v>
@@ -2439,7 +2439,7 @@
     </row>
     <row r="111" spans="1:4">
       <c r="A111" s="2">
-        <v>46137</v>
+        <v>46177</v>
       </c>
       <c r="B111">
         <v>23</v>
@@ -2453,7 +2453,7 @@
     </row>
     <row r="112" spans="1:4">
       <c r="A112" s="2">
-        <v>46137</v>
+        <v>46177</v>
       </c>
       <c r="B112">
         <v>24</v>
@@ -2467,7 +2467,7 @@
     </row>
     <row r="113" spans="1:4">
       <c r="A113" s="2">
-        <v>46138</v>
+        <v>46178</v>
       </c>
       <c r="B113">
         <v>1</v>
@@ -2481,7 +2481,7 @@
     </row>
     <row r="114" spans="1:4">
       <c r="A114" s="2">
-        <v>46138</v>
+        <v>46178</v>
       </c>
       <c r="B114">
         <v>2</v>
@@ -2495,7 +2495,7 @@
     </row>
     <row r="115" spans="1:4">
       <c r="A115" s="2">
-        <v>46138</v>
+        <v>46178</v>
       </c>
       <c r="B115">
         <v>3</v>
@@ -2509,7 +2509,7 @@
     </row>
     <row r="116" spans="1:4">
       <c r="A116" s="2">
-        <v>46138</v>
+        <v>46178</v>
       </c>
       <c r="B116">
         <v>4</v>
@@ -2523,7 +2523,7 @@
     </row>
     <row r="117" spans="1:4">
       <c r="A117" s="2">
-        <v>46138</v>
+        <v>46178</v>
       </c>
       <c r="B117">
         <v>5</v>
@@ -2537,7 +2537,7 @@
     </row>
     <row r="118" spans="1:4">
       <c r="A118" s="2">
-        <v>46138</v>
+        <v>46178</v>
       </c>
       <c r="B118">
         <v>6</v>
@@ -2551,13 +2551,13 @@
     </row>
     <row r="119" spans="1:4">
       <c r="A119" s="2">
-        <v>46138</v>
+        <v>46178</v>
       </c>
       <c r="B119">
         <v>7</v>
       </c>
       <c r="C119">
-        <v>0.029</v>
+        <v>0.07199999999999999</v>
       </c>
       <c r="D119" t="s">
         <v>121</v>
@@ -2565,13 +2565,13 @@
     </row>
     <row r="120" spans="1:4">
       <c r="A120" s="2">
-        <v>46138</v>
+        <v>46178</v>
       </c>
       <c r="B120">
         <v>8</v>
       </c>
       <c r="C120">
-        <v>0.37</v>
+        <v>0.424</v>
       </c>
       <c r="D120" t="s">
         <v>122</v>
@@ -2579,13 +2579,13 @@
     </row>
     <row r="121" spans="1:4">
       <c r="A121" s="2">
-        <v>46138</v>
+        <v>46178</v>
       </c>
       <c r="B121">
         <v>9</v>
       </c>
       <c r="C121">
-        <v>1.048</v>
+        <v>0.978</v>
       </c>
       <c r="D121" t="s">
         <v>123</v>
@@ -2593,13 +2593,13 @@
     </row>
     <row r="122" spans="1:4">
       <c r="A122" s="2">
-        <v>46138</v>
+        <v>46178</v>
       </c>
       <c r="B122">
         <v>10</v>
       </c>
       <c r="C122">
-        <v>1.783</v>
+        <v>1.477</v>
       </c>
       <c r="D122" t="s">
         <v>124</v>
@@ -2607,13 +2607,13 @@
     </row>
     <row r="123" spans="1:4">
       <c r="A123" s="2">
-        <v>46138</v>
+        <v>46178</v>
       </c>
       <c r="B123">
         <v>11</v>
       </c>
       <c r="C123">
-        <v>2.024</v>
+        <v>1.879</v>
       </c>
       <c r="D123" t="s">
         <v>125</v>
@@ -2621,13 +2621,13 @@
     </row>
     <row r="124" spans="1:4">
       <c r="A124" s="2">
-        <v>46138</v>
+        <v>46178</v>
       </c>
       <c r="B124">
         <v>12</v>
       </c>
       <c r="C124">
-        <v>1.998</v>
+        <v>2.223</v>
       </c>
       <c r="D124" t="s">
         <v>126</v>
@@ -2635,13 +2635,13 @@
     </row>
     <row r="125" spans="1:4">
       <c r="A125" s="2">
-        <v>46138</v>
+        <v>46178</v>
       </c>
       <c r="B125">
         <v>13</v>
       </c>
       <c r="C125">
-        <v>1.963</v>
+        <v>2.395</v>
       </c>
       <c r="D125" t="s">
         <v>127</v>
@@ -2649,13 +2649,13 @@
     </row>
     <row r="126" spans="1:4">
       <c r="A126" s="2">
-        <v>46138</v>
+        <v>46178</v>
       </c>
       <c r="B126">
         <v>14</v>
       </c>
       <c r="C126">
-        <v>1.939</v>
+        <v>2.411</v>
       </c>
       <c r="D126" t="s">
         <v>128</v>
@@ -2663,13 +2663,13 @@
     </row>
     <row r="127" spans="1:4">
       <c r="A127" s="2">
-        <v>46138</v>
+        <v>46178</v>
       </c>
       <c r="B127">
         <v>15</v>
       </c>
       <c r="C127">
-        <v>1.977</v>
+        <v>2.431</v>
       </c>
       <c r="D127" t="s">
         <v>129</v>
@@ -2677,13 +2677,13 @@
     </row>
     <row r="128" spans="1:4">
       <c r="A128" s="2">
-        <v>46138</v>
+        <v>46178</v>
       </c>
       <c r="B128">
         <v>16</v>
       </c>
       <c r="C128">
-        <v>1.942</v>
+        <v>1.983</v>
       </c>
       <c r="D128" t="s">
         <v>130</v>
@@ -2691,13 +2691,13 @@
     </row>
     <row r="129" spans="1:4">
       <c r="A129" s="2">
-        <v>46138</v>
+        <v>46178</v>
       </c>
       <c r="B129">
         <v>17</v>
       </c>
       <c r="C129">
-        <v>1.588</v>
+        <v>1.7</v>
       </c>
       <c r="D129" t="s">
         <v>131</v>
@@ -2705,13 +2705,13 @@
     </row>
     <row r="130" spans="1:4">
       <c r="A130" s="2">
-        <v>46138</v>
+        <v>46178</v>
       </c>
       <c r="B130">
         <v>18</v>
       </c>
       <c r="C130">
-        <v>1.197</v>
+        <v>1.145</v>
       </c>
       <c r="D130" t="s">
         <v>132</v>
@@ -2719,13 +2719,13 @@
     </row>
     <row r="131" spans="1:4">
       <c r="A131" s="2">
-        <v>46138</v>
+        <v>46178</v>
       </c>
       <c r="B131">
         <v>19</v>
       </c>
       <c r="C131">
-        <v>0.465</v>
+        <v>0.618</v>
       </c>
       <c r="D131" t="s">
         <v>133</v>
@@ -2733,13 +2733,13 @@
     </row>
     <row r="132" spans="1:4">
       <c r="A132" s="2">
-        <v>46138</v>
+        <v>46178</v>
       </c>
       <c r="B132">
         <v>20</v>
       </c>
       <c r="C132">
-        <v>0.106</v>
+        <v>0.275</v>
       </c>
       <c r="D132" t="s">
         <v>134</v>
@@ -2747,13 +2747,13 @@
     </row>
     <row r="133" spans="1:4">
       <c r="A133" s="2">
-        <v>46138</v>
+        <v>46178</v>
       </c>
       <c r="B133">
         <v>21</v>
       </c>
       <c r="C133">
-        <v>0</v>
+        <v>0.046</v>
       </c>
       <c r="D133" t="s">
         <v>135</v>
@@ -2761,7 +2761,7 @@
     </row>
     <row r="134" spans="1:4">
       <c r="A134" s="2">
-        <v>46138</v>
+        <v>46178</v>
       </c>
       <c r="B134">
         <v>22</v>
@@ -2775,7 +2775,7 @@
     </row>
     <row r="135" spans="1:4">
       <c r="A135" s="2">
-        <v>46138</v>
+        <v>46178</v>
       </c>
       <c r="B135">
         <v>23</v>
@@ -2789,7 +2789,7 @@
     </row>
     <row r="136" spans="1:4">
       <c r="A136" s="2">
-        <v>46138</v>
+        <v>46178</v>
       </c>
       <c r="B136">
         <v>24</v>
@@ -2803,7 +2803,7 @@
     </row>
     <row r="137" spans="1:4">
       <c r="A137" s="2">
-        <v>46139</v>
+        <v>46179</v>
       </c>
       <c r="B137">
         <v>1</v>
@@ -2817,7 +2817,7 @@
     </row>
     <row r="138" spans="1:4">
       <c r="A138" s="2">
-        <v>46139</v>
+        <v>46179</v>
       </c>
       <c r="B138">
         <v>2</v>
@@ -2831,7 +2831,7 @@
     </row>
     <row r="139" spans="1:4">
       <c r="A139" s="2">
-        <v>46139</v>
+        <v>46179</v>
       </c>
       <c r="B139">
         <v>3</v>
@@ -2845,7 +2845,7 @@
     </row>
     <row r="140" spans="1:4">
       <c r="A140" s="2">
-        <v>46139</v>
+        <v>46179</v>
       </c>
       <c r="B140">
         <v>4</v>
@@ -2859,7 +2859,7 @@
     </row>
     <row r="141" spans="1:4">
       <c r="A141" s="2">
-        <v>46139</v>
+        <v>46179</v>
       </c>
       <c r="B141">
         <v>5</v>
@@ -2873,7 +2873,7 @@
     </row>
     <row r="142" spans="1:4">
       <c r="A142" s="2">
-        <v>46139</v>
+        <v>46179</v>
       </c>
       <c r="B142">
         <v>6</v>
@@ -2887,13 +2887,13 @@
     </row>
     <row r="143" spans="1:4">
       <c r="A143" s="2">
-        <v>46139</v>
+        <v>46179</v>
       </c>
       <c r="B143">
         <v>7</v>
       </c>
       <c r="C143">
-        <v>0.03</v>
+        <v>0.075</v>
       </c>
       <c r="D143" t="s">
         <v>145</v>
@@ -2901,13 +2901,13 @@
     </row>
     <row r="144" spans="1:4">
       <c r="A144" s="2">
-        <v>46139</v>
+        <v>46179</v>
       </c>
       <c r="B144">
         <v>8</v>
       </c>
       <c r="C144">
-        <v>0.455</v>
+        <v>0.446</v>
       </c>
       <c r="D144" t="s">
         <v>146</v>
@@ -2915,13 +2915,13 @@
     </row>
     <row r="145" spans="1:4">
       <c r="A145" s="2">
-        <v>46139</v>
+        <v>46179</v>
       </c>
       <c r="B145">
         <v>9</v>
       </c>
       <c r="C145">
-        <v>1.222</v>
+        <v>0.9330000000000001</v>
       </c>
       <c r="D145" t="s">
         <v>147</v>
@@ -2929,13 +2929,13 @@
     </row>
     <row r="146" spans="1:4">
       <c r="A146" s="2">
-        <v>46139</v>
+        <v>46179</v>
       </c>
       <c r="B146">
         <v>10</v>
       </c>
       <c r="C146">
-        <v>2.16</v>
+        <v>1.612</v>
       </c>
       <c r="D146" t="s">
         <v>148</v>
@@ -2943,13 +2943,13 @@
     </row>
     <row r="147" spans="1:4">
       <c r="A147" s="2">
-        <v>46139</v>
+        <v>46179</v>
       </c>
       <c r="B147">
         <v>11</v>
       </c>
       <c r="C147">
-        <v>2.899</v>
+        <v>2.014</v>
       </c>
       <c r="D147" t="s">
         <v>149</v>
@@ -2957,13 +2957,13 @@
     </row>
     <row r="148" spans="1:4">
       <c r="A148" s="2">
-        <v>46139</v>
+        <v>46179</v>
       </c>
       <c r="B148">
         <v>12</v>
       </c>
       <c r="C148">
-        <v>3.232</v>
+        <v>2.365</v>
       </c>
       <c r="D148" t="s">
         <v>150</v>
@@ -2971,13 +2971,13 @@
     </row>
     <row r="149" spans="1:4">
       <c r="A149" s="2">
-        <v>46139</v>
+        <v>46179</v>
       </c>
       <c r="B149">
         <v>13</v>
       </c>
       <c r="C149">
-        <v>3.232</v>
+        <v>2.428</v>
       </c>
       <c r="D149" t="s">
         <v>151</v>
@@ -2985,13 +2985,13 @@
     </row>
     <row r="150" spans="1:4">
       <c r="A150" s="2">
-        <v>46139</v>
+        <v>46179</v>
       </c>
       <c r="B150">
         <v>14</v>
       </c>
       <c r="C150">
-        <v>3.158</v>
+        <v>2.376</v>
       </c>
       <c r="D150" t="s">
         <v>152</v>
@@ -2999,13 +2999,13 @@
     </row>
     <row r="151" spans="1:4">
       <c r="A151" s="2">
-        <v>46139</v>
+        <v>46179</v>
       </c>
       <c r="B151">
         <v>15</v>
       </c>
       <c r="C151">
-        <v>3.133</v>
+        <v>2.269</v>
       </c>
       <c r="D151" t="s">
         <v>153</v>
@@ -3013,13 +3013,13 @@
     </row>
     <row r="152" spans="1:4">
       <c r="A152" s="2">
-        <v>46139</v>
+        <v>46179</v>
       </c>
       <c r="B152">
         <v>16</v>
       </c>
       <c r="C152">
-        <v>2.778</v>
+        <v>1.91</v>
       </c>
       <c r="D152" t="s">
         <v>154</v>
@@ -3027,13 +3027,13 @@
     </row>
     <row r="153" spans="1:4">
       <c r="A153" s="2">
-        <v>46139</v>
+        <v>46179</v>
       </c>
       <c r="B153">
         <v>17</v>
       </c>
       <c r="C153">
-        <v>2.192</v>
+        <v>1.651</v>
       </c>
       <c r="D153" t="s">
         <v>155</v>
@@ -3041,13 +3041,13 @@
     </row>
     <row r="154" spans="1:4">
       <c r="A154" s="2">
-        <v>46139</v>
+        <v>46179</v>
       </c>
       <c r="B154">
         <v>18</v>
       </c>
       <c r="C154">
-        <v>1.444</v>
+        <v>1.065</v>
       </c>
       <c r="D154" t="s">
         <v>156</v>
@@ -3055,13 +3055,13 @@
     </row>
     <row r="155" spans="1:4">
       <c r="A155" s="2">
-        <v>46139</v>
+        <v>46179</v>
       </c>
       <c r="B155">
         <v>19</v>
       </c>
       <c r="C155">
-        <v>0.621</v>
+        <v>0.593</v>
       </c>
       <c r="D155" t="s">
         <v>157</v>
@@ -3069,13 +3069,13 @@
     </row>
     <row r="156" spans="1:4">
       <c r="A156" s="2">
-        <v>46139</v>
+        <v>46179</v>
       </c>
       <c r="B156">
         <v>20</v>
       </c>
       <c r="C156">
-        <v>0.136</v>
+        <v>0.301</v>
       </c>
       <c r="D156" t="s">
         <v>158</v>
@@ -3083,13 +3083,13 @@
     </row>
     <row r="157" spans="1:4">
       <c r="A157" s="2">
-        <v>46139</v>
+        <v>46179</v>
       </c>
       <c r="B157">
         <v>21</v>
       </c>
       <c r="C157">
-        <v>0</v>
+        <v>0.05</v>
       </c>
       <c r="D157" t="s">
         <v>159</v>
@@ -3097,7 +3097,7 @@
     </row>
     <row r="158" spans="1:4">
       <c r="A158" s="2">
-        <v>46139</v>
+        <v>46179</v>
       </c>
       <c r="B158">
         <v>22</v>
@@ -3111,7 +3111,7 @@
     </row>
     <row r="159" spans="1:4">
       <c r="A159" s="2">
-        <v>46139</v>
+        <v>46179</v>
       </c>
       <c r="B159">
         <v>23</v>
@@ -3125,7 +3125,7 @@
     </row>
     <row r="160" spans="1:4">
       <c r="A160" s="2">
-        <v>46139</v>
+        <v>46179</v>
       </c>
       <c r="B160">
         <v>24</v>
@@ -3139,7 +3139,7 @@
     </row>
     <row r="161" spans="1:4">
       <c r="A161" s="2">
-        <v>46140</v>
+        <v>46180</v>
       </c>
       <c r="B161">
         <v>1</v>
@@ -3153,7 +3153,7 @@
     </row>
     <row r="162" spans="1:4">
       <c r="A162" s="2">
-        <v>46140</v>
+        <v>46180</v>
       </c>
       <c r="B162">
         <v>2</v>
@@ -3167,7 +3167,7 @@
     </row>
     <row r="163" spans="1:4">
       <c r="A163" s="2">
-        <v>46140</v>
+        <v>46180</v>
       </c>
       <c r="B163">
         <v>3</v>
@@ -3181,7 +3181,7 @@
     </row>
     <row r="164" spans="1:4">
       <c r="A164" s="2">
-        <v>46140</v>
+        <v>46180</v>
       </c>
       <c r="B164">
         <v>4</v>
@@ -3195,7 +3195,7 @@
     </row>
     <row r="165" spans="1:4">
       <c r="A165" s="2">
-        <v>46140</v>
+        <v>46180</v>
       </c>
       <c r="B165">
         <v>5</v>
@@ -3209,7 +3209,7 @@
     </row>
     <row r="166" spans="1:4">
       <c r="A166" s="2">
-        <v>46140</v>
+        <v>46180</v>
       </c>
       <c r="B166">
         <v>6</v>
@@ -3223,13 +3223,13 @@
     </row>
     <row r="167" spans="1:4">
       <c r="A167" s="2">
-        <v>46140</v>
+        <v>46180</v>
       </c>
       <c r="B167">
         <v>7</v>
       </c>
       <c r="C167">
-        <v>0.028</v>
+        <v>0.075</v>
       </c>
       <c r="D167" t="s">
         <v>169</v>
@@ -3237,13 +3237,13 @@
     </row>
     <row r="168" spans="1:4">
       <c r="A168" s="2">
-        <v>46140</v>
+        <v>46180</v>
       </c>
       <c r="B168">
         <v>8</v>
       </c>
       <c r="C168">
-        <v>0.42</v>
+        <v>0.451</v>
       </c>
       <c r="D168" t="s">
         <v>170</v>
@@ -3251,13 +3251,13 @@
     </row>
     <row r="169" spans="1:4">
       <c r="A169" s="2">
-        <v>46140</v>
+        <v>46180</v>
       </c>
       <c r="B169">
         <v>9</v>
       </c>
       <c r="C169">
-        <v>1.064</v>
+        <v>0.8120000000000001</v>
       </c>
       <c r="D169" t="s">
         <v>171</v>
@@ -3265,13 +3265,13 @@
     </row>
     <row r="170" spans="1:4">
       <c r="A170" s="2">
-        <v>46140</v>
+        <v>46180</v>
       </c>
       <c r="B170">
         <v>10</v>
       </c>
       <c r="C170">
-        <v>2.105</v>
+        <v>1.382</v>
       </c>
       <c r="D170" t="s">
         <v>172</v>

</xml_diff>

<commit_message>
Updating the model for Astro
</commit_message>
<xml_diff>
--- a/Astro/Results_Production_Astro_xgb.xlsx
+++ b/Astro/Results_Production_Astro_xgb.xlsx
@@ -28,312 +28,6 @@
     <t>Lookup</t>
   </si>
   <si>
-    <t>31.05.202610</t>
-  </si>
-  <si>
-    <t>31.05.202611</t>
-  </si>
-  <si>
-    <t>31.05.202612</t>
-  </si>
-  <si>
-    <t>31.05.202613</t>
-  </si>
-  <si>
-    <t>31.05.202614</t>
-  </si>
-  <si>
-    <t>31.05.202615</t>
-  </si>
-  <si>
-    <t>31.05.202616</t>
-  </si>
-  <si>
-    <t>31.05.202617</t>
-  </si>
-  <si>
-    <t>31.05.202618</t>
-  </si>
-  <si>
-    <t>31.05.202619</t>
-  </si>
-  <si>
-    <t>31.05.202620</t>
-  </si>
-  <si>
-    <t>31.05.202621</t>
-  </si>
-  <si>
-    <t>31.05.202622</t>
-  </si>
-  <si>
-    <t>31.05.202623</t>
-  </si>
-  <si>
-    <t>31.05.202624</t>
-  </si>
-  <si>
-    <t>01.06.20261</t>
-  </si>
-  <si>
-    <t>01.06.20262</t>
-  </si>
-  <si>
-    <t>01.06.20263</t>
-  </si>
-  <si>
-    <t>01.06.20264</t>
-  </si>
-  <si>
-    <t>01.06.20265</t>
-  </si>
-  <si>
-    <t>01.06.20266</t>
-  </si>
-  <si>
-    <t>01.06.20267</t>
-  </si>
-  <si>
-    <t>01.06.20268</t>
-  </si>
-  <si>
-    <t>01.06.20269</t>
-  </si>
-  <si>
-    <t>01.06.202610</t>
-  </si>
-  <si>
-    <t>01.06.202611</t>
-  </si>
-  <si>
-    <t>01.06.202612</t>
-  </si>
-  <si>
-    <t>01.06.202613</t>
-  </si>
-  <si>
-    <t>01.06.202614</t>
-  </si>
-  <si>
-    <t>01.06.202615</t>
-  </si>
-  <si>
-    <t>01.06.202616</t>
-  </si>
-  <si>
-    <t>01.06.202617</t>
-  </si>
-  <si>
-    <t>01.06.202618</t>
-  </si>
-  <si>
-    <t>01.06.202619</t>
-  </si>
-  <si>
-    <t>01.06.202620</t>
-  </si>
-  <si>
-    <t>01.06.202621</t>
-  </si>
-  <si>
-    <t>01.06.202622</t>
-  </si>
-  <si>
-    <t>01.06.202623</t>
-  </si>
-  <si>
-    <t>01.06.202624</t>
-  </si>
-  <si>
-    <t>02.06.20261</t>
-  </si>
-  <si>
-    <t>02.06.20262</t>
-  </si>
-  <si>
-    <t>02.06.20263</t>
-  </si>
-  <si>
-    <t>02.06.20264</t>
-  </si>
-  <si>
-    <t>02.06.20265</t>
-  </si>
-  <si>
-    <t>02.06.20266</t>
-  </si>
-  <si>
-    <t>02.06.20267</t>
-  </si>
-  <si>
-    <t>02.06.20268</t>
-  </si>
-  <si>
-    <t>02.06.20269</t>
-  </si>
-  <si>
-    <t>02.06.202610</t>
-  </si>
-  <si>
-    <t>02.06.202611</t>
-  </si>
-  <si>
-    <t>02.06.202612</t>
-  </si>
-  <si>
-    <t>02.06.202613</t>
-  </si>
-  <si>
-    <t>02.06.202614</t>
-  </si>
-  <si>
-    <t>02.06.202615</t>
-  </si>
-  <si>
-    <t>02.06.202616</t>
-  </si>
-  <si>
-    <t>02.06.202617</t>
-  </si>
-  <si>
-    <t>02.06.202618</t>
-  </si>
-  <si>
-    <t>02.06.202619</t>
-  </si>
-  <si>
-    <t>02.06.202620</t>
-  </si>
-  <si>
-    <t>02.06.202621</t>
-  </si>
-  <si>
-    <t>02.06.202622</t>
-  </si>
-  <si>
-    <t>02.06.202623</t>
-  </si>
-  <si>
-    <t>02.06.202624</t>
-  </si>
-  <si>
-    <t>03.06.20261</t>
-  </si>
-  <si>
-    <t>03.06.20262</t>
-  </si>
-  <si>
-    <t>03.06.20263</t>
-  </si>
-  <si>
-    <t>03.06.20264</t>
-  </si>
-  <si>
-    <t>03.06.20265</t>
-  </si>
-  <si>
-    <t>03.06.20266</t>
-  </si>
-  <si>
-    <t>03.06.20267</t>
-  </si>
-  <si>
-    <t>03.06.20268</t>
-  </si>
-  <si>
-    <t>03.06.20269</t>
-  </si>
-  <si>
-    <t>03.06.202610</t>
-  </si>
-  <si>
-    <t>03.06.202611</t>
-  </si>
-  <si>
-    <t>03.06.202612</t>
-  </si>
-  <si>
-    <t>03.06.202613</t>
-  </si>
-  <si>
-    <t>03.06.202614</t>
-  </si>
-  <si>
-    <t>03.06.202615</t>
-  </si>
-  <si>
-    <t>03.06.202616</t>
-  </si>
-  <si>
-    <t>03.06.202617</t>
-  </si>
-  <si>
-    <t>03.06.202618</t>
-  </si>
-  <si>
-    <t>03.06.202619</t>
-  </si>
-  <si>
-    <t>03.06.202620</t>
-  </si>
-  <si>
-    <t>03.06.202621</t>
-  </si>
-  <si>
-    <t>03.06.202622</t>
-  </si>
-  <si>
-    <t>03.06.202623</t>
-  </si>
-  <si>
-    <t>03.06.202624</t>
-  </si>
-  <si>
-    <t>04.06.20261</t>
-  </si>
-  <si>
-    <t>04.06.20262</t>
-  </si>
-  <si>
-    <t>04.06.20263</t>
-  </si>
-  <si>
-    <t>04.06.20264</t>
-  </si>
-  <si>
-    <t>04.06.20265</t>
-  </si>
-  <si>
-    <t>04.06.20266</t>
-  </si>
-  <si>
-    <t>04.06.20267</t>
-  </si>
-  <si>
-    <t>04.06.20268</t>
-  </si>
-  <si>
-    <t>04.06.20269</t>
-  </si>
-  <si>
-    <t>04.06.202610</t>
-  </si>
-  <si>
-    <t>04.06.202611</t>
-  </si>
-  <si>
-    <t>04.06.202612</t>
-  </si>
-  <si>
-    <t>04.06.202613</t>
-  </si>
-  <si>
-    <t>04.06.202614</t>
-  </si>
-  <si>
-    <t>04.06.202615</t>
-  </si>
-  <si>
     <t>04.06.202616</t>
   </si>
   <si>
@@ -533,6 +227,312 @@
   </si>
   <si>
     <t>07.06.202610</t>
+  </si>
+  <si>
+    <t>07.06.202611</t>
+  </si>
+  <si>
+    <t>07.06.202612</t>
+  </si>
+  <si>
+    <t>07.06.202613</t>
+  </si>
+  <si>
+    <t>07.06.202614</t>
+  </si>
+  <si>
+    <t>07.06.202615</t>
+  </si>
+  <si>
+    <t>07.06.202616</t>
+  </si>
+  <si>
+    <t>07.06.202617</t>
+  </si>
+  <si>
+    <t>07.06.202618</t>
+  </si>
+  <si>
+    <t>07.06.202619</t>
+  </si>
+  <si>
+    <t>07.06.202620</t>
+  </si>
+  <si>
+    <t>07.06.202621</t>
+  </si>
+  <si>
+    <t>07.06.202622</t>
+  </si>
+  <si>
+    <t>07.06.202623</t>
+  </si>
+  <si>
+    <t>07.06.202624</t>
+  </si>
+  <si>
+    <t>08.06.20261</t>
+  </si>
+  <si>
+    <t>08.06.20262</t>
+  </si>
+  <si>
+    <t>08.06.20263</t>
+  </si>
+  <si>
+    <t>08.06.20264</t>
+  </si>
+  <si>
+    <t>08.06.20265</t>
+  </si>
+  <si>
+    <t>08.06.20266</t>
+  </si>
+  <si>
+    <t>08.06.20267</t>
+  </si>
+  <si>
+    <t>08.06.20268</t>
+  </si>
+  <si>
+    <t>08.06.20269</t>
+  </si>
+  <si>
+    <t>08.06.202610</t>
+  </si>
+  <si>
+    <t>08.06.202611</t>
+  </si>
+  <si>
+    <t>08.06.202612</t>
+  </si>
+  <si>
+    <t>08.06.202613</t>
+  </si>
+  <si>
+    <t>08.06.202614</t>
+  </si>
+  <si>
+    <t>08.06.202615</t>
+  </si>
+  <si>
+    <t>08.06.202616</t>
+  </si>
+  <si>
+    <t>08.06.202617</t>
+  </si>
+  <si>
+    <t>08.06.202618</t>
+  </si>
+  <si>
+    <t>08.06.202619</t>
+  </si>
+  <si>
+    <t>08.06.202620</t>
+  </si>
+  <si>
+    <t>08.06.202621</t>
+  </si>
+  <si>
+    <t>08.06.202622</t>
+  </si>
+  <si>
+    <t>08.06.202623</t>
+  </si>
+  <si>
+    <t>08.06.202624</t>
+  </si>
+  <si>
+    <t>09.06.20261</t>
+  </si>
+  <si>
+    <t>09.06.20262</t>
+  </si>
+  <si>
+    <t>09.06.20263</t>
+  </si>
+  <si>
+    <t>09.06.20264</t>
+  </si>
+  <si>
+    <t>09.06.20265</t>
+  </si>
+  <si>
+    <t>09.06.20266</t>
+  </si>
+  <si>
+    <t>09.06.20267</t>
+  </si>
+  <si>
+    <t>09.06.20268</t>
+  </si>
+  <si>
+    <t>09.06.20269</t>
+  </si>
+  <si>
+    <t>09.06.202610</t>
+  </si>
+  <si>
+    <t>09.06.202611</t>
+  </si>
+  <si>
+    <t>09.06.202612</t>
+  </si>
+  <si>
+    <t>09.06.202613</t>
+  </si>
+  <si>
+    <t>09.06.202614</t>
+  </si>
+  <si>
+    <t>09.06.202615</t>
+  </si>
+  <si>
+    <t>09.06.202616</t>
+  </si>
+  <si>
+    <t>09.06.202617</t>
+  </si>
+  <si>
+    <t>09.06.202618</t>
+  </si>
+  <si>
+    <t>09.06.202619</t>
+  </si>
+  <si>
+    <t>09.06.202620</t>
+  </si>
+  <si>
+    <t>09.06.202621</t>
+  </si>
+  <si>
+    <t>09.06.202622</t>
+  </si>
+  <si>
+    <t>09.06.202623</t>
+  </si>
+  <si>
+    <t>09.06.202624</t>
+  </si>
+  <si>
+    <t>10.06.20261</t>
+  </si>
+  <si>
+    <t>10.06.20262</t>
+  </si>
+  <si>
+    <t>10.06.20263</t>
+  </si>
+  <si>
+    <t>10.06.20264</t>
+  </si>
+  <si>
+    <t>10.06.20265</t>
+  </si>
+  <si>
+    <t>10.06.20266</t>
+  </si>
+  <si>
+    <t>10.06.20267</t>
+  </si>
+  <si>
+    <t>10.06.20268</t>
+  </si>
+  <si>
+    <t>10.06.20269</t>
+  </si>
+  <si>
+    <t>10.06.202610</t>
+  </si>
+  <si>
+    <t>10.06.202611</t>
+  </si>
+  <si>
+    <t>10.06.202612</t>
+  </si>
+  <si>
+    <t>10.06.202613</t>
+  </si>
+  <si>
+    <t>10.06.202614</t>
+  </si>
+  <si>
+    <t>10.06.202615</t>
+  </si>
+  <si>
+    <t>10.06.202616</t>
+  </si>
+  <si>
+    <t>10.06.202617</t>
+  </si>
+  <si>
+    <t>10.06.202618</t>
+  </si>
+  <si>
+    <t>10.06.202619</t>
+  </si>
+  <si>
+    <t>10.06.202620</t>
+  </si>
+  <si>
+    <t>10.06.202621</t>
+  </si>
+  <si>
+    <t>10.06.202622</t>
+  </si>
+  <si>
+    <t>10.06.202623</t>
+  </si>
+  <si>
+    <t>10.06.202624</t>
+  </si>
+  <si>
+    <t>11.06.20261</t>
+  </si>
+  <si>
+    <t>11.06.20262</t>
+  </si>
+  <si>
+    <t>11.06.20263</t>
+  </si>
+  <si>
+    <t>11.06.20264</t>
+  </si>
+  <si>
+    <t>11.06.20265</t>
+  </si>
+  <si>
+    <t>11.06.20266</t>
+  </si>
+  <si>
+    <t>11.06.20267</t>
+  </si>
+  <si>
+    <t>11.06.20268</t>
+  </si>
+  <si>
+    <t>11.06.20269</t>
+  </si>
+  <si>
+    <t>11.06.202610</t>
+  </si>
+  <si>
+    <t>11.06.202611</t>
+  </si>
+  <si>
+    <t>11.06.202612</t>
+  </si>
+  <si>
+    <t>11.06.202613</t>
+  </si>
+  <si>
+    <t>11.06.202614</t>
+  </si>
+  <si>
+    <t>11.06.202615</t>
+  </si>
+  <si>
+    <t>11.06.202616</t>
   </si>
 </sst>
 </file>
@@ -913,10 +913,10 @@
     </row>
     <row r="2" spans="1:4">
       <c r="A2" s="2">
-        <v>46173</v>
+        <v>46177</v>
       </c>
       <c r="B2">
-        <v>10</v>
+        <v>16</v>
       </c>
       <c r="C2">
         <v>0</v>
@@ -927,10 +927,10 @@
     </row>
     <row r="3" spans="1:4">
       <c r="A3" s="2">
-        <v>46173</v>
+        <v>46177</v>
       </c>
       <c r="B3">
-        <v>11</v>
+        <v>17</v>
       </c>
       <c r="C3">
         <v>0</v>
@@ -941,13 +941,13 @@
     </row>
     <row r="4" spans="1:4">
       <c r="A4" s="2">
-        <v>46173</v>
+        <v>46177</v>
       </c>
       <c r="B4">
-        <v>12</v>
+        <v>18</v>
       </c>
       <c r="C4">
-        <v>2.055</v>
+        <v>1.326</v>
       </c>
       <c r="D4" t="s">
         <v>6</v>
@@ -955,13 +955,13 @@
     </row>
     <row r="5" spans="1:4">
       <c r="A5" s="2">
-        <v>46173</v>
+        <v>46177</v>
       </c>
       <c r="B5">
-        <v>13</v>
+        <v>19</v>
       </c>
       <c r="C5">
-        <v>2.39</v>
+        <v>0.514</v>
       </c>
       <c r="D5" t="s">
         <v>7</v>
@@ -969,13 +969,13 @@
     </row>
     <row r="6" spans="1:4">
       <c r="A6" s="2">
-        <v>46173</v>
+        <v>46177</v>
       </c>
       <c r="B6">
-        <v>14</v>
+        <v>20</v>
       </c>
       <c r="C6">
-        <v>2.833</v>
+        <v>0.239</v>
       </c>
       <c r="D6" t="s">
         <v>8</v>
@@ -983,13 +983,13 @@
     </row>
     <row r="7" spans="1:4">
       <c r="A7" s="2">
-        <v>46173</v>
+        <v>46177</v>
       </c>
       <c r="B7">
-        <v>15</v>
+        <v>21</v>
       </c>
       <c r="C7">
-        <v>2.705</v>
+        <v>0.05</v>
       </c>
       <c r="D7" t="s">
         <v>9</v>
@@ -997,13 +997,13 @@
     </row>
     <row r="8" spans="1:4">
       <c r="A8" s="2">
-        <v>46173</v>
+        <v>46177</v>
       </c>
       <c r="B8">
-        <v>16</v>
+        <v>22</v>
       </c>
       <c r="C8">
-        <v>2.305</v>
+        <v>0</v>
       </c>
       <c r="D8" t="s">
         <v>10</v>
@@ -1011,13 +1011,13 @@
     </row>
     <row r="9" spans="1:4">
       <c r="A9" s="2">
-        <v>46173</v>
+        <v>46177</v>
       </c>
       <c r="B9">
-        <v>17</v>
+        <v>23</v>
       </c>
       <c r="C9">
-        <v>1.945</v>
+        <v>0</v>
       </c>
       <c r="D9" t="s">
         <v>11</v>
@@ -1025,13 +1025,13 @@
     </row>
     <row r="10" spans="1:4">
       <c r="A10" s="2">
-        <v>46173</v>
+        <v>46177</v>
       </c>
       <c r="B10">
-        <v>18</v>
+        <v>24</v>
       </c>
       <c r="C10">
-        <v>1.419</v>
+        <v>0</v>
       </c>
       <c r="D10" t="s">
         <v>12</v>
@@ -1039,13 +1039,13 @@
     </row>
     <row r="11" spans="1:4">
       <c r="A11" s="2">
-        <v>46173</v>
+        <v>46178</v>
       </c>
       <c r="B11">
-        <v>19</v>
+        <v>1</v>
       </c>
       <c r="C11">
-        <v>0.8159999999999999</v>
+        <v>0</v>
       </c>
       <c r="D11" t="s">
         <v>13</v>
@@ -1053,13 +1053,13 @@
     </row>
     <row r="12" spans="1:4">
       <c r="A12" s="2">
-        <v>46173</v>
+        <v>46178</v>
       </c>
       <c r="B12">
-        <v>20</v>
+        <v>2</v>
       </c>
       <c r="C12">
-        <v>0.282</v>
+        <v>0</v>
       </c>
       <c r="D12" t="s">
         <v>14</v>
@@ -1067,13 +1067,13 @@
     </row>
     <row r="13" spans="1:4">
       <c r="A13" s="2">
-        <v>46173</v>
+        <v>46178</v>
       </c>
       <c r="B13">
-        <v>21</v>
+        <v>3</v>
       </c>
       <c r="C13">
-        <v>0.057</v>
+        <v>0</v>
       </c>
       <c r="D13" t="s">
         <v>15</v>
@@ -1081,10 +1081,10 @@
     </row>
     <row r="14" spans="1:4">
       <c r="A14" s="2">
-        <v>46173</v>
+        <v>46178</v>
       </c>
       <c r="B14">
-        <v>22</v>
+        <v>4</v>
       </c>
       <c r="C14">
         <v>0</v>
@@ -1095,10 +1095,10 @@
     </row>
     <row r="15" spans="1:4">
       <c r="A15" s="2">
-        <v>46173</v>
+        <v>46178</v>
       </c>
       <c r="B15">
-        <v>23</v>
+        <v>5</v>
       </c>
       <c r="C15">
         <v>0</v>
@@ -1109,10 +1109,10 @@
     </row>
     <row r="16" spans="1:4">
       <c r="A16" s="2">
-        <v>46173</v>
+        <v>46178</v>
       </c>
       <c r="B16">
-        <v>24</v>
+        <v>6</v>
       </c>
       <c r="C16">
         <v>0</v>
@@ -1123,13 +1123,13 @@
     </row>
     <row r="17" spans="1:4">
       <c r="A17" s="2">
-        <v>46174</v>
+        <v>46178</v>
       </c>
       <c r="B17">
-        <v>1</v>
+        <v>7</v>
       </c>
       <c r="C17">
-        <v>0</v>
+        <v>0.091</v>
       </c>
       <c r="D17" t="s">
         <v>19</v>
@@ -1137,13 +1137,13 @@
     </row>
     <row r="18" spans="1:4">
       <c r="A18" s="2">
-        <v>46174</v>
+        <v>46178</v>
       </c>
       <c r="B18">
-        <v>2</v>
+        <v>8</v>
       </c>
       <c r="C18">
-        <v>0</v>
+        <v>0.398</v>
       </c>
       <c r="D18" t="s">
         <v>20</v>
@@ -1151,13 +1151,13 @@
     </row>
     <row r="19" spans="1:4">
       <c r="A19" s="2">
-        <v>46174</v>
+        <v>46178</v>
       </c>
       <c r="B19">
-        <v>3</v>
+        <v>9</v>
       </c>
       <c r="C19">
-        <v>0</v>
+        <v>0.832</v>
       </c>
       <c r="D19" t="s">
         <v>21</v>
@@ -1165,13 +1165,13 @@
     </row>
     <row r="20" spans="1:4">
       <c r="A20" s="2">
-        <v>46174</v>
+        <v>46178</v>
       </c>
       <c r="B20">
-        <v>4</v>
+        <v>10</v>
       </c>
       <c r="C20">
-        <v>0</v>
+        <v>1.493</v>
       </c>
       <c r="D20" t="s">
         <v>22</v>
@@ -1179,13 +1179,13 @@
     </row>
     <row r="21" spans="1:4">
       <c r="A21" s="2">
-        <v>46174</v>
+        <v>46178</v>
       </c>
       <c r="B21">
-        <v>5</v>
+        <v>11</v>
       </c>
       <c r="C21">
-        <v>0</v>
+        <v>1.924</v>
       </c>
       <c r="D21" t="s">
         <v>23</v>
@@ -1193,13 +1193,13 @@
     </row>
     <row r="22" spans="1:4">
       <c r="A22" s="2">
-        <v>46174</v>
+        <v>46178</v>
       </c>
       <c r="B22">
-        <v>6</v>
+        <v>12</v>
       </c>
       <c r="C22">
-        <v>0</v>
+        <v>2.421</v>
       </c>
       <c r="D22" t="s">
         <v>24</v>
@@ -1207,13 +1207,13 @@
     </row>
     <row r="23" spans="1:4">
       <c r="A23" s="2">
-        <v>46174</v>
+        <v>46178</v>
       </c>
       <c r="B23">
-        <v>7</v>
+        <v>13</v>
       </c>
       <c r="C23">
-        <v>0.068</v>
+        <v>2.591</v>
       </c>
       <c r="D23" t="s">
         <v>25</v>
@@ -1221,13 +1221,13 @@
     </row>
     <row r="24" spans="1:4">
       <c r="A24" s="2">
-        <v>46174</v>
+        <v>46178</v>
       </c>
       <c r="B24">
-        <v>8</v>
+        <v>14</v>
       </c>
       <c r="C24">
-        <v>0.283</v>
+        <v>2.638</v>
       </c>
       <c r="D24" t="s">
         <v>26</v>
@@ -1235,13 +1235,13 @@
     </row>
     <row r="25" spans="1:4">
       <c r="A25" s="2">
-        <v>46174</v>
+        <v>46178</v>
       </c>
       <c r="B25">
-        <v>9</v>
+        <v>15</v>
       </c>
       <c r="C25">
-        <v>0.642</v>
+        <v>2.459</v>
       </c>
       <c r="D25" t="s">
         <v>27</v>
@@ -1249,13 +1249,13 @@
     </row>
     <row r="26" spans="1:4">
       <c r="A26" s="2">
-        <v>46174</v>
+        <v>46178</v>
       </c>
       <c r="B26">
-        <v>10</v>
+        <v>16</v>
       </c>
       <c r="C26">
-        <v>0.744</v>
+        <v>1.983</v>
       </c>
       <c r="D26" t="s">
         <v>28</v>
@@ -1263,13 +1263,13 @@
     </row>
     <row r="27" spans="1:4">
       <c r="A27" s="2">
-        <v>46174</v>
+        <v>46178</v>
       </c>
       <c r="B27">
-        <v>11</v>
+        <v>17</v>
       </c>
       <c r="C27">
-        <v>0.853</v>
+        <v>1.579</v>
       </c>
       <c r="D27" t="s">
         <v>29</v>
@@ -1277,13 +1277,13 @@
     </row>
     <row r="28" spans="1:4">
       <c r="A28" s="2">
-        <v>46174</v>
+        <v>46178</v>
       </c>
       <c r="B28">
-        <v>12</v>
+        <v>18</v>
       </c>
       <c r="C28">
-        <v>0.792</v>
+        <v>1.061</v>
       </c>
       <c r="D28" t="s">
         <v>30</v>
@@ -1291,13 +1291,13 @@
     </row>
     <row r="29" spans="1:4">
       <c r="A29" s="2">
-        <v>46174</v>
+        <v>46178</v>
       </c>
       <c r="B29">
-        <v>13</v>
+        <v>19</v>
       </c>
       <c r="C29">
-        <v>0.742</v>
+        <v>0.588</v>
       </c>
       <c r="D29" t="s">
         <v>31</v>
@@ -1305,13 +1305,13 @@
     </row>
     <row r="30" spans="1:4">
       <c r="A30" s="2">
-        <v>46174</v>
+        <v>46178</v>
       </c>
       <c r="B30">
-        <v>14</v>
+        <v>20</v>
       </c>
       <c r="C30">
-        <v>0.705</v>
+        <v>0.266</v>
       </c>
       <c r="D30" t="s">
         <v>32</v>
@@ -1319,13 +1319,13 @@
     </row>
     <row r="31" spans="1:4">
       <c r="A31" s="2">
-        <v>46174</v>
+        <v>46178</v>
       </c>
       <c r="B31">
-        <v>15</v>
+        <v>21</v>
       </c>
       <c r="C31">
-        <v>0.673</v>
+        <v>0.055</v>
       </c>
       <c r="D31" t="s">
         <v>33</v>
@@ -1333,13 +1333,13 @@
     </row>
     <row r="32" spans="1:4">
       <c r="A32" s="2">
-        <v>46174</v>
+        <v>46178</v>
       </c>
       <c r="B32">
-        <v>16</v>
+        <v>22</v>
       </c>
       <c r="C32">
-        <v>0.5600000000000001</v>
+        <v>0</v>
       </c>
       <c r="D32" t="s">
         <v>34</v>
@@ -1347,13 +1347,13 @@
     </row>
     <row r="33" spans="1:4">
       <c r="A33" s="2">
-        <v>46174</v>
+        <v>46178</v>
       </c>
       <c r="B33">
-        <v>17</v>
+        <v>23</v>
       </c>
       <c r="C33">
-        <v>0.466</v>
+        <v>0</v>
       </c>
       <c r="D33" t="s">
         <v>35</v>
@@ -1361,13 +1361,13 @@
     </row>
     <row r="34" spans="1:4">
       <c r="A34" s="2">
-        <v>46174</v>
+        <v>46178</v>
       </c>
       <c r="B34">
-        <v>18</v>
+        <v>24</v>
       </c>
       <c r="C34">
-        <v>0.348</v>
+        <v>0</v>
       </c>
       <c r="D34" t="s">
         <v>36</v>
@@ -1375,13 +1375,13 @@
     </row>
     <row r="35" spans="1:4">
       <c r="A35" s="2">
-        <v>46174</v>
+        <v>46179</v>
       </c>
       <c r="B35">
-        <v>19</v>
+        <v>1</v>
       </c>
       <c r="C35">
-        <v>0.152</v>
+        <v>0</v>
       </c>
       <c r="D35" t="s">
         <v>37</v>
@@ -1389,13 +1389,13 @@
     </row>
     <row r="36" spans="1:4">
       <c r="A36" s="2">
-        <v>46174</v>
+        <v>46179</v>
       </c>
       <c r="B36">
-        <v>20</v>
+        <v>2</v>
       </c>
       <c r="C36">
-        <v>0.063</v>
+        <v>0</v>
       </c>
       <c r="D36" t="s">
         <v>38</v>
@@ -1403,10 +1403,10 @@
     </row>
     <row r="37" spans="1:4">
       <c r="A37" s="2">
-        <v>46174</v>
+        <v>46179</v>
       </c>
       <c r="B37">
-        <v>21</v>
+        <v>3</v>
       </c>
       <c r="C37">
         <v>0</v>
@@ -1417,10 +1417,10 @@
     </row>
     <row r="38" spans="1:4">
       <c r="A38" s="2">
-        <v>46174</v>
+        <v>46179</v>
       </c>
       <c r="B38">
-        <v>22</v>
+        <v>4</v>
       </c>
       <c r="C38">
         <v>0</v>
@@ -1431,10 +1431,10 @@
     </row>
     <row r="39" spans="1:4">
       <c r="A39" s="2">
-        <v>46174</v>
+        <v>46179</v>
       </c>
       <c r="B39">
-        <v>23</v>
+        <v>5</v>
       </c>
       <c r="C39">
         <v>0</v>
@@ -1445,10 +1445,10 @@
     </row>
     <row r="40" spans="1:4">
       <c r="A40" s="2">
-        <v>46174</v>
+        <v>46179</v>
       </c>
       <c r="B40">
-        <v>24</v>
+        <v>6</v>
       </c>
       <c r="C40">
         <v>0</v>
@@ -1459,13 +1459,13 @@
     </row>
     <row r="41" spans="1:4">
       <c r="A41" s="2">
-        <v>46175</v>
+        <v>46179</v>
       </c>
       <c r="B41">
-        <v>1</v>
+        <v>7</v>
       </c>
       <c r="C41">
-        <v>0</v>
+        <v>0.07199999999999999</v>
       </c>
       <c r="D41" t="s">
         <v>43</v>
@@ -1473,13 +1473,13 @@
     </row>
     <row r="42" spans="1:4">
       <c r="A42" s="2">
-        <v>46175</v>
+        <v>46179</v>
       </c>
       <c r="B42">
-        <v>2</v>
+        <v>8</v>
       </c>
       <c r="C42">
-        <v>0</v>
+        <v>0.405</v>
       </c>
       <c r="D42" t="s">
         <v>44</v>
@@ -1487,13 +1487,13 @@
     </row>
     <row r="43" spans="1:4">
       <c r="A43" s="2">
-        <v>46175</v>
+        <v>46179</v>
       </c>
       <c r="B43">
-        <v>3</v>
+        <v>9</v>
       </c>
       <c r="C43">
-        <v>0</v>
+        <v>0.838</v>
       </c>
       <c r="D43" t="s">
         <v>45</v>
@@ -1501,13 +1501,13 @@
     </row>
     <row r="44" spans="1:4">
       <c r="A44" s="2">
-        <v>46175</v>
+        <v>46179</v>
       </c>
       <c r="B44">
-        <v>4</v>
+        <v>10</v>
       </c>
       <c r="C44">
-        <v>0</v>
+        <v>1.228</v>
       </c>
       <c r="D44" t="s">
         <v>46</v>
@@ -1515,13 +1515,13 @@
     </row>
     <row r="45" spans="1:4">
       <c r="A45" s="2">
-        <v>46175</v>
+        <v>46179</v>
       </c>
       <c r="B45">
-        <v>5</v>
+        <v>11</v>
       </c>
       <c r="C45">
-        <v>0</v>
+        <v>1.563</v>
       </c>
       <c r="D45" t="s">
         <v>47</v>
@@ -1529,13 +1529,13 @@
     </row>
     <row r="46" spans="1:4">
       <c r="A46" s="2">
-        <v>46175</v>
+        <v>46179</v>
       </c>
       <c r="B46">
-        <v>6</v>
+        <v>12</v>
       </c>
       <c r="C46">
-        <v>0</v>
+        <v>1.729</v>
       </c>
       <c r="D46" t="s">
         <v>48</v>
@@ -1543,13 +1543,13 @@
     </row>
     <row r="47" spans="1:4">
       <c r="A47" s="2">
-        <v>46175</v>
+        <v>46179</v>
       </c>
       <c r="B47">
-        <v>7</v>
+        <v>13</v>
       </c>
       <c r="C47">
-        <v>0.05</v>
+        <v>1.827</v>
       </c>
       <c r="D47" t="s">
         <v>49</v>
@@ -1557,13 +1557,13 @@
     </row>
     <row r="48" spans="1:4">
       <c r="A48" s="2">
-        <v>46175</v>
+        <v>46179</v>
       </c>
       <c r="B48">
-        <v>8</v>
+        <v>14</v>
       </c>
       <c r="C48">
-        <v>0.19</v>
+        <v>2.067</v>
       </c>
       <c r="D48" t="s">
         <v>50</v>
@@ -1571,13 +1571,13 @@
     </row>
     <row r="49" spans="1:4">
       <c r="A49" s="2">
-        <v>46175</v>
+        <v>46179</v>
       </c>
       <c r="B49">
-        <v>9</v>
+        <v>15</v>
       </c>
       <c r="C49">
-        <v>0.386</v>
+        <v>2.205</v>
       </c>
       <c r="D49" t="s">
         <v>51</v>
@@ -1585,13 +1585,13 @@
     </row>
     <row r="50" spans="1:4">
       <c r="A50" s="2">
-        <v>46175</v>
+        <v>46179</v>
       </c>
       <c r="B50">
-        <v>10</v>
+        <v>16</v>
       </c>
       <c r="C50">
-        <v>0.732</v>
+        <v>1.911</v>
       </c>
       <c r="D50" t="s">
         <v>52</v>
@@ -1599,13 +1599,13 @@
     </row>
     <row r="51" spans="1:4">
       <c r="A51" s="2">
-        <v>46175</v>
+        <v>46179</v>
       </c>
       <c r="B51">
-        <v>11</v>
+        <v>17</v>
       </c>
       <c r="C51">
-        <v>1.102</v>
+        <v>1.601</v>
       </c>
       <c r="D51" t="s">
         <v>53</v>
@@ -1613,13 +1613,13 @@
     </row>
     <row r="52" spans="1:4">
       <c r="A52" s="2">
-        <v>46175</v>
+        <v>46179</v>
       </c>
       <c r="B52">
-        <v>12</v>
+        <v>18</v>
       </c>
       <c r="C52">
-        <v>1.205</v>
+        <v>1.093</v>
       </c>
       <c r="D52" t="s">
         <v>54</v>
@@ -1627,13 +1627,13 @@
     </row>
     <row r="53" spans="1:4">
       <c r="A53" s="2">
-        <v>46175</v>
+        <v>46179</v>
       </c>
       <c r="B53">
-        <v>13</v>
+        <v>19</v>
       </c>
       <c r="C53">
-        <v>1.319</v>
+        <v>0.618</v>
       </c>
       <c r="D53" t="s">
         <v>55</v>
@@ -1641,13 +1641,13 @@
     </row>
     <row r="54" spans="1:4">
       <c r="A54" s="2">
-        <v>46175</v>
+        <v>46179</v>
       </c>
       <c r="B54">
-        <v>14</v>
+        <v>20</v>
       </c>
       <c r="C54">
-        <v>1.291</v>
+        <v>0.297</v>
       </c>
       <c r="D54" t="s">
         <v>56</v>
@@ -1655,13 +1655,13 @@
     </row>
     <row r="55" spans="1:4">
       <c r="A55" s="2">
-        <v>46175</v>
+        <v>46179</v>
       </c>
       <c r="B55">
-        <v>15</v>
+        <v>21</v>
       </c>
       <c r="C55">
-        <v>1.193</v>
+        <v>0.056</v>
       </c>
       <c r="D55" t="s">
         <v>57</v>
@@ -1669,13 +1669,13 @@
     </row>
     <row r="56" spans="1:4">
       <c r="A56" s="2">
-        <v>46175</v>
+        <v>46179</v>
       </c>
       <c r="B56">
-        <v>16</v>
+        <v>22</v>
       </c>
       <c r="C56">
-        <v>0.913</v>
+        <v>0</v>
       </c>
       <c r="D56" t="s">
         <v>58</v>
@@ -1683,13 +1683,13 @@
     </row>
     <row r="57" spans="1:4">
       <c r="A57" s="2">
-        <v>46175</v>
+        <v>46179</v>
       </c>
       <c r="B57">
-        <v>17</v>
+        <v>23</v>
       </c>
       <c r="C57">
-        <v>1.028</v>
+        <v>0</v>
       </c>
       <c r="D57" t="s">
         <v>59</v>
@@ -1697,13 +1697,13 @@
     </row>
     <row r="58" spans="1:4">
       <c r="A58" s="2">
-        <v>46175</v>
+        <v>46179</v>
       </c>
       <c r="B58">
-        <v>18</v>
+        <v>24</v>
       </c>
       <c r="C58">
-        <v>0.8110000000000001</v>
+        <v>0</v>
       </c>
       <c r="D58" t="s">
         <v>60</v>
@@ -1711,13 +1711,13 @@
     </row>
     <row r="59" spans="1:4">
       <c r="A59" s="2">
-        <v>46175</v>
+        <v>46180</v>
       </c>
       <c r="B59">
-        <v>19</v>
+        <v>1</v>
       </c>
       <c r="C59">
-        <v>0.421</v>
+        <v>0</v>
       </c>
       <c r="D59" t="s">
         <v>61</v>
@@ -1725,13 +1725,13 @@
     </row>
     <row r="60" spans="1:4">
       <c r="A60" s="2">
-        <v>46175</v>
+        <v>46180</v>
       </c>
       <c r="B60">
-        <v>20</v>
+        <v>2</v>
       </c>
       <c r="C60">
-        <v>0.224</v>
+        <v>0</v>
       </c>
       <c r="D60" t="s">
         <v>62</v>
@@ -1739,13 +1739,13 @@
     </row>
     <row r="61" spans="1:4">
       <c r="A61" s="2">
-        <v>46175</v>
+        <v>46180</v>
       </c>
       <c r="B61">
-        <v>21</v>
+        <v>3</v>
       </c>
       <c r="C61">
-        <v>0.043</v>
+        <v>0</v>
       </c>
       <c r="D61" t="s">
         <v>63</v>
@@ -1753,10 +1753,10 @@
     </row>
     <row r="62" spans="1:4">
       <c r="A62" s="2">
-        <v>46175</v>
+        <v>46180</v>
       </c>
       <c r="B62">
-        <v>22</v>
+        <v>4</v>
       </c>
       <c r="C62">
         <v>0</v>
@@ -1767,10 +1767,10 @@
     </row>
     <row r="63" spans="1:4">
       <c r="A63" s="2">
-        <v>46175</v>
+        <v>46180</v>
       </c>
       <c r="B63">
-        <v>23</v>
+        <v>5</v>
       </c>
       <c r="C63">
         <v>0</v>
@@ -1781,10 +1781,10 @@
     </row>
     <row r="64" spans="1:4">
       <c r="A64" s="2">
-        <v>46175</v>
+        <v>46180</v>
       </c>
       <c r="B64">
-        <v>24</v>
+        <v>6</v>
       </c>
       <c r="C64">
         <v>0</v>
@@ -1795,13 +1795,13 @@
     </row>
     <row r="65" spans="1:4">
       <c r="A65" s="2">
-        <v>46176</v>
+        <v>46180</v>
       </c>
       <c r="B65">
-        <v>1</v>
+        <v>7</v>
       </c>
       <c r="C65">
-        <v>0</v>
+        <v>0.061</v>
       </c>
       <c r="D65" t="s">
         <v>67</v>
@@ -1809,13 +1809,13 @@
     </row>
     <row r="66" spans="1:4">
       <c r="A66" s="2">
-        <v>46176</v>
+        <v>46180</v>
       </c>
       <c r="B66">
-        <v>2</v>
+        <v>8</v>
       </c>
       <c r="C66">
-        <v>0</v>
+        <v>0.236</v>
       </c>
       <c r="D66" t="s">
         <v>68</v>
@@ -1823,13 +1823,13 @@
     </row>
     <row r="67" spans="1:4">
       <c r="A67" s="2">
-        <v>46176</v>
+        <v>46180</v>
       </c>
       <c r="B67">
-        <v>3</v>
+        <v>9</v>
       </c>
       <c r="C67">
-        <v>0</v>
+        <v>0.704</v>
       </c>
       <c r="D67" t="s">
         <v>69</v>
@@ -1837,13 +1837,13 @@
     </row>
     <row r="68" spans="1:4">
       <c r="A68" s="2">
-        <v>46176</v>
+        <v>46180</v>
       </c>
       <c r="B68">
-        <v>4</v>
+        <v>10</v>
       </c>
       <c r="C68">
-        <v>0</v>
+        <v>0.962</v>
       </c>
       <c r="D68" t="s">
         <v>70</v>
@@ -1851,13 +1851,13 @@
     </row>
     <row r="69" spans="1:4">
       <c r="A69" s="2">
-        <v>46176</v>
+        <v>46180</v>
       </c>
       <c r="B69">
-        <v>5</v>
+        <v>11</v>
       </c>
       <c r="C69">
-        <v>0</v>
+        <v>1.575</v>
       </c>
       <c r="D69" t="s">
         <v>71</v>
@@ -1865,13 +1865,13 @@
     </row>
     <row r="70" spans="1:4">
       <c r="A70" s="2">
-        <v>46176</v>
+        <v>46180</v>
       </c>
       <c r="B70">
-        <v>6</v>
+        <v>12</v>
       </c>
       <c r="C70">
-        <v>0</v>
+        <v>2.076</v>
       </c>
       <c r="D70" t="s">
         <v>72</v>
@@ -1879,13 +1879,13 @@
     </row>
     <row r="71" spans="1:4">
       <c r="A71" s="2">
-        <v>46176</v>
+        <v>46180</v>
       </c>
       <c r="B71">
-        <v>7</v>
+        <v>13</v>
       </c>
       <c r="C71">
-        <v>0.091</v>
+        <v>2.492</v>
       </c>
       <c r="D71" t="s">
         <v>73</v>
@@ -1893,13 +1893,13 @@
     </row>
     <row r="72" spans="1:4">
       <c r="A72" s="2">
-        <v>46176</v>
+        <v>46180</v>
       </c>
       <c r="B72">
-        <v>8</v>
+        <v>14</v>
       </c>
       <c r="C72">
-        <v>0.405</v>
+        <v>2.809</v>
       </c>
       <c r="D72" t="s">
         <v>74</v>
@@ -1907,13 +1907,13 @@
     </row>
     <row r="73" spans="1:4">
       <c r="A73" s="2">
-        <v>46176</v>
+        <v>46180</v>
       </c>
       <c r="B73">
-        <v>9</v>
+        <v>15</v>
       </c>
       <c r="C73">
-        <v>0.98</v>
+        <v>2.698</v>
       </c>
       <c r="D73" t="s">
         <v>75</v>
@@ -1921,13 +1921,13 @@
     </row>
     <row r="74" spans="1:4">
       <c r="A74" s="2">
-        <v>46176</v>
+        <v>46180</v>
       </c>
       <c r="B74">
-        <v>10</v>
+        <v>16</v>
       </c>
       <c r="C74">
-        <v>1.532</v>
+        <v>2.282</v>
       </c>
       <c r="D74" t="s">
         <v>76</v>
@@ -1935,13 +1935,13 @@
     </row>
     <row r="75" spans="1:4">
       <c r="A75" s="2">
-        <v>46176</v>
+        <v>46180</v>
       </c>
       <c r="B75">
-        <v>11</v>
+        <v>17</v>
       </c>
       <c r="C75">
-        <v>2.061</v>
+        <v>1.94</v>
       </c>
       <c r="D75" t="s">
         <v>77</v>
@@ -1949,13 +1949,13 @@
     </row>
     <row r="76" spans="1:4">
       <c r="A76" s="2">
-        <v>46176</v>
+        <v>46180</v>
       </c>
       <c r="B76">
-        <v>12</v>
+        <v>18</v>
       </c>
       <c r="C76">
-        <v>2.462</v>
+        <v>1.339</v>
       </c>
       <c r="D76" t="s">
         <v>78</v>
@@ -1963,13 +1963,13 @@
     </row>
     <row r="77" spans="1:4">
       <c r="A77" s="2">
-        <v>46176</v>
+        <v>46180</v>
       </c>
       <c r="B77">
-        <v>13</v>
+        <v>19</v>
       </c>
       <c r="C77">
-        <v>2.819</v>
+        <v>0.862</v>
       </c>
       <c r="D77" t="s">
         <v>79</v>
@@ -1977,13 +1977,13 @@
     </row>
     <row r="78" spans="1:4">
       <c r="A78" s="2">
-        <v>46176</v>
+        <v>46180</v>
       </c>
       <c r="B78">
-        <v>14</v>
+        <v>20</v>
       </c>
       <c r="C78">
-        <v>2.875</v>
+        <v>0.276</v>
       </c>
       <c r="D78" t="s">
         <v>80</v>
@@ -1991,13 +1991,13 @@
     </row>
     <row r="79" spans="1:4">
       <c r="A79" s="2">
-        <v>46176</v>
+        <v>46180</v>
       </c>
       <c r="B79">
-        <v>15</v>
+        <v>21</v>
       </c>
       <c r="C79">
-        <v>2.691</v>
+        <v>0.076</v>
       </c>
       <c r="D79" t="s">
         <v>81</v>
@@ -2005,13 +2005,13 @@
     </row>
     <row r="80" spans="1:4">
       <c r="A80" s="2">
-        <v>46176</v>
+        <v>46180</v>
       </c>
       <c r="B80">
-        <v>16</v>
+        <v>22</v>
       </c>
       <c r="C80">
-        <v>2.326</v>
+        <v>0</v>
       </c>
       <c r="D80" t="s">
         <v>82</v>
@@ -2019,13 +2019,13 @@
     </row>
     <row r="81" spans="1:4">
       <c r="A81" s="2">
-        <v>46176</v>
+        <v>46180</v>
       </c>
       <c r="B81">
-        <v>17</v>
+        <v>23</v>
       </c>
       <c r="C81">
-        <v>1.916</v>
+        <v>0</v>
       </c>
       <c r="D81" t="s">
         <v>83</v>
@@ -2033,13 +2033,13 @@
     </row>
     <row r="82" spans="1:4">
       <c r="A82" s="2">
-        <v>46176</v>
+        <v>46180</v>
       </c>
       <c r="B82">
-        <v>18</v>
+        <v>24</v>
       </c>
       <c r="C82">
-        <v>1.398</v>
+        <v>0</v>
       </c>
       <c r="D82" t="s">
         <v>84</v>
@@ -2047,13 +2047,13 @@
     </row>
     <row r="83" spans="1:4">
       <c r="A83" s="2">
-        <v>46176</v>
+        <v>46181</v>
       </c>
       <c r="B83">
-        <v>19</v>
+        <v>1</v>
       </c>
       <c r="C83">
-        <v>0.822</v>
+        <v>0</v>
       </c>
       <c r="D83" t="s">
         <v>85</v>
@@ -2061,13 +2061,13 @@
     </row>
     <row r="84" spans="1:4">
       <c r="A84" s="2">
-        <v>46176</v>
+        <v>46181</v>
       </c>
       <c r="B84">
-        <v>20</v>
+        <v>2</v>
       </c>
       <c r="C84">
-        <v>0.344</v>
+        <v>0</v>
       </c>
       <c r="D84" t="s">
         <v>86</v>
@@ -2075,13 +2075,13 @@
     </row>
     <row r="85" spans="1:4">
       <c r="A85" s="2">
-        <v>46176</v>
+        <v>46181</v>
       </c>
       <c r="B85">
-        <v>21</v>
+        <v>3</v>
       </c>
       <c r="C85">
-        <v>0.056</v>
+        <v>0</v>
       </c>
       <c r="D85" t="s">
         <v>87</v>
@@ -2089,10 +2089,10 @@
     </row>
     <row r="86" spans="1:4">
       <c r="A86" s="2">
-        <v>46176</v>
+        <v>46181</v>
       </c>
       <c r="B86">
-        <v>22</v>
+        <v>4</v>
       </c>
       <c r="C86">
         <v>0</v>
@@ -2103,10 +2103,10 @@
     </row>
     <row r="87" spans="1:4">
       <c r="A87" s="2">
-        <v>46176</v>
+        <v>46181</v>
       </c>
       <c r="B87">
-        <v>23</v>
+        <v>5</v>
       </c>
       <c r="C87">
         <v>0</v>
@@ -2117,10 +2117,10 @@
     </row>
     <row r="88" spans="1:4">
       <c r="A88" s="2">
-        <v>46176</v>
+        <v>46181</v>
       </c>
       <c r="B88">
-        <v>24</v>
+        <v>6</v>
       </c>
       <c r="C88">
         <v>0</v>
@@ -2131,13 +2131,13 @@
     </row>
     <row r="89" spans="1:4">
       <c r="A89" s="2">
-        <v>46177</v>
+        <v>46181</v>
       </c>
       <c r="B89">
-        <v>1</v>
+        <v>7</v>
       </c>
       <c r="C89">
-        <v>0</v>
+        <v>0.097</v>
       </c>
       <c r="D89" t="s">
         <v>91</v>
@@ -2145,13 +2145,13 @@
     </row>
     <row r="90" spans="1:4">
       <c r="A90" s="2">
-        <v>46177</v>
+        <v>46181</v>
       </c>
       <c r="B90">
-        <v>2</v>
+        <v>8</v>
       </c>
       <c r="C90">
-        <v>0</v>
+        <v>0.521</v>
       </c>
       <c r="D90" t="s">
         <v>92</v>
@@ -2159,13 +2159,13 @@
     </row>
     <row r="91" spans="1:4">
       <c r="A91" s="2">
-        <v>46177</v>
+        <v>46181</v>
       </c>
       <c r="B91">
-        <v>3</v>
+        <v>9</v>
       </c>
       <c r="C91">
-        <v>0</v>
+        <v>1.136</v>
       </c>
       <c r="D91" t="s">
         <v>93</v>
@@ -2173,13 +2173,13 @@
     </row>
     <row r="92" spans="1:4">
       <c r="A92" s="2">
-        <v>46177</v>
+        <v>46181</v>
       </c>
       <c r="B92">
-        <v>4</v>
+        <v>10</v>
       </c>
       <c r="C92">
-        <v>0</v>
+        <v>1.856</v>
       </c>
       <c r="D92" t="s">
         <v>94</v>
@@ -2187,13 +2187,13 @@
     </row>
     <row r="93" spans="1:4">
       <c r="A93" s="2">
-        <v>46177</v>
+        <v>46181</v>
       </c>
       <c r="B93">
-        <v>5</v>
+        <v>11</v>
       </c>
       <c r="C93">
-        <v>0</v>
+        <v>2.417</v>
       </c>
       <c r="D93" t="s">
         <v>95</v>
@@ -2201,13 +2201,13 @@
     </row>
     <row r="94" spans="1:4">
       <c r="A94" s="2">
-        <v>46177</v>
+        <v>46181</v>
       </c>
       <c r="B94">
-        <v>6</v>
+        <v>12</v>
       </c>
       <c r="C94">
-        <v>0</v>
+        <v>2.652</v>
       </c>
       <c r="D94" t="s">
         <v>96</v>
@@ -2215,13 +2215,13 @@
     </row>
     <row r="95" spans="1:4">
       <c r="A95" s="2">
-        <v>46177</v>
+        <v>46181</v>
       </c>
       <c r="B95">
-        <v>7</v>
+        <v>13</v>
       </c>
       <c r="C95">
-        <v>0.105</v>
+        <v>2.971</v>
       </c>
       <c r="D95" t="s">
         <v>97</v>
@@ -2229,13 +2229,13 @@
     </row>
     <row r="96" spans="1:4">
       <c r="A96" s="2">
-        <v>46177</v>
+        <v>46181</v>
       </c>
       <c r="B96">
-        <v>8</v>
+        <v>14</v>
       </c>
       <c r="C96">
-        <v>0.417</v>
+        <v>2.966</v>
       </c>
       <c r="D96" t="s">
         <v>98</v>
@@ -2243,13 +2243,13 @@
     </row>
     <row r="97" spans="1:4">
       <c r="A97" s="2">
-        <v>46177</v>
+        <v>46181</v>
       </c>
       <c r="B97">
-        <v>9</v>
+        <v>15</v>
       </c>
       <c r="C97">
-        <v>0.928</v>
+        <v>2.765</v>
       </c>
       <c r="D97" t="s">
         <v>99</v>
@@ -2257,13 +2257,13 @@
     </row>
     <row r="98" spans="1:4">
       <c r="A98" s="2">
-        <v>46177</v>
+        <v>46181</v>
       </c>
       <c r="B98">
-        <v>10</v>
+        <v>16</v>
       </c>
       <c r="C98">
-        <v>1.543</v>
+        <v>2.368</v>
       </c>
       <c r="D98" t="s">
         <v>100</v>
@@ -2271,13 +2271,13 @@
     </row>
     <row r="99" spans="1:4">
       <c r="A99" s="2">
-        <v>46177</v>
+        <v>46181</v>
       </c>
       <c r="B99">
-        <v>11</v>
+        <v>17</v>
       </c>
       <c r="C99">
-        <v>2.028</v>
+        <v>2.099</v>
       </c>
       <c r="D99" t="s">
         <v>101</v>
@@ -2285,13 +2285,13 @@
     </row>
     <row r="100" spans="1:4">
       <c r="A100" s="2">
-        <v>46177</v>
+        <v>46181</v>
       </c>
       <c r="B100">
-        <v>12</v>
+        <v>18</v>
       </c>
       <c r="C100">
-        <v>2.455</v>
+        <v>1.45</v>
       </c>
       <c r="D100" t="s">
         <v>102</v>
@@ -2299,13 +2299,13 @@
     </row>
     <row r="101" spans="1:4">
       <c r="A101" s="2">
-        <v>46177</v>
+        <v>46181</v>
       </c>
       <c r="B101">
-        <v>13</v>
+        <v>19</v>
       </c>
       <c r="C101">
-        <v>2.47</v>
+        <v>0.8159999999999999</v>
       </c>
       <c r="D101" t="s">
         <v>103</v>
@@ -2313,13 +2313,13 @@
     </row>
     <row r="102" spans="1:4">
       <c r="A102" s="2">
-        <v>46177</v>
+        <v>46181</v>
       </c>
       <c r="B102">
-        <v>14</v>
+        <v>20</v>
       </c>
       <c r="C102">
-        <v>2.442</v>
+        <v>0.313</v>
       </c>
       <c r="D102" t="s">
         <v>104</v>
@@ -2327,13 +2327,13 @@
     </row>
     <row r="103" spans="1:4">
       <c r="A103" s="2">
-        <v>46177</v>
+        <v>46181</v>
       </c>
       <c r="B103">
-        <v>15</v>
+        <v>21</v>
       </c>
       <c r="C103">
-        <v>2.15</v>
+        <v>0.056</v>
       </c>
       <c r="D103" t="s">
         <v>105</v>
@@ -2341,13 +2341,13 @@
     </row>
     <row r="104" spans="1:4">
       <c r="A104" s="2">
-        <v>46177</v>
+        <v>46181</v>
       </c>
       <c r="B104">
-        <v>16</v>
+        <v>22</v>
       </c>
       <c r="C104">
-        <v>1.809</v>
+        <v>0</v>
       </c>
       <c r="D104" t="s">
         <v>106</v>
@@ -2355,13 +2355,13 @@
     </row>
     <row r="105" spans="1:4">
       <c r="A105" s="2">
-        <v>46177</v>
+        <v>46181</v>
       </c>
       <c r="B105">
-        <v>17</v>
+        <v>23</v>
       </c>
       <c r="C105">
-        <v>1.677</v>
+        <v>0</v>
       </c>
       <c r="D105" t="s">
         <v>107</v>
@@ -2369,13 +2369,13 @@
     </row>
     <row r="106" spans="1:4">
       <c r="A106" s="2">
-        <v>46177</v>
+        <v>46181</v>
       </c>
       <c r="B106">
-        <v>18</v>
+        <v>24</v>
       </c>
       <c r="C106">
-        <v>1.124</v>
+        <v>0</v>
       </c>
       <c r="D106" t="s">
         <v>108</v>
@@ -2383,13 +2383,13 @@
     </row>
     <row r="107" spans="1:4">
       <c r="A107" s="2">
-        <v>46177</v>
+        <v>46182</v>
       </c>
       <c r="B107">
-        <v>19</v>
+        <v>1</v>
       </c>
       <c r="C107">
-        <v>0.635</v>
+        <v>0</v>
       </c>
       <c r="D107" t="s">
         <v>109</v>
@@ -2397,13 +2397,13 @@
     </row>
     <row r="108" spans="1:4">
       <c r="A108" s="2">
-        <v>46177</v>
+        <v>46182</v>
       </c>
       <c r="B108">
-        <v>20</v>
+        <v>2</v>
       </c>
       <c r="C108">
-        <v>0.272</v>
+        <v>0</v>
       </c>
       <c r="D108" t="s">
         <v>110</v>
@@ -2411,13 +2411,13 @@
     </row>
     <row r="109" spans="1:4">
       <c r="A109" s="2">
-        <v>46177</v>
+        <v>46182</v>
       </c>
       <c r="B109">
-        <v>21</v>
+        <v>3</v>
       </c>
       <c r="C109">
-        <v>0.046</v>
+        <v>0</v>
       </c>
       <c r="D109" t="s">
         <v>111</v>
@@ -2425,10 +2425,10 @@
     </row>
     <row r="110" spans="1:4">
       <c r="A110" s="2">
-        <v>46177</v>
+        <v>46182</v>
       </c>
       <c r="B110">
-        <v>22</v>
+        <v>4</v>
       </c>
       <c r="C110">
         <v>0</v>
@@ -2439,10 +2439,10 @@
     </row>
     <row r="111" spans="1:4">
       <c r="A111" s="2">
-        <v>46177</v>
+        <v>46182</v>
       </c>
       <c r="B111">
-        <v>23</v>
+        <v>5</v>
       </c>
       <c r="C111">
         <v>0</v>
@@ -2453,10 +2453,10 @@
     </row>
     <row r="112" spans="1:4">
       <c r="A112" s="2">
-        <v>46177</v>
+        <v>46182</v>
       </c>
       <c r="B112">
-        <v>24</v>
+        <v>6</v>
       </c>
       <c r="C112">
         <v>0</v>
@@ -2467,13 +2467,13 @@
     </row>
     <row r="113" spans="1:4">
       <c r="A113" s="2">
-        <v>46178</v>
+        <v>46182</v>
       </c>
       <c r="B113">
-        <v>1</v>
+        <v>7</v>
       </c>
       <c r="C113">
-        <v>0</v>
+        <v>0.08500000000000001</v>
       </c>
       <c r="D113" t="s">
         <v>115</v>
@@ -2481,13 +2481,13 @@
     </row>
     <row r="114" spans="1:4">
       <c r="A114" s="2">
-        <v>46178</v>
+        <v>46182</v>
       </c>
       <c r="B114">
-        <v>2</v>
+        <v>8</v>
       </c>
       <c r="C114">
-        <v>0</v>
+        <v>0.458</v>
       </c>
       <c r="D114" t="s">
         <v>116</v>
@@ -2495,13 +2495,13 @@
     </row>
     <row r="115" spans="1:4">
       <c r="A115" s="2">
-        <v>46178</v>
+        <v>46182</v>
       </c>
       <c r="B115">
-        <v>3</v>
+        <v>9</v>
       </c>
       <c r="C115">
-        <v>0</v>
+        <v>1.129</v>
       </c>
       <c r="D115" t="s">
         <v>117</v>
@@ -2509,13 +2509,13 @@
     </row>
     <row r="116" spans="1:4">
       <c r="A116" s="2">
-        <v>46178</v>
+        <v>46182</v>
       </c>
       <c r="B116">
-        <v>4</v>
+        <v>10</v>
       </c>
       <c r="C116">
-        <v>0</v>
+        <v>1.839</v>
       </c>
       <c r="D116" t="s">
         <v>118</v>
@@ -2523,13 +2523,13 @@
     </row>
     <row r="117" spans="1:4">
       <c r="A117" s="2">
-        <v>46178</v>
+        <v>46182</v>
       </c>
       <c r="B117">
-        <v>5</v>
+        <v>11</v>
       </c>
       <c r="C117">
-        <v>0</v>
+        <v>2.462</v>
       </c>
       <c r="D117" t="s">
         <v>119</v>
@@ -2537,13 +2537,13 @@
     </row>
     <row r="118" spans="1:4">
       <c r="A118" s="2">
-        <v>46178</v>
+        <v>46182</v>
       </c>
       <c r="B118">
-        <v>6</v>
+        <v>12</v>
       </c>
       <c r="C118">
-        <v>0</v>
+        <v>2.808</v>
       </c>
       <c r="D118" t="s">
         <v>120</v>
@@ -2551,13 +2551,13 @@
     </row>
     <row r="119" spans="1:4">
       <c r="A119" s="2">
-        <v>46178</v>
+        <v>46182</v>
       </c>
       <c r="B119">
-        <v>7</v>
+        <v>13</v>
       </c>
       <c r="C119">
-        <v>0.07199999999999999</v>
+        <v>2.985</v>
       </c>
       <c r="D119" t="s">
         <v>121</v>
@@ -2565,13 +2565,13 @@
     </row>
     <row r="120" spans="1:4">
       <c r="A120" s="2">
-        <v>46178</v>
+        <v>46182</v>
       </c>
       <c r="B120">
-        <v>8</v>
+        <v>14</v>
       </c>
       <c r="C120">
-        <v>0.424</v>
+        <v>2.929</v>
       </c>
       <c r="D120" t="s">
         <v>122</v>
@@ -2579,13 +2579,13 @@
     </row>
     <row r="121" spans="1:4">
       <c r="A121" s="2">
-        <v>46178</v>
+        <v>46182</v>
       </c>
       <c r="B121">
-        <v>9</v>
+        <v>15</v>
       </c>
       <c r="C121">
-        <v>0.978</v>
+        <v>2.798</v>
       </c>
       <c r="D121" t="s">
         <v>123</v>
@@ -2593,13 +2593,13 @@
     </row>
     <row r="122" spans="1:4">
       <c r="A122" s="2">
-        <v>46178</v>
+        <v>46182</v>
       </c>
       <c r="B122">
-        <v>10</v>
+        <v>16</v>
       </c>
       <c r="C122">
-        <v>1.477</v>
+        <v>2.569</v>
       </c>
       <c r="D122" t="s">
         <v>124</v>
@@ -2607,13 +2607,13 @@
     </row>
     <row r="123" spans="1:4">
       <c r="A123" s="2">
-        <v>46178</v>
+        <v>46182</v>
       </c>
       <c r="B123">
-        <v>11</v>
+        <v>17</v>
       </c>
       <c r="C123">
-        <v>1.879</v>
+        <v>2.109</v>
       </c>
       <c r="D123" t="s">
         <v>125</v>
@@ -2621,13 +2621,13 @@
     </row>
     <row r="124" spans="1:4">
       <c r="A124" s="2">
-        <v>46178</v>
+        <v>46182</v>
       </c>
       <c r="B124">
-        <v>12</v>
+        <v>18</v>
       </c>
       <c r="C124">
-        <v>2.223</v>
+        <v>1.44</v>
       </c>
       <c r="D124" t="s">
         <v>126</v>
@@ -2635,13 +2635,13 @@
     </row>
     <row r="125" spans="1:4">
       <c r="A125" s="2">
-        <v>46178</v>
+        <v>46182</v>
       </c>
       <c r="B125">
-        <v>13</v>
+        <v>19</v>
       </c>
       <c r="C125">
-        <v>2.395</v>
+        <v>0.788</v>
       </c>
       <c r="D125" t="s">
         <v>127</v>
@@ -2649,13 +2649,13 @@
     </row>
     <row r="126" spans="1:4">
       <c r="A126" s="2">
-        <v>46178</v>
+        <v>46182</v>
       </c>
       <c r="B126">
-        <v>14</v>
+        <v>20</v>
       </c>
       <c r="C126">
-        <v>2.411</v>
+        <v>0.281</v>
       </c>
       <c r="D126" t="s">
         <v>128</v>
@@ -2663,13 +2663,13 @@
     </row>
     <row r="127" spans="1:4">
       <c r="A127" s="2">
-        <v>46178</v>
+        <v>46182</v>
       </c>
       <c r="B127">
-        <v>15</v>
+        <v>21</v>
       </c>
       <c r="C127">
-        <v>2.431</v>
+        <v>0.059</v>
       </c>
       <c r="D127" t="s">
         <v>129</v>
@@ -2677,13 +2677,13 @@
     </row>
     <row r="128" spans="1:4">
       <c r="A128" s="2">
-        <v>46178</v>
+        <v>46182</v>
       </c>
       <c r="B128">
-        <v>16</v>
+        <v>22</v>
       </c>
       <c r="C128">
-        <v>1.983</v>
+        <v>0</v>
       </c>
       <c r="D128" t="s">
         <v>130</v>
@@ -2691,13 +2691,13 @@
     </row>
     <row r="129" spans="1:4">
       <c r="A129" s="2">
-        <v>46178</v>
+        <v>46182</v>
       </c>
       <c r="B129">
-        <v>17</v>
+        <v>23</v>
       </c>
       <c r="C129">
-        <v>1.7</v>
+        <v>0</v>
       </c>
       <c r="D129" t="s">
         <v>131</v>
@@ -2705,13 +2705,13 @@
     </row>
     <row r="130" spans="1:4">
       <c r="A130" s="2">
-        <v>46178</v>
+        <v>46182</v>
       </c>
       <c r="B130">
-        <v>18</v>
+        <v>24</v>
       </c>
       <c r="C130">
-        <v>1.145</v>
+        <v>0</v>
       </c>
       <c r="D130" t="s">
         <v>132</v>
@@ -2719,13 +2719,13 @@
     </row>
     <row r="131" spans="1:4">
       <c r="A131" s="2">
-        <v>46178</v>
+        <v>46183</v>
       </c>
       <c r="B131">
-        <v>19</v>
+        <v>1</v>
       </c>
       <c r="C131">
-        <v>0.618</v>
+        <v>0</v>
       </c>
       <c r="D131" t="s">
         <v>133</v>
@@ -2733,13 +2733,13 @@
     </row>
     <row r="132" spans="1:4">
       <c r="A132" s="2">
-        <v>46178</v>
+        <v>46183</v>
       </c>
       <c r="B132">
-        <v>20</v>
+        <v>2</v>
       </c>
       <c r="C132">
-        <v>0.275</v>
+        <v>0</v>
       </c>
       <c r="D132" t="s">
         <v>134</v>
@@ -2747,13 +2747,13 @@
     </row>
     <row r="133" spans="1:4">
       <c r="A133" s="2">
-        <v>46178</v>
+        <v>46183</v>
       </c>
       <c r="B133">
-        <v>21</v>
+        <v>3</v>
       </c>
       <c r="C133">
-        <v>0.046</v>
+        <v>0</v>
       </c>
       <c r="D133" t="s">
         <v>135</v>
@@ -2761,10 +2761,10 @@
     </row>
     <row r="134" spans="1:4">
       <c r="A134" s="2">
-        <v>46178</v>
+        <v>46183</v>
       </c>
       <c r="B134">
-        <v>22</v>
+        <v>4</v>
       </c>
       <c r="C134">
         <v>0</v>
@@ -2775,10 +2775,10 @@
     </row>
     <row r="135" spans="1:4">
       <c r="A135" s="2">
-        <v>46178</v>
+        <v>46183</v>
       </c>
       <c r="B135">
-        <v>23</v>
+        <v>5</v>
       </c>
       <c r="C135">
         <v>0</v>
@@ -2789,10 +2789,10 @@
     </row>
     <row r="136" spans="1:4">
       <c r="A136" s="2">
-        <v>46178</v>
+        <v>46183</v>
       </c>
       <c r="B136">
-        <v>24</v>
+        <v>6</v>
       </c>
       <c r="C136">
         <v>0</v>
@@ -2803,13 +2803,13 @@
     </row>
     <row r="137" spans="1:4">
       <c r="A137" s="2">
-        <v>46179</v>
+        <v>46183</v>
       </c>
       <c r="B137">
-        <v>1</v>
+        <v>7</v>
       </c>
       <c r="C137">
-        <v>0</v>
+        <v>0.08</v>
       </c>
       <c r="D137" t="s">
         <v>139</v>
@@ -2817,13 +2817,13 @@
     </row>
     <row r="138" spans="1:4">
       <c r="A138" s="2">
-        <v>46179</v>
+        <v>46183</v>
       </c>
       <c r="B138">
-        <v>2</v>
+        <v>8</v>
       </c>
       <c r="C138">
-        <v>0</v>
+        <v>0.436</v>
       </c>
       <c r="D138" t="s">
         <v>140</v>
@@ -2831,13 +2831,13 @@
     </row>
     <row r="139" spans="1:4">
       <c r="A139" s="2">
-        <v>46179</v>
+        <v>46183</v>
       </c>
       <c r="B139">
-        <v>3</v>
+        <v>9</v>
       </c>
       <c r="C139">
-        <v>0</v>
+        <v>0.97</v>
       </c>
       <c r="D139" t="s">
         <v>141</v>
@@ -2845,13 +2845,13 @@
     </row>
     <row r="140" spans="1:4">
       <c r="A140" s="2">
-        <v>46179</v>
+        <v>46183</v>
       </c>
       <c r="B140">
-        <v>4</v>
+        <v>10</v>
       </c>
       <c r="C140">
-        <v>0</v>
+        <v>1.395</v>
       </c>
       <c r="D140" t="s">
         <v>142</v>
@@ -2859,13 +2859,13 @@
     </row>
     <row r="141" spans="1:4">
       <c r="A141" s="2">
-        <v>46179</v>
+        <v>46183</v>
       </c>
       <c r="B141">
-        <v>5</v>
+        <v>11</v>
       </c>
       <c r="C141">
-        <v>0</v>
+        <v>1.898</v>
       </c>
       <c r="D141" t="s">
         <v>143</v>
@@ -2873,13 +2873,13 @@
     </row>
     <row r="142" spans="1:4">
       <c r="A142" s="2">
-        <v>46179</v>
+        <v>46183</v>
       </c>
       <c r="B142">
-        <v>6</v>
+        <v>12</v>
       </c>
       <c r="C142">
-        <v>0</v>
+        <v>2.313</v>
       </c>
       <c r="D142" t="s">
         <v>144</v>
@@ -2887,13 +2887,13 @@
     </row>
     <row r="143" spans="1:4">
       <c r="A143" s="2">
-        <v>46179</v>
+        <v>46183</v>
       </c>
       <c r="B143">
-        <v>7</v>
+        <v>13</v>
       </c>
       <c r="C143">
-        <v>0.075</v>
+        <v>2.404</v>
       </c>
       <c r="D143" t="s">
         <v>145</v>
@@ -2901,13 +2901,13 @@
     </row>
     <row r="144" spans="1:4">
       <c r="A144" s="2">
-        <v>46179</v>
+        <v>46183</v>
       </c>
       <c r="B144">
-        <v>8</v>
+        <v>14</v>
       </c>
       <c r="C144">
-        <v>0.446</v>
+        <v>2.553</v>
       </c>
       <c r="D144" t="s">
         <v>146</v>
@@ -2915,13 +2915,13 @@
     </row>
     <row r="145" spans="1:4">
       <c r="A145" s="2">
-        <v>46179</v>
+        <v>46183</v>
       </c>
       <c r="B145">
-        <v>9</v>
+        <v>15</v>
       </c>
       <c r="C145">
-        <v>0.9330000000000001</v>
+        <v>2.524</v>
       </c>
       <c r="D145" t="s">
         <v>147</v>
@@ -2929,13 +2929,13 @@
     </row>
     <row r="146" spans="1:4">
       <c r="A146" s="2">
-        <v>46179</v>
+        <v>46183</v>
       </c>
       <c r="B146">
-        <v>10</v>
+        <v>16</v>
       </c>
       <c r="C146">
-        <v>1.612</v>
+        <v>2.128</v>
       </c>
       <c r="D146" t="s">
         <v>148</v>
@@ -2943,13 +2943,13 @@
     </row>
     <row r="147" spans="1:4">
       <c r="A147" s="2">
-        <v>46179</v>
+        <v>46183</v>
       </c>
       <c r="B147">
-        <v>11</v>
+        <v>17</v>
       </c>
       <c r="C147">
-        <v>2.014</v>
+        <v>1.759</v>
       </c>
       <c r="D147" t="s">
         <v>149</v>
@@ -2957,13 +2957,13 @@
     </row>
     <row r="148" spans="1:4">
       <c r="A148" s="2">
-        <v>46179</v>
+        <v>46183</v>
       </c>
       <c r="B148">
-        <v>12</v>
+        <v>18</v>
       </c>
       <c r="C148">
-        <v>2.365</v>
+        <v>1.259</v>
       </c>
       <c r="D148" t="s">
         <v>150</v>
@@ -2971,13 +2971,13 @@
     </row>
     <row r="149" spans="1:4">
       <c r="A149" s="2">
-        <v>46179</v>
+        <v>46183</v>
       </c>
       <c r="B149">
-        <v>13</v>
+        <v>19</v>
       </c>
       <c r="C149">
-        <v>2.428</v>
+        <v>0.671</v>
       </c>
       <c r="D149" t="s">
         <v>151</v>
@@ -2985,13 +2985,13 @@
     </row>
     <row r="150" spans="1:4">
       <c r="A150" s="2">
-        <v>46179</v>
+        <v>46183</v>
       </c>
       <c r="B150">
-        <v>14</v>
+        <v>20</v>
       </c>
       <c r="C150">
-        <v>2.376</v>
+        <v>0.277</v>
       </c>
       <c r="D150" t="s">
         <v>152</v>
@@ -2999,13 +2999,13 @@
     </row>
     <row r="151" spans="1:4">
       <c r="A151" s="2">
-        <v>46179</v>
+        <v>46183</v>
       </c>
       <c r="B151">
-        <v>15</v>
+        <v>21</v>
       </c>
       <c r="C151">
-        <v>2.269</v>
+        <v>0.047</v>
       </c>
       <c r="D151" t="s">
         <v>153</v>
@@ -3013,13 +3013,13 @@
     </row>
     <row r="152" spans="1:4">
       <c r="A152" s="2">
-        <v>46179</v>
+        <v>46183</v>
       </c>
       <c r="B152">
-        <v>16</v>
+        <v>22</v>
       </c>
       <c r="C152">
-        <v>1.91</v>
+        <v>0</v>
       </c>
       <c r="D152" t="s">
         <v>154</v>
@@ -3027,13 +3027,13 @@
     </row>
     <row r="153" spans="1:4">
       <c r="A153" s="2">
-        <v>46179</v>
+        <v>46183</v>
       </c>
       <c r="B153">
-        <v>17</v>
+        <v>23</v>
       </c>
       <c r="C153">
-        <v>1.651</v>
+        <v>0</v>
       </c>
       <c r="D153" t="s">
         <v>155</v>
@@ -3041,13 +3041,13 @@
     </row>
     <row r="154" spans="1:4">
       <c r="A154" s="2">
-        <v>46179</v>
+        <v>46183</v>
       </c>
       <c r="B154">
-        <v>18</v>
+        <v>24</v>
       </c>
       <c r="C154">
-        <v>1.065</v>
+        <v>0</v>
       </c>
       <c r="D154" t="s">
         <v>156</v>
@@ -3055,13 +3055,13 @@
     </row>
     <row r="155" spans="1:4">
       <c r="A155" s="2">
-        <v>46179</v>
+        <v>46184</v>
       </c>
       <c r="B155">
-        <v>19</v>
+        <v>1</v>
       </c>
       <c r="C155">
-        <v>0.593</v>
+        <v>0</v>
       </c>
       <c r="D155" t="s">
         <v>157</v>
@@ -3069,13 +3069,13 @@
     </row>
     <row r="156" spans="1:4">
       <c r="A156" s="2">
-        <v>46179</v>
+        <v>46184</v>
       </c>
       <c r="B156">
-        <v>20</v>
+        <v>2</v>
       </c>
       <c r="C156">
-        <v>0.301</v>
+        <v>0</v>
       </c>
       <c r="D156" t="s">
         <v>158</v>
@@ -3083,13 +3083,13 @@
     </row>
     <row r="157" spans="1:4">
       <c r="A157" s="2">
-        <v>46179</v>
+        <v>46184</v>
       </c>
       <c r="B157">
-        <v>21</v>
+        <v>3</v>
       </c>
       <c r="C157">
-        <v>0.05</v>
+        <v>0</v>
       </c>
       <c r="D157" t="s">
         <v>159</v>
@@ -3097,10 +3097,10 @@
     </row>
     <row r="158" spans="1:4">
       <c r="A158" s="2">
-        <v>46179</v>
+        <v>46184</v>
       </c>
       <c r="B158">
-        <v>22</v>
+        <v>4</v>
       </c>
       <c r="C158">
         <v>0</v>
@@ -3111,10 +3111,10 @@
     </row>
     <row r="159" spans="1:4">
       <c r="A159" s="2">
-        <v>46179</v>
+        <v>46184</v>
       </c>
       <c r="B159">
-        <v>23</v>
+        <v>5</v>
       </c>
       <c r="C159">
         <v>0</v>
@@ -3125,10 +3125,10 @@
     </row>
     <row r="160" spans="1:4">
       <c r="A160" s="2">
-        <v>46179</v>
+        <v>46184</v>
       </c>
       <c r="B160">
-        <v>24</v>
+        <v>6</v>
       </c>
       <c r="C160">
         <v>0</v>
@@ -3139,13 +3139,13 @@
     </row>
     <row r="161" spans="1:4">
       <c r="A161" s="2">
-        <v>46180</v>
+        <v>46184</v>
       </c>
       <c r="B161">
-        <v>1</v>
+        <v>7</v>
       </c>
       <c r="C161">
-        <v>0</v>
+        <v>0.082</v>
       </c>
       <c r="D161" t="s">
         <v>163</v>
@@ -3153,13 +3153,13 @@
     </row>
     <row r="162" spans="1:4">
       <c r="A162" s="2">
-        <v>46180</v>
+        <v>46184</v>
       </c>
       <c r="B162">
-        <v>2</v>
+        <v>8</v>
       </c>
       <c r="C162">
-        <v>0</v>
+        <v>0.427</v>
       </c>
       <c r="D162" t="s">
         <v>164</v>
@@ -3167,13 +3167,13 @@
     </row>
     <row r="163" spans="1:4">
       <c r="A163" s="2">
-        <v>46180</v>
+        <v>46184</v>
       </c>
       <c r="B163">
-        <v>3</v>
+        <v>9</v>
       </c>
       <c r="C163">
-        <v>0</v>
+        <v>1.012</v>
       </c>
       <c r="D163" t="s">
         <v>165</v>
@@ -3181,13 +3181,13 @@
     </row>
     <row r="164" spans="1:4">
       <c r="A164" s="2">
-        <v>46180</v>
+        <v>46184</v>
       </c>
       <c r="B164">
-        <v>4</v>
+        <v>10</v>
       </c>
       <c r="C164">
-        <v>0</v>
+        <v>1.555</v>
       </c>
       <c r="D164" t="s">
         <v>166</v>
@@ -3195,13 +3195,13 @@
     </row>
     <row r="165" spans="1:4">
       <c r="A165" s="2">
-        <v>46180</v>
+        <v>46184</v>
       </c>
       <c r="B165">
-        <v>5</v>
+        <v>11</v>
       </c>
       <c r="C165">
-        <v>0</v>
+        <v>1.919</v>
       </c>
       <c r="D165" t="s">
         <v>167</v>
@@ -3209,13 +3209,13 @@
     </row>
     <row r="166" spans="1:4">
       <c r="A166" s="2">
-        <v>46180</v>
+        <v>46184</v>
       </c>
       <c r="B166">
-        <v>6</v>
+        <v>12</v>
       </c>
       <c r="C166">
-        <v>0</v>
+        <v>2.349</v>
       </c>
       <c r="D166" t="s">
         <v>168</v>
@@ -3223,13 +3223,13 @@
     </row>
     <row r="167" spans="1:4">
       <c r="A167" s="2">
-        <v>46180</v>
+        <v>46184</v>
       </c>
       <c r="B167">
-        <v>7</v>
+        <v>13</v>
       </c>
       <c r="C167">
-        <v>0.075</v>
+        <v>2.644</v>
       </c>
       <c r="D167" t="s">
         <v>169</v>
@@ -3237,13 +3237,13 @@
     </row>
     <row r="168" spans="1:4">
       <c r="A168" s="2">
-        <v>46180</v>
+        <v>46184</v>
       </c>
       <c r="B168">
-        <v>8</v>
+        <v>14</v>
       </c>
       <c r="C168">
-        <v>0.451</v>
+        <v>2.764</v>
       </c>
       <c r="D168" t="s">
         <v>170</v>
@@ -3251,13 +3251,13 @@
     </row>
     <row r="169" spans="1:4">
       <c r="A169" s="2">
-        <v>46180</v>
+        <v>46184</v>
       </c>
       <c r="B169">
-        <v>9</v>
+        <v>15</v>
       </c>
       <c r="C169">
-        <v>0.8120000000000001</v>
+        <v>2.679</v>
       </c>
       <c r="D169" t="s">
         <v>171</v>
@@ -3265,13 +3265,13 @@
     </row>
     <row r="170" spans="1:4">
       <c r="A170" s="2">
-        <v>46180</v>
+        <v>46184</v>
       </c>
       <c r="B170">
-        <v>10</v>
+        <v>16</v>
       </c>
       <c r="C170">
-        <v>1.382</v>
+        <v>2.271</v>
       </c>
       <c r="D170" t="s">
         <v>172</v>

</xml_diff>

<commit_message>
Updating the model for GESS
</commit_message>
<xml_diff>
--- a/Astro/Results_Production_Astro_xgb.xlsx
+++ b/Astro/Results_Production_Astro_xgb.xlsx
@@ -28,511 +28,511 @@
     <t>Lookup</t>
   </si>
   <si>
-    <t>16.07.202617</t>
-  </si>
-  <si>
-    <t>16.07.202618</t>
-  </si>
-  <si>
-    <t>16.07.202619</t>
-  </si>
-  <si>
-    <t>16.07.202620</t>
-  </si>
-  <si>
-    <t>16.07.202621</t>
-  </si>
-  <si>
-    <t>16.07.202622</t>
-  </si>
-  <si>
-    <t>16.07.202623</t>
-  </si>
-  <si>
-    <t>16.07.202624</t>
-  </si>
-  <si>
-    <t>17.07.20261</t>
-  </si>
-  <si>
-    <t>17.07.20262</t>
-  </si>
-  <si>
-    <t>17.07.20263</t>
-  </si>
-  <si>
-    <t>17.07.20264</t>
-  </si>
-  <si>
-    <t>17.07.20265</t>
-  </si>
-  <si>
-    <t>17.07.20266</t>
-  </si>
-  <si>
-    <t>17.07.20267</t>
-  </si>
-  <si>
-    <t>17.07.20268</t>
-  </si>
-  <si>
-    <t>17.07.20269</t>
-  </si>
-  <si>
-    <t>17.07.202610</t>
-  </si>
-  <si>
-    <t>17.07.202611</t>
-  </si>
-  <si>
-    <t>17.07.202612</t>
-  </si>
-  <si>
-    <t>17.07.202613</t>
-  </si>
-  <si>
-    <t>17.07.202614</t>
-  </si>
-  <si>
-    <t>17.07.202615</t>
-  </si>
-  <si>
-    <t>17.07.202616</t>
-  </si>
-  <si>
-    <t>17.07.202617</t>
-  </si>
-  <si>
-    <t>17.07.202618</t>
-  </si>
-  <si>
-    <t>17.07.202619</t>
-  </si>
-  <si>
-    <t>17.07.202620</t>
-  </si>
-  <si>
-    <t>17.07.202621</t>
-  </si>
-  <si>
-    <t>17.07.202622</t>
-  </si>
-  <si>
-    <t>17.07.202623</t>
-  </si>
-  <si>
-    <t>17.07.202624</t>
-  </si>
-  <si>
-    <t>18.07.20261</t>
-  </si>
-  <si>
-    <t>18.07.20262</t>
-  </si>
-  <si>
-    <t>18.07.20263</t>
-  </si>
-  <si>
-    <t>18.07.20264</t>
-  </si>
-  <si>
-    <t>18.07.20265</t>
-  </si>
-  <si>
-    <t>18.07.20266</t>
-  </si>
-  <si>
-    <t>18.07.20267</t>
-  </si>
-  <si>
-    <t>18.07.20268</t>
-  </si>
-  <si>
-    <t>18.07.20269</t>
-  </si>
-  <si>
-    <t>18.07.202610</t>
-  </si>
-  <si>
-    <t>18.07.202611</t>
-  </si>
-  <si>
-    <t>18.07.202612</t>
-  </si>
-  <si>
-    <t>18.07.202613</t>
-  </si>
-  <si>
-    <t>18.07.202614</t>
-  </si>
-  <si>
-    <t>18.07.202615</t>
-  </si>
-  <si>
-    <t>18.07.202616</t>
-  </si>
-  <si>
-    <t>18.07.202617</t>
-  </si>
-  <si>
-    <t>18.07.202618</t>
-  </si>
-  <si>
-    <t>18.07.202619</t>
-  </si>
-  <si>
-    <t>18.07.202620</t>
-  </si>
-  <si>
-    <t>18.07.202621</t>
-  </si>
-  <si>
-    <t>18.07.202622</t>
-  </si>
-  <si>
-    <t>18.07.202623</t>
-  </si>
-  <si>
-    <t>18.07.202624</t>
-  </si>
-  <si>
-    <t>19.07.20261</t>
-  </si>
-  <si>
-    <t>19.07.20262</t>
-  </si>
-  <si>
-    <t>19.07.20263</t>
-  </si>
-  <si>
-    <t>19.07.20264</t>
-  </si>
-  <si>
-    <t>19.07.20265</t>
-  </si>
-  <si>
-    <t>19.07.20266</t>
-  </si>
-  <si>
-    <t>19.07.20267</t>
-  </si>
-  <si>
-    <t>19.07.20268</t>
-  </si>
-  <si>
-    <t>19.07.20269</t>
-  </si>
-  <si>
-    <t>19.07.202610</t>
-  </si>
-  <si>
-    <t>19.07.202611</t>
-  </si>
-  <si>
-    <t>19.07.202612</t>
-  </si>
-  <si>
-    <t>19.07.202613</t>
-  </si>
-  <si>
-    <t>19.07.202614</t>
-  </si>
-  <si>
-    <t>19.07.202615</t>
-  </si>
-  <si>
-    <t>19.07.202616</t>
-  </si>
-  <si>
-    <t>19.07.202617</t>
-  </si>
-  <si>
-    <t>19.07.202618</t>
-  </si>
-  <si>
-    <t>19.07.202619</t>
-  </si>
-  <si>
-    <t>19.07.202620</t>
-  </si>
-  <si>
-    <t>19.07.202621</t>
-  </si>
-  <si>
-    <t>19.07.202622</t>
-  </si>
-  <si>
-    <t>19.07.202623</t>
-  </si>
-  <si>
-    <t>19.07.202624</t>
-  </si>
-  <si>
-    <t>20.07.20261</t>
-  </si>
-  <si>
-    <t>20.07.20262</t>
-  </si>
-  <si>
-    <t>20.07.20263</t>
-  </si>
-  <si>
-    <t>20.07.20264</t>
-  </si>
-  <si>
-    <t>20.07.20265</t>
-  </si>
-  <si>
-    <t>20.07.20266</t>
-  </si>
-  <si>
-    <t>20.07.20267</t>
-  </si>
-  <si>
-    <t>20.07.20268</t>
-  </si>
-  <si>
-    <t>20.07.20269</t>
-  </si>
-  <si>
-    <t>20.07.202610</t>
-  </si>
-  <si>
-    <t>20.07.202611</t>
-  </si>
-  <si>
-    <t>20.07.202612</t>
-  </si>
-  <si>
-    <t>20.07.202613</t>
-  </si>
-  <si>
-    <t>20.07.202614</t>
-  </si>
-  <si>
-    <t>20.07.202615</t>
-  </si>
-  <si>
-    <t>20.07.202616</t>
-  </si>
-  <si>
-    <t>20.07.202617</t>
-  </si>
-  <si>
-    <t>20.07.202618</t>
-  </si>
-  <si>
-    <t>20.07.202619</t>
-  </si>
-  <si>
-    <t>20.07.202620</t>
-  </si>
-  <si>
-    <t>20.07.202621</t>
-  </si>
-  <si>
-    <t>20.07.202622</t>
-  </si>
-  <si>
-    <t>20.07.202623</t>
-  </si>
-  <si>
-    <t>20.07.202624</t>
-  </si>
-  <si>
-    <t>21.07.20261</t>
-  </si>
-  <si>
-    <t>21.07.20262</t>
-  </si>
-  <si>
-    <t>21.07.20263</t>
-  </si>
-  <si>
-    <t>21.07.20264</t>
-  </si>
-  <si>
-    <t>21.07.20265</t>
-  </si>
-  <si>
-    <t>21.07.20266</t>
-  </si>
-  <si>
-    <t>21.07.20267</t>
-  </si>
-  <si>
-    <t>21.07.20268</t>
-  </si>
-  <si>
-    <t>21.07.20269</t>
-  </si>
-  <si>
-    <t>21.07.202610</t>
-  </si>
-  <si>
-    <t>21.07.202611</t>
-  </si>
-  <si>
-    <t>21.07.202612</t>
-  </si>
-  <si>
-    <t>21.07.202613</t>
-  </si>
-  <si>
-    <t>21.07.202614</t>
-  </si>
-  <si>
-    <t>21.07.202615</t>
-  </si>
-  <si>
-    <t>21.07.202616</t>
-  </si>
-  <si>
-    <t>21.07.202617</t>
-  </si>
-  <si>
-    <t>21.07.202618</t>
-  </si>
-  <si>
-    <t>21.07.202619</t>
-  </si>
-  <si>
-    <t>21.07.202620</t>
-  </si>
-  <si>
-    <t>21.07.202621</t>
-  </si>
-  <si>
-    <t>21.07.202622</t>
-  </si>
-  <si>
-    <t>21.07.202623</t>
-  </si>
-  <si>
-    <t>21.07.202624</t>
-  </si>
-  <si>
-    <t>22.07.20261</t>
-  </si>
-  <si>
-    <t>22.07.20262</t>
-  </si>
-  <si>
-    <t>22.07.20263</t>
-  </si>
-  <si>
-    <t>22.07.20264</t>
-  </si>
-  <si>
-    <t>22.07.20265</t>
-  </si>
-  <si>
-    <t>22.07.20266</t>
-  </si>
-  <si>
-    <t>22.07.20267</t>
-  </si>
-  <si>
-    <t>22.07.20268</t>
-  </si>
-  <si>
-    <t>22.07.20269</t>
-  </si>
-  <si>
-    <t>22.07.202610</t>
-  </si>
-  <si>
-    <t>22.07.202611</t>
-  </si>
-  <si>
-    <t>22.07.202612</t>
-  </si>
-  <si>
-    <t>22.07.202613</t>
-  </si>
-  <si>
-    <t>22.07.202614</t>
-  </si>
-  <si>
-    <t>22.07.202615</t>
-  </si>
-  <si>
-    <t>22.07.202616</t>
-  </si>
-  <si>
-    <t>22.07.202617</t>
-  </si>
-  <si>
-    <t>22.07.202618</t>
-  </si>
-  <si>
-    <t>22.07.202619</t>
-  </si>
-  <si>
-    <t>22.07.202620</t>
-  </si>
-  <si>
-    <t>22.07.202621</t>
-  </si>
-  <si>
-    <t>22.07.202622</t>
-  </si>
-  <si>
-    <t>22.07.202623</t>
-  </si>
-  <si>
-    <t>22.07.202624</t>
-  </si>
-  <si>
-    <t>23.07.20261</t>
-  </si>
-  <si>
-    <t>23.07.20262</t>
-  </si>
-  <si>
-    <t>23.07.20263</t>
-  </si>
-  <si>
-    <t>23.07.20264</t>
-  </si>
-  <si>
-    <t>23.07.20265</t>
-  </si>
-  <si>
-    <t>23.07.20266</t>
-  </si>
-  <si>
-    <t>23.07.20267</t>
-  </si>
-  <si>
-    <t>23.07.20268</t>
-  </si>
-  <si>
-    <t>23.07.20269</t>
-  </si>
-  <si>
-    <t>23.07.202610</t>
-  </si>
-  <si>
-    <t>23.07.202611</t>
-  </si>
-  <si>
-    <t>23.07.202612</t>
-  </si>
-  <si>
-    <t>23.07.202613</t>
-  </si>
-  <si>
-    <t>23.07.202614</t>
-  </si>
-  <si>
-    <t>23.07.202615</t>
-  </si>
-  <si>
-    <t>23.07.202616</t>
-  </si>
-  <si>
-    <t>23.07.202617</t>
+    <t>24.07.20267</t>
+  </si>
+  <si>
+    <t>24.07.20268</t>
+  </si>
+  <si>
+    <t>24.07.20269</t>
+  </si>
+  <si>
+    <t>24.07.202610</t>
+  </si>
+  <si>
+    <t>24.07.202611</t>
+  </si>
+  <si>
+    <t>24.07.202612</t>
+  </si>
+  <si>
+    <t>24.07.202613</t>
+  </si>
+  <si>
+    <t>24.07.202614</t>
+  </si>
+  <si>
+    <t>24.07.202615</t>
+  </si>
+  <si>
+    <t>24.07.202616</t>
+  </si>
+  <si>
+    <t>24.07.202617</t>
+  </si>
+  <si>
+    <t>24.07.202618</t>
+  </si>
+  <si>
+    <t>24.07.202619</t>
+  </si>
+  <si>
+    <t>24.07.202620</t>
+  </si>
+  <si>
+    <t>24.07.202621</t>
+  </si>
+  <si>
+    <t>24.07.202622</t>
+  </si>
+  <si>
+    <t>24.07.202623</t>
+  </si>
+  <si>
+    <t>24.07.202624</t>
+  </si>
+  <si>
+    <t>25.07.20261</t>
+  </si>
+  <si>
+    <t>25.07.20262</t>
+  </si>
+  <si>
+    <t>25.07.20263</t>
+  </si>
+  <si>
+    <t>25.07.20264</t>
+  </si>
+  <si>
+    <t>25.07.20265</t>
+  </si>
+  <si>
+    <t>25.07.20266</t>
+  </si>
+  <si>
+    <t>25.07.20267</t>
+  </si>
+  <si>
+    <t>25.07.20268</t>
+  </si>
+  <si>
+    <t>25.07.20269</t>
+  </si>
+  <si>
+    <t>25.07.202610</t>
+  </si>
+  <si>
+    <t>25.07.202611</t>
+  </si>
+  <si>
+    <t>25.07.202612</t>
+  </si>
+  <si>
+    <t>25.07.202613</t>
+  </si>
+  <si>
+    <t>25.07.202614</t>
+  </si>
+  <si>
+    <t>25.07.202615</t>
+  </si>
+  <si>
+    <t>25.07.202616</t>
+  </si>
+  <si>
+    <t>25.07.202617</t>
+  </si>
+  <si>
+    <t>25.07.202618</t>
+  </si>
+  <si>
+    <t>25.07.202619</t>
+  </si>
+  <si>
+    <t>25.07.202620</t>
+  </si>
+  <si>
+    <t>25.07.202621</t>
+  </si>
+  <si>
+    <t>25.07.202622</t>
+  </si>
+  <si>
+    <t>25.07.202623</t>
+  </si>
+  <si>
+    <t>25.07.202624</t>
+  </si>
+  <si>
+    <t>26.07.20261</t>
+  </si>
+  <si>
+    <t>26.07.20262</t>
+  </si>
+  <si>
+    <t>26.07.20263</t>
+  </si>
+  <si>
+    <t>26.07.20264</t>
+  </si>
+  <si>
+    <t>26.07.20265</t>
+  </si>
+  <si>
+    <t>26.07.20266</t>
+  </si>
+  <si>
+    <t>26.07.20267</t>
+  </si>
+  <si>
+    <t>26.07.20268</t>
+  </si>
+  <si>
+    <t>26.07.20269</t>
+  </si>
+  <si>
+    <t>26.07.202610</t>
+  </si>
+  <si>
+    <t>26.07.202611</t>
+  </si>
+  <si>
+    <t>26.07.202612</t>
+  </si>
+  <si>
+    <t>26.07.202613</t>
+  </si>
+  <si>
+    <t>26.07.202614</t>
+  </si>
+  <si>
+    <t>26.07.202615</t>
+  </si>
+  <si>
+    <t>26.07.202616</t>
+  </si>
+  <si>
+    <t>26.07.202617</t>
+  </si>
+  <si>
+    <t>26.07.202618</t>
+  </si>
+  <si>
+    <t>26.07.202619</t>
+  </si>
+  <si>
+    <t>26.07.202620</t>
+  </si>
+  <si>
+    <t>26.07.202621</t>
+  </si>
+  <si>
+    <t>26.07.202622</t>
+  </si>
+  <si>
+    <t>26.07.202623</t>
+  </si>
+  <si>
+    <t>26.07.202624</t>
+  </si>
+  <si>
+    <t>27.07.20261</t>
+  </si>
+  <si>
+    <t>27.07.20262</t>
+  </si>
+  <si>
+    <t>27.07.20263</t>
+  </si>
+  <si>
+    <t>27.07.20264</t>
+  </si>
+  <si>
+    <t>27.07.20265</t>
+  </si>
+  <si>
+    <t>27.07.20266</t>
+  </si>
+  <si>
+    <t>27.07.20267</t>
+  </si>
+  <si>
+    <t>27.07.20268</t>
+  </si>
+  <si>
+    <t>27.07.20269</t>
+  </si>
+  <si>
+    <t>27.07.202610</t>
+  </si>
+  <si>
+    <t>27.07.202611</t>
+  </si>
+  <si>
+    <t>27.07.202612</t>
+  </si>
+  <si>
+    <t>27.07.202613</t>
+  </si>
+  <si>
+    <t>27.07.202614</t>
+  </si>
+  <si>
+    <t>27.07.202615</t>
+  </si>
+  <si>
+    <t>27.07.202616</t>
+  </si>
+  <si>
+    <t>27.07.202617</t>
+  </si>
+  <si>
+    <t>27.07.202618</t>
+  </si>
+  <si>
+    <t>27.07.202619</t>
+  </si>
+  <si>
+    <t>27.07.202620</t>
+  </si>
+  <si>
+    <t>27.07.202621</t>
+  </si>
+  <si>
+    <t>27.07.202622</t>
+  </si>
+  <si>
+    <t>27.07.202623</t>
+  </si>
+  <si>
+    <t>27.07.202624</t>
+  </si>
+  <si>
+    <t>28.07.20261</t>
+  </si>
+  <si>
+    <t>28.07.20262</t>
+  </si>
+  <si>
+    <t>28.07.20263</t>
+  </si>
+  <si>
+    <t>28.07.20264</t>
+  </si>
+  <si>
+    <t>28.07.20265</t>
+  </si>
+  <si>
+    <t>28.07.20266</t>
+  </si>
+  <si>
+    <t>28.07.20267</t>
+  </si>
+  <si>
+    <t>28.07.20268</t>
+  </si>
+  <si>
+    <t>28.07.20269</t>
+  </si>
+  <si>
+    <t>28.07.202610</t>
+  </si>
+  <si>
+    <t>28.07.202611</t>
+  </si>
+  <si>
+    <t>28.07.202612</t>
+  </si>
+  <si>
+    <t>28.07.202613</t>
+  </si>
+  <si>
+    <t>28.07.202614</t>
+  </si>
+  <si>
+    <t>28.07.202615</t>
+  </si>
+  <si>
+    <t>28.07.202616</t>
+  </si>
+  <si>
+    <t>28.07.202617</t>
+  </si>
+  <si>
+    <t>28.07.202618</t>
+  </si>
+  <si>
+    <t>28.07.202619</t>
+  </si>
+  <si>
+    <t>28.07.202620</t>
+  </si>
+  <si>
+    <t>28.07.202621</t>
+  </si>
+  <si>
+    <t>28.07.202622</t>
+  </si>
+  <si>
+    <t>28.07.202623</t>
+  </si>
+  <si>
+    <t>28.07.202624</t>
+  </si>
+  <si>
+    <t>29.07.20261</t>
+  </si>
+  <si>
+    <t>29.07.20262</t>
+  </si>
+  <si>
+    <t>29.07.20263</t>
+  </si>
+  <si>
+    <t>29.07.20264</t>
+  </si>
+  <si>
+    <t>29.07.20265</t>
+  </si>
+  <si>
+    <t>29.07.20266</t>
+  </si>
+  <si>
+    <t>29.07.20267</t>
+  </si>
+  <si>
+    <t>29.07.20268</t>
+  </si>
+  <si>
+    <t>29.07.20269</t>
+  </si>
+  <si>
+    <t>29.07.202610</t>
+  </si>
+  <si>
+    <t>29.07.202611</t>
+  </si>
+  <si>
+    <t>29.07.202612</t>
+  </si>
+  <si>
+    <t>29.07.202613</t>
+  </si>
+  <si>
+    <t>29.07.202614</t>
+  </si>
+  <si>
+    <t>29.07.202615</t>
+  </si>
+  <si>
+    <t>29.07.202616</t>
+  </si>
+  <si>
+    <t>29.07.202617</t>
+  </si>
+  <si>
+    <t>29.07.202618</t>
+  </si>
+  <si>
+    <t>29.07.202619</t>
+  </si>
+  <si>
+    <t>29.07.202620</t>
+  </si>
+  <si>
+    <t>29.07.202621</t>
+  </si>
+  <si>
+    <t>29.07.202622</t>
+  </si>
+  <si>
+    <t>29.07.202623</t>
+  </si>
+  <si>
+    <t>29.07.202624</t>
+  </si>
+  <si>
+    <t>30.07.20261</t>
+  </si>
+  <si>
+    <t>30.07.20262</t>
+  </si>
+  <si>
+    <t>30.07.20263</t>
+  </si>
+  <si>
+    <t>30.07.20264</t>
+  </si>
+  <si>
+    <t>30.07.20265</t>
+  </si>
+  <si>
+    <t>30.07.20266</t>
+  </si>
+  <si>
+    <t>30.07.20267</t>
+  </si>
+  <si>
+    <t>30.07.20268</t>
+  </si>
+  <si>
+    <t>30.07.20269</t>
+  </si>
+  <si>
+    <t>30.07.202610</t>
+  </si>
+  <si>
+    <t>30.07.202611</t>
+  </si>
+  <si>
+    <t>30.07.202612</t>
+  </si>
+  <si>
+    <t>30.07.202613</t>
+  </si>
+  <si>
+    <t>30.07.202614</t>
+  </si>
+  <si>
+    <t>30.07.202615</t>
+  </si>
+  <si>
+    <t>30.07.202616</t>
+  </si>
+  <si>
+    <t>30.07.202617</t>
+  </si>
+  <si>
+    <t>30.07.202618</t>
+  </si>
+  <si>
+    <t>30.07.202619</t>
+  </si>
+  <si>
+    <t>30.07.202620</t>
+  </si>
+  <si>
+    <t>30.07.202621</t>
+  </si>
+  <si>
+    <t>30.07.202622</t>
+  </si>
+  <si>
+    <t>30.07.202623</t>
+  </si>
+  <si>
+    <t>30.07.202624</t>
+  </si>
+  <si>
+    <t>31.07.20261</t>
+  </si>
+  <si>
+    <t>31.07.20262</t>
+  </si>
+  <si>
+    <t>31.07.20263</t>
+  </si>
+  <si>
+    <t>31.07.20264</t>
+  </si>
+  <si>
+    <t>31.07.20265</t>
+  </si>
+  <si>
+    <t>31.07.20266</t>
+  </si>
+  <si>
+    <t>31.07.20267</t>
   </si>
 </sst>
 </file>
@@ -913,10 +913,10 @@
     </row>
     <row r="2" spans="1:4">
       <c r="A2" s="2">
-        <v>46219</v>
+        <v>46227</v>
       </c>
       <c r="B2">
-        <v>17</v>
+        <v>7</v>
       </c>
       <c r="C2">
         <v>0</v>
@@ -927,10 +927,10 @@
     </row>
     <row r="3" spans="1:4">
       <c r="A3" s="2">
-        <v>46219</v>
+        <v>46227</v>
       </c>
       <c r="B3">
-        <v>18</v>
+        <v>8</v>
       </c>
       <c r="C3">
         <v>0</v>
@@ -941,13 +941,13 @@
     </row>
     <row r="4" spans="1:4">
       <c r="A4" s="2">
-        <v>46219</v>
+        <v>46227</v>
       </c>
       <c r="B4">
-        <v>19</v>
+        <v>9</v>
       </c>
       <c r="C4">
-        <v>0.839</v>
+        <v>1.116</v>
       </c>
       <c r="D4" t="s">
         <v>6</v>
@@ -955,13 +955,13 @@
     </row>
     <row r="5" spans="1:4">
       <c r="A5" s="2">
-        <v>46219</v>
+        <v>46227</v>
       </c>
       <c r="B5">
-        <v>20</v>
+        <v>10</v>
       </c>
       <c r="C5">
-        <v>0.273</v>
+        <v>1.909</v>
       </c>
       <c r="D5" t="s">
         <v>7</v>
@@ -969,13 +969,13 @@
     </row>
     <row r="6" spans="1:4">
       <c r="A6" s="2">
-        <v>46219</v>
+        <v>46227</v>
       </c>
       <c r="B6">
-        <v>21</v>
+        <v>11</v>
       </c>
       <c r="C6">
-        <v>0.066</v>
+        <v>2.225</v>
       </c>
       <c r="D6" t="s">
         <v>8</v>
@@ -983,13 +983,13 @@
     </row>
     <row r="7" spans="1:4">
       <c r="A7" s="2">
-        <v>46219</v>
+        <v>46227</v>
       </c>
       <c r="B7">
-        <v>22</v>
+        <v>12</v>
       </c>
       <c r="C7">
-        <v>0</v>
+        <v>2.444</v>
       </c>
       <c r="D7" t="s">
         <v>9</v>
@@ -997,13 +997,13 @@
     </row>
     <row r="8" spans="1:4">
       <c r="A8" s="2">
-        <v>46219</v>
+        <v>46227</v>
       </c>
       <c r="B8">
-        <v>23</v>
+        <v>13</v>
       </c>
       <c r="C8">
-        <v>0</v>
+        <v>2.401</v>
       </c>
       <c r="D8" t="s">
         <v>10</v>
@@ -1011,13 +1011,13 @@
     </row>
     <row r="9" spans="1:4">
       <c r="A9" s="2">
-        <v>46219</v>
+        <v>46227</v>
       </c>
       <c r="B9">
-        <v>24</v>
+        <v>14</v>
       </c>
       <c r="C9">
-        <v>0</v>
+        <v>2.375</v>
       </c>
       <c r="D9" t="s">
         <v>11</v>
@@ -1025,13 +1025,13 @@
     </row>
     <row r="10" spans="1:4">
       <c r="A10" s="2">
-        <v>46220</v>
+        <v>46227</v>
       </c>
       <c r="B10">
-        <v>1</v>
+        <v>15</v>
       </c>
       <c r="C10">
-        <v>0</v>
+        <v>2.132</v>
       </c>
       <c r="D10" t="s">
         <v>12</v>
@@ -1039,13 +1039,13 @@
     </row>
     <row r="11" spans="1:4">
       <c r="A11" s="2">
-        <v>46220</v>
+        <v>46227</v>
       </c>
       <c r="B11">
-        <v>2</v>
+        <v>16</v>
       </c>
       <c r="C11">
-        <v>0</v>
+        <v>1.857</v>
       </c>
       <c r="D11" t="s">
         <v>13</v>
@@ -1053,13 +1053,13 @@
     </row>
     <row r="12" spans="1:4">
       <c r="A12" s="2">
-        <v>46220</v>
+        <v>46227</v>
       </c>
       <c r="B12">
-        <v>3</v>
+        <v>17</v>
       </c>
       <c r="C12">
-        <v>0</v>
+        <v>1.719</v>
       </c>
       <c r="D12" t="s">
         <v>14</v>
@@ -1067,13 +1067,13 @@
     </row>
     <row r="13" spans="1:4">
       <c r="A13" s="2">
-        <v>46220</v>
+        <v>46227</v>
       </c>
       <c r="B13">
-        <v>4</v>
+        <v>18</v>
       </c>
       <c r="C13">
-        <v>0</v>
+        <v>1.145</v>
       </c>
       <c r="D13" t="s">
         <v>15</v>
@@ -1081,13 +1081,13 @@
     </row>
     <row r="14" spans="1:4">
       <c r="A14" s="2">
-        <v>46220</v>
+        <v>46227</v>
       </c>
       <c r="B14">
-        <v>5</v>
+        <v>19</v>
       </c>
       <c r="C14">
-        <v>0</v>
+        <v>0.648</v>
       </c>
       <c r="D14" t="s">
         <v>16</v>
@@ -1095,13 +1095,13 @@
     </row>
     <row r="15" spans="1:4">
       <c r="A15" s="2">
-        <v>46220</v>
+        <v>46227</v>
       </c>
       <c r="B15">
-        <v>6</v>
+        <v>20</v>
       </c>
       <c r="C15">
-        <v>0</v>
+        <v>0.306</v>
       </c>
       <c r="D15" t="s">
         <v>17</v>
@@ -1109,13 +1109,13 @@
     </row>
     <row r="16" spans="1:4">
       <c r="A16" s="2">
-        <v>46220</v>
+        <v>46227</v>
       </c>
       <c r="B16">
-        <v>7</v>
+        <v>21</v>
       </c>
       <c r="C16">
-        <v>0.063</v>
+        <v>0.066</v>
       </c>
       <c r="D16" t="s">
         <v>18</v>
@@ -1123,13 +1123,13 @@
     </row>
     <row r="17" spans="1:4">
       <c r="A17" s="2">
-        <v>46220</v>
+        <v>46227</v>
       </c>
       <c r="B17">
-        <v>8</v>
+        <v>22</v>
       </c>
       <c r="C17">
-        <v>0.364</v>
+        <v>0</v>
       </c>
       <c r="D17" t="s">
         <v>19</v>
@@ -1137,13 +1137,13 @@
     </row>
     <row r="18" spans="1:4">
       <c r="A18" s="2">
-        <v>46220</v>
+        <v>46227</v>
       </c>
       <c r="B18">
-        <v>9</v>
+        <v>23</v>
       </c>
       <c r="C18">
-        <v>1.009</v>
+        <v>0</v>
       </c>
       <c r="D18" t="s">
         <v>20</v>
@@ -1151,13 +1151,13 @@
     </row>
     <row r="19" spans="1:4">
       <c r="A19" s="2">
-        <v>46220</v>
+        <v>46227</v>
       </c>
       <c r="B19">
-        <v>10</v>
+        <v>24</v>
       </c>
       <c r="C19">
-        <v>1.777</v>
+        <v>0</v>
       </c>
       <c r="D19" t="s">
         <v>21</v>
@@ -1165,13 +1165,13 @@
     </row>
     <row r="20" spans="1:4">
       <c r="A20" s="2">
-        <v>46220</v>
+        <v>46228</v>
       </c>
       <c r="B20">
-        <v>11</v>
+        <v>1</v>
       </c>
       <c r="C20">
-        <v>2.373</v>
+        <v>0</v>
       </c>
       <c r="D20" t="s">
         <v>22</v>
@@ -1179,13 +1179,13 @@
     </row>
     <row r="21" spans="1:4">
       <c r="A21" s="2">
-        <v>46220</v>
+        <v>46228</v>
       </c>
       <c r="B21">
-        <v>12</v>
+        <v>2</v>
       </c>
       <c r="C21">
-        <v>2.694</v>
+        <v>0</v>
       </c>
       <c r="D21" t="s">
         <v>23</v>
@@ -1193,13 +1193,13 @@
     </row>
     <row r="22" spans="1:4">
       <c r="A22" s="2">
-        <v>46220</v>
+        <v>46228</v>
       </c>
       <c r="B22">
-        <v>13</v>
+        <v>3</v>
       </c>
       <c r="C22">
-        <v>2.873</v>
+        <v>0</v>
       </c>
       <c r="D22" t="s">
         <v>24</v>
@@ -1207,13 +1207,13 @@
     </row>
     <row r="23" spans="1:4">
       <c r="A23" s="2">
-        <v>46220</v>
+        <v>46228</v>
       </c>
       <c r="B23">
-        <v>14</v>
+        <v>4</v>
       </c>
       <c r="C23">
-        <v>2.791</v>
+        <v>0</v>
       </c>
       <c r="D23" t="s">
         <v>25</v>
@@ -1221,13 +1221,13 @@
     </row>
     <row r="24" spans="1:4">
       <c r="A24" s="2">
-        <v>46220</v>
+        <v>46228</v>
       </c>
       <c r="B24">
-        <v>15</v>
+        <v>5</v>
       </c>
       <c r="C24">
-        <v>2.508</v>
+        <v>0</v>
       </c>
       <c r="D24" t="s">
         <v>26</v>
@@ -1235,13 +1235,13 @@
     </row>
     <row r="25" spans="1:4">
       <c r="A25" s="2">
-        <v>46220</v>
+        <v>46228</v>
       </c>
       <c r="B25">
-        <v>16</v>
+        <v>6</v>
       </c>
       <c r="C25">
-        <v>2.156</v>
+        <v>0</v>
       </c>
       <c r="D25" t="s">
         <v>27</v>
@@ -1249,13 +1249,13 @@
     </row>
     <row r="26" spans="1:4">
       <c r="A26" s="2">
-        <v>46220</v>
+        <v>46228</v>
       </c>
       <c r="B26">
-        <v>17</v>
+        <v>7</v>
       </c>
       <c r="C26">
-        <v>1.622</v>
+        <v>0.059</v>
       </c>
       <c r="D26" t="s">
         <v>28</v>
@@ -1263,13 +1263,13 @@
     </row>
     <row r="27" spans="1:4">
       <c r="A27" s="2">
-        <v>46220</v>
+        <v>46228</v>
       </c>
       <c r="B27">
-        <v>18</v>
+        <v>8</v>
       </c>
       <c r="C27">
-        <v>1.18</v>
+        <v>0.372</v>
       </c>
       <c r="D27" t="s">
         <v>29</v>
@@ -1277,13 +1277,13 @@
     </row>
     <row r="28" spans="1:4">
       <c r="A28" s="2">
-        <v>46220</v>
+        <v>46228</v>
       </c>
       <c r="B28">
-        <v>19</v>
+        <v>9</v>
       </c>
       <c r="C28">
-        <v>0.787</v>
+        <v>1.095</v>
       </c>
       <c r="D28" t="s">
         <v>30</v>
@@ -1291,13 +1291,13 @@
     </row>
     <row r="29" spans="1:4">
       <c r="A29" s="2">
-        <v>46220</v>
+        <v>46228</v>
       </c>
       <c r="B29">
-        <v>20</v>
+        <v>10</v>
       </c>
       <c r="C29">
-        <v>0.303</v>
+        <v>1.84</v>
       </c>
       <c r="D29" t="s">
         <v>31</v>
@@ -1305,13 +1305,13 @@
     </row>
     <row r="30" spans="1:4">
       <c r="A30" s="2">
-        <v>46220</v>
+        <v>46228</v>
       </c>
       <c r="B30">
-        <v>21</v>
+        <v>11</v>
       </c>
       <c r="C30">
-        <v>0.061</v>
+        <v>2.311</v>
       </c>
       <c r="D30" t="s">
         <v>32</v>
@@ -1319,13 +1319,13 @@
     </row>
     <row r="31" spans="1:4">
       <c r="A31" s="2">
-        <v>46220</v>
+        <v>46228</v>
       </c>
       <c r="B31">
-        <v>22</v>
+        <v>12</v>
       </c>
       <c r="C31">
-        <v>0</v>
+        <v>2.444</v>
       </c>
       <c r="D31" t="s">
         <v>33</v>
@@ -1333,13 +1333,13 @@
     </row>
     <row r="32" spans="1:4">
       <c r="A32" s="2">
-        <v>46220</v>
+        <v>46228</v>
       </c>
       <c r="B32">
-        <v>23</v>
+        <v>13</v>
       </c>
       <c r="C32">
-        <v>0</v>
+        <v>2.695</v>
       </c>
       <c r="D32" t="s">
         <v>34</v>
@@ -1347,13 +1347,13 @@
     </row>
     <row r="33" spans="1:4">
       <c r="A33" s="2">
-        <v>46220</v>
+        <v>46228</v>
       </c>
       <c r="B33">
-        <v>24</v>
+        <v>14</v>
       </c>
       <c r="C33">
-        <v>0</v>
+        <v>2.715</v>
       </c>
       <c r="D33" t="s">
         <v>35</v>
@@ -1361,13 +1361,13 @@
     </row>
     <row r="34" spans="1:4">
       <c r="A34" s="2">
-        <v>46221</v>
+        <v>46228</v>
       </c>
       <c r="B34">
-        <v>1</v>
+        <v>15</v>
       </c>
       <c r="C34">
-        <v>0</v>
+        <v>2.632</v>
       </c>
       <c r="D34" t="s">
         <v>36</v>
@@ -1375,13 +1375,13 @@
     </row>
     <row r="35" spans="1:4">
       <c r="A35" s="2">
-        <v>46221</v>
+        <v>46228</v>
       </c>
       <c r="B35">
-        <v>2</v>
+        <v>16</v>
       </c>
       <c r="C35">
-        <v>0</v>
+        <v>2.204</v>
       </c>
       <c r="D35" t="s">
         <v>37</v>
@@ -1389,13 +1389,13 @@
     </row>
     <row r="36" spans="1:4">
       <c r="A36" s="2">
-        <v>46221</v>
+        <v>46228</v>
       </c>
       <c r="B36">
-        <v>3</v>
+        <v>17</v>
       </c>
       <c r="C36">
-        <v>0</v>
+        <v>1.96</v>
       </c>
       <c r="D36" t="s">
         <v>38</v>
@@ -1403,13 +1403,13 @@
     </row>
     <row r="37" spans="1:4">
       <c r="A37" s="2">
-        <v>46221</v>
+        <v>46228</v>
       </c>
       <c r="B37">
-        <v>4</v>
+        <v>18</v>
       </c>
       <c r="C37">
-        <v>0</v>
+        <v>1.367</v>
       </c>
       <c r="D37" t="s">
         <v>39</v>
@@ -1417,13 +1417,13 @@
     </row>
     <row r="38" spans="1:4">
       <c r="A38" s="2">
-        <v>46221</v>
+        <v>46228</v>
       </c>
       <c r="B38">
-        <v>5</v>
+        <v>19</v>
       </c>
       <c r="C38">
-        <v>0</v>
+        <v>0.863</v>
       </c>
       <c r="D38" t="s">
         <v>40</v>
@@ -1431,13 +1431,13 @@
     </row>
     <row r="39" spans="1:4">
       <c r="A39" s="2">
-        <v>46221</v>
+        <v>46228</v>
       </c>
       <c r="B39">
-        <v>6</v>
+        <v>20</v>
       </c>
       <c r="C39">
-        <v>0</v>
+        <v>0.282</v>
       </c>
       <c r="D39" t="s">
         <v>41</v>
@@ -1445,13 +1445,13 @@
     </row>
     <row r="40" spans="1:4">
       <c r="A40" s="2">
-        <v>46221</v>
+        <v>46228</v>
       </c>
       <c r="B40">
-        <v>7</v>
+        <v>21</v>
       </c>
       <c r="C40">
-        <v>0.07000000000000001</v>
+        <v>0.052</v>
       </c>
       <c r="D40" t="s">
         <v>42</v>
@@ -1459,13 +1459,13 @@
     </row>
     <row r="41" spans="1:4">
       <c r="A41" s="2">
-        <v>46221</v>
+        <v>46228</v>
       </c>
       <c r="B41">
-        <v>8</v>
+        <v>22</v>
       </c>
       <c r="C41">
-        <v>0.365</v>
+        <v>0</v>
       </c>
       <c r="D41" t="s">
         <v>43</v>
@@ -1473,13 +1473,13 @@
     </row>
     <row r="42" spans="1:4">
       <c r="A42" s="2">
-        <v>46221</v>
+        <v>46228</v>
       </c>
       <c r="B42">
-        <v>9</v>
+        <v>23</v>
       </c>
       <c r="C42">
-        <v>0.84</v>
+        <v>0</v>
       </c>
       <c r="D42" t="s">
         <v>44</v>
@@ -1487,13 +1487,13 @@
     </row>
     <row r="43" spans="1:4">
       <c r="A43" s="2">
-        <v>46221</v>
+        <v>46228</v>
       </c>
       <c r="B43">
-        <v>10</v>
+        <v>24</v>
       </c>
       <c r="C43">
-        <v>1.418</v>
+        <v>0</v>
       </c>
       <c r="D43" t="s">
         <v>45</v>
@@ -1501,13 +1501,13 @@
     </row>
     <row r="44" spans="1:4">
       <c r="A44" s="2">
-        <v>46221</v>
+        <v>46229</v>
       </c>
       <c r="B44">
-        <v>11</v>
+        <v>1</v>
       </c>
       <c r="C44">
-        <v>1.792</v>
+        <v>0</v>
       </c>
       <c r="D44" t="s">
         <v>46</v>
@@ -1515,13 +1515,13 @@
     </row>
     <row r="45" spans="1:4">
       <c r="A45" s="2">
-        <v>46221</v>
+        <v>46229</v>
       </c>
       <c r="B45">
-        <v>12</v>
+        <v>2</v>
       </c>
       <c r="C45">
-        <v>2.252</v>
+        <v>0</v>
       </c>
       <c r="D45" t="s">
         <v>47</v>
@@ -1529,13 +1529,13 @@
     </row>
     <row r="46" spans="1:4">
       <c r="A46" s="2">
-        <v>46221</v>
+        <v>46229</v>
       </c>
       <c r="B46">
-        <v>13</v>
+        <v>3</v>
       </c>
       <c r="C46">
-        <v>2.479</v>
+        <v>0</v>
       </c>
       <c r="D46" t="s">
         <v>48</v>
@@ -1543,13 +1543,13 @@
     </row>
     <row r="47" spans="1:4">
       <c r="A47" s="2">
-        <v>46221</v>
+        <v>46229</v>
       </c>
       <c r="B47">
-        <v>14</v>
+        <v>4</v>
       </c>
       <c r="C47">
-        <v>2.557</v>
+        <v>0</v>
       </c>
       <c r="D47" t="s">
         <v>49</v>
@@ -1557,13 +1557,13 @@
     </row>
     <row r="48" spans="1:4">
       <c r="A48" s="2">
-        <v>46221</v>
+        <v>46229</v>
       </c>
       <c r="B48">
-        <v>15</v>
+        <v>5</v>
       </c>
       <c r="C48">
-        <v>2.175</v>
+        <v>0</v>
       </c>
       <c r="D48" t="s">
         <v>50</v>
@@ -1571,13 +1571,13 @@
     </row>
     <row r="49" spans="1:4">
       <c r="A49" s="2">
-        <v>46221</v>
+        <v>46229</v>
       </c>
       <c r="B49">
-        <v>16</v>
+        <v>6</v>
       </c>
       <c r="C49">
-        <v>1.738</v>
+        <v>0</v>
       </c>
       <c r="D49" t="s">
         <v>51</v>
@@ -1585,13 +1585,13 @@
     </row>
     <row r="50" spans="1:4">
       <c r="A50" s="2">
-        <v>46221</v>
+        <v>46229</v>
       </c>
       <c r="B50">
-        <v>17</v>
+        <v>7</v>
       </c>
       <c r="C50">
-        <v>1.583</v>
+        <v>0.057</v>
       </c>
       <c r="D50" t="s">
         <v>52</v>
@@ -1599,13 +1599,13 @@
     </row>
     <row r="51" spans="1:4">
       <c r="A51" s="2">
-        <v>46221</v>
+        <v>46229</v>
       </c>
       <c r="B51">
-        <v>18</v>
+        <v>8</v>
       </c>
       <c r="C51">
-        <v>1.181</v>
+        <v>0.393</v>
       </c>
       <c r="D51" t="s">
         <v>53</v>
@@ -1613,13 +1613,13 @@
     </row>
     <row r="52" spans="1:4">
       <c r="A52" s="2">
-        <v>46221</v>
+        <v>46229</v>
       </c>
       <c r="B52">
-        <v>19</v>
+        <v>9</v>
       </c>
       <c r="C52">
-        <v>0.649</v>
+        <v>1.136</v>
       </c>
       <c r="D52" t="s">
         <v>54</v>
@@ -1627,13 +1627,13 @@
     </row>
     <row r="53" spans="1:4">
       <c r="A53" s="2">
-        <v>46221</v>
+        <v>46229</v>
       </c>
       <c r="B53">
-        <v>20</v>
+        <v>10</v>
       </c>
       <c r="C53">
-        <v>0.309</v>
+        <v>1.825</v>
       </c>
       <c r="D53" t="s">
         <v>55</v>
@@ -1641,13 +1641,13 @@
     </row>
     <row r="54" spans="1:4">
       <c r="A54" s="2">
-        <v>46221</v>
+        <v>46229</v>
       </c>
       <c r="B54">
-        <v>21</v>
+        <v>11</v>
       </c>
       <c r="C54">
-        <v>0.055</v>
+        <v>2.494</v>
       </c>
       <c r="D54" t="s">
         <v>56</v>
@@ -1655,13 +1655,13 @@
     </row>
     <row r="55" spans="1:4">
       <c r="A55" s="2">
-        <v>46221</v>
+        <v>46229</v>
       </c>
       <c r="B55">
-        <v>22</v>
+        <v>12</v>
       </c>
       <c r="C55">
-        <v>0</v>
+        <v>2.878</v>
       </c>
       <c r="D55" t="s">
         <v>57</v>
@@ -1669,13 +1669,13 @@
     </row>
     <row r="56" spans="1:4">
       <c r="A56" s="2">
-        <v>46221</v>
+        <v>46229</v>
       </c>
       <c r="B56">
-        <v>23</v>
+        <v>13</v>
       </c>
       <c r="C56">
-        <v>0</v>
+        <v>3.069</v>
       </c>
       <c r="D56" t="s">
         <v>58</v>
@@ -1683,13 +1683,13 @@
     </row>
     <row r="57" spans="1:4">
       <c r="A57" s="2">
-        <v>46221</v>
+        <v>46229</v>
       </c>
       <c r="B57">
-        <v>24</v>
+        <v>14</v>
       </c>
       <c r="C57">
-        <v>0</v>
+        <v>3.015</v>
       </c>
       <c r="D57" t="s">
         <v>59</v>
@@ -1697,13 +1697,13 @@
     </row>
     <row r="58" spans="1:4">
       <c r="A58" s="2">
-        <v>46222</v>
+        <v>46229</v>
       </c>
       <c r="B58">
-        <v>1</v>
+        <v>15</v>
       </c>
       <c r="C58">
-        <v>0</v>
+        <v>2.845</v>
       </c>
       <c r="D58" t="s">
         <v>60</v>
@@ -1711,13 +1711,13 @@
     </row>
     <row r="59" spans="1:4">
       <c r="A59" s="2">
-        <v>46222</v>
+        <v>46229</v>
       </c>
       <c r="B59">
-        <v>2</v>
+        <v>16</v>
       </c>
       <c r="C59">
-        <v>0</v>
+        <v>2.56</v>
       </c>
       <c r="D59" t="s">
         <v>61</v>
@@ -1725,13 +1725,13 @@
     </row>
     <row r="60" spans="1:4">
       <c r="A60" s="2">
-        <v>46222</v>
+        <v>46229</v>
       </c>
       <c r="B60">
-        <v>3</v>
+        <v>17</v>
       </c>
       <c r="C60">
-        <v>0</v>
+        <v>1.954</v>
       </c>
       <c r="D60" t="s">
         <v>62</v>
@@ -1739,13 +1739,13 @@
     </row>
     <row r="61" spans="1:4">
       <c r="A61" s="2">
-        <v>46222</v>
+        <v>46229</v>
       </c>
       <c r="B61">
-        <v>4</v>
+        <v>18</v>
       </c>
       <c r="C61">
-        <v>0</v>
+        <v>1.336</v>
       </c>
       <c r="D61" t="s">
         <v>63</v>
@@ -1753,13 +1753,13 @@
     </row>
     <row r="62" spans="1:4">
       <c r="A62" s="2">
-        <v>46222</v>
+        <v>46229</v>
       </c>
       <c r="B62">
-        <v>5</v>
+        <v>19</v>
       </c>
       <c r="C62">
-        <v>0</v>
+        <v>0.832</v>
       </c>
       <c r="D62" t="s">
         <v>64</v>
@@ -1767,13 +1767,13 @@
     </row>
     <row r="63" spans="1:4">
       <c r="A63" s="2">
-        <v>46222</v>
+        <v>46229</v>
       </c>
       <c r="B63">
-        <v>6</v>
+        <v>20</v>
       </c>
       <c r="C63">
-        <v>0</v>
+        <v>0.301</v>
       </c>
       <c r="D63" t="s">
         <v>65</v>
@@ -1781,13 +1781,13 @@
     </row>
     <row r="64" spans="1:4">
       <c r="A64" s="2">
-        <v>46222</v>
+        <v>46229</v>
       </c>
       <c r="B64">
-        <v>7</v>
+        <v>21</v>
       </c>
       <c r="C64">
-        <v>0.04</v>
+        <v>0.051</v>
       </c>
       <c r="D64" t="s">
         <v>66</v>
@@ -1795,13 +1795,13 @@
     </row>
     <row r="65" spans="1:4">
       <c r="A65" s="2">
-        <v>46222</v>
+        <v>46229</v>
       </c>
       <c r="B65">
-        <v>8</v>
+        <v>22</v>
       </c>
       <c r="C65">
-        <v>0.295</v>
+        <v>0</v>
       </c>
       <c r="D65" t="s">
         <v>67</v>
@@ -1809,13 +1809,13 @@
     </row>
     <row r="66" spans="1:4">
       <c r="A66" s="2">
-        <v>46222</v>
+        <v>46229</v>
       </c>
       <c r="B66">
-        <v>9</v>
+        <v>23</v>
       </c>
       <c r="C66">
-        <v>0.773</v>
+        <v>0</v>
       </c>
       <c r="D66" t="s">
         <v>68</v>
@@ -1823,13 +1823,13 @@
     </row>
     <row r="67" spans="1:4">
       <c r="A67" s="2">
-        <v>46222</v>
+        <v>46229</v>
       </c>
       <c r="B67">
-        <v>10</v>
+        <v>24</v>
       </c>
       <c r="C67">
-        <v>1.223</v>
+        <v>0</v>
       </c>
       <c r="D67" t="s">
         <v>69</v>
@@ -1837,13 +1837,13 @@
     </row>
     <row r="68" spans="1:4">
       <c r="A68" s="2">
-        <v>46222</v>
+        <v>46230</v>
       </c>
       <c r="B68">
-        <v>11</v>
+        <v>1</v>
       </c>
       <c r="C68">
-        <v>1.551</v>
+        <v>0</v>
       </c>
       <c r="D68" t="s">
         <v>70</v>
@@ -1851,13 +1851,13 @@
     </row>
     <row r="69" spans="1:4">
       <c r="A69" s="2">
-        <v>46222</v>
+        <v>46230</v>
       </c>
       <c r="B69">
-        <v>12</v>
+        <v>2</v>
       </c>
       <c r="C69">
-        <v>1.698</v>
+        <v>0</v>
       </c>
       <c r="D69" t="s">
         <v>71</v>
@@ -1865,13 +1865,13 @@
     </row>
     <row r="70" spans="1:4">
       <c r="A70" s="2">
-        <v>46222</v>
+        <v>46230</v>
       </c>
       <c r="B70">
-        <v>13</v>
+        <v>3</v>
       </c>
       <c r="C70">
-        <v>1.756</v>
+        <v>0</v>
       </c>
       <c r="D70" t="s">
         <v>72</v>
@@ -1879,13 +1879,13 @@
     </row>
     <row r="71" spans="1:4">
       <c r="A71" s="2">
-        <v>46222</v>
+        <v>46230</v>
       </c>
       <c r="B71">
-        <v>14</v>
+        <v>4</v>
       </c>
       <c r="C71">
-        <v>1.825</v>
+        <v>0</v>
       </c>
       <c r="D71" t="s">
         <v>73</v>
@@ -1893,13 +1893,13 @@
     </row>
     <row r="72" spans="1:4">
       <c r="A72" s="2">
-        <v>46222</v>
+        <v>46230</v>
       </c>
       <c r="B72">
-        <v>15</v>
+        <v>5</v>
       </c>
       <c r="C72">
-        <v>1.979</v>
+        <v>0</v>
       </c>
       <c r="D72" t="s">
         <v>74</v>
@@ -1907,13 +1907,13 @@
     </row>
     <row r="73" spans="1:4">
       <c r="A73" s="2">
-        <v>46222</v>
+        <v>46230</v>
       </c>
       <c r="B73">
-        <v>16</v>
+        <v>6</v>
       </c>
       <c r="C73">
-        <v>1.819</v>
+        <v>0</v>
       </c>
       <c r="D73" t="s">
         <v>75</v>
@@ -1921,13 +1921,13 @@
     </row>
     <row r="74" spans="1:4">
       <c r="A74" s="2">
-        <v>46222</v>
+        <v>46230</v>
       </c>
       <c r="B74">
-        <v>17</v>
+        <v>7</v>
       </c>
       <c r="C74">
-        <v>1.717</v>
+        <v>0.034</v>
       </c>
       <c r="D74" t="s">
         <v>76</v>
@@ -1935,13 +1935,13 @@
     </row>
     <row r="75" spans="1:4">
       <c r="A75" s="2">
-        <v>46222</v>
+        <v>46230</v>
       </c>
       <c r="B75">
-        <v>18</v>
+        <v>8</v>
       </c>
       <c r="C75">
-        <v>1.085</v>
+        <v>0.306</v>
       </c>
       <c r="D75" t="s">
         <v>77</v>
@@ -1949,13 +1949,13 @@
     </row>
     <row r="76" spans="1:4">
       <c r="A76" s="2">
-        <v>46222</v>
+        <v>46230</v>
       </c>
       <c r="B76">
-        <v>19</v>
+        <v>9</v>
       </c>
       <c r="C76">
-        <v>0.606</v>
+        <v>0.755</v>
       </c>
       <c r="D76" t="s">
         <v>78</v>
@@ -1963,13 +1963,13 @@
     </row>
     <row r="77" spans="1:4">
       <c r="A77" s="2">
-        <v>46222</v>
+        <v>46230</v>
       </c>
       <c r="B77">
-        <v>20</v>
+        <v>10</v>
       </c>
       <c r="C77">
-        <v>0.382</v>
+        <v>1.128</v>
       </c>
       <c r="D77" t="s">
         <v>79</v>
@@ -1977,13 +1977,13 @@
     </row>
     <row r="78" spans="1:4">
       <c r="A78" s="2">
-        <v>46222</v>
+        <v>46230</v>
       </c>
       <c r="B78">
-        <v>21</v>
+        <v>11</v>
       </c>
       <c r="C78">
-        <v>0.055</v>
+        <v>1.64</v>
       </c>
       <c r="D78" t="s">
         <v>80</v>
@@ -1991,13 +1991,13 @@
     </row>
     <row r="79" spans="1:4">
       <c r="A79" s="2">
-        <v>46222</v>
+        <v>46230</v>
       </c>
       <c r="B79">
-        <v>22</v>
+        <v>12</v>
       </c>
       <c r="C79">
-        <v>0</v>
+        <v>1.791</v>
       </c>
       <c r="D79" t="s">
         <v>81</v>
@@ -2005,13 +2005,13 @@
     </row>
     <row r="80" spans="1:4">
       <c r="A80" s="2">
-        <v>46222</v>
+        <v>46230</v>
       </c>
       <c r="B80">
-        <v>23</v>
+        <v>13</v>
       </c>
       <c r="C80">
-        <v>0</v>
+        <v>2.071</v>
       </c>
       <c r="D80" t="s">
         <v>82</v>
@@ -2019,13 +2019,13 @@
     </row>
     <row r="81" spans="1:4">
       <c r="A81" s="2">
-        <v>46222</v>
+        <v>46230</v>
       </c>
       <c r="B81">
-        <v>24</v>
+        <v>14</v>
       </c>
       <c r="C81">
-        <v>0</v>
+        <v>2.281</v>
       </c>
       <c r="D81" t="s">
         <v>83</v>
@@ -2033,13 +2033,13 @@
     </row>
     <row r="82" spans="1:4">
       <c r="A82" s="2">
-        <v>46223</v>
+        <v>46230</v>
       </c>
       <c r="B82">
-        <v>1</v>
+        <v>15</v>
       </c>
       <c r="C82">
-        <v>0</v>
+        <v>1.894</v>
       </c>
       <c r="D82" t="s">
         <v>84</v>
@@ -2047,13 +2047,13 @@
     </row>
     <row r="83" spans="1:4">
       <c r="A83" s="2">
-        <v>46223</v>
+        <v>46230</v>
       </c>
       <c r="B83">
-        <v>2</v>
+        <v>16</v>
       </c>
       <c r="C83">
-        <v>0</v>
+        <v>1.555</v>
       </c>
       <c r="D83" t="s">
         <v>85</v>
@@ -2061,13 +2061,13 @@
     </row>
     <row r="84" spans="1:4">
       <c r="A84" s="2">
-        <v>46223</v>
+        <v>46230</v>
       </c>
       <c r="B84">
-        <v>3</v>
+        <v>17</v>
       </c>
       <c r="C84">
-        <v>0</v>
+        <v>1.299</v>
       </c>
       <c r="D84" t="s">
         <v>86</v>
@@ -2075,13 +2075,13 @@
     </row>
     <row r="85" spans="1:4">
       <c r="A85" s="2">
-        <v>46223</v>
+        <v>46230</v>
       </c>
       <c r="B85">
-        <v>4</v>
+        <v>18</v>
       </c>
       <c r="C85">
-        <v>0</v>
+        <v>0.8129999999999999</v>
       </c>
       <c r="D85" t="s">
         <v>87</v>
@@ -2089,13 +2089,13 @@
     </row>
     <row r="86" spans="1:4">
       <c r="A86" s="2">
-        <v>46223</v>
+        <v>46230</v>
       </c>
       <c r="B86">
-        <v>5</v>
+        <v>19</v>
       </c>
       <c r="C86">
-        <v>0</v>
+        <v>0.498</v>
       </c>
       <c r="D86" t="s">
         <v>88</v>
@@ -2103,13 +2103,13 @@
     </row>
     <row r="87" spans="1:4">
       <c r="A87" s="2">
-        <v>46223</v>
+        <v>46230</v>
       </c>
       <c r="B87">
-        <v>6</v>
+        <v>20</v>
       </c>
       <c r="C87">
-        <v>0</v>
+        <v>0.219</v>
       </c>
       <c r="D87" t="s">
         <v>89</v>
@@ -2117,13 +2117,13 @@
     </row>
     <row r="88" spans="1:4">
       <c r="A88" s="2">
-        <v>46223</v>
+        <v>46230</v>
       </c>
       <c r="B88">
-        <v>7</v>
+        <v>21</v>
       </c>
       <c r="C88">
-        <v>0.049</v>
+        <v>0.036</v>
       </c>
       <c r="D88" t="s">
         <v>90</v>
@@ -2131,13 +2131,13 @@
     </row>
     <row r="89" spans="1:4">
       <c r="A89" s="2">
-        <v>46223</v>
+        <v>46230</v>
       </c>
       <c r="B89">
-        <v>8</v>
+        <v>22</v>
       </c>
       <c r="C89">
-        <v>0.359</v>
+        <v>0</v>
       </c>
       <c r="D89" t="s">
         <v>91</v>
@@ -2145,13 +2145,13 @@
     </row>
     <row r="90" spans="1:4">
       <c r="A90" s="2">
-        <v>46223</v>
+        <v>46230</v>
       </c>
       <c r="B90">
-        <v>9</v>
+        <v>23</v>
       </c>
       <c r="C90">
-        <v>0.8159999999999999</v>
+        <v>0</v>
       </c>
       <c r="D90" t="s">
         <v>92</v>
@@ -2159,13 +2159,13 @@
     </row>
     <row r="91" spans="1:4">
       <c r="A91" s="2">
-        <v>46223</v>
+        <v>46230</v>
       </c>
       <c r="B91">
-        <v>10</v>
+        <v>24</v>
       </c>
       <c r="C91">
-        <v>1.246</v>
+        <v>0</v>
       </c>
       <c r="D91" t="s">
         <v>93</v>
@@ -2173,13 +2173,13 @@
     </row>
     <row r="92" spans="1:4">
       <c r="A92" s="2">
-        <v>46223</v>
+        <v>46231</v>
       </c>
       <c r="B92">
-        <v>11</v>
+        <v>1</v>
       </c>
       <c r="C92">
-        <v>1.757</v>
+        <v>0</v>
       </c>
       <c r="D92" t="s">
         <v>94</v>
@@ -2187,13 +2187,13 @@
     </row>
     <row r="93" spans="1:4">
       <c r="A93" s="2">
-        <v>46223</v>
+        <v>46231</v>
       </c>
       <c r="B93">
-        <v>12</v>
+        <v>2</v>
       </c>
       <c r="C93">
-        <v>1.846</v>
+        <v>0</v>
       </c>
       <c r="D93" t="s">
         <v>95</v>
@@ -2201,13 +2201,13 @@
     </row>
     <row r="94" spans="1:4">
       <c r="A94" s="2">
-        <v>46223</v>
+        <v>46231</v>
       </c>
       <c r="B94">
-        <v>13</v>
+        <v>3</v>
       </c>
       <c r="C94">
-        <v>1.801</v>
+        <v>0</v>
       </c>
       <c r="D94" t="s">
         <v>96</v>
@@ -2215,13 +2215,13 @@
     </row>
     <row r="95" spans="1:4">
       <c r="A95" s="2">
-        <v>46223</v>
+        <v>46231</v>
       </c>
       <c r="B95">
-        <v>14</v>
+        <v>4</v>
       </c>
       <c r="C95">
-        <v>1.822</v>
+        <v>0</v>
       </c>
       <c r="D95" t="s">
         <v>97</v>
@@ -2229,13 +2229,13 @@
     </row>
     <row r="96" spans="1:4">
       <c r="A96" s="2">
-        <v>46223</v>
+        <v>46231</v>
       </c>
       <c r="B96">
-        <v>15</v>
+        <v>5</v>
       </c>
       <c r="C96">
-        <v>1.825</v>
+        <v>0</v>
       </c>
       <c r="D96" t="s">
         <v>98</v>
@@ -2243,13 +2243,13 @@
     </row>
     <row r="97" spans="1:4">
       <c r="A97" s="2">
-        <v>46223</v>
+        <v>46231</v>
       </c>
       <c r="B97">
-        <v>16</v>
+        <v>6</v>
       </c>
       <c r="C97">
-        <v>1.682</v>
+        <v>0</v>
       </c>
       <c r="D97" t="s">
         <v>99</v>
@@ -2257,13 +2257,13 @@
     </row>
     <row r="98" spans="1:4">
       <c r="A98" s="2">
-        <v>46223</v>
+        <v>46231</v>
       </c>
       <c r="B98">
-        <v>17</v>
+        <v>7</v>
       </c>
       <c r="C98">
-        <v>1.388</v>
+        <v>0.035</v>
       </c>
       <c r="D98" t="s">
         <v>100</v>
@@ -2271,13 +2271,13 @@
     </row>
     <row r="99" spans="1:4">
       <c r="A99" s="2">
-        <v>46223</v>
+        <v>46231</v>
       </c>
       <c r="B99">
-        <v>18</v>
+        <v>8</v>
       </c>
       <c r="C99">
-        <v>1.117</v>
+        <v>0.248</v>
       </c>
       <c r="D99" t="s">
         <v>101</v>
@@ -2285,13 +2285,13 @@
     </row>
     <row r="100" spans="1:4">
       <c r="A100" s="2">
-        <v>46223</v>
+        <v>46231</v>
       </c>
       <c r="B100">
-        <v>19</v>
+        <v>9</v>
       </c>
       <c r="C100">
-        <v>0.646</v>
+        <v>0.757</v>
       </c>
       <c r="D100" t="s">
         <v>102</v>
@@ -2299,13 +2299,13 @@
     </row>
     <row r="101" spans="1:4">
       <c r="A101" s="2">
-        <v>46223</v>
+        <v>46231</v>
       </c>
       <c r="B101">
-        <v>20</v>
+        <v>10</v>
       </c>
       <c r="C101">
-        <v>0.324</v>
+        <v>1.254</v>
       </c>
       <c r="D101" t="s">
         <v>103</v>
@@ -2313,13 +2313,13 @@
     </row>
     <row r="102" spans="1:4">
       <c r="A102" s="2">
-        <v>46223</v>
+        <v>46231</v>
       </c>
       <c r="B102">
-        <v>21</v>
+        <v>11</v>
       </c>
       <c r="C102">
-        <v>0.055</v>
+        <v>1.613</v>
       </c>
       <c r="D102" t="s">
         <v>104</v>
@@ -2327,13 +2327,13 @@
     </row>
     <row r="103" spans="1:4">
       <c r="A103" s="2">
-        <v>46223</v>
+        <v>46231</v>
       </c>
       <c r="B103">
-        <v>22</v>
+        <v>12</v>
       </c>
       <c r="C103">
-        <v>0</v>
+        <v>1.842</v>
       </c>
       <c r="D103" t="s">
         <v>105</v>
@@ -2341,13 +2341,13 @@
     </row>
     <row r="104" spans="1:4">
       <c r="A104" s="2">
-        <v>46223</v>
+        <v>46231</v>
       </c>
       <c r="B104">
-        <v>23</v>
+        <v>13</v>
       </c>
       <c r="C104">
-        <v>0</v>
+        <v>2.238</v>
       </c>
       <c r="D104" t="s">
         <v>106</v>
@@ -2355,13 +2355,13 @@
     </row>
     <row r="105" spans="1:4">
       <c r="A105" s="2">
-        <v>46223</v>
+        <v>46231</v>
       </c>
       <c r="B105">
-        <v>24</v>
+        <v>14</v>
       </c>
       <c r="C105">
-        <v>0</v>
+        <v>2.484</v>
       </c>
       <c r="D105" t="s">
         <v>107</v>
@@ -2369,13 +2369,13 @@
     </row>
     <row r="106" spans="1:4">
       <c r="A106" s="2">
-        <v>46224</v>
+        <v>46231</v>
       </c>
       <c r="B106">
-        <v>1</v>
+        <v>15</v>
       </c>
       <c r="C106">
-        <v>0</v>
+        <v>2.615</v>
       </c>
       <c r="D106" t="s">
         <v>108</v>
@@ -2383,13 +2383,13 @@
     </row>
     <row r="107" spans="1:4">
       <c r="A107" s="2">
-        <v>46224</v>
+        <v>46231</v>
       </c>
       <c r="B107">
-        <v>2</v>
+        <v>16</v>
       </c>
       <c r="C107">
-        <v>0</v>
+        <v>2.181</v>
       </c>
       <c r="D107" t="s">
         <v>109</v>
@@ -2397,13 +2397,13 @@
     </row>
     <row r="108" spans="1:4">
       <c r="A108" s="2">
-        <v>46224</v>
+        <v>46231</v>
       </c>
       <c r="B108">
-        <v>3</v>
+        <v>17</v>
       </c>
       <c r="C108">
-        <v>0</v>
+        <v>1.918</v>
       </c>
       <c r="D108" t="s">
         <v>110</v>
@@ -2411,13 +2411,13 @@
     </row>
     <row r="109" spans="1:4">
       <c r="A109" s="2">
-        <v>46224</v>
+        <v>46231</v>
       </c>
       <c r="B109">
-        <v>4</v>
+        <v>18</v>
       </c>
       <c r="C109">
-        <v>0</v>
+        <v>1.393</v>
       </c>
       <c r="D109" t="s">
         <v>111</v>
@@ -2425,13 +2425,13 @@
     </row>
     <row r="110" spans="1:4">
       <c r="A110" s="2">
-        <v>46224</v>
+        <v>46231</v>
       </c>
       <c r="B110">
-        <v>5</v>
+        <v>19</v>
       </c>
       <c r="C110">
-        <v>0</v>
+        <v>0.777</v>
       </c>
       <c r="D110" t="s">
         <v>112</v>
@@ -2439,13 +2439,13 @@
     </row>
     <row r="111" spans="1:4">
       <c r="A111" s="2">
-        <v>46224</v>
+        <v>46231</v>
       </c>
       <c r="B111">
-        <v>6</v>
+        <v>20</v>
       </c>
       <c r="C111">
-        <v>0</v>
+        <v>0.245</v>
       </c>
       <c r="D111" t="s">
         <v>113</v>
@@ -2453,13 +2453,13 @@
     </row>
     <row r="112" spans="1:4">
       <c r="A112" s="2">
-        <v>46224</v>
+        <v>46231</v>
       </c>
       <c r="B112">
-        <v>7</v>
+        <v>21</v>
       </c>
       <c r="C112">
-        <v>0.046</v>
+        <v>0.039</v>
       </c>
       <c r="D112" t="s">
         <v>114</v>
@@ -2467,13 +2467,13 @@
     </row>
     <row r="113" spans="1:4">
       <c r="A113" s="2">
-        <v>46224</v>
+        <v>46231</v>
       </c>
       <c r="B113">
-        <v>8</v>
+        <v>22</v>
       </c>
       <c r="C113">
-        <v>0.31</v>
+        <v>0</v>
       </c>
       <c r="D113" t="s">
         <v>115</v>
@@ -2481,13 +2481,13 @@
     </row>
     <row r="114" spans="1:4">
       <c r="A114" s="2">
-        <v>46224</v>
+        <v>46231</v>
       </c>
       <c r="B114">
-        <v>9</v>
+        <v>23</v>
       </c>
       <c r="C114">
-        <v>0.874</v>
+        <v>0</v>
       </c>
       <c r="D114" t="s">
         <v>116</v>
@@ -2495,13 +2495,13 @@
     </row>
     <row r="115" spans="1:4">
       <c r="A115" s="2">
-        <v>46224</v>
+        <v>46231</v>
       </c>
       <c r="B115">
-        <v>10</v>
+        <v>24</v>
       </c>
       <c r="C115">
-        <v>1.484</v>
+        <v>0</v>
       </c>
       <c r="D115" t="s">
         <v>117</v>
@@ -2509,13 +2509,13 @@
     </row>
     <row r="116" spans="1:4">
       <c r="A116" s="2">
-        <v>46224</v>
+        <v>46232</v>
       </c>
       <c r="B116">
-        <v>11</v>
+        <v>1</v>
       </c>
       <c r="C116">
-        <v>1.813</v>
+        <v>0</v>
       </c>
       <c r="D116" t="s">
         <v>118</v>
@@ -2523,13 +2523,13 @@
     </row>
     <row r="117" spans="1:4">
       <c r="A117" s="2">
-        <v>46224</v>
+        <v>46232</v>
       </c>
       <c r="B117">
-        <v>12</v>
+        <v>2</v>
       </c>
       <c r="C117">
-        <v>2.359</v>
+        <v>0</v>
       </c>
       <c r="D117" t="s">
         <v>119</v>
@@ -2537,13 +2537,13 @@
     </row>
     <row r="118" spans="1:4">
       <c r="A118" s="2">
-        <v>46224</v>
+        <v>46232</v>
       </c>
       <c r="B118">
-        <v>13</v>
+        <v>3</v>
       </c>
       <c r="C118">
-        <v>2.526</v>
+        <v>0</v>
       </c>
       <c r="D118" t="s">
         <v>120</v>
@@ -2551,13 +2551,13 @@
     </row>
     <row r="119" spans="1:4">
       <c r="A119" s="2">
-        <v>46224</v>
+        <v>46232</v>
       </c>
       <c r="B119">
-        <v>14</v>
+        <v>4</v>
       </c>
       <c r="C119">
-        <v>2.423</v>
+        <v>0</v>
       </c>
       <c r="D119" t="s">
         <v>121</v>
@@ -2565,13 +2565,13 @@
     </row>
     <row r="120" spans="1:4">
       <c r="A120" s="2">
-        <v>46224</v>
+        <v>46232</v>
       </c>
       <c r="B120">
-        <v>15</v>
+        <v>5</v>
       </c>
       <c r="C120">
-        <v>2.434</v>
+        <v>0</v>
       </c>
       <c r="D120" t="s">
         <v>122</v>
@@ -2579,13 +2579,13 @@
     </row>
     <row r="121" spans="1:4">
       <c r="A121" s="2">
-        <v>46224</v>
+        <v>46232</v>
       </c>
       <c r="B121">
-        <v>16</v>
+        <v>6</v>
       </c>
       <c r="C121">
-        <v>2.036</v>
+        <v>0</v>
       </c>
       <c r="D121" t="s">
         <v>123</v>
@@ -2593,13 +2593,13 @@
     </row>
     <row r="122" spans="1:4">
       <c r="A122" s="2">
-        <v>46224</v>
+        <v>46232</v>
       </c>
       <c r="B122">
-        <v>17</v>
+        <v>7</v>
       </c>
       <c r="C122">
-        <v>1.613</v>
+        <v>0.045</v>
       </c>
       <c r="D122" t="s">
         <v>124</v>
@@ -2607,13 +2607,13 @@
     </row>
     <row r="123" spans="1:4">
       <c r="A123" s="2">
-        <v>46224</v>
+        <v>46232</v>
       </c>
       <c r="B123">
-        <v>18</v>
+        <v>8</v>
       </c>
       <c r="C123">
-        <v>1.126</v>
+        <v>0.342</v>
       </c>
       <c r="D123" t="s">
         <v>125</v>
@@ -2621,13 +2621,13 @@
     </row>
     <row r="124" spans="1:4">
       <c r="A124" s="2">
-        <v>46224</v>
+        <v>46232</v>
       </c>
       <c r="B124">
-        <v>19</v>
+        <v>9</v>
       </c>
       <c r="C124">
-        <v>0.598</v>
+        <v>1.056</v>
       </c>
       <c r="D124" t="s">
         <v>126</v>
@@ -2635,13 +2635,13 @@
     </row>
     <row r="125" spans="1:4">
       <c r="A125" s="2">
-        <v>46224</v>
+        <v>46232</v>
       </c>
       <c r="B125">
-        <v>20</v>
+        <v>10</v>
       </c>
       <c r="C125">
-        <v>0.304</v>
+        <v>1.812</v>
       </c>
       <c r="D125" t="s">
         <v>127</v>
@@ -2649,13 +2649,13 @@
     </row>
     <row r="126" spans="1:4">
       <c r="A126" s="2">
-        <v>46224</v>
+        <v>46232</v>
       </c>
       <c r="B126">
-        <v>21</v>
+        <v>11</v>
       </c>
       <c r="C126">
-        <v>0.06</v>
+        <v>2.454</v>
       </c>
       <c r="D126" t="s">
         <v>128</v>
@@ -2663,13 +2663,13 @@
     </row>
     <row r="127" spans="1:4">
       <c r="A127" s="2">
-        <v>46224</v>
+        <v>46232</v>
       </c>
       <c r="B127">
-        <v>22</v>
+        <v>12</v>
       </c>
       <c r="C127">
-        <v>0</v>
+        <v>2.842</v>
       </c>
       <c r="D127" t="s">
         <v>129</v>
@@ -2677,13 +2677,13 @@
     </row>
     <row r="128" spans="1:4">
       <c r="A128" s="2">
-        <v>46224</v>
+        <v>46232</v>
       </c>
       <c r="B128">
-        <v>23</v>
+        <v>13</v>
       </c>
       <c r="C128">
-        <v>0</v>
+        <v>3.097</v>
       </c>
       <c r="D128" t="s">
         <v>130</v>
@@ -2691,13 +2691,13 @@
     </row>
     <row r="129" spans="1:4">
       <c r="A129" s="2">
-        <v>46224</v>
+        <v>46232</v>
       </c>
       <c r="B129">
-        <v>24</v>
+        <v>14</v>
       </c>
       <c r="C129">
-        <v>0</v>
+        <v>3.142</v>
       </c>
       <c r="D129" t="s">
         <v>131</v>
@@ -2705,13 +2705,13 @@
     </row>
     <row r="130" spans="1:4">
       <c r="A130" s="2">
-        <v>46225</v>
+        <v>46232</v>
       </c>
       <c r="B130">
-        <v>1</v>
+        <v>15</v>
       </c>
       <c r="C130">
-        <v>0</v>
+        <v>3.013</v>
       </c>
       <c r="D130" t="s">
         <v>132</v>
@@ -2719,13 +2719,13 @@
     </row>
     <row r="131" spans="1:4">
       <c r="A131" s="2">
-        <v>46225</v>
+        <v>46232</v>
       </c>
       <c r="B131">
-        <v>2</v>
+        <v>16</v>
       </c>
       <c r="C131">
-        <v>0</v>
+        <v>2.734</v>
       </c>
       <c r="D131" t="s">
         <v>133</v>
@@ -2733,13 +2733,13 @@
     </row>
     <row r="132" spans="1:4">
       <c r="A132" s="2">
-        <v>46225</v>
+        <v>46232</v>
       </c>
       <c r="B132">
-        <v>3</v>
+        <v>17</v>
       </c>
       <c r="C132">
-        <v>0</v>
+        <v>2.187</v>
       </c>
       <c r="D132" t="s">
         <v>134</v>
@@ -2747,13 +2747,13 @@
     </row>
     <row r="133" spans="1:4">
       <c r="A133" s="2">
-        <v>46225</v>
+        <v>46232</v>
       </c>
       <c r="B133">
-        <v>4</v>
+        <v>18</v>
       </c>
       <c r="C133">
-        <v>0</v>
+        <v>1.564</v>
       </c>
       <c r="D133" t="s">
         <v>135</v>
@@ -2761,13 +2761,13 @@
     </row>
     <row r="134" spans="1:4">
       <c r="A134" s="2">
-        <v>46225</v>
+        <v>46232</v>
       </c>
       <c r="B134">
-        <v>5</v>
+        <v>19</v>
       </c>
       <c r="C134">
-        <v>0</v>
+        <v>0.83</v>
       </c>
       <c r="D134" t="s">
         <v>136</v>
@@ -2775,13 +2775,13 @@
     </row>
     <row r="135" spans="1:4">
       <c r="A135" s="2">
-        <v>46225</v>
+        <v>46232</v>
       </c>
       <c r="B135">
-        <v>6</v>
+        <v>20</v>
       </c>
       <c r="C135">
-        <v>0</v>
+        <v>0.206</v>
       </c>
       <c r="D135" t="s">
         <v>137</v>
@@ -2789,13 +2789,13 @@
     </row>
     <row r="136" spans="1:4">
       <c r="A136" s="2">
-        <v>46225</v>
+        <v>46232</v>
       </c>
       <c r="B136">
-        <v>7</v>
+        <v>21</v>
       </c>
       <c r="C136">
-        <v>0.056</v>
+        <v>0.04</v>
       </c>
       <c r="D136" t="s">
         <v>138</v>
@@ -2803,13 +2803,13 @@
     </row>
     <row r="137" spans="1:4">
       <c r="A137" s="2">
-        <v>46225</v>
+        <v>46232</v>
       </c>
       <c r="B137">
-        <v>8</v>
+        <v>22</v>
       </c>
       <c r="C137">
-        <v>0.379</v>
+        <v>0</v>
       </c>
       <c r="D137" t="s">
         <v>139</v>
@@ -2817,13 +2817,13 @@
     </row>
     <row r="138" spans="1:4">
       <c r="A138" s="2">
-        <v>46225</v>
+        <v>46232</v>
       </c>
       <c r="B138">
-        <v>9</v>
+        <v>23</v>
       </c>
       <c r="C138">
-        <v>1.039</v>
+        <v>0</v>
       </c>
       <c r="D138" t="s">
         <v>140</v>
@@ -2831,13 +2831,13 @@
     </row>
     <row r="139" spans="1:4">
       <c r="A139" s="2">
-        <v>46225</v>
+        <v>46232</v>
       </c>
       <c r="B139">
-        <v>10</v>
+        <v>24</v>
       </c>
       <c r="C139">
-        <v>1.784</v>
+        <v>0</v>
       </c>
       <c r="D139" t="s">
         <v>141</v>
@@ -2845,13 +2845,13 @@
     </row>
     <row r="140" spans="1:4">
       <c r="A140" s="2">
-        <v>46225</v>
+        <v>46233</v>
       </c>
       <c r="B140">
-        <v>11</v>
+        <v>1</v>
       </c>
       <c r="C140">
-        <v>2.328</v>
+        <v>0</v>
       </c>
       <c r="D140" t="s">
         <v>142</v>
@@ -2859,13 +2859,13 @@
     </row>
     <row r="141" spans="1:4">
       <c r="A141" s="2">
-        <v>46225</v>
+        <v>46233</v>
       </c>
       <c r="B141">
-        <v>12</v>
+        <v>2</v>
       </c>
       <c r="C141">
-        <v>2.654</v>
+        <v>0</v>
       </c>
       <c r="D141" t="s">
         <v>143</v>
@@ -2873,13 +2873,13 @@
     </row>
     <row r="142" spans="1:4">
       <c r="A142" s="2">
-        <v>46225</v>
+        <v>46233</v>
       </c>
       <c r="B142">
-        <v>13</v>
+        <v>3</v>
       </c>
       <c r="C142">
-        <v>2.969</v>
+        <v>0</v>
       </c>
       <c r="D142" t="s">
         <v>144</v>
@@ -2887,13 +2887,13 @@
     </row>
     <row r="143" spans="1:4">
       <c r="A143" s="2">
-        <v>46225</v>
+        <v>46233</v>
       </c>
       <c r="B143">
-        <v>14</v>
+        <v>4</v>
       </c>
       <c r="C143">
-        <v>2.993</v>
+        <v>0</v>
       </c>
       <c r="D143" t="s">
         <v>145</v>
@@ -2901,13 +2901,13 @@
     </row>
     <row r="144" spans="1:4">
       <c r="A144" s="2">
-        <v>46225</v>
+        <v>46233</v>
       </c>
       <c r="B144">
-        <v>15</v>
+        <v>5</v>
       </c>
       <c r="C144">
-        <v>2.86</v>
+        <v>0</v>
       </c>
       <c r="D144" t="s">
         <v>146</v>
@@ -2915,13 +2915,13 @@
     </row>
     <row r="145" spans="1:4">
       <c r="A145" s="2">
-        <v>46225</v>
+        <v>46233</v>
       </c>
       <c r="B145">
-        <v>16</v>
+        <v>6</v>
       </c>
       <c r="C145">
-        <v>2.586</v>
+        <v>0</v>
       </c>
       <c r="D145" t="s">
         <v>147</v>
@@ -2929,13 +2929,13 @@
     </row>
     <row r="146" spans="1:4">
       <c r="A146" s="2">
-        <v>46225</v>
+        <v>46233</v>
       </c>
       <c r="B146">
-        <v>17</v>
+        <v>7</v>
       </c>
       <c r="C146">
-        <v>2.14</v>
+        <v>0.047</v>
       </c>
       <c r="D146" t="s">
         <v>148</v>
@@ -2943,13 +2943,13 @@
     </row>
     <row r="147" spans="1:4">
       <c r="A147" s="2">
-        <v>46225</v>
+        <v>46233</v>
       </c>
       <c r="B147">
-        <v>18</v>
+        <v>8</v>
       </c>
       <c r="C147">
-        <v>1.427</v>
+        <v>0.376</v>
       </c>
       <c r="D147" t="s">
         <v>149</v>
@@ -2957,13 +2957,13 @@
     </row>
     <row r="148" spans="1:4">
       <c r="A148" s="2">
-        <v>46225</v>
+        <v>46233</v>
       </c>
       <c r="B148">
-        <v>19</v>
+        <v>9</v>
       </c>
       <c r="C148">
-        <v>0.888</v>
+        <v>1.035</v>
       </c>
       <c r="D148" t="s">
         <v>150</v>
@@ -2971,13 +2971,13 @@
     </row>
     <row r="149" spans="1:4">
       <c r="A149" s="2">
-        <v>46225</v>
+        <v>46233</v>
       </c>
       <c r="B149">
-        <v>20</v>
+        <v>10</v>
       </c>
       <c r="C149">
-        <v>0.295</v>
+        <v>1.74</v>
       </c>
       <c r="D149" t="s">
         <v>151</v>
@@ -2985,13 +2985,13 @@
     </row>
     <row r="150" spans="1:4">
       <c r="A150" s="2">
-        <v>46225</v>
+        <v>46233</v>
       </c>
       <c r="B150">
-        <v>21</v>
+        <v>11</v>
       </c>
       <c r="C150">
-        <v>0.053</v>
+        <v>2.336</v>
       </c>
       <c r="D150" t="s">
         <v>152</v>
@@ -2999,13 +2999,13 @@
     </row>
     <row r="151" spans="1:4">
       <c r="A151" s="2">
-        <v>46225</v>
+        <v>46233</v>
       </c>
       <c r="B151">
-        <v>22</v>
+        <v>12</v>
       </c>
       <c r="C151">
-        <v>0</v>
+        <v>2.639</v>
       </c>
       <c r="D151" t="s">
         <v>153</v>
@@ -3013,13 +3013,13 @@
     </row>
     <row r="152" spans="1:4">
       <c r="A152" s="2">
-        <v>46225</v>
+        <v>46233</v>
       </c>
       <c r="B152">
-        <v>23</v>
+        <v>13</v>
       </c>
       <c r="C152">
-        <v>0</v>
+        <v>2.851</v>
       </c>
       <c r="D152" t="s">
         <v>154</v>
@@ -3027,13 +3027,13 @@
     </row>
     <row r="153" spans="1:4">
       <c r="A153" s="2">
-        <v>46225</v>
+        <v>46233</v>
       </c>
       <c r="B153">
-        <v>24</v>
+        <v>14</v>
       </c>
       <c r="C153">
-        <v>0</v>
+        <v>2.955</v>
       </c>
       <c r="D153" t="s">
         <v>155</v>
@@ -3041,13 +3041,13 @@
     </row>
     <row r="154" spans="1:4">
       <c r="A154" s="2">
-        <v>46226</v>
+        <v>46233</v>
       </c>
       <c r="B154">
-        <v>1</v>
+        <v>15</v>
       </c>
       <c r="C154">
-        <v>0</v>
+        <v>2.786</v>
       </c>
       <c r="D154" t="s">
         <v>156</v>
@@ -3055,13 +3055,13 @@
     </row>
     <row r="155" spans="1:4">
       <c r="A155" s="2">
-        <v>46226</v>
+        <v>46233</v>
       </c>
       <c r="B155">
-        <v>2</v>
+        <v>16</v>
       </c>
       <c r="C155">
-        <v>0</v>
+        <v>2.474</v>
       </c>
       <c r="D155" t="s">
         <v>157</v>
@@ -3069,13 +3069,13 @@
     </row>
     <row r="156" spans="1:4">
       <c r="A156" s="2">
-        <v>46226</v>
+        <v>46233</v>
       </c>
       <c r="B156">
-        <v>3</v>
+        <v>17</v>
       </c>
       <c r="C156">
-        <v>0</v>
+        <v>2.016</v>
       </c>
       <c r="D156" t="s">
         <v>158</v>
@@ -3083,13 +3083,13 @@
     </row>
     <row r="157" spans="1:4">
       <c r="A157" s="2">
-        <v>46226</v>
+        <v>46233</v>
       </c>
       <c r="B157">
-        <v>4</v>
+        <v>18</v>
       </c>
       <c r="C157">
-        <v>0</v>
+        <v>1.473</v>
       </c>
       <c r="D157" t="s">
         <v>159</v>
@@ -3097,13 +3097,13 @@
     </row>
     <row r="158" spans="1:4">
       <c r="A158" s="2">
-        <v>46226</v>
+        <v>46233</v>
       </c>
       <c r="B158">
-        <v>5</v>
+        <v>19</v>
       </c>
       <c r="C158">
-        <v>0</v>
+        <v>0.773</v>
       </c>
       <c r="D158" t="s">
         <v>160</v>
@@ -3111,13 +3111,13 @@
     </row>
     <row r="159" spans="1:4">
       <c r="A159" s="2">
-        <v>46226</v>
+        <v>46233</v>
       </c>
       <c r="B159">
-        <v>6</v>
+        <v>20</v>
       </c>
       <c r="C159">
-        <v>0</v>
+        <v>0.215</v>
       </c>
       <c r="D159" t="s">
         <v>161</v>
@@ -3125,13 +3125,13 @@
     </row>
     <row r="160" spans="1:4">
       <c r="A160" s="2">
-        <v>46226</v>
+        <v>46233</v>
       </c>
       <c r="B160">
-        <v>7</v>
+        <v>21</v>
       </c>
       <c r="C160">
-        <v>0.065</v>
+        <v>0.042</v>
       </c>
       <c r="D160" t="s">
         <v>162</v>
@@ -3139,13 +3139,13 @@
     </row>
     <row r="161" spans="1:4">
       <c r="A161" s="2">
-        <v>46226</v>
+        <v>46233</v>
       </c>
       <c r="B161">
-        <v>8</v>
+        <v>22</v>
       </c>
       <c r="C161">
-        <v>0.39</v>
+        <v>0</v>
       </c>
       <c r="D161" t="s">
         <v>163</v>
@@ -3153,13 +3153,13 @@
     </row>
     <row r="162" spans="1:4">
       <c r="A162" s="2">
-        <v>46226</v>
+        <v>46233</v>
       </c>
       <c r="B162">
-        <v>9</v>
+        <v>23</v>
       </c>
       <c r="C162">
-        <v>1.071</v>
+        <v>0</v>
       </c>
       <c r="D162" t="s">
         <v>164</v>
@@ -3167,13 +3167,13 @@
     </row>
     <row r="163" spans="1:4">
       <c r="A163" s="2">
-        <v>46226</v>
+        <v>46233</v>
       </c>
       <c r="B163">
-        <v>10</v>
+        <v>24</v>
       </c>
       <c r="C163">
-        <v>1.669</v>
+        <v>0</v>
       </c>
       <c r="D163" t="s">
         <v>165</v>
@@ -3181,13 +3181,13 @@
     </row>
     <row r="164" spans="1:4">
       <c r="A164" s="2">
-        <v>46226</v>
+        <v>46234</v>
       </c>
       <c r="B164">
-        <v>11</v>
+        <v>1</v>
       </c>
       <c r="C164">
-        <v>1.926</v>
+        <v>0</v>
       </c>
       <c r="D164" t="s">
         <v>166</v>
@@ -3195,13 +3195,13 @@
     </row>
     <row r="165" spans="1:4">
       <c r="A165" s="2">
-        <v>46226</v>
+        <v>46234</v>
       </c>
       <c r="B165">
-        <v>12</v>
+        <v>2</v>
       </c>
       <c r="C165">
-        <v>2.258</v>
+        <v>0</v>
       </c>
       <c r="D165" t="s">
         <v>167</v>
@@ -3209,13 +3209,13 @@
     </row>
     <row r="166" spans="1:4">
       <c r="A166" s="2">
-        <v>46226</v>
+        <v>46234</v>
       </c>
       <c r="B166">
-        <v>13</v>
+        <v>3</v>
       </c>
       <c r="C166">
-        <v>2.358</v>
+        <v>0</v>
       </c>
       <c r="D166" t="s">
         <v>168</v>
@@ -3223,13 +3223,13 @@
     </row>
     <row r="167" spans="1:4">
       <c r="A167" s="2">
-        <v>46226</v>
+        <v>46234</v>
       </c>
       <c r="B167">
-        <v>14</v>
+        <v>4</v>
       </c>
       <c r="C167">
-        <v>2.356</v>
+        <v>0</v>
       </c>
       <c r="D167" t="s">
         <v>169</v>
@@ -3237,13 +3237,13 @@
     </row>
     <row r="168" spans="1:4">
       <c r="A168" s="2">
-        <v>46226</v>
+        <v>46234</v>
       </c>
       <c r="B168">
-        <v>15</v>
+        <v>5</v>
       </c>
       <c r="C168">
-        <v>2.22</v>
+        <v>0</v>
       </c>
       <c r="D168" t="s">
         <v>170</v>
@@ -3251,13 +3251,13 @@
     </row>
     <row r="169" spans="1:4">
       <c r="A169" s="2">
-        <v>46226</v>
+        <v>46234</v>
       </c>
       <c r="B169">
-        <v>16</v>
+        <v>6</v>
       </c>
       <c r="C169">
-        <v>1.772</v>
+        <v>0</v>
       </c>
       <c r="D169" t="s">
         <v>171</v>
@@ -3265,13 +3265,13 @@
     </row>
     <row r="170" spans="1:4">
       <c r="A170" s="2">
-        <v>46226</v>
+        <v>46234</v>
       </c>
       <c r="B170">
-        <v>17</v>
+        <v>7</v>
       </c>
       <c r="C170">
-        <v>1.577</v>
+        <v>0.043</v>
       </c>
       <c r="D170" t="s">
         <v>172</v>

</xml_diff>

<commit_message>
Adding the HNG model to the p[ortfolio forecast
</commit_message>
<xml_diff>
--- a/Astro/Results_Production_Astro_xgb.xlsx
+++ b/Astro/Results_Production_Astro_xgb.xlsx
@@ -28,21 +28,6 @@
     <t>Lookup</t>
   </si>
   <si>
-    <t>24.07.20267</t>
-  </si>
-  <si>
-    <t>24.07.20268</t>
-  </si>
-  <si>
-    <t>24.07.20269</t>
-  </si>
-  <si>
-    <t>24.07.202610</t>
-  </si>
-  <si>
-    <t>24.07.202611</t>
-  </si>
-  <si>
     <t>24.07.202612</t>
   </si>
   <si>
@@ -533,6 +518,21 @@
   </si>
   <si>
     <t>31.07.20267</t>
+  </si>
+  <si>
+    <t>31.07.20268</t>
+  </si>
+  <si>
+    <t>31.07.20269</t>
+  </si>
+  <si>
+    <t>31.07.202610</t>
+  </si>
+  <si>
+    <t>31.07.202611</t>
+  </si>
+  <si>
+    <t>31.07.202612</t>
   </si>
 </sst>
 </file>
@@ -916,7 +916,7 @@
         <v>46227</v>
       </c>
       <c r="B2">
-        <v>7</v>
+        <v>12</v>
       </c>
       <c r="C2">
         <v>0</v>
@@ -930,7 +930,7 @@
         <v>46227</v>
       </c>
       <c r="B3">
-        <v>8</v>
+        <v>13</v>
       </c>
       <c r="C3">
         <v>0</v>
@@ -944,10 +944,10 @@
         <v>46227</v>
       </c>
       <c r="B4">
-        <v>9</v>
+        <v>14</v>
       </c>
       <c r="C4">
-        <v>1.116</v>
+        <v>2.235</v>
       </c>
       <c r="D4" t="s">
         <v>6</v>
@@ -958,10 +958,10 @@
         <v>46227</v>
       </c>
       <c r="B5">
-        <v>10</v>
+        <v>15</v>
       </c>
       <c r="C5">
-        <v>1.909</v>
+        <v>1.846</v>
       </c>
       <c r="D5" t="s">
         <v>7</v>
@@ -972,10 +972,10 @@
         <v>46227</v>
       </c>
       <c r="B6">
-        <v>11</v>
+        <v>16</v>
       </c>
       <c r="C6">
-        <v>2.225</v>
+        <v>1.81</v>
       </c>
       <c r="D6" t="s">
         <v>8</v>
@@ -986,10 +986,10 @@
         <v>46227</v>
       </c>
       <c r="B7">
-        <v>12</v>
+        <v>17</v>
       </c>
       <c r="C7">
-        <v>2.444</v>
+        <v>1.721</v>
       </c>
       <c r="D7" t="s">
         <v>9</v>
@@ -1000,10 +1000,10 @@
         <v>46227</v>
       </c>
       <c r="B8">
-        <v>13</v>
+        <v>18</v>
       </c>
       <c r="C8">
-        <v>2.401</v>
+        <v>1.186</v>
       </c>
       <c r="D8" t="s">
         <v>10</v>
@@ -1014,10 +1014,10 @@
         <v>46227</v>
       </c>
       <c r="B9">
-        <v>14</v>
+        <v>19</v>
       </c>
       <c r="C9">
-        <v>2.375</v>
+        <v>0.593</v>
       </c>
       <c r="D9" t="s">
         <v>11</v>
@@ -1028,10 +1028,10 @@
         <v>46227</v>
       </c>
       <c r="B10">
-        <v>15</v>
+        <v>20</v>
       </c>
       <c r="C10">
-        <v>2.132</v>
+        <v>0.302</v>
       </c>
       <c r="D10" t="s">
         <v>12</v>
@@ -1042,10 +1042,10 @@
         <v>46227</v>
       </c>
       <c r="B11">
-        <v>16</v>
+        <v>21</v>
       </c>
       <c r="C11">
-        <v>1.857</v>
+        <v>0.05</v>
       </c>
       <c r="D11" t="s">
         <v>13</v>
@@ -1056,10 +1056,10 @@
         <v>46227</v>
       </c>
       <c r="B12">
-        <v>17</v>
+        <v>22</v>
       </c>
       <c r="C12">
-        <v>1.719</v>
+        <v>0</v>
       </c>
       <c r="D12" t="s">
         <v>14</v>
@@ -1070,10 +1070,10 @@
         <v>46227</v>
       </c>
       <c r="B13">
-        <v>18</v>
+        <v>23</v>
       </c>
       <c r="C13">
-        <v>1.145</v>
+        <v>0</v>
       </c>
       <c r="D13" t="s">
         <v>15</v>
@@ -1084,10 +1084,10 @@
         <v>46227</v>
       </c>
       <c r="B14">
-        <v>19</v>
+        <v>24</v>
       </c>
       <c r="C14">
-        <v>0.648</v>
+        <v>0</v>
       </c>
       <c r="D14" t="s">
         <v>16</v>
@@ -1095,13 +1095,13 @@
     </row>
     <row r="15" spans="1:4">
       <c r="A15" s="2">
-        <v>46227</v>
+        <v>46228</v>
       </c>
       <c r="B15">
-        <v>20</v>
+        <v>1</v>
       </c>
       <c r="C15">
-        <v>0.306</v>
+        <v>0</v>
       </c>
       <c r="D15" t="s">
         <v>17</v>
@@ -1109,13 +1109,13 @@
     </row>
     <row r="16" spans="1:4">
       <c r="A16" s="2">
-        <v>46227</v>
+        <v>46228</v>
       </c>
       <c r="B16">
-        <v>21</v>
+        <v>2</v>
       </c>
       <c r="C16">
-        <v>0.066</v>
+        <v>0</v>
       </c>
       <c r="D16" t="s">
         <v>18</v>
@@ -1123,10 +1123,10 @@
     </row>
     <row r="17" spans="1:4">
       <c r="A17" s="2">
-        <v>46227</v>
+        <v>46228</v>
       </c>
       <c r="B17">
-        <v>22</v>
+        <v>3</v>
       </c>
       <c r="C17">
         <v>0</v>
@@ -1137,10 +1137,10 @@
     </row>
     <row r="18" spans="1:4">
       <c r="A18" s="2">
-        <v>46227</v>
+        <v>46228</v>
       </c>
       <c r="B18">
-        <v>23</v>
+        <v>4</v>
       </c>
       <c r="C18">
         <v>0</v>
@@ -1151,10 +1151,10 @@
     </row>
     <row r="19" spans="1:4">
       <c r="A19" s="2">
-        <v>46227</v>
+        <v>46228</v>
       </c>
       <c r="B19">
-        <v>24</v>
+        <v>5</v>
       </c>
       <c r="C19">
         <v>0</v>
@@ -1168,7 +1168,7 @@
         <v>46228</v>
       </c>
       <c r="B20">
-        <v>1</v>
+        <v>6</v>
       </c>
       <c r="C20">
         <v>0</v>
@@ -1182,10 +1182,10 @@
         <v>46228</v>
       </c>
       <c r="B21">
-        <v>2</v>
+        <v>7</v>
       </c>
       <c r="C21">
-        <v>0</v>
+        <v>0.055</v>
       </c>
       <c r="D21" t="s">
         <v>23</v>
@@ -1196,10 +1196,10 @@
         <v>46228</v>
       </c>
       <c r="B22">
-        <v>3</v>
+        <v>8</v>
       </c>
       <c r="C22">
-        <v>0</v>
+        <v>0.371</v>
       </c>
       <c r="D22" t="s">
         <v>24</v>
@@ -1210,10 +1210,10 @@
         <v>46228</v>
       </c>
       <c r="B23">
-        <v>4</v>
+        <v>9</v>
       </c>
       <c r="C23">
-        <v>0</v>
+        <v>1.094</v>
       </c>
       <c r="D23" t="s">
         <v>25</v>
@@ -1224,10 +1224,10 @@
         <v>46228</v>
       </c>
       <c r="B24">
-        <v>5</v>
+        <v>10</v>
       </c>
       <c r="C24">
-        <v>0</v>
+        <v>1.863</v>
       </c>
       <c r="D24" t="s">
         <v>26</v>
@@ -1238,10 +1238,10 @@
         <v>46228</v>
       </c>
       <c r="B25">
-        <v>6</v>
+        <v>11</v>
       </c>
       <c r="C25">
-        <v>0</v>
+        <v>2.277</v>
       </c>
       <c r="D25" t="s">
         <v>27</v>
@@ -1252,10 +1252,10 @@
         <v>46228</v>
       </c>
       <c r="B26">
-        <v>7</v>
+        <v>12</v>
       </c>
       <c r="C26">
-        <v>0.059</v>
+        <v>2.426</v>
       </c>
       <c r="D26" t="s">
         <v>28</v>
@@ -1266,10 +1266,10 @@
         <v>46228</v>
       </c>
       <c r="B27">
-        <v>8</v>
+        <v>13</v>
       </c>
       <c r="C27">
-        <v>0.372</v>
+        <v>2.655</v>
       </c>
       <c r="D27" t="s">
         <v>29</v>
@@ -1280,10 +1280,10 @@
         <v>46228</v>
       </c>
       <c r="B28">
-        <v>9</v>
+        <v>14</v>
       </c>
       <c r="C28">
-        <v>1.095</v>
+        <v>2.7</v>
       </c>
       <c r="D28" t="s">
         <v>30</v>
@@ -1294,10 +1294,10 @@
         <v>46228</v>
       </c>
       <c r="B29">
-        <v>10</v>
+        <v>15</v>
       </c>
       <c r="C29">
-        <v>1.84</v>
+        <v>2.641</v>
       </c>
       <c r="D29" t="s">
         <v>31</v>
@@ -1308,10 +1308,10 @@
         <v>46228</v>
       </c>
       <c r="B30">
-        <v>11</v>
+        <v>16</v>
       </c>
       <c r="C30">
-        <v>2.311</v>
+        <v>2.206</v>
       </c>
       <c r="D30" t="s">
         <v>32</v>
@@ -1322,10 +1322,10 @@
         <v>46228</v>
       </c>
       <c r="B31">
-        <v>12</v>
+        <v>17</v>
       </c>
       <c r="C31">
-        <v>2.444</v>
+        <v>1.918</v>
       </c>
       <c r="D31" t="s">
         <v>33</v>
@@ -1336,10 +1336,10 @@
         <v>46228</v>
       </c>
       <c r="B32">
-        <v>13</v>
+        <v>18</v>
       </c>
       <c r="C32">
-        <v>2.695</v>
+        <v>1.351</v>
       </c>
       <c r="D32" t="s">
         <v>34</v>
@@ -1350,10 +1350,10 @@
         <v>46228</v>
       </c>
       <c r="B33">
-        <v>14</v>
+        <v>19</v>
       </c>
       <c r="C33">
-        <v>2.715</v>
+        <v>0.757</v>
       </c>
       <c r="D33" t="s">
         <v>35</v>
@@ -1364,10 +1364,10 @@
         <v>46228</v>
       </c>
       <c r="B34">
-        <v>15</v>
+        <v>20</v>
       </c>
       <c r="C34">
-        <v>2.632</v>
+        <v>0.262</v>
       </c>
       <c r="D34" t="s">
         <v>36</v>
@@ -1378,10 +1378,10 @@
         <v>46228</v>
       </c>
       <c r="B35">
-        <v>16</v>
+        <v>21</v>
       </c>
       <c r="C35">
-        <v>2.204</v>
+        <v>0.06</v>
       </c>
       <c r="D35" t="s">
         <v>37</v>
@@ -1392,10 +1392,10 @@
         <v>46228</v>
       </c>
       <c r="B36">
-        <v>17</v>
+        <v>22</v>
       </c>
       <c r="C36">
-        <v>1.96</v>
+        <v>0</v>
       </c>
       <c r="D36" t="s">
         <v>38</v>
@@ -1406,10 +1406,10 @@
         <v>46228</v>
       </c>
       <c r="B37">
-        <v>18</v>
+        <v>23</v>
       </c>
       <c r="C37">
-        <v>1.367</v>
+        <v>0</v>
       </c>
       <c r="D37" t="s">
         <v>39</v>
@@ -1420,10 +1420,10 @@
         <v>46228</v>
       </c>
       <c r="B38">
-        <v>19</v>
+        <v>24</v>
       </c>
       <c r="C38">
-        <v>0.863</v>
+        <v>0</v>
       </c>
       <c r="D38" t="s">
         <v>40</v>
@@ -1431,13 +1431,13 @@
     </row>
     <row r="39" spans="1:4">
       <c r="A39" s="2">
-        <v>46228</v>
+        <v>46229</v>
       </c>
       <c r="B39">
-        <v>20</v>
+        <v>1</v>
       </c>
       <c r="C39">
-        <v>0.282</v>
+        <v>0</v>
       </c>
       <c r="D39" t="s">
         <v>41</v>
@@ -1445,13 +1445,13 @@
     </row>
     <row r="40" spans="1:4">
       <c r="A40" s="2">
-        <v>46228</v>
+        <v>46229</v>
       </c>
       <c r="B40">
-        <v>21</v>
+        <v>2</v>
       </c>
       <c r="C40">
-        <v>0.052</v>
+        <v>0</v>
       </c>
       <c r="D40" t="s">
         <v>42</v>
@@ -1459,10 +1459,10 @@
     </row>
     <row r="41" spans="1:4">
       <c r="A41" s="2">
-        <v>46228</v>
+        <v>46229</v>
       </c>
       <c r="B41">
-        <v>22</v>
+        <v>3</v>
       </c>
       <c r="C41">
         <v>0</v>
@@ -1473,10 +1473,10 @@
     </row>
     <row r="42" spans="1:4">
       <c r="A42" s="2">
-        <v>46228</v>
+        <v>46229</v>
       </c>
       <c r="B42">
-        <v>23</v>
+        <v>4</v>
       </c>
       <c r="C42">
         <v>0</v>
@@ -1487,10 +1487,10 @@
     </row>
     <row r="43" spans="1:4">
       <c r="A43" s="2">
-        <v>46228</v>
+        <v>46229</v>
       </c>
       <c r="B43">
-        <v>24</v>
+        <v>5</v>
       </c>
       <c r="C43">
         <v>0</v>
@@ -1504,7 +1504,7 @@
         <v>46229</v>
       </c>
       <c r="B44">
-        <v>1</v>
+        <v>6</v>
       </c>
       <c r="C44">
         <v>0</v>
@@ -1518,10 +1518,10 @@
         <v>46229</v>
       </c>
       <c r="B45">
-        <v>2</v>
+        <v>7</v>
       </c>
       <c r="C45">
-        <v>0</v>
+        <v>0.056</v>
       </c>
       <c r="D45" t="s">
         <v>47</v>
@@ -1532,10 +1532,10 @@
         <v>46229</v>
       </c>
       <c r="B46">
-        <v>3</v>
+        <v>8</v>
       </c>
       <c r="C46">
-        <v>0</v>
+        <v>0.356</v>
       </c>
       <c r="D46" t="s">
         <v>48</v>
@@ -1546,10 +1546,10 @@
         <v>46229</v>
       </c>
       <c r="B47">
-        <v>4</v>
+        <v>9</v>
       </c>
       <c r="C47">
-        <v>0</v>
+        <v>1.113</v>
       </c>
       <c r="D47" t="s">
         <v>49</v>
@@ -1560,10 +1560,10 @@
         <v>46229</v>
       </c>
       <c r="B48">
-        <v>5</v>
+        <v>10</v>
       </c>
       <c r="C48">
-        <v>0</v>
+        <v>1.864</v>
       </c>
       <c r="D48" t="s">
         <v>50</v>
@@ -1574,10 +1574,10 @@
         <v>46229</v>
       </c>
       <c r="B49">
-        <v>6</v>
+        <v>11</v>
       </c>
       <c r="C49">
-        <v>0</v>
+        <v>2.487</v>
       </c>
       <c r="D49" t="s">
         <v>51</v>
@@ -1588,10 +1588,10 @@
         <v>46229</v>
       </c>
       <c r="B50">
-        <v>7</v>
+        <v>12</v>
       </c>
       <c r="C50">
-        <v>0.057</v>
+        <v>2.846</v>
       </c>
       <c r="D50" t="s">
         <v>52</v>
@@ -1602,10 +1602,10 @@
         <v>46229</v>
       </c>
       <c r="B51">
-        <v>8</v>
+        <v>13</v>
       </c>
       <c r="C51">
-        <v>0.393</v>
+        <v>3.02</v>
       </c>
       <c r="D51" t="s">
         <v>53</v>
@@ -1616,10 +1616,10 @@
         <v>46229</v>
       </c>
       <c r="B52">
-        <v>9</v>
+        <v>14</v>
       </c>
       <c r="C52">
-        <v>1.136</v>
+        <v>2.996</v>
       </c>
       <c r="D52" t="s">
         <v>54</v>
@@ -1630,10 +1630,10 @@
         <v>46229</v>
       </c>
       <c r="B53">
-        <v>10</v>
+        <v>15</v>
       </c>
       <c r="C53">
-        <v>1.825</v>
+        <v>2.903</v>
       </c>
       <c r="D53" t="s">
         <v>55</v>
@@ -1644,10 +1644,10 @@
         <v>46229</v>
       </c>
       <c r="B54">
-        <v>11</v>
+        <v>16</v>
       </c>
       <c r="C54">
-        <v>2.494</v>
+        <v>2.593</v>
       </c>
       <c r="D54" t="s">
         <v>56</v>
@@ -1658,10 +1658,10 @@
         <v>46229</v>
       </c>
       <c r="B55">
-        <v>12</v>
+        <v>17</v>
       </c>
       <c r="C55">
-        <v>2.878</v>
+        <v>2.003</v>
       </c>
       <c r="D55" t="s">
         <v>57</v>
@@ -1672,10 +1672,10 @@
         <v>46229</v>
       </c>
       <c r="B56">
-        <v>13</v>
+        <v>18</v>
       </c>
       <c r="C56">
-        <v>3.069</v>
+        <v>1.337</v>
       </c>
       <c r="D56" t="s">
         <v>58</v>
@@ -1686,10 +1686,10 @@
         <v>46229</v>
       </c>
       <c r="B57">
-        <v>14</v>
+        <v>19</v>
       </c>
       <c r="C57">
-        <v>3.015</v>
+        <v>0.827</v>
       </c>
       <c r="D57" t="s">
         <v>59</v>
@@ -1700,10 +1700,10 @@
         <v>46229</v>
       </c>
       <c r="B58">
-        <v>15</v>
+        <v>20</v>
       </c>
       <c r="C58">
-        <v>2.845</v>
+        <v>0.274</v>
       </c>
       <c r="D58" t="s">
         <v>60</v>
@@ -1714,10 +1714,10 @@
         <v>46229</v>
       </c>
       <c r="B59">
-        <v>16</v>
+        <v>21</v>
       </c>
       <c r="C59">
-        <v>2.56</v>
+        <v>0.051</v>
       </c>
       <c r="D59" t="s">
         <v>61</v>
@@ -1728,10 +1728,10 @@
         <v>46229</v>
       </c>
       <c r="B60">
-        <v>17</v>
+        <v>22</v>
       </c>
       <c r="C60">
-        <v>1.954</v>
+        <v>0</v>
       </c>
       <c r="D60" t="s">
         <v>62</v>
@@ -1742,10 +1742,10 @@
         <v>46229</v>
       </c>
       <c r="B61">
-        <v>18</v>
+        <v>23</v>
       </c>
       <c r="C61">
-        <v>1.336</v>
+        <v>0</v>
       </c>
       <c r="D61" t="s">
         <v>63</v>
@@ -1756,10 +1756,10 @@
         <v>46229</v>
       </c>
       <c r="B62">
-        <v>19</v>
+        <v>24</v>
       </c>
       <c r="C62">
-        <v>0.832</v>
+        <v>0</v>
       </c>
       <c r="D62" t="s">
         <v>64</v>
@@ -1767,13 +1767,13 @@
     </row>
     <row r="63" spans="1:4">
       <c r="A63" s="2">
-        <v>46229</v>
+        <v>46230</v>
       </c>
       <c r="B63">
-        <v>20</v>
+        <v>1</v>
       </c>
       <c r="C63">
-        <v>0.301</v>
+        <v>0</v>
       </c>
       <c r="D63" t="s">
         <v>65</v>
@@ -1781,13 +1781,13 @@
     </row>
     <row r="64" spans="1:4">
       <c r="A64" s="2">
-        <v>46229</v>
+        <v>46230</v>
       </c>
       <c r="B64">
-        <v>21</v>
+        <v>2</v>
       </c>
       <c r="C64">
-        <v>0.051</v>
+        <v>0</v>
       </c>
       <c r="D64" t="s">
         <v>66</v>
@@ -1795,10 +1795,10 @@
     </row>
     <row r="65" spans="1:4">
       <c r="A65" s="2">
-        <v>46229</v>
+        <v>46230</v>
       </c>
       <c r="B65">
-        <v>22</v>
+        <v>3</v>
       </c>
       <c r="C65">
         <v>0</v>
@@ -1809,10 +1809,10 @@
     </row>
     <row r="66" spans="1:4">
       <c r="A66" s="2">
-        <v>46229</v>
+        <v>46230</v>
       </c>
       <c r="B66">
-        <v>23</v>
+        <v>4</v>
       </c>
       <c r="C66">
         <v>0</v>
@@ -1823,10 +1823,10 @@
     </row>
     <row r="67" spans="1:4">
       <c r="A67" s="2">
-        <v>46229</v>
+        <v>46230</v>
       </c>
       <c r="B67">
-        <v>24</v>
+        <v>5</v>
       </c>
       <c r="C67">
         <v>0</v>
@@ -1840,7 +1840,7 @@
         <v>46230</v>
       </c>
       <c r="B68">
-        <v>1</v>
+        <v>6</v>
       </c>
       <c r="C68">
         <v>0</v>
@@ -1854,10 +1854,10 @@
         <v>46230</v>
       </c>
       <c r="B69">
-        <v>2</v>
+        <v>7</v>
       </c>
       <c r="C69">
-        <v>0</v>
+        <v>0.042</v>
       </c>
       <c r="D69" t="s">
         <v>71</v>
@@ -1868,10 +1868,10 @@
         <v>46230</v>
       </c>
       <c r="B70">
-        <v>3</v>
+        <v>8</v>
       </c>
       <c r="C70">
-        <v>0</v>
+        <v>0.305</v>
       </c>
       <c r="D70" t="s">
         <v>72</v>
@@ -1882,10 +1882,10 @@
         <v>46230</v>
       </c>
       <c r="B71">
-        <v>4</v>
+        <v>9</v>
       </c>
       <c r="C71">
-        <v>0</v>
+        <v>0.77</v>
       </c>
       <c r="D71" t="s">
         <v>73</v>
@@ -1896,10 +1896,10 @@
         <v>46230</v>
       </c>
       <c r="B72">
-        <v>5</v>
+        <v>10</v>
       </c>
       <c r="C72">
-        <v>0</v>
+        <v>1.175</v>
       </c>
       <c r="D72" t="s">
         <v>74</v>
@@ -1910,10 +1910,10 @@
         <v>46230</v>
       </c>
       <c r="B73">
-        <v>6</v>
+        <v>11</v>
       </c>
       <c r="C73">
-        <v>0</v>
+        <v>1.715</v>
       </c>
       <c r="D73" t="s">
         <v>75</v>
@@ -1924,10 +1924,10 @@
         <v>46230</v>
       </c>
       <c r="B74">
-        <v>7</v>
+        <v>12</v>
       </c>
       <c r="C74">
-        <v>0.034</v>
+        <v>1.832</v>
       </c>
       <c r="D74" t="s">
         <v>76</v>
@@ -1938,10 +1938,10 @@
         <v>46230</v>
       </c>
       <c r="B75">
-        <v>8</v>
+        <v>13</v>
       </c>
       <c r="C75">
-        <v>0.306</v>
+        <v>2.281</v>
       </c>
       <c r="D75" t="s">
         <v>77</v>
@@ -1952,10 +1952,10 @@
         <v>46230</v>
       </c>
       <c r="B76">
-        <v>9</v>
+        <v>14</v>
       </c>
       <c r="C76">
-        <v>0.755</v>
+        <v>2.505</v>
       </c>
       <c r="D76" t="s">
         <v>78</v>
@@ -1966,10 +1966,10 @@
         <v>46230</v>
       </c>
       <c r="B77">
-        <v>10</v>
+        <v>15</v>
       </c>
       <c r="C77">
-        <v>1.128</v>
+        <v>2.144</v>
       </c>
       <c r="D77" t="s">
         <v>79</v>
@@ -1980,10 +1980,10 @@
         <v>46230</v>
       </c>
       <c r="B78">
-        <v>11</v>
+        <v>16</v>
       </c>
       <c r="C78">
-        <v>1.64</v>
+        <v>1.685</v>
       </c>
       <c r="D78" t="s">
         <v>80</v>
@@ -1994,10 +1994,10 @@
         <v>46230</v>
       </c>
       <c r="B79">
-        <v>12</v>
+        <v>17</v>
       </c>
       <c r="C79">
-        <v>1.791</v>
+        <v>1.483</v>
       </c>
       <c r="D79" t="s">
         <v>81</v>
@@ -2008,10 +2008,10 @@
         <v>46230</v>
       </c>
       <c r="B80">
-        <v>13</v>
+        <v>18</v>
       </c>
       <c r="C80">
-        <v>2.071</v>
+        <v>1.014</v>
       </c>
       <c r="D80" t="s">
         <v>82</v>
@@ -2022,10 +2022,10 @@
         <v>46230</v>
       </c>
       <c r="B81">
-        <v>14</v>
+        <v>19</v>
       </c>
       <c r="C81">
-        <v>2.281</v>
+        <v>0.491</v>
       </c>
       <c r="D81" t="s">
         <v>83</v>
@@ -2036,10 +2036,10 @@
         <v>46230</v>
       </c>
       <c r="B82">
-        <v>15</v>
+        <v>20</v>
       </c>
       <c r="C82">
-        <v>1.894</v>
+        <v>0.229</v>
       </c>
       <c r="D82" t="s">
         <v>84</v>
@@ -2050,10 +2050,10 @@
         <v>46230</v>
       </c>
       <c r="B83">
-        <v>16</v>
+        <v>21</v>
       </c>
       <c r="C83">
-        <v>1.555</v>
+        <v>0.029</v>
       </c>
       <c r="D83" t="s">
         <v>85</v>
@@ -2064,10 +2064,10 @@
         <v>46230</v>
       </c>
       <c r="B84">
-        <v>17</v>
+        <v>22</v>
       </c>
       <c r="C84">
-        <v>1.299</v>
+        <v>0</v>
       </c>
       <c r="D84" t="s">
         <v>86</v>
@@ -2078,10 +2078,10 @@
         <v>46230</v>
       </c>
       <c r="B85">
-        <v>18</v>
+        <v>23</v>
       </c>
       <c r="C85">
-        <v>0.8129999999999999</v>
+        <v>0</v>
       </c>
       <c r="D85" t="s">
         <v>87</v>
@@ -2092,10 +2092,10 @@
         <v>46230</v>
       </c>
       <c r="B86">
-        <v>19</v>
+        <v>24</v>
       </c>
       <c r="C86">
-        <v>0.498</v>
+        <v>0</v>
       </c>
       <c r="D86" t="s">
         <v>88</v>
@@ -2103,13 +2103,13 @@
     </row>
     <row r="87" spans="1:4">
       <c r="A87" s="2">
-        <v>46230</v>
+        <v>46231</v>
       </c>
       <c r="B87">
-        <v>20</v>
+        <v>1</v>
       </c>
       <c r="C87">
-        <v>0.219</v>
+        <v>0</v>
       </c>
       <c r="D87" t="s">
         <v>89</v>
@@ -2117,13 +2117,13 @@
     </row>
     <row r="88" spans="1:4">
       <c r="A88" s="2">
-        <v>46230</v>
+        <v>46231</v>
       </c>
       <c r="B88">
-        <v>21</v>
+        <v>2</v>
       </c>
       <c r="C88">
-        <v>0.036</v>
+        <v>0</v>
       </c>
       <c r="D88" t="s">
         <v>90</v>
@@ -2131,10 +2131,10 @@
     </row>
     <row r="89" spans="1:4">
       <c r="A89" s="2">
-        <v>46230</v>
+        <v>46231</v>
       </c>
       <c r="B89">
-        <v>22</v>
+        <v>3</v>
       </c>
       <c r="C89">
         <v>0</v>
@@ -2145,10 +2145,10 @@
     </row>
     <row r="90" spans="1:4">
       <c r="A90" s="2">
-        <v>46230</v>
+        <v>46231</v>
       </c>
       <c r="B90">
-        <v>23</v>
+        <v>4</v>
       </c>
       <c r="C90">
         <v>0</v>
@@ -2159,10 +2159,10 @@
     </row>
     <row r="91" spans="1:4">
       <c r="A91" s="2">
-        <v>46230</v>
+        <v>46231</v>
       </c>
       <c r="B91">
-        <v>24</v>
+        <v>5</v>
       </c>
       <c r="C91">
         <v>0</v>
@@ -2176,7 +2176,7 @@
         <v>46231</v>
       </c>
       <c r="B92">
-        <v>1</v>
+        <v>6</v>
       </c>
       <c r="C92">
         <v>0</v>
@@ -2190,10 +2190,10 @@
         <v>46231</v>
       </c>
       <c r="B93">
-        <v>2</v>
+        <v>7</v>
       </c>
       <c r="C93">
-        <v>0</v>
+        <v>0.046</v>
       </c>
       <c r="D93" t="s">
         <v>95</v>
@@ -2204,10 +2204,10 @@
         <v>46231</v>
       </c>
       <c r="B94">
-        <v>3</v>
+        <v>8</v>
       </c>
       <c r="C94">
-        <v>0</v>
+        <v>0.352</v>
       </c>
       <c r="D94" t="s">
         <v>96</v>
@@ -2218,10 +2218,10 @@
         <v>46231</v>
       </c>
       <c r="B95">
-        <v>4</v>
+        <v>9</v>
       </c>
       <c r="C95">
-        <v>0</v>
+        <v>0.861</v>
       </c>
       <c r="D95" t="s">
         <v>97</v>
@@ -2232,10 +2232,10 @@
         <v>46231</v>
       </c>
       <c r="B96">
-        <v>5</v>
+        <v>10</v>
       </c>
       <c r="C96">
-        <v>0</v>
+        <v>1.462</v>
       </c>
       <c r="D96" t="s">
         <v>98</v>
@@ -2246,10 +2246,10 @@
         <v>46231</v>
       </c>
       <c r="B97">
-        <v>6</v>
+        <v>11</v>
       </c>
       <c r="C97">
-        <v>0</v>
+        <v>2.023</v>
       </c>
       <c r="D97" t="s">
         <v>99</v>
@@ -2260,10 +2260,10 @@
         <v>46231</v>
       </c>
       <c r="B98">
-        <v>7</v>
+        <v>12</v>
       </c>
       <c r="C98">
-        <v>0.035</v>
+        <v>2.305</v>
       </c>
       <c r="D98" t="s">
         <v>100</v>
@@ -2274,10 +2274,10 @@
         <v>46231</v>
       </c>
       <c r="B99">
-        <v>8</v>
+        <v>13</v>
       </c>
       <c r="C99">
-        <v>0.248</v>
+        <v>2.65</v>
       </c>
       <c r="D99" t="s">
         <v>101</v>
@@ -2288,10 +2288,10 @@
         <v>46231</v>
       </c>
       <c r="B100">
-        <v>9</v>
+        <v>14</v>
       </c>
       <c r="C100">
-        <v>0.757</v>
+        <v>2.822</v>
       </c>
       <c r="D100" t="s">
         <v>102</v>
@@ -2302,10 +2302,10 @@
         <v>46231</v>
       </c>
       <c r="B101">
-        <v>10</v>
+        <v>15</v>
       </c>
       <c r="C101">
-        <v>1.254</v>
+        <v>2.76</v>
       </c>
       <c r="D101" t="s">
         <v>103</v>
@@ -2316,10 +2316,10 @@
         <v>46231</v>
       </c>
       <c r="B102">
-        <v>11</v>
+        <v>16</v>
       </c>
       <c r="C102">
-        <v>1.613</v>
+        <v>2.574</v>
       </c>
       <c r="D102" t="s">
         <v>104</v>
@@ -2330,10 +2330,10 @@
         <v>46231</v>
       </c>
       <c r="B103">
-        <v>12</v>
+        <v>17</v>
       </c>
       <c r="C103">
-        <v>1.842</v>
+        <v>2.049</v>
       </c>
       <c r="D103" t="s">
         <v>105</v>
@@ -2344,10 +2344,10 @@
         <v>46231</v>
       </c>
       <c r="B104">
-        <v>13</v>
+        <v>18</v>
       </c>
       <c r="C104">
-        <v>2.238</v>
+        <v>1.483</v>
       </c>
       <c r="D104" t="s">
         <v>106</v>
@@ -2358,10 +2358,10 @@
         <v>46231</v>
       </c>
       <c r="B105">
-        <v>14</v>
+        <v>19</v>
       </c>
       <c r="C105">
-        <v>2.484</v>
+        <v>0.8120000000000001</v>
       </c>
       <c r="D105" t="s">
         <v>107</v>
@@ -2372,10 +2372,10 @@
         <v>46231</v>
       </c>
       <c r="B106">
-        <v>15</v>
+        <v>20</v>
       </c>
       <c r="C106">
-        <v>2.615</v>
+        <v>0.24</v>
       </c>
       <c r="D106" t="s">
         <v>108</v>
@@ -2386,10 +2386,10 @@
         <v>46231</v>
       </c>
       <c r="B107">
-        <v>16</v>
+        <v>21</v>
       </c>
       <c r="C107">
-        <v>2.181</v>
+        <v>0.041</v>
       </c>
       <c r="D107" t="s">
         <v>109</v>
@@ -2400,10 +2400,10 @@
         <v>46231</v>
       </c>
       <c r="B108">
-        <v>17</v>
+        <v>22</v>
       </c>
       <c r="C108">
-        <v>1.918</v>
+        <v>0</v>
       </c>
       <c r="D108" t="s">
         <v>110</v>
@@ -2414,10 +2414,10 @@
         <v>46231</v>
       </c>
       <c r="B109">
-        <v>18</v>
+        <v>23</v>
       </c>
       <c r="C109">
-        <v>1.393</v>
+        <v>0</v>
       </c>
       <c r="D109" t="s">
         <v>111</v>
@@ -2428,10 +2428,10 @@
         <v>46231</v>
       </c>
       <c r="B110">
-        <v>19</v>
+        <v>24</v>
       </c>
       <c r="C110">
-        <v>0.777</v>
+        <v>0</v>
       </c>
       <c r="D110" t="s">
         <v>112</v>
@@ -2439,13 +2439,13 @@
     </row>
     <row r="111" spans="1:4">
       <c r="A111" s="2">
-        <v>46231</v>
+        <v>46232</v>
       </c>
       <c r="B111">
-        <v>20</v>
+        <v>1</v>
       </c>
       <c r="C111">
-        <v>0.245</v>
+        <v>0</v>
       </c>
       <c r="D111" t="s">
         <v>113</v>
@@ -2453,13 +2453,13 @@
     </row>
     <row r="112" spans="1:4">
       <c r="A112" s="2">
-        <v>46231</v>
+        <v>46232</v>
       </c>
       <c r="B112">
-        <v>21</v>
+        <v>2</v>
       </c>
       <c r="C112">
-        <v>0.039</v>
+        <v>0</v>
       </c>
       <c r="D112" t="s">
         <v>114</v>
@@ -2467,10 +2467,10 @@
     </row>
     <row r="113" spans="1:4">
       <c r="A113" s="2">
-        <v>46231</v>
+        <v>46232</v>
       </c>
       <c r="B113">
-        <v>22</v>
+        <v>3</v>
       </c>
       <c r="C113">
         <v>0</v>
@@ -2481,10 +2481,10 @@
     </row>
     <row r="114" spans="1:4">
       <c r="A114" s="2">
-        <v>46231</v>
+        <v>46232</v>
       </c>
       <c r="B114">
-        <v>23</v>
+        <v>4</v>
       </c>
       <c r="C114">
         <v>0</v>
@@ -2495,10 +2495,10 @@
     </row>
     <row r="115" spans="1:4">
       <c r="A115" s="2">
-        <v>46231</v>
+        <v>46232</v>
       </c>
       <c r="B115">
-        <v>24</v>
+        <v>5</v>
       </c>
       <c r="C115">
         <v>0</v>
@@ -2512,7 +2512,7 @@
         <v>46232</v>
       </c>
       <c r="B116">
-        <v>1</v>
+        <v>6</v>
       </c>
       <c r="C116">
         <v>0</v>
@@ -2526,10 +2526,10 @@
         <v>46232</v>
       </c>
       <c r="B117">
-        <v>2</v>
+        <v>7</v>
       </c>
       <c r="C117">
-        <v>0</v>
+        <v>0.046</v>
       </c>
       <c r="D117" t="s">
         <v>119</v>
@@ -2540,10 +2540,10 @@
         <v>46232</v>
       </c>
       <c r="B118">
-        <v>3</v>
+        <v>8</v>
       </c>
       <c r="C118">
-        <v>0</v>
+        <v>0.351</v>
       </c>
       <c r="D118" t="s">
         <v>120</v>
@@ -2554,10 +2554,10 @@
         <v>46232</v>
       </c>
       <c r="B119">
-        <v>4</v>
+        <v>9</v>
       </c>
       <c r="C119">
-        <v>0</v>
+        <v>1.069</v>
       </c>
       <c r="D119" t="s">
         <v>121</v>
@@ -2568,10 +2568,10 @@
         <v>46232</v>
       </c>
       <c r="B120">
-        <v>5</v>
+        <v>10</v>
       </c>
       <c r="C120">
-        <v>0</v>
+        <v>1.792</v>
       </c>
       <c r="D120" t="s">
         <v>122</v>
@@ -2582,10 +2582,10 @@
         <v>46232</v>
       </c>
       <c r="B121">
-        <v>6</v>
+        <v>11</v>
       </c>
       <c r="C121">
-        <v>0</v>
+        <v>2.456</v>
       </c>
       <c r="D121" t="s">
         <v>123</v>
@@ -2596,10 +2596,10 @@
         <v>46232</v>
       </c>
       <c r="B122">
-        <v>7</v>
+        <v>12</v>
       </c>
       <c r="C122">
-        <v>0.045</v>
+        <v>2.851</v>
       </c>
       <c r="D122" t="s">
         <v>124</v>
@@ -2610,10 +2610,10 @@
         <v>46232</v>
       </c>
       <c r="B123">
-        <v>8</v>
+        <v>13</v>
       </c>
       <c r="C123">
-        <v>0.342</v>
+        <v>3.098</v>
       </c>
       <c r="D123" t="s">
         <v>125</v>
@@ -2624,10 +2624,10 @@
         <v>46232</v>
       </c>
       <c r="B124">
-        <v>9</v>
+        <v>14</v>
       </c>
       <c r="C124">
-        <v>1.056</v>
+        <v>3.143</v>
       </c>
       <c r="D124" t="s">
         <v>126</v>
@@ -2638,10 +2638,10 @@
         <v>46232</v>
       </c>
       <c r="B125">
-        <v>10</v>
+        <v>15</v>
       </c>
       <c r="C125">
-        <v>1.812</v>
+        <v>3.018</v>
       </c>
       <c r="D125" t="s">
         <v>127</v>
@@ -2652,10 +2652,10 @@
         <v>46232</v>
       </c>
       <c r="B126">
-        <v>11</v>
+        <v>16</v>
       </c>
       <c r="C126">
-        <v>2.454</v>
+        <v>2.732</v>
       </c>
       <c r="D126" t="s">
         <v>128</v>
@@ -2666,10 +2666,10 @@
         <v>46232</v>
       </c>
       <c r="B127">
-        <v>12</v>
+        <v>17</v>
       </c>
       <c r="C127">
-        <v>2.842</v>
+        <v>2.189</v>
       </c>
       <c r="D127" t="s">
         <v>129</v>
@@ -2680,10 +2680,10 @@
         <v>46232</v>
       </c>
       <c r="B128">
-        <v>13</v>
+        <v>18</v>
       </c>
       <c r="C128">
-        <v>3.097</v>
+        <v>1.575</v>
       </c>
       <c r="D128" t="s">
         <v>130</v>
@@ -2694,10 +2694,10 @@
         <v>46232</v>
       </c>
       <c r="B129">
-        <v>14</v>
+        <v>19</v>
       </c>
       <c r="C129">
-        <v>3.142</v>
+        <v>0.827</v>
       </c>
       <c r="D129" t="s">
         <v>131</v>
@@ -2708,10 +2708,10 @@
         <v>46232</v>
       </c>
       <c r="B130">
-        <v>15</v>
+        <v>20</v>
       </c>
       <c r="C130">
-        <v>3.013</v>
+        <v>0.205</v>
       </c>
       <c r="D130" t="s">
         <v>132</v>
@@ -2722,10 +2722,10 @@
         <v>46232</v>
       </c>
       <c r="B131">
-        <v>16</v>
+        <v>21</v>
       </c>
       <c r="C131">
-        <v>2.734</v>
+        <v>0.04</v>
       </c>
       <c r="D131" t="s">
         <v>133</v>
@@ -2736,10 +2736,10 @@
         <v>46232</v>
       </c>
       <c r="B132">
-        <v>17</v>
+        <v>22</v>
       </c>
       <c r="C132">
-        <v>2.187</v>
+        <v>0</v>
       </c>
       <c r="D132" t="s">
         <v>134</v>
@@ -2750,10 +2750,10 @@
         <v>46232</v>
       </c>
       <c r="B133">
-        <v>18</v>
+        <v>23</v>
       </c>
       <c r="C133">
-        <v>1.564</v>
+        <v>0</v>
       </c>
       <c r="D133" t="s">
         <v>135</v>
@@ -2764,10 +2764,10 @@
         <v>46232</v>
       </c>
       <c r="B134">
-        <v>19</v>
+        <v>24</v>
       </c>
       <c r="C134">
-        <v>0.83</v>
+        <v>0</v>
       </c>
       <c r="D134" t="s">
         <v>136</v>
@@ -2775,13 +2775,13 @@
     </row>
     <row r="135" spans="1:4">
       <c r="A135" s="2">
-        <v>46232</v>
+        <v>46233</v>
       </c>
       <c r="B135">
-        <v>20</v>
+        <v>1</v>
       </c>
       <c r="C135">
-        <v>0.206</v>
+        <v>0</v>
       </c>
       <c r="D135" t="s">
         <v>137</v>
@@ -2789,13 +2789,13 @@
     </row>
     <row r="136" spans="1:4">
       <c r="A136" s="2">
-        <v>46232</v>
+        <v>46233</v>
       </c>
       <c r="B136">
-        <v>21</v>
+        <v>2</v>
       </c>
       <c r="C136">
-        <v>0.04</v>
+        <v>0</v>
       </c>
       <c r="D136" t="s">
         <v>138</v>
@@ -2803,10 +2803,10 @@
     </row>
     <row r="137" spans="1:4">
       <c r="A137" s="2">
-        <v>46232</v>
+        <v>46233</v>
       </c>
       <c r="B137">
-        <v>22</v>
+        <v>3</v>
       </c>
       <c r="C137">
         <v>0</v>
@@ -2817,10 +2817,10 @@
     </row>
     <row r="138" spans="1:4">
       <c r="A138" s="2">
-        <v>46232</v>
+        <v>46233</v>
       </c>
       <c r="B138">
-        <v>23</v>
+        <v>4</v>
       </c>
       <c r="C138">
         <v>0</v>
@@ -2831,10 +2831,10 @@
     </row>
     <row r="139" spans="1:4">
       <c r="A139" s="2">
-        <v>46232</v>
+        <v>46233</v>
       </c>
       <c r="B139">
-        <v>24</v>
+        <v>5</v>
       </c>
       <c r="C139">
         <v>0</v>
@@ -2848,7 +2848,7 @@
         <v>46233</v>
       </c>
       <c r="B140">
-        <v>1</v>
+        <v>6</v>
       </c>
       <c r="C140">
         <v>0</v>
@@ -2862,10 +2862,10 @@
         <v>46233</v>
       </c>
       <c r="B141">
-        <v>2</v>
+        <v>7</v>
       </c>
       <c r="C141">
-        <v>0</v>
+        <v>0.046</v>
       </c>
       <c r="D141" t="s">
         <v>143</v>
@@ -2876,10 +2876,10 @@
         <v>46233</v>
       </c>
       <c r="B142">
-        <v>3</v>
+        <v>8</v>
       </c>
       <c r="C142">
-        <v>0</v>
+        <v>0.365</v>
       </c>
       <c r="D142" t="s">
         <v>144</v>
@@ -2890,10 +2890,10 @@
         <v>46233</v>
       </c>
       <c r="B143">
-        <v>4</v>
+        <v>9</v>
       </c>
       <c r="C143">
-        <v>0</v>
+        <v>1.037</v>
       </c>
       <c r="D143" t="s">
         <v>145</v>
@@ -2904,10 +2904,10 @@
         <v>46233</v>
       </c>
       <c r="B144">
-        <v>5</v>
+        <v>10</v>
       </c>
       <c r="C144">
-        <v>0</v>
+        <v>1.786</v>
       </c>
       <c r="D144" t="s">
         <v>146</v>
@@ -2918,10 +2918,10 @@
         <v>46233</v>
       </c>
       <c r="B145">
-        <v>6</v>
+        <v>11</v>
       </c>
       <c r="C145">
-        <v>0</v>
+        <v>2.343</v>
       </c>
       <c r="D145" t="s">
         <v>147</v>
@@ -2932,10 +2932,10 @@
         <v>46233</v>
       </c>
       <c r="B146">
-        <v>7</v>
+        <v>12</v>
       </c>
       <c r="C146">
-        <v>0.047</v>
+        <v>2.64</v>
       </c>
       <c r="D146" t="s">
         <v>148</v>
@@ -2946,10 +2946,10 @@
         <v>46233</v>
       </c>
       <c r="B147">
-        <v>8</v>
+        <v>13</v>
       </c>
       <c r="C147">
-        <v>0.376</v>
+        <v>2.874</v>
       </c>
       <c r="D147" t="s">
         <v>149</v>
@@ -2960,10 +2960,10 @@
         <v>46233</v>
       </c>
       <c r="B148">
-        <v>9</v>
+        <v>14</v>
       </c>
       <c r="C148">
-        <v>1.035</v>
+        <v>3.058</v>
       </c>
       <c r="D148" t="s">
         <v>150</v>
@@ -2974,10 +2974,10 @@
         <v>46233</v>
       </c>
       <c r="B149">
-        <v>10</v>
+        <v>15</v>
       </c>
       <c r="C149">
-        <v>1.74</v>
+        <v>3.031</v>
       </c>
       <c r="D149" t="s">
         <v>151</v>
@@ -2988,10 +2988,10 @@
         <v>46233</v>
       </c>
       <c r="B150">
-        <v>11</v>
+        <v>16</v>
       </c>
       <c r="C150">
-        <v>2.336</v>
+        <v>2.562</v>
       </c>
       <c r="D150" t="s">
         <v>152</v>
@@ -3002,10 +3002,10 @@
         <v>46233</v>
       </c>
       <c r="B151">
-        <v>12</v>
+        <v>17</v>
       </c>
       <c r="C151">
-        <v>2.639</v>
+        <v>1.98</v>
       </c>
       <c r="D151" t="s">
         <v>153</v>
@@ -3016,10 +3016,10 @@
         <v>46233</v>
       </c>
       <c r="B152">
-        <v>13</v>
+        <v>18</v>
       </c>
       <c r="C152">
-        <v>2.851</v>
+        <v>1.378</v>
       </c>
       <c r="D152" t="s">
         <v>154</v>
@@ -3030,10 +3030,10 @@
         <v>46233</v>
       </c>
       <c r="B153">
-        <v>14</v>
+        <v>19</v>
       </c>
       <c r="C153">
-        <v>2.955</v>
+        <v>0.747</v>
       </c>
       <c r="D153" t="s">
         <v>155</v>
@@ -3044,10 +3044,10 @@
         <v>46233</v>
       </c>
       <c r="B154">
-        <v>15</v>
+        <v>20</v>
       </c>
       <c r="C154">
-        <v>2.786</v>
+        <v>0.248</v>
       </c>
       <c r="D154" t="s">
         <v>156</v>
@@ -3058,10 +3058,10 @@
         <v>46233</v>
       </c>
       <c r="B155">
-        <v>16</v>
+        <v>21</v>
       </c>
       <c r="C155">
-        <v>2.474</v>
+        <v>0.048</v>
       </c>
       <c r="D155" t="s">
         <v>157</v>
@@ -3072,10 +3072,10 @@
         <v>46233</v>
       </c>
       <c r="B156">
-        <v>17</v>
+        <v>22</v>
       </c>
       <c r="C156">
-        <v>2.016</v>
+        <v>0</v>
       </c>
       <c r="D156" t="s">
         <v>158</v>
@@ -3086,10 +3086,10 @@
         <v>46233</v>
       </c>
       <c r="B157">
-        <v>18</v>
+        <v>23</v>
       </c>
       <c r="C157">
-        <v>1.473</v>
+        <v>0</v>
       </c>
       <c r="D157" t="s">
         <v>159</v>
@@ -3100,10 +3100,10 @@
         <v>46233</v>
       </c>
       <c r="B158">
-        <v>19</v>
+        <v>24</v>
       </c>
       <c r="C158">
-        <v>0.773</v>
+        <v>0</v>
       </c>
       <c r="D158" t="s">
         <v>160</v>
@@ -3111,13 +3111,13 @@
     </row>
     <row r="159" spans="1:4">
       <c r="A159" s="2">
-        <v>46233</v>
+        <v>46234</v>
       </c>
       <c r="B159">
-        <v>20</v>
+        <v>1</v>
       </c>
       <c r="C159">
-        <v>0.215</v>
+        <v>0</v>
       </c>
       <c r="D159" t="s">
         <v>161</v>
@@ -3125,13 +3125,13 @@
     </row>
     <row r="160" spans="1:4">
       <c r="A160" s="2">
-        <v>46233</v>
+        <v>46234</v>
       </c>
       <c r="B160">
-        <v>21</v>
+        <v>2</v>
       </c>
       <c r="C160">
-        <v>0.042</v>
+        <v>0</v>
       </c>
       <c r="D160" t="s">
         <v>162</v>
@@ -3139,10 +3139,10 @@
     </row>
     <row r="161" spans="1:4">
       <c r="A161" s="2">
-        <v>46233</v>
+        <v>46234</v>
       </c>
       <c r="B161">
-        <v>22</v>
+        <v>3</v>
       </c>
       <c r="C161">
         <v>0</v>
@@ -3153,10 +3153,10 @@
     </row>
     <row r="162" spans="1:4">
       <c r="A162" s="2">
-        <v>46233</v>
+        <v>46234</v>
       </c>
       <c r="B162">
-        <v>23</v>
+        <v>4</v>
       </c>
       <c r="C162">
         <v>0</v>
@@ -3167,10 +3167,10 @@
     </row>
     <row r="163" spans="1:4">
       <c r="A163" s="2">
-        <v>46233</v>
+        <v>46234</v>
       </c>
       <c r="B163">
-        <v>24</v>
+        <v>5</v>
       </c>
       <c r="C163">
         <v>0</v>
@@ -3184,7 +3184,7 @@
         <v>46234</v>
       </c>
       <c r="B164">
-        <v>1</v>
+        <v>6</v>
       </c>
       <c r="C164">
         <v>0</v>
@@ -3198,10 +3198,10 @@
         <v>46234</v>
       </c>
       <c r="B165">
-        <v>2</v>
+        <v>7</v>
       </c>
       <c r="C165">
-        <v>0</v>
+        <v>0.039</v>
       </c>
       <c r="D165" t="s">
         <v>167</v>
@@ -3212,10 +3212,10 @@
         <v>46234</v>
       </c>
       <c r="B166">
-        <v>3</v>
+        <v>8</v>
       </c>
       <c r="C166">
-        <v>0</v>
+        <v>0.36</v>
       </c>
       <c r="D166" t="s">
         <v>168</v>
@@ -3226,10 +3226,10 @@
         <v>46234</v>
       </c>
       <c r="B167">
-        <v>4</v>
+        <v>9</v>
       </c>
       <c r="C167">
-        <v>0</v>
+        <v>0.994</v>
       </c>
       <c r="D167" t="s">
         <v>169</v>
@@ -3240,10 +3240,10 @@
         <v>46234</v>
       </c>
       <c r="B168">
-        <v>5</v>
+        <v>10</v>
       </c>
       <c r="C168">
-        <v>0</v>
+        <v>1.729</v>
       </c>
       <c r="D168" t="s">
         <v>170</v>
@@ -3254,10 +3254,10 @@
         <v>46234</v>
       </c>
       <c r="B169">
-        <v>6</v>
+        <v>11</v>
       </c>
       <c r="C169">
-        <v>0</v>
+        <v>2.347</v>
       </c>
       <c r="D169" t="s">
         <v>171</v>
@@ -3268,10 +3268,10 @@
         <v>46234</v>
       </c>
       <c r="B170">
-        <v>7</v>
+        <v>12</v>
       </c>
       <c r="C170">
-        <v>0.043</v>
+        <v>2.688</v>
       </c>
       <c r="D170" t="s">
         <v>172</v>

</xml_diff>

<commit_message>
Updating the model for Elnet
</commit_message>
<xml_diff>
--- a/Astro/Results_Production_Astro_xgb.xlsx
+++ b/Astro/Results_Production_Astro_xgb.xlsx
@@ -28,511 +28,511 @@
     <t>Lookup</t>
   </si>
   <si>
-    <t>24.07.202612</t>
-  </si>
-  <si>
-    <t>24.07.202613</t>
-  </si>
-  <si>
-    <t>24.07.202614</t>
-  </si>
-  <si>
-    <t>24.07.202615</t>
-  </si>
-  <si>
-    <t>24.07.202616</t>
-  </si>
-  <si>
-    <t>24.07.202617</t>
-  </si>
-  <si>
-    <t>24.07.202618</t>
-  </si>
-  <si>
-    <t>24.07.202619</t>
-  </si>
-  <si>
-    <t>24.07.202620</t>
-  </si>
-  <si>
-    <t>24.07.202621</t>
-  </si>
-  <si>
-    <t>24.07.202622</t>
-  </si>
-  <si>
-    <t>24.07.202623</t>
-  </si>
-  <si>
-    <t>24.07.202624</t>
-  </si>
-  <si>
-    <t>25.07.20261</t>
-  </si>
-  <si>
-    <t>25.07.20262</t>
-  </si>
-  <si>
-    <t>25.07.20263</t>
-  </si>
-  <si>
-    <t>25.07.20264</t>
-  </si>
-  <si>
-    <t>25.07.20265</t>
-  </si>
-  <si>
-    <t>25.07.20266</t>
-  </si>
-  <si>
-    <t>25.07.20267</t>
-  </si>
-  <si>
-    <t>25.07.20268</t>
-  </si>
-  <si>
-    <t>25.07.20269</t>
-  </si>
-  <si>
-    <t>25.07.202610</t>
-  </si>
-  <si>
-    <t>25.07.202611</t>
-  </si>
-  <si>
-    <t>25.07.202612</t>
-  </si>
-  <si>
-    <t>25.07.202613</t>
-  </si>
-  <si>
-    <t>25.07.202614</t>
-  </si>
-  <si>
-    <t>25.07.202615</t>
-  </si>
-  <si>
-    <t>25.07.202616</t>
-  </si>
-  <si>
-    <t>25.07.202617</t>
-  </si>
-  <si>
-    <t>25.07.202618</t>
-  </si>
-  <si>
-    <t>25.07.202619</t>
-  </si>
-  <si>
-    <t>25.07.202620</t>
-  </si>
-  <si>
-    <t>25.07.202621</t>
-  </si>
-  <si>
-    <t>25.07.202622</t>
-  </si>
-  <si>
-    <t>25.07.202623</t>
-  </si>
-  <si>
-    <t>25.07.202624</t>
-  </si>
-  <si>
-    <t>26.07.20261</t>
-  </si>
-  <si>
-    <t>26.07.20262</t>
-  </si>
-  <si>
-    <t>26.07.20263</t>
-  </si>
-  <si>
-    <t>26.07.20264</t>
-  </si>
-  <si>
-    <t>26.07.20265</t>
-  </si>
-  <si>
-    <t>26.07.20266</t>
-  </si>
-  <si>
-    <t>26.07.20267</t>
-  </si>
-  <si>
-    <t>26.07.20268</t>
-  </si>
-  <si>
-    <t>26.07.20269</t>
-  </si>
-  <si>
-    <t>26.07.202610</t>
-  </si>
-  <si>
-    <t>26.07.202611</t>
-  </si>
-  <si>
-    <t>26.07.202612</t>
-  </si>
-  <si>
-    <t>26.07.202613</t>
-  </si>
-  <si>
-    <t>26.07.202614</t>
-  </si>
-  <si>
-    <t>26.07.202615</t>
-  </si>
-  <si>
-    <t>26.07.202616</t>
-  </si>
-  <si>
-    <t>26.07.202617</t>
-  </si>
-  <si>
-    <t>26.07.202618</t>
-  </si>
-  <si>
-    <t>26.07.202619</t>
-  </si>
-  <si>
-    <t>26.07.202620</t>
-  </si>
-  <si>
-    <t>26.07.202621</t>
-  </si>
-  <si>
-    <t>26.07.202622</t>
-  </si>
-  <si>
-    <t>26.07.202623</t>
-  </si>
-  <si>
-    <t>26.07.202624</t>
-  </si>
-  <si>
-    <t>27.07.20261</t>
-  </si>
-  <si>
-    <t>27.07.20262</t>
-  </si>
-  <si>
-    <t>27.07.20263</t>
-  </si>
-  <si>
-    <t>27.07.20264</t>
-  </si>
-  <si>
-    <t>27.07.20265</t>
-  </si>
-  <si>
-    <t>27.07.20266</t>
-  </si>
-  <si>
-    <t>27.07.20267</t>
-  </si>
-  <si>
-    <t>27.07.20268</t>
-  </si>
-  <si>
-    <t>27.07.20269</t>
-  </si>
-  <si>
-    <t>27.07.202610</t>
-  </si>
-  <si>
-    <t>27.07.202611</t>
-  </si>
-  <si>
-    <t>27.07.202612</t>
-  </si>
-  <si>
-    <t>27.07.202613</t>
-  </si>
-  <si>
-    <t>27.07.202614</t>
-  </si>
-  <si>
-    <t>27.07.202615</t>
-  </si>
-  <si>
-    <t>27.07.202616</t>
-  </si>
-  <si>
-    <t>27.07.202617</t>
-  </si>
-  <si>
-    <t>27.07.202618</t>
-  </si>
-  <si>
-    <t>27.07.202619</t>
-  </si>
-  <si>
-    <t>27.07.202620</t>
-  </si>
-  <si>
-    <t>27.07.202621</t>
-  </si>
-  <si>
-    <t>27.07.202622</t>
-  </si>
-  <si>
-    <t>27.07.202623</t>
-  </si>
-  <si>
-    <t>27.07.202624</t>
-  </si>
-  <si>
-    <t>28.07.20261</t>
-  </si>
-  <si>
-    <t>28.07.20262</t>
-  </si>
-  <si>
-    <t>28.07.20263</t>
-  </si>
-  <si>
-    <t>28.07.20264</t>
-  </si>
-  <si>
-    <t>28.07.20265</t>
-  </si>
-  <si>
-    <t>28.07.20266</t>
-  </si>
-  <si>
-    <t>28.07.20267</t>
-  </si>
-  <si>
-    <t>28.07.20268</t>
-  </si>
-  <si>
-    <t>28.07.20269</t>
-  </si>
-  <si>
-    <t>28.07.202610</t>
-  </si>
-  <si>
-    <t>28.07.202611</t>
-  </si>
-  <si>
-    <t>28.07.202612</t>
-  </si>
-  <si>
-    <t>28.07.202613</t>
-  </si>
-  <si>
-    <t>28.07.202614</t>
-  </si>
-  <si>
-    <t>28.07.202615</t>
-  </si>
-  <si>
-    <t>28.07.202616</t>
-  </si>
-  <si>
-    <t>28.07.202617</t>
-  </si>
-  <si>
-    <t>28.07.202618</t>
-  </si>
-  <si>
-    <t>28.07.202619</t>
-  </si>
-  <si>
-    <t>28.07.202620</t>
-  </si>
-  <si>
-    <t>28.07.202621</t>
-  </si>
-  <si>
-    <t>28.07.202622</t>
-  </si>
-  <si>
-    <t>28.07.202623</t>
-  </si>
-  <si>
-    <t>28.07.202624</t>
-  </si>
-  <si>
-    <t>29.07.20261</t>
-  </si>
-  <si>
-    <t>29.07.20262</t>
-  </si>
-  <si>
-    <t>29.07.20263</t>
-  </si>
-  <si>
-    <t>29.07.20264</t>
-  </si>
-  <si>
-    <t>29.07.20265</t>
-  </si>
-  <si>
-    <t>29.07.20266</t>
-  </si>
-  <si>
-    <t>29.07.20267</t>
-  </si>
-  <si>
-    <t>29.07.20268</t>
-  </si>
-  <si>
-    <t>29.07.20269</t>
-  </si>
-  <si>
-    <t>29.07.202610</t>
-  </si>
-  <si>
-    <t>29.07.202611</t>
-  </si>
-  <si>
-    <t>29.07.202612</t>
-  </si>
-  <si>
-    <t>29.07.202613</t>
-  </si>
-  <si>
-    <t>29.07.202614</t>
-  </si>
-  <si>
-    <t>29.07.202615</t>
-  </si>
-  <si>
-    <t>29.07.202616</t>
-  </si>
-  <si>
-    <t>29.07.202617</t>
-  </si>
-  <si>
-    <t>29.07.202618</t>
-  </si>
-  <si>
-    <t>29.07.202619</t>
-  </si>
-  <si>
-    <t>29.07.202620</t>
-  </si>
-  <si>
-    <t>29.07.202621</t>
-  </si>
-  <si>
-    <t>29.07.202622</t>
-  </si>
-  <si>
-    <t>29.07.202623</t>
-  </si>
-  <si>
-    <t>29.07.202624</t>
-  </si>
-  <si>
-    <t>30.07.20261</t>
-  </si>
-  <si>
-    <t>30.07.20262</t>
-  </si>
-  <si>
-    <t>30.07.20263</t>
-  </si>
-  <si>
-    <t>30.07.20264</t>
-  </si>
-  <si>
-    <t>30.07.20265</t>
-  </si>
-  <si>
-    <t>30.07.20266</t>
-  </si>
-  <si>
-    <t>30.07.20267</t>
-  </si>
-  <si>
-    <t>30.07.20268</t>
-  </si>
-  <si>
-    <t>30.07.20269</t>
-  </si>
-  <si>
-    <t>30.07.202610</t>
-  </si>
-  <si>
-    <t>30.07.202611</t>
-  </si>
-  <si>
-    <t>30.07.202612</t>
-  </si>
-  <si>
-    <t>30.07.202613</t>
-  </si>
-  <si>
-    <t>30.07.202614</t>
-  </si>
-  <si>
-    <t>30.07.202615</t>
-  </si>
-  <si>
-    <t>30.07.202616</t>
-  </si>
-  <si>
-    <t>30.07.202617</t>
-  </si>
-  <si>
-    <t>30.07.202618</t>
-  </si>
-  <si>
-    <t>30.07.202619</t>
-  </si>
-  <si>
-    <t>30.07.202620</t>
-  </si>
-  <si>
-    <t>30.07.202621</t>
-  </si>
-  <si>
-    <t>30.07.202622</t>
-  </si>
-  <si>
-    <t>30.07.202623</t>
-  </si>
-  <si>
-    <t>30.07.202624</t>
-  </si>
-  <si>
-    <t>31.07.20261</t>
-  </si>
-  <si>
-    <t>31.07.20262</t>
-  </si>
-  <si>
-    <t>31.07.20263</t>
-  </si>
-  <si>
-    <t>31.07.20264</t>
-  </si>
-  <si>
-    <t>31.07.20265</t>
-  </si>
-  <si>
-    <t>31.07.20266</t>
-  </si>
-  <si>
-    <t>31.07.20267</t>
-  </si>
-  <si>
-    <t>31.07.20268</t>
-  </si>
-  <si>
-    <t>31.07.20269</t>
-  </si>
-  <si>
-    <t>31.07.202610</t>
-  </si>
-  <si>
-    <t>31.07.202611</t>
-  </si>
-  <si>
-    <t>31.07.202612</t>
+    <t>11.08.202614</t>
+  </si>
+  <si>
+    <t>11.08.202615</t>
+  </si>
+  <si>
+    <t>11.08.202616</t>
+  </si>
+  <si>
+    <t>11.08.202617</t>
+  </si>
+  <si>
+    <t>11.08.202618</t>
+  </si>
+  <si>
+    <t>11.08.202619</t>
+  </si>
+  <si>
+    <t>11.08.202620</t>
+  </si>
+  <si>
+    <t>11.08.202621</t>
+  </si>
+  <si>
+    <t>11.08.202622</t>
+  </si>
+  <si>
+    <t>11.08.202623</t>
+  </si>
+  <si>
+    <t>11.08.202624</t>
+  </si>
+  <si>
+    <t>12.08.20261</t>
+  </si>
+  <si>
+    <t>12.08.20262</t>
+  </si>
+  <si>
+    <t>12.08.20263</t>
+  </si>
+  <si>
+    <t>12.08.20264</t>
+  </si>
+  <si>
+    <t>12.08.20265</t>
+  </si>
+  <si>
+    <t>12.08.20266</t>
+  </si>
+  <si>
+    <t>12.08.20267</t>
+  </si>
+  <si>
+    <t>12.08.20268</t>
+  </si>
+  <si>
+    <t>12.08.20269</t>
+  </si>
+  <si>
+    <t>12.08.202610</t>
+  </si>
+  <si>
+    <t>12.08.202611</t>
+  </si>
+  <si>
+    <t>12.08.202612</t>
+  </si>
+  <si>
+    <t>12.08.202613</t>
+  </si>
+  <si>
+    <t>12.08.202614</t>
+  </si>
+  <si>
+    <t>12.08.202615</t>
+  </si>
+  <si>
+    <t>12.08.202616</t>
+  </si>
+  <si>
+    <t>12.08.202617</t>
+  </si>
+  <si>
+    <t>12.08.202618</t>
+  </si>
+  <si>
+    <t>12.08.202619</t>
+  </si>
+  <si>
+    <t>12.08.202620</t>
+  </si>
+  <si>
+    <t>12.08.202621</t>
+  </si>
+  <si>
+    <t>12.08.202622</t>
+  </si>
+  <si>
+    <t>12.08.202623</t>
+  </si>
+  <si>
+    <t>12.08.202624</t>
+  </si>
+  <si>
+    <t>13.08.20261</t>
+  </si>
+  <si>
+    <t>13.08.20262</t>
+  </si>
+  <si>
+    <t>13.08.20263</t>
+  </si>
+  <si>
+    <t>13.08.20264</t>
+  </si>
+  <si>
+    <t>13.08.20265</t>
+  </si>
+  <si>
+    <t>13.08.20266</t>
+  </si>
+  <si>
+    <t>13.08.20267</t>
+  </si>
+  <si>
+    <t>13.08.20268</t>
+  </si>
+  <si>
+    <t>13.08.20269</t>
+  </si>
+  <si>
+    <t>13.08.202610</t>
+  </si>
+  <si>
+    <t>13.08.202611</t>
+  </si>
+  <si>
+    <t>13.08.202612</t>
+  </si>
+  <si>
+    <t>13.08.202613</t>
+  </si>
+  <si>
+    <t>13.08.202614</t>
+  </si>
+  <si>
+    <t>13.08.202615</t>
+  </si>
+  <si>
+    <t>13.08.202616</t>
+  </si>
+  <si>
+    <t>13.08.202617</t>
+  </si>
+  <si>
+    <t>13.08.202618</t>
+  </si>
+  <si>
+    <t>13.08.202619</t>
+  </si>
+  <si>
+    <t>13.08.202620</t>
+  </si>
+  <si>
+    <t>13.08.202621</t>
+  </si>
+  <si>
+    <t>13.08.202622</t>
+  </si>
+  <si>
+    <t>13.08.202623</t>
+  </si>
+  <si>
+    <t>13.08.202624</t>
+  </si>
+  <si>
+    <t>14.08.20261</t>
+  </si>
+  <si>
+    <t>14.08.20262</t>
+  </si>
+  <si>
+    <t>14.08.20263</t>
+  </si>
+  <si>
+    <t>14.08.20264</t>
+  </si>
+  <si>
+    <t>14.08.20265</t>
+  </si>
+  <si>
+    <t>14.08.20266</t>
+  </si>
+  <si>
+    <t>14.08.20267</t>
+  </si>
+  <si>
+    <t>14.08.20268</t>
+  </si>
+  <si>
+    <t>14.08.20269</t>
+  </si>
+  <si>
+    <t>14.08.202610</t>
+  </si>
+  <si>
+    <t>14.08.202611</t>
+  </si>
+  <si>
+    <t>14.08.202612</t>
+  </si>
+  <si>
+    <t>14.08.202613</t>
+  </si>
+  <si>
+    <t>14.08.202614</t>
+  </si>
+  <si>
+    <t>14.08.202615</t>
+  </si>
+  <si>
+    <t>14.08.202616</t>
+  </si>
+  <si>
+    <t>14.08.202617</t>
+  </si>
+  <si>
+    <t>14.08.202618</t>
+  </si>
+  <si>
+    <t>14.08.202619</t>
+  </si>
+  <si>
+    <t>14.08.202620</t>
+  </si>
+  <si>
+    <t>14.08.202621</t>
+  </si>
+  <si>
+    <t>14.08.202622</t>
+  </si>
+  <si>
+    <t>14.08.202623</t>
+  </si>
+  <si>
+    <t>14.08.202624</t>
+  </si>
+  <si>
+    <t>15.08.20261</t>
+  </si>
+  <si>
+    <t>15.08.20262</t>
+  </si>
+  <si>
+    <t>15.08.20263</t>
+  </si>
+  <si>
+    <t>15.08.20264</t>
+  </si>
+  <si>
+    <t>15.08.20265</t>
+  </si>
+  <si>
+    <t>15.08.20266</t>
+  </si>
+  <si>
+    <t>15.08.20267</t>
+  </si>
+  <si>
+    <t>15.08.20268</t>
+  </si>
+  <si>
+    <t>15.08.20269</t>
+  </si>
+  <si>
+    <t>15.08.202610</t>
+  </si>
+  <si>
+    <t>15.08.202611</t>
+  </si>
+  <si>
+    <t>15.08.202612</t>
+  </si>
+  <si>
+    <t>15.08.202613</t>
+  </si>
+  <si>
+    <t>15.08.202614</t>
+  </si>
+  <si>
+    <t>15.08.202615</t>
+  </si>
+  <si>
+    <t>15.08.202616</t>
+  </si>
+  <si>
+    <t>15.08.202617</t>
+  </si>
+  <si>
+    <t>15.08.202618</t>
+  </si>
+  <si>
+    <t>15.08.202619</t>
+  </si>
+  <si>
+    <t>15.08.202620</t>
+  </si>
+  <si>
+    <t>15.08.202621</t>
+  </si>
+  <si>
+    <t>15.08.202622</t>
+  </si>
+  <si>
+    <t>15.08.202623</t>
+  </si>
+  <si>
+    <t>15.08.202624</t>
+  </si>
+  <si>
+    <t>16.08.20261</t>
+  </si>
+  <si>
+    <t>16.08.20262</t>
+  </si>
+  <si>
+    <t>16.08.20263</t>
+  </si>
+  <si>
+    <t>16.08.20264</t>
+  </si>
+  <si>
+    <t>16.08.20265</t>
+  </si>
+  <si>
+    <t>16.08.20266</t>
+  </si>
+  <si>
+    <t>16.08.20267</t>
+  </si>
+  <si>
+    <t>16.08.20268</t>
+  </si>
+  <si>
+    <t>16.08.20269</t>
+  </si>
+  <si>
+    <t>16.08.202610</t>
+  </si>
+  <si>
+    <t>16.08.202611</t>
+  </si>
+  <si>
+    <t>16.08.202612</t>
+  </si>
+  <si>
+    <t>16.08.202613</t>
+  </si>
+  <si>
+    <t>16.08.202614</t>
+  </si>
+  <si>
+    <t>16.08.202615</t>
+  </si>
+  <si>
+    <t>16.08.202616</t>
+  </si>
+  <si>
+    <t>16.08.202617</t>
+  </si>
+  <si>
+    <t>16.08.202618</t>
+  </si>
+  <si>
+    <t>16.08.202619</t>
+  </si>
+  <si>
+    <t>16.08.202620</t>
+  </si>
+  <si>
+    <t>16.08.202621</t>
+  </si>
+  <si>
+    <t>16.08.202622</t>
+  </si>
+  <si>
+    <t>16.08.202623</t>
+  </si>
+  <si>
+    <t>16.08.202624</t>
+  </si>
+  <si>
+    <t>17.08.20261</t>
+  </si>
+  <si>
+    <t>17.08.20262</t>
+  </si>
+  <si>
+    <t>17.08.20263</t>
+  </si>
+  <si>
+    <t>17.08.20264</t>
+  </si>
+  <si>
+    <t>17.08.20265</t>
+  </si>
+  <si>
+    <t>17.08.20266</t>
+  </si>
+  <si>
+    <t>17.08.20267</t>
+  </si>
+  <si>
+    <t>17.08.20268</t>
+  </si>
+  <si>
+    <t>17.08.20269</t>
+  </si>
+  <si>
+    <t>17.08.202610</t>
+  </si>
+  <si>
+    <t>17.08.202611</t>
+  </si>
+  <si>
+    <t>17.08.202612</t>
+  </si>
+  <si>
+    <t>17.08.202613</t>
+  </si>
+  <si>
+    <t>17.08.202614</t>
+  </si>
+  <si>
+    <t>17.08.202615</t>
+  </si>
+  <si>
+    <t>17.08.202616</t>
+  </si>
+  <si>
+    <t>17.08.202617</t>
+  </si>
+  <si>
+    <t>17.08.202618</t>
+  </si>
+  <si>
+    <t>17.08.202619</t>
+  </si>
+  <si>
+    <t>17.08.202620</t>
+  </si>
+  <si>
+    <t>17.08.202621</t>
+  </si>
+  <si>
+    <t>17.08.202622</t>
+  </si>
+  <si>
+    <t>17.08.202623</t>
+  </si>
+  <si>
+    <t>17.08.202624</t>
+  </si>
+  <si>
+    <t>18.08.20261</t>
+  </si>
+  <si>
+    <t>18.08.20262</t>
+  </si>
+  <si>
+    <t>18.08.20263</t>
+  </si>
+  <si>
+    <t>18.08.20264</t>
+  </si>
+  <si>
+    <t>18.08.20265</t>
+  </si>
+  <si>
+    <t>18.08.20266</t>
+  </si>
+  <si>
+    <t>18.08.20267</t>
+  </si>
+  <si>
+    <t>18.08.20268</t>
+  </si>
+  <si>
+    <t>18.08.20269</t>
+  </si>
+  <si>
+    <t>18.08.202610</t>
+  </si>
+  <si>
+    <t>18.08.202611</t>
+  </si>
+  <si>
+    <t>18.08.202612</t>
+  </si>
+  <si>
+    <t>18.08.202613</t>
+  </si>
+  <si>
+    <t>18.08.202614</t>
   </si>
 </sst>
 </file>
@@ -913,10 +913,10 @@
     </row>
     <row r="2" spans="1:4">
       <c r="A2" s="2">
-        <v>46227</v>
+        <v>46245</v>
       </c>
       <c r="B2">
-        <v>12</v>
+        <v>14</v>
       </c>
       <c r="C2">
         <v>0</v>
@@ -927,10 +927,10 @@
     </row>
     <row r="3" spans="1:4">
       <c r="A3" s="2">
-        <v>46227</v>
+        <v>46245</v>
       </c>
       <c r="B3">
-        <v>13</v>
+        <v>15</v>
       </c>
       <c r="C3">
         <v>0</v>
@@ -941,13 +941,13 @@
     </row>
     <row r="4" spans="1:4">
       <c r="A4" s="2">
-        <v>46227</v>
+        <v>46245</v>
       </c>
       <c r="B4">
-        <v>14</v>
+        <v>16</v>
       </c>
       <c r="C4">
-        <v>2.235</v>
+        <v>2.668</v>
       </c>
       <c r="D4" t="s">
         <v>6</v>
@@ -955,13 +955,13 @@
     </row>
     <row r="5" spans="1:4">
       <c r="A5" s="2">
-        <v>46227</v>
+        <v>46245</v>
       </c>
       <c r="B5">
-        <v>15</v>
+        <v>17</v>
       </c>
       <c r="C5">
-        <v>1.846</v>
+        <v>2.021</v>
       </c>
       <c r="D5" t="s">
         <v>7</v>
@@ -969,13 +969,13 @@
     </row>
     <row r="6" spans="1:4">
       <c r="A6" s="2">
-        <v>46227</v>
+        <v>46245</v>
       </c>
       <c r="B6">
-        <v>16</v>
+        <v>18</v>
       </c>
       <c r="C6">
-        <v>1.81</v>
+        <v>1.268</v>
       </c>
       <c r="D6" t="s">
         <v>8</v>
@@ -983,13 +983,13 @@
     </row>
     <row r="7" spans="1:4">
       <c r="A7" s="2">
-        <v>46227</v>
+        <v>46245</v>
       </c>
       <c r="B7">
-        <v>17</v>
+        <v>19</v>
       </c>
       <c r="C7">
-        <v>1.721</v>
+        <v>0.613</v>
       </c>
       <c r="D7" t="s">
         <v>9</v>
@@ -997,13 +997,13 @@
     </row>
     <row r="8" spans="1:4">
       <c r="A8" s="2">
-        <v>46227</v>
+        <v>46245</v>
       </c>
       <c r="B8">
-        <v>18</v>
+        <v>20</v>
       </c>
       <c r="C8">
-        <v>1.186</v>
+        <v>0.182</v>
       </c>
       <c r="D8" t="s">
         <v>10</v>
@@ -1011,13 +1011,13 @@
     </row>
     <row r="9" spans="1:4">
       <c r="A9" s="2">
-        <v>46227</v>
+        <v>46245</v>
       </c>
       <c r="B9">
-        <v>19</v>
+        <v>21</v>
       </c>
       <c r="C9">
-        <v>0.593</v>
+        <v>0.021</v>
       </c>
       <c r="D9" t="s">
         <v>11</v>
@@ -1025,13 +1025,13 @@
     </row>
     <row r="10" spans="1:4">
       <c r="A10" s="2">
-        <v>46227</v>
+        <v>46245</v>
       </c>
       <c r="B10">
-        <v>20</v>
+        <v>22</v>
       </c>
       <c r="C10">
-        <v>0.302</v>
+        <v>0</v>
       </c>
       <c r="D10" t="s">
         <v>12</v>
@@ -1039,13 +1039,13 @@
     </row>
     <row r="11" spans="1:4">
       <c r="A11" s="2">
-        <v>46227</v>
+        <v>46245</v>
       </c>
       <c r="B11">
-        <v>21</v>
+        <v>23</v>
       </c>
       <c r="C11">
-        <v>0.05</v>
+        <v>0</v>
       </c>
       <c r="D11" t="s">
         <v>13</v>
@@ -1053,10 +1053,10 @@
     </row>
     <row r="12" spans="1:4">
       <c r="A12" s="2">
-        <v>46227</v>
+        <v>46245</v>
       </c>
       <c r="B12">
-        <v>22</v>
+        <v>24</v>
       </c>
       <c r="C12">
         <v>0</v>
@@ -1067,10 +1067,10 @@
     </row>
     <row r="13" spans="1:4">
       <c r="A13" s="2">
-        <v>46227</v>
+        <v>46246</v>
       </c>
       <c r="B13">
-        <v>23</v>
+        <v>1</v>
       </c>
       <c r="C13">
         <v>0</v>
@@ -1081,10 +1081,10 @@
     </row>
     <row r="14" spans="1:4">
       <c r="A14" s="2">
-        <v>46227</v>
+        <v>46246</v>
       </c>
       <c r="B14">
-        <v>24</v>
+        <v>2</v>
       </c>
       <c r="C14">
         <v>0</v>
@@ -1095,10 +1095,10 @@
     </row>
     <row r="15" spans="1:4">
       <c r="A15" s="2">
-        <v>46228</v>
+        <v>46246</v>
       </c>
       <c r="B15">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="C15">
         <v>0</v>
@@ -1109,10 +1109,10 @@
     </row>
     <row r="16" spans="1:4">
       <c r="A16" s="2">
-        <v>46228</v>
+        <v>46246</v>
       </c>
       <c r="B16">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="C16">
         <v>0</v>
@@ -1123,10 +1123,10 @@
     </row>
     <row r="17" spans="1:4">
       <c r="A17" s="2">
-        <v>46228</v>
+        <v>46246</v>
       </c>
       <c r="B17">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="C17">
         <v>0</v>
@@ -1137,10 +1137,10 @@
     </row>
     <row r="18" spans="1:4">
       <c r="A18" s="2">
-        <v>46228</v>
+        <v>46246</v>
       </c>
       <c r="B18">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="C18">
         <v>0</v>
@@ -1151,13 +1151,13 @@
     </row>
     <row r="19" spans="1:4">
       <c r="A19" s="2">
-        <v>46228</v>
+        <v>46246</v>
       </c>
       <c r="B19">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="C19">
-        <v>0</v>
+        <v>0.018</v>
       </c>
       <c r="D19" t="s">
         <v>21</v>
@@ -1165,13 +1165,13 @@
     </row>
     <row r="20" spans="1:4">
       <c r="A20" s="2">
-        <v>46228</v>
+        <v>46246</v>
       </c>
       <c r="B20">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="C20">
-        <v>0</v>
+        <v>0.256</v>
       </c>
       <c r="D20" t="s">
         <v>22</v>
@@ -1179,13 +1179,13 @@
     </row>
     <row r="21" spans="1:4">
       <c r="A21" s="2">
-        <v>46228</v>
+        <v>46246</v>
       </c>
       <c r="B21">
-        <v>7</v>
+        <v>9</v>
       </c>
       <c r="C21">
-        <v>0.055</v>
+        <v>0.9320000000000001</v>
       </c>
       <c r="D21" t="s">
         <v>23</v>
@@ -1193,13 +1193,13 @@
     </row>
     <row r="22" spans="1:4">
       <c r="A22" s="2">
-        <v>46228</v>
+        <v>46246</v>
       </c>
       <c r="B22">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="C22">
-        <v>0.371</v>
+        <v>1.686</v>
       </c>
       <c r="D22" t="s">
         <v>24</v>
@@ -1207,13 +1207,13 @@
     </row>
     <row r="23" spans="1:4">
       <c r="A23" s="2">
-        <v>46228</v>
+        <v>46246</v>
       </c>
       <c r="B23">
-        <v>9</v>
+        <v>11</v>
       </c>
       <c r="C23">
-        <v>1.094</v>
+        <v>2.328</v>
       </c>
       <c r="D23" t="s">
         <v>25</v>
@@ -1221,13 +1221,13 @@
     </row>
     <row r="24" spans="1:4">
       <c r="A24" s="2">
-        <v>46228</v>
+        <v>46246</v>
       </c>
       <c r="B24">
-        <v>10</v>
+        <v>12</v>
       </c>
       <c r="C24">
-        <v>1.863</v>
+        <v>2.829</v>
       </c>
       <c r="D24" t="s">
         <v>26</v>
@@ -1235,13 +1235,13 @@
     </row>
     <row r="25" spans="1:4">
       <c r="A25" s="2">
-        <v>46228</v>
+        <v>46246</v>
       </c>
       <c r="B25">
-        <v>11</v>
+        <v>13</v>
       </c>
       <c r="C25">
-        <v>2.277</v>
+        <v>3.033</v>
       </c>
       <c r="D25" t="s">
         <v>27</v>
@@ -1249,13 +1249,13 @@
     </row>
     <row r="26" spans="1:4">
       <c r="A26" s="2">
-        <v>46228</v>
+        <v>46246</v>
       </c>
       <c r="B26">
-        <v>12</v>
+        <v>14</v>
       </c>
       <c r="C26">
-        <v>2.426</v>
+        <v>3.102</v>
       </c>
       <c r="D26" t="s">
         <v>28</v>
@@ -1263,13 +1263,13 @@
     </row>
     <row r="27" spans="1:4">
       <c r="A27" s="2">
-        <v>46228</v>
+        <v>46246</v>
       </c>
       <c r="B27">
-        <v>13</v>
+        <v>15</v>
       </c>
       <c r="C27">
-        <v>2.655</v>
+        <v>2.719</v>
       </c>
       <c r="D27" t="s">
         <v>29</v>
@@ -1277,13 +1277,13 @@
     </row>
     <row r="28" spans="1:4">
       <c r="A28" s="2">
-        <v>46228</v>
+        <v>46246</v>
       </c>
       <c r="B28">
-        <v>14</v>
+        <v>16</v>
       </c>
       <c r="C28">
-        <v>2.7</v>
+        <v>2.38</v>
       </c>
       <c r="D28" t="s">
         <v>30</v>
@@ -1291,13 +1291,13 @@
     </row>
     <row r="29" spans="1:4">
       <c r="A29" s="2">
-        <v>46228</v>
+        <v>46246</v>
       </c>
       <c r="B29">
-        <v>15</v>
+        <v>17</v>
       </c>
       <c r="C29">
-        <v>2.641</v>
+        <v>2.04</v>
       </c>
       <c r="D29" t="s">
         <v>31</v>
@@ -1305,13 +1305,13 @@
     </row>
     <row r="30" spans="1:4">
       <c r="A30" s="2">
-        <v>46228</v>
+        <v>46246</v>
       </c>
       <c r="B30">
-        <v>16</v>
+        <v>18</v>
       </c>
       <c r="C30">
-        <v>2.206</v>
+        <v>1.363</v>
       </c>
       <c r="D30" t="s">
         <v>32</v>
@@ -1319,13 +1319,13 @@
     </row>
     <row r="31" spans="1:4">
       <c r="A31" s="2">
-        <v>46228</v>
+        <v>46246</v>
       </c>
       <c r="B31">
-        <v>17</v>
+        <v>19</v>
       </c>
       <c r="C31">
-        <v>1.918</v>
+        <v>0.754</v>
       </c>
       <c r="D31" t="s">
         <v>33</v>
@@ -1333,13 +1333,13 @@
     </row>
     <row r="32" spans="1:4">
       <c r="A32" s="2">
-        <v>46228</v>
+        <v>46246</v>
       </c>
       <c r="B32">
-        <v>18</v>
+        <v>20</v>
       </c>
       <c r="C32">
-        <v>1.351</v>
+        <v>0.204</v>
       </c>
       <c r="D32" t="s">
         <v>34</v>
@@ -1347,13 +1347,13 @@
     </row>
     <row r="33" spans="1:4">
       <c r="A33" s="2">
-        <v>46228</v>
+        <v>46246</v>
       </c>
       <c r="B33">
-        <v>19</v>
+        <v>21</v>
       </c>
       <c r="C33">
-        <v>0.757</v>
+        <v>0.021</v>
       </c>
       <c r="D33" t="s">
         <v>35</v>
@@ -1361,13 +1361,13 @@
     </row>
     <row r="34" spans="1:4">
       <c r="A34" s="2">
-        <v>46228</v>
+        <v>46246</v>
       </c>
       <c r="B34">
-        <v>20</v>
+        <v>22</v>
       </c>
       <c r="C34">
-        <v>0.262</v>
+        <v>0</v>
       </c>
       <c r="D34" t="s">
         <v>36</v>
@@ -1375,13 +1375,13 @@
     </row>
     <row r="35" spans="1:4">
       <c r="A35" s="2">
-        <v>46228</v>
+        <v>46246</v>
       </c>
       <c r="B35">
-        <v>21</v>
+        <v>23</v>
       </c>
       <c r="C35">
-        <v>0.06</v>
+        <v>0</v>
       </c>
       <c r="D35" t="s">
         <v>37</v>
@@ -1389,10 +1389,10 @@
     </row>
     <row r="36" spans="1:4">
       <c r="A36" s="2">
-        <v>46228</v>
+        <v>46246</v>
       </c>
       <c r="B36">
-        <v>22</v>
+        <v>24</v>
       </c>
       <c r="C36">
         <v>0</v>
@@ -1403,10 +1403,10 @@
     </row>
     <row r="37" spans="1:4">
       <c r="A37" s="2">
-        <v>46228</v>
+        <v>46247</v>
       </c>
       <c r="B37">
-        <v>23</v>
+        <v>1</v>
       </c>
       <c r="C37">
         <v>0</v>
@@ -1417,10 +1417,10 @@
     </row>
     <row r="38" spans="1:4">
       <c r="A38" s="2">
-        <v>46228</v>
+        <v>46247</v>
       </c>
       <c r="B38">
-        <v>24</v>
+        <v>2</v>
       </c>
       <c r="C38">
         <v>0</v>
@@ -1431,10 +1431,10 @@
     </row>
     <row r="39" spans="1:4">
       <c r="A39" s="2">
-        <v>46229</v>
+        <v>46247</v>
       </c>
       <c r="B39">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="C39">
         <v>0</v>
@@ -1445,10 +1445,10 @@
     </row>
     <row r="40" spans="1:4">
       <c r="A40" s="2">
-        <v>46229</v>
+        <v>46247</v>
       </c>
       <c r="B40">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="C40">
         <v>0</v>
@@ -1459,10 +1459,10 @@
     </row>
     <row r="41" spans="1:4">
       <c r="A41" s="2">
-        <v>46229</v>
+        <v>46247</v>
       </c>
       <c r="B41">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="C41">
         <v>0</v>
@@ -1473,10 +1473,10 @@
     </row>
     <row r="42" spans="1:4">
       <c r="A42" s="2">
-        <v>46229</v>
+        <v>46247</v>
       </c>
       <c r="B42">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="C42">
         <v>0</v>
@@ -1487,13 +1487,13 @@
     </row>
     <row r="43" spans="1:4">
       <c r="A43" s="2">
-        <v>46229</v>
+        <v>46247</v>
       </c>
       <c r="B43">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="C43">
-        <v>0</v>
+        <v>0.024</v>
       </c>
       <c r="D43" t="s">
         <v>45</v>
@@ -1501,13 +1501,13 @@
     </row>
     <row r="44" spans="1:4">
       <c r="A44" s="2">
-        <v>46229</v>
+        <v>46247</v>
       </c>
       <c r="B44">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="C44">
-        <v>0</v>
+        <v>0.303</v>
       </c>
       <c r="D44" t="s">
         <v>46</v>
@@ -1515,13 +1515,13 @@
     </row>
     <row r="45" spans="1:4">
       <c r="A45" s="2">
-        <v>46229</v>
+        <v>46247</v>
       </c>
       <c r="B45">
-        <v>7</v>
+        <v>9</v>
       </c>
       <c r="C45">
-        <v>0.056</v>
+        <v>1.001</v>
       </c>
       <c r="D45" t="s">
         <v>47</v>
@@ -1529,13 +1529,13 @@
     </row>
     <row r="46" spans="1:4">
       <c r="A46" s="2">
-        <v>46229</v>
+        <v>46247</v>
       </c>
       <c r="B46">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="C46">
-        <v>0.356</v>
+        <v>1.634</v>
       </c>
       <c r="D46" t="s">
         <v>48</v>
@@ -1543,13 +1543,13 @@
     </row>
     <row r="47" spans="1:4">
       <c r="A47" s="2">
-        <v>46229</v>
+        <v>46247</v>
       </c>
       <c r="B47">
-        <v>9</v>
+        <v>11</v>
       </c>
       <c r="C47">
-        <v>1.113</v>
+        <v>2.017</v>
       </c>
       <c r="D47" t="s">
         <v>49</v>
@@ -1557,13 +1557,13 @@
     </row>
     <row r="48" spans="1:4">
       <c r="A48" s="2">
-        <v>46229</v>
+        <v>46247</v>
       </c>
       <c r="B48">
-        <v>10</v>
+        <v>12</v>
       </c>
       <c r="C48">
-        <v>1.864</v>
+        <v>2.325</v>
       </c>
       <c r="D48" t="s">
         <v>50</v>
@@ -1571,13 +1571,13 @@
     </row>
     <row r="49" spans="1:4">
       <c r="A49" s="2">
-        <v>46229</v>
+        <v>46247</v>
       </c>
       <c r="B49">
-        <v>11</v>
+        <v>13</v>
       </c>
       <c r="C49">
-        <v>2.487</v>
+        <v>2.607</v>
       </c>
       <c r="D49" t="s">
         <v>51</v>
@@ -1585,13 +1585,13 @@
     </row>
     <row r="50" spans="1:4">
       <c r="A50" s="2">
-        <v>46229</v>
+        <v>46247</v>
       </c>
       <c r="B50">
-        <v>12</v>
+        <v>14</v>
       </c>
       <c r="C50">
-        <v>2.846</v>
+        <v>2.584</v>
       </c>
       <c r="D50" t="s">
         <v>52</v>
@@ -1599,13 +1599,13 @@
     </row>
     <row r="51" spans="1:4">
       <c r="A51" s="2">
-        <v>46229</v>
+        <v>46247</v>
       </c>
       <c r="B51">
-        <v>13</v>
+        <v>15</v>
       </c>
       <c r="C51">
-        <v>3.02</v>
+        <v>2.514</v>
       </c>
       <c r="D51" t="s">
         <v>53</v>
@@ -1613,13 +1613,13 @@
     </row>
     <row r="52" spans="1:4">
       <c r="A52" s="2">
-        <v>46229</v>
+        <v>46247</v>
       </c>
       <c r="B52">
-        <v>14</v>
+        <v>16</v>
       </c>
       <c r="C52">
-        <v>2.996</v>
+        <v>2.118</v>
       </c>
       <c r="D52" t="s">
         <v>54</v>
@@ -1627,13 +1627,13 @@
     </row>
     <row r="53" spans="1:4">
       <c r="A53" s="2">
-        <v>46229</v>
+        <v>46247</v>
       </c>
       <c r="B53">
-        <v>15</v>
+        <v>17</v>
       </c>
       <c r="C53">
-        <v>2.903</v>
+        <v>1.582</v>
       </c>
       <c r="D53" t="s">
         <v>55</v>
@@ -1641,13 +1641,13 @@
     </row>
     <row r="54" spans="1:4">
       <c r="A54" s="2">
-        <v>46229</v>
+        <v>46247</v>
       </c>
       <c r="B54">
-        <v>16</v>
+        <v>18</v>
       </c>
       <c r="C54">
-        <v>2.593</v>
+        <v>1.096</v>
       </c>
       <c r="D54" t="s">
         <v>56</v>
@@ -1655,13 +1655,13 @@
     </row>
     <row r="55" spans="1:4">
       <c r="A55" s="2">
-        <v>46229</v>
+        <v>46247</v>
       </c>
       <c r="B55">
-        <v>17</v>
+        <v>19</v>
       </c>
       <c r="C55">
-        <v>2.003</v>
+        <v>0.586</v>
       </c>
       <c r="D55" t="s">
         <v>57</v>
@@ -1669,13 +1669,13 @@
     </row>
     <row r="56" spans="1:4">
       <c r="A56" s="2">
-        <v>46229</v>
+        <v>46247</v>
       </c>
       <c r="B56">
-        <v>18</v>
+        <v>20</v>
       </c>
       <c r="C56">
-        <v>1.337</v>
+        <v>0.204</v>
       </c>
       <c r="D56" t="s">
         <v>58</v>
@@ -1683,13 +1683,13 @@
     </row>
     <row r="57" spans="1:4">
       <c r="A57" s="2">
-        <v>46229</v>
+        <v>46247</v>
       </c>
       <c r="B57">
-        <v>19</v>
+        <v>21</v>
       </c>
       <c r="C57">
-        <v>0.827</v>
+        <v>0.023</v>
       </c>
       <c r="D57" t="s">
         <v>59</v>
@@ -1697,13 +1697,13 @@
     </row>
     <row r="58" spans="1:4">
       <c r="A58" s="2">
-        <v>46229</v>
+        <v>46247</v>
       </c>
       <c r="B58">
-        <v>20</v>
+        <v>22</v>
       </c>
       <c r="C58">
-        <v>0.274</v>
+        <v>0</v>
       </c>
       <c r="D58" t="s">
         <v>60</v>
@@ -1711,13 +1711,13 @@
     </row>
     <row r="59" spans="1:4">
       <c r="A59" s="2">
-        <v>46229</v>
+        <v>46247</v>
       </c>
       <c r="B59">
-        <v>21</v>
+        <v>23</v>
       </c>
       <c r="C59">
-        <v>0.051</v>
+        <v>0</v>
       </c>
       <c r="D59" t="s">
         <v>61</v>
@@ -1725,10 +1725,10 @@
     </row>
     <row r="60" spans="1:4">
       <c r="A60" s="2">
-        <v>46229</v>
+        <v>46247</v>
       </c>
       <c r="B60">
-        <v>22</v>
+        <v>24</v>
       </c>
       <c r="C60">
         <v>0</v>
@@ -1739,10 +1739,10 @@
     </row>
     <row r="61" spans="1:4">
       <c r="A61" s="2">
-        <v>46229</v>
+        <v>46248</v>
       </c>
       <c r="B61">
-        <v>23</v>
+        <v>1</v>
       </c>
       <c r="C61">
         <v>0</v>
@@ -1753,10 +1753,10 @@
     </row>
     <row r="62" spans="1:4">
       <c r="A62" s="2">
-        <v>46229</v>
+        <v>46248</v>
       </c>
       <c r="B62">
-        <v>24</v>
+        <v>2</v>
       </c>
       <c r="C62">
         <v>0</v>
@@ -1767,10 +1767,10 @@
     </row>
     <row r="63" spans="1:4">
       <c r="A63" s="2">
-        <v>46230</v>
+        <v>46248</v>
       </c>
       <c r="B63">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="C63">
         <v>0</v>
@@ -1781,10 +1781,10 @@
     </row>
     <row r="64" spans="1:4">
       <c r="A64" s="2">
-        <v>46230</v>
+        <v>46248</v>
       </c>
       <c r="B64">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="C64">
         <v>0</v>
@@ -1795,10 +1795,10 @@
     </row>
     <row r="65" spans="1:4">
       <c r="A65" s="2">
-        <v>46230</v>
+        <v>46248</v>
       </c>
       <c r="B65">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="C65">
         <v>0</v>
@@ -1809,10 +1809,10 @@
     </row>
     <row r="66" spans="1:4">
       <c r="A66" s="2">
-        <v>46230</v>
+        <v>46248</v>
       </c>
       <c r="B66">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="C66">
         <v>0</v>
@@ -1823,13 +1823,13 @@
     </row>
     <row r="67" spans="1:4">
       <c r="A67" s="2">
-        <v>46230</v>
+        <v>46248</v>
       </c>
       <c r="B67">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="C67">
-        <v>0</v>
+        <v>0.022</v>
       </c>
       <c r="D67" t="s">
         <v>69</v>
@@ -1837,13 +1837,13 @@
     </row>
     <row r="68" spans="1:4">
       <c r="A68" s="2">
-        <v>46230</v>
+        <v>46248</v>
       </c>
       <c r="B68">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="C68">
-        <v>0</v>
+        <v>0.285</v>
       </c>
       <c r="D68" t="s">
         <v>70</v>
@@ -1851,13 +1851,13 @@
     </row>
     <row r="69" spans="1:4">
       <c r="A69" s="2">
-        <v>46230</v>
+        <v>46248</v>
       </c>
       <c r="B69">
-        <v>7</v>
+        <v>9</v>
       </c>
       <c r="C69">
-        <v>0.042</v>
+        <v>0.918</v>
       </c>
       <c r="D69" t="s">
         <v>71</v>
@@ -1865,13 +1865,13 @@
     </row>
     <row r="70" spans="1:4">
       <c r="A70" s="2">
-        <v>46230</v>
+        <v>46248</v>
       </c>
       <c r="B70">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="C70">
-        <v>0.305</v>
+        <v>1.602</v>
       </c>
       <c r="D70" t="s">
         <v>72</v>
@@ -1879,13 +1879,13 @@
     </row>
     <row r="71" spans="1:4">
       <c r="A71" s="2">
-        <v>46230</v>
+        <v>46248</v>
       </c>
       <c r="B71">
-        <v>9</v>
+        <v>11</v>
       </c>
       <c r="C71">
-        <v>0.77</v>
+        <v>2.025</v>
       </c>
       <c r="D71" t="s">
         <v>73</v>
@@ -1893,13 +1893,13 @@
     </row>
     <row r="72" spans="1:4">
       <c r="A72" s="2">
-        <v>46230</v>
+        <v>46248</v>
       </c>
       <c r="B72">
-        <v>10</v>
+        <v>12</v>
       </c>
       <c r="C72">
-        <v>1.175</v>
+        <v>2.372</v>
       </c>
       <c r="D72" t="s">
         <v>74</v>
@@ -1907,13 +1907,13 @@
     </row>
     <row r="73" spans="1:4">
       <c r="A73" s="2">
-        <v>46230</v>
+        <v>46248</v>
       </c>
       <c r="B73">
-        <v>11</v>
+        <v>13</v>
       </c>
       <c r="C73">
-        <v>1.715</v>
+        <v>2.694</v>
       </c>
       <c r="D73" t="s">
         <v>75</v>
@@ -1921,13 +1921,13 @@
     </row>
     <row r="74" spans="1:4">
       <c r="A74" s="2">
-        <v>46230</v>
+        <v>46248</v>
       </c>
       <c r="B74">
-        <v>12</v>
+        <v>14</v>
       </c>
       <c r="C74">
-        <v>1.832</v>
+        <v>2.6</v>
       </c>
       <c r="D74" t="s">
         <v>76</v>
@@ -1935,13 +1935,13 @@
     </row>
     <row r="75" spans="1:4">
       <c r="A75" s="2">
-        <v>46230</v>
+        <v>46248</v>
       </c>
       <c r="B75">
-        <v>13</v>
+        <v>15</v>
       </c>
       <c r="C75">
-        <v>2.281</v>
+        <v>2.622</v>
       </c>
       <c r="D75" t="s">
         <v>77</v>
@@ -1949,13 +1949,13 @@
     </row>
     <row r="76" spans="1:4">
       <c r="A76" s="2">
-        <v>46230</v>
+        <v>46248</v>
       </c>
       <c r="B76">
-        <v>14</v>
+        <v>16</v>
       </c>
       <c r="C76">
-        <v>2.505</v>
+        <v>2.449</v>
       </c>
       <c r="D76" t="s">
         <v>78</v>
@@ -1963,13 +1963,13 @@
     </row>
     <row r="77" spans="1:4">
       <c r="A77" s="2">
-        <v>46230</v>
+        <v>46248</v>
       </c>
       <c r="B77">
-        <v>15</v>
+        <v>17</v>
       </c>
       <c r="C77">
-        <v>2.144</v>
+        <v>2.081</v>
       </c>
       <c r="D77" t="s">
         <v>79</v>
@@ -1977,13 +1977,13 @@
     </row>
     <row r="78" spans="1:4">
       <c r="A78" s="2">
-        <v>46230</v>
+        <v>46248</v>
       </c>
       <c r="B78">
-        <v>16</v>
+        <v>18</v>
       </c>
       <c r="C78">
-        <v>1.685</v>
+        <v>1.445</v>
       </c>
       <c r="D78" t="s">
         <v>80</v>
@@ -1991,13 +1991,13 @@
     </row>
     <row r="79" spans="1:4">
       <c r="A79" s="2">
-        <v>46230</v>
+        <v>46248</v>
       </c>
       <c r="B79">
-        <v>17</v>
+        <v>19</v>
       </c>
       <c r="C79">
-        <v>1.483</v>
+        <v>0.74</v>
       </c>
       <c r="D79" t="s">
         <v>81</v>
@@ -2005,13 +2005,13 @@
     </row>
     <row r="80" spans="1:4">
       <c r="A80" s="2">
-        <v>46230</v>
+        <v>46248</v>
       </c>
       <c r="B80">
-        <v>18</v>
+        <v>20</v>
       </c>
       <c r="C80">
-        <v>1.014</v>
+        <v>0.172</v>
       </c>
       <c r="D80" t="s">
         <v>82</v>
@@ -2019,13 +2019,13 @@
     </row>
     <row r="81" spans="1:4">
       <c r="A81" s="2">
-        <v>46230</v>
+        <v>46248</v>
       </c>
       <c r="B81">
-        <v>19</v>
+        <v>21</v>
       </c>
       <c r="C81">
-        <v>0.491</v>
+        <v>0.02</v>
       </c>
       <c r="D81" t="s">
         <v>83</v>
@@ -2033,13 +2033,13 @@
     </row>
     <row r="82" spans="1:4">
       <c r="A82" s="2">
-        <v>46230</v>
+        <v>46248</v>
       </c>
       <c r="B82">
-        <v>20</v>
+        <v>22</v>
       </c>
       <c r="C82">
-        <v>0.229</v>
+        <v>0</v>
       </c>
       <c r="D82" t="s">
         <v>84</v>
@@ -2047,13 +2047,13 @@
     </row>
     <row r="83" spans="1:4">
       <c r="A83" s="2">
-        <v>46230</v>
+        <v>46248</v>
       </c>
       <c r="B83">
-        <v>21</v>
+        <v>23</v>
       </c>
       <c r="C83">
-        <v>0.029</v>
+        <v>0</v>
       </c>
       <c r="D83" t="s">
         <v>85</v>
@@ -2061,10 +2061,10 @@
     </row>
     <row r="84" spans="1:4">
       <c r="A84" s="2">
-        <v>46230</v>
+        <v>46248</v>
       </c>
       <c r="B84">
-        <v>22</v>
+        <v>24</v>
       </c>
       <c r="C84">
         <v>0</v>
@@ -2075,10 +2075,10 @@
     </row>
     <row r="85" spans="1:4">
       <c r="A85" s="2">
-        <v>46230</v>
+        <v>46249</v>
       </c>
       <c r="B85">
-        <v>23</v>
+        <v>1</v>
       </c>
       <c r="C85">
         <v>0</v>
@@ -2089,10 +2089,10 @@
     </row>
     <row r="86" spans="1:4">
       <c r="A86" s="2">
-        <v>46230</v>
+        <v>46249</v>
       </c>
       <c r="B86">
-        <v>24</v>
+        <v>2</v>
       </c>
       <c r="C86">
         <v>0</v>
@@ -2103,10 +2103,10 @@
     </row>
     <row r="87" spans="1:4">
       <c r="A87" s="2">
-        <v>46231</v>
+        <v>46249</v>
       </c>
       <c r="B87">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="C87">
         <v>0</v>
@@ -2117,10 +2117,10 @@
     </row>
     <row r="88" spans="1:4">
       <c r="A88" s="2">
-        <v>46231</v>
+        <v>46249</v>
       </c>
       <c r="B88">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="C88">
         <v>0</v>
@@ -2131,10 +2131,10 @@
     </row>
     <row r="89" spans="1:4">
       <c r="A89" s="2">
-        <v>46231</v>
+        <v>46249</v>
       </c>
       <c r="B89">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="C89">
         <v>0</v>
@@ -2145,10 +2145,10 @@
     </row>
     <row r="90" spans="1:4">
       <c r="A90" s="2">
-        <v>46231</v>
+        <v>46249</v>
       </c>
       <c r="B90">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="C90">
         <v>0</v>
@@ -2159,13 +2159,13 @@
     </row>
     <row r="91" spans="1:4">
       <c r="A91" s="2">
-        <v>46231</v>
+        <v>46249</v>
       </c>
       <c r="B91">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="C91">
-        <v>0</v>
+        <v>0.024</v>
       </c>
       <c r="D91" t="s">
         <v>93</v>
@@ -2173,13 +2173,13 @@
     </row>
     <row r="92" spans="1:4">
       <c r="A92" s="2">
-        <v>46231</v>
+        <v>46249</v>
       </c>
       <c r="B92">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="C92">
-        <v>0</v>
+        <v>0.276</v>
       </c>
       <c r="D92" t="s">
         <v>94</v>
@@ -2187,13 +2187,13 @@
     </row>
     <row r="93" spans="1:4">
       <c r="A93" s="2">
-        <v>46231</v>
+        <v>46249</v>
       </c>
       <c r="B93">
-        <v>7</v>
+        <v>9</v>
       </c>
       <c r="C93">
-        <v>0.046</v>
+        <v>1.006</v>
       </c>
       <c r="D93" t="s">
         <v>95</v>
@@ -2201,13 +2201,13 @@
     </row>
     <row r="94" spans="1:4">
       <c r="A94" s="2">
-        <v>46231</v>
+        <v>46249</v>
       </c>
       <c r="B94">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="C94">
-        <v>0.352</v>
+        <v>1.668</v>
       </c>
       <c r="D94" t="s">
         <v>96</v>
@@ -2215,13 +2215,13 @@
     </row>
     <row r="95" spans="1:4">
       <c r="A95" s="2">
-        <v>46231</v>
+        <v>46249</v>
       </c>
       <c r="B95">
-        <v>9</v>
+        <v>11</v>
       </c>
       <c r="C95">
-        <v>0.861</v>
+        <v>2.317</v>
       </c>
       <c r="D95" t="s">
         <v>97</v>
@@ -2229,13 +2229,13 @@
     </row>
     <row r="96" spans="1:4">
       <c r="A96" s="2">
-        <v>46231</v>
+        <v>46249</v>
       </c>
       <c r="B96">
-        <v>10</v>
+        <v>12</v>
       </c>
       <c r="C96">
-        <v>1.462</v>
+        <v>2.652</v>
       </c>
       <c r="D96" t="s">
         <v>98</v>
@@ -2243,13 +2243,13 @@
     </row>
     <row r="97" spans="1:4">
       <c r="A97" s="2">
-        <v>46231</v>
+        <v>46249</v>
       </c>
       <c r="B97">
-        <v>11</v>
+        <v>13</v>
       </c>
       <c r="C97">
-        <v>2.023</v>
+        <v>2.828</v>
       </c>
       <c r="D97" t="s">
         <v>99</v>
@@ -2257,13 +2257,13 @@
     </row>
     <row r="98" spans="1:4">
       <c r="A98" s="2">
-        <v>46231</v>
+        <v>46249</v>
       </c>
       <c r="B98">
-        <v>12</v>
+        <v>14</v>
       </c>
       <c r="C98">
-        <v>2.305</v>
+        <v>3.109</v>
       </c>
       <c r="D98" t="s">
         <v>100</v>
@@ -2271,13 +2271,13 @@
     </row>
     <row r="99" spans="1:4">
       <c r="A99" s="2">
-        <v>46231</v>
+        <v>46249</v>
       </c>
       <c r="B99">
-        <v>13</v>
+        <v>15</v>
       </c>
       <c r="C99">
-        <v>2.65</v>
+        <v>3.026</v>
       </c>
       <c r="D99" t="s">
         <v>101</v>
@@ -2285,13 +2285,13 @@
     </row>
     <row r="100" spans="1:4">
       <c r="A100" s="2">
-        <v>46231</v>
+        <v>46249</v>
       </c>
       <c r="B100">
-        <v>14</v>
+        <v>16</v>
       </c>
       <c r="C100">
-        <v>2.822</v>
+        <v>2.643</v>
       </c>
       <c r="D100" t="s">
         <v>102</v>
@@ -2299,13 +2299,13 @@
     </row>
     <row r="101" spans="1:4">
       <c r="A101" s="2">
-        <v>46231</v>
+        <v>46249</v>
       </c>
       <c r="B101">
-        <v>15</v>
+        <v>17</v>
       </c>
       <c r="C101">
-        <v>2.76</v>
+        <v>2.085</v>
       </c>
       <c r="D101" t="s">
         <v>103</v>
@@ -2313,13 +2313,13 @@
     </row>
     <row r="102" spans="1:4">
       <c r="A102" s="2">
-        <v>46231</v>
+        <v>46249</v>
       </c>
       <c r="B102">
-        <v>16</v>
+        <v>18</v>
       </c>
       <c r="C102">
-        <v>2.574</v>
+        <v>1.488</v>
       </c>
       <c r="D102" t="s">
         <v>104</v>
@@ -2327,13 +2327,13 @@
     </row>
     <row r="103" spans="1:4">
       <c r="A103" s="2">
-        <v>46231</v>
+        <v>46249</v>
       </c>
       <c r="B103">
-        <v>17</v>
+        <v>19</v>
       </c>
       <c r="C103">
-        <v>2.049</v>
+        <v>0.6929999999999999</v>
       </c>
       <c r="D103" t="s">
         <v>105</v>
@@ -2341,13 +2341,13 @@
     </row>
     <row r="104" spans="1:4">
       <c r="A104" s="2">
-        <v>46231</v>
+        <v>46249</v>
       </c>
       <c r="B104">
-        <v>18</v>
+        <v>20</v>
       </c>
       <c r="C104">
-        <v>1.483</v>
+        <v>0.149</v>
       </c>
       <c r="D104" t="s">
         <v>106</v>
@@ -2355,13 +2355,13 @@
     </row>
     <row r="105" spans="1:4">
       <c r="A105" s="2">
-        <v>46231</v>
+        <v>46249</v>
       </c>
       <c r="B105">
-        <v>19</v>
+        <v>21</v>
       </c>
       <c r="C105">
-        <v>0.8120000000000001</v>
+        <v>0.02</v>
       </c>
       <c r="D105" t="s">
         <v>107</v>
@@ -2369,13 +2369,13 @@
     </row>
     <row r="106" spans="1:4">
       <c r="A106" s="2">
-        <v>46231</v>
+        <v>46249</v>
       </c>
       <c r="B106">
-        <v>20</v>
+        <v>22</v>
       </c>
       <c r="C106">
-        <v>0.24</v>
+        <v>0</v>
       </c>
       <c r="D106" t="s">
         <v>108</v>
@@ -2383,13 +2383,13 @@
     </row>
     <row r="107" spans="1:4">
       <c r="A107" s="2">
-        <v>46231</v>
+        <v>46249</v>
       </c>
       <c r="B107">
-        <v>21</v>
+        <v>23</v>
       </c>
       <c r="C107">
-        <v>0.041</v>
+        <v>0</v>
       </c>
       <c r="D107" t="s">
         <v>109</v>
@@ -2397,10 +2397,10 @@
     </row>
     <row r="108" spans="1:4">
       <c r="A108" s="2">
-        <v>46231</v>
+        <v>46249</v>
       </c>
       <c r="B108">
-        <v>22</v>
+        <v>24</v>
       </c>
       <c r="C108">
         <v>0</v>
@@ -2411,10 +2411,10 @@
     </row>
     <row r="109" spans="1:4">
       <c r="A109" s="2">
-        <v>46231</v>
+        <v>46250</v>
       </c>
       <c r="B109">
-        <v>23</v>
+        <v>1</v>
       </c>
       <c r="C109">
         <v>0</v>
@@ -2425,10 +2425,10 @@
     </row>
     <row r="110" spans="1:4">
       <c r="A110" s="2">
-        <v>46231</v>
+        <v>46250</v>
       </c>
       <c r="B110">
-        <v>24</v>
+        <v>2</v>
       </c>
       <c r="C110">
         <v>0</v>
@@ -2439,10 +2439,10 @@
     </row>
     <row r="111" spans="1:4">
       <c r="A111" s="2">
-        <v>46232</v>
+        <v>46250</v>
       </c>
       <c r="B111">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="C111">
         <v>0</v>
@@ -2453,10 +2453,10 @@
     </row>
     <row r="112" spans="1:4">
       <c r="A112" s="2">
-        <v>46232</v>
+        <v>46250</v>
       </c>
       <c r="B112">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="C112">
         <v>0</v>
@@ -2467,10 +2467,10 @@
     </row>
     <row r="113" spans="1:4">
       <c r="A113" s="2">
-        <v>46232</v>
+        <v>46250</v>
       </c>
       <c r="B113">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="C113">
         <v>0</v>
@@ -2481,10 +2481,10 @@
     </row>
     <row r="114" spans="1:4">
       <c r="A114" s="2">
-        <v>46232</v>
+        <v>46250</v>
       </c>
       <c r="B114">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="C114">
         <v>0</v>
@@ -2495,13 +2495,13 @@
     </row>
     <row r="115" spans="1:4">
       <c r="A115" s="2">
-        <v>46232</v>
+        <v>46250</v>
       </c>
       <c r="B115">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="C115">
-        <v>0</v>
+        <v>0.024</v>
       </c>
       <c r="D115" t="s">
         <v>117</v>
@@ -2509,13 +2509,13 @@
     </row>
     <row r="116" spans="1:4">
       <c r="A116" s="2">
-        <v>46232</v>
+        <v>46250</v>
       </c>
       <c r="B116">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="C116">
-        <v>0</v>
+        <v>0.238</v>
       </c>
       <c r="D116" t="s">
         <v>118</v>
@@ -2523,13 +2523,13 @@
     </row>
     <row r="117" spans="1:4">
       <c r="A117" s="2">
-        <v>46232</v>
+        <v>46250</v>
       </c>
       <c r="B117">
-        <v>7</v>
+        <v>9</v>
       </c>
       <c r="C117">
-        <v>0.046</v>
+        <v>1.008</v>
       </c>
       <c r="D117" t="s">
         <v>119</v>
@@ -2537,13 +2537,13 @@
     </row>
     <row r="118" spans="1:4">
       <c r="A118" s="2">
-        <v>46232</v>
+        <v>46250</v>
       </c>
       <c r="B118">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="C118">
-        <v>0.351</v>
+        <v>1.721</v>
       </c>
       <c r="D118" t="s">
         <v>120</v>
@@ -2551,13 +2551,13 @@
     </row>
     <row r="119" spans="1:4">
       <c r="A119" s="2">
-        <v>46232</v>
+        <v>46250</v>
       </c>
       <c r="B119">
-        <v>9</v>
+        <v>11</v>
       </c>
       <c r="C119">
-        <v>1.069</v>
+        <v>2.386</v>
       </c>
       <c r="D119" t="s">
         <v>121</v>
@@ -2565,13 +2565,13 @@
     </row>
     <row r="120" spans="1:4">
       <c r="A120" s="2">
-        <v>46232</v>
+        <v>46250</v>
       </c>
       <c r="B120">
-        <v>10</v>
+        <v>12</v>
       </c>
       <c r="C120">
-        <v>1.792</v>
+        <v>2.863</v>
       </c>
       <c r="D120" t="s">
         <v>122</v>
@@ -2579,13 +2579,13 @@
     </row>
     <row r="121" spans="1:4">
       <c r="A121" s="2">
-        <v>46232</v>
+        <v>46250</v>
       </c>
       <c r="B121">
-        <v>11</v>
+        <v>13</v>
       </c>
       <c r="C121">
-        <v>2.456</v>
+        <v>3.08</v>
       </c>
       <c r="D121" t="s">
         <v>123</v>
@@ -2593,13 +2593,13 @@
     </row>
     <row r="122" spans="1:4">
       <c r="A122" s="2">
-        <v>46232</v>
+        <v>46250</v>
       </c>
       <c r="B122">
-        <v>12</v>
+        <v>14</v>
       </c>
       <c r="C122">
-        <v>2.851</v>
+        <v>3.141</v>
       </c>
       <c r="D122" t="s">
         <v>124</v>
@@ -2607,13 +2607,13 @@
     </row>
     <row r="123" spans="1:4">
       <c r="A123" s="2">
-        <v>46232</v>
+        <v>46250</v>
       </c>
       <c r="B123">
-        <v>13</v>
+        <v>15</v>
       </c>
       <c r="C123">
-        <v>3.098</v>
+        <v>3.006</v>
       </c>
       <c r="D123" t="s">
         <v>125</v>
@@ -2621,13 +2621,13 @@
     </row>
     <row r="124" spans="1:4">
       <c r="A124" s="2">
-        <v>46232</v>
+        <v>46250</v>
       </c>
       <c r="B124">
-        <v>14</v>
+        <v>16</v>
       </c>
       <c r="C124">
-        <v>3.143</v>
+        <v>2.646</v>
       </c>
       <c r="D124" t="s">
         <v>126</v>
@@ -2635,13 +2635,13 @@
     </row>
     <row r="125" spans="1:4">
       <c r="A125" s="2">
-        <v>46232</v>
+        <v>46250</v>
       </c>
       <c r="B125">
-        <v>15</v>
+        <v>17</v>
       </c>
       <c r="C125">
-        <v>3.018</v>
+        <v>2.076</v>
       </c>
       <c r="D125" t="s">
         <v>127</v>
@@ -2649,13 +2649,13 @@
     </row>
     <row r="126" spans="1:4">
       <c r="A126" s="2">
-        <v>46232</v>
+        <v>46250</v>
       </c>
       <c r="B126">
-        <v>16</v>
+        <v>18</v>
       </c>
       <c r="C126">
-        <v>2.732</v>
+        <v>1.488</v>
       </c>
       <c r="D126" t="s">
         <v>128</v>
@@ -2663,13 +2663,13 @@
     </row>
     <row r="127" spans="1:4">
       <c r="A127" s="2">
-        <v>46232</v>
+        <v>46250</v>
       </c>
       <c r="B127">
-        <v>17</v>
+        <v>19</v>
       </c>
       <c r="C127">
-        <v>2.189</v>
+        <v>0.637</v>
       </c>
       <c r="D127" t="s">
         <v>129</v>
@@ -2677,13 +2677,13 @@
     </row>
     <row r="128" spans="1:4">
       <c r="A128" s="2">
-        <v>46232</v>
+        <v>46250</v>
       </c>
       <c r="B128">
-        <v>18</v>
+        <v>20</v>
       </c>
       <c r="C128">
-        <v>1.575</v>
+        <v>0.16</v>
       </c>
       <c r="D128" t="s">
         <v>130</v>
@@ -2691,13 +2691,13 @@
     </row>
     <row r="129" spans="1:4">
       <c r="A129" s="2">
-        <v>46232</v>
+        <v>46250</v>
       </c>
       <c r="B129">
-        <v>19</v>
+        <v>21</v>
       </c>
       <c r="C129">
-        <v>0.827</v>
+        <v>0.014</v>
       </c>
       <c r="D129" t="s">
         <v>131</v>
@@ -2705,13 +2705,13 @@
     </row>
     <row r="130" spans="1:4">
       <c r="A130" s="2">
-        <v>46232</v>
+        <v>46250</v>
       </c>
       <c r="B130">
-        <v>20</v>
+        <v>22</v>
       </c>
       <c r="C130">
-        <v>0.205</v>
+        <v>0</v>
       </c>
       <c r="D130" t="s">
         <v>132</v>
@@ -2719,13 +2719,13 @@
     </row>
     <row r="131" spans="1:4">
       <c r="A131" s="2">
-        <v>46232</v>
+        <v>46250</v>
       </c>
       <c r="B131">
-        <v>21</v>
+        <v>23</v>
       </c>
       <c r="C131">
-        <v>0.04</v>
+        <v>0</v>
       </c>
       <c r="D131" t="s">
         <v>133</v>
@@ -2733,10 +2733,10 @@
     </row>
     <row r="132" spans="1:4">
       <c r="A132" s="2">
-        <v>46232</v>
+        <v>46250</v>
       </c>
       <c r="B132">
-        <v>22</v>
+        <v>24</v>
       </c>
       <c r="C132">
         <v>0</v>
@@ -2747,10 +2747,10 @@
     </row>
     <row r="133" spans="1:4">
       <c r="A133" s="2">
-        <v>46232</v>
+        <v>46251</v>
       </c>
       <c r="B133">
-        <v>23</v>
+        <v>1</v>
       </c>
       <c r="C133">
         <v>0</v>
@@ -2761,10 +2761,10 @@
     </row>
     <row r="134" spans="1:4">
       <c r="A134" s="2">
-        <v>46232</v>
+        <v>46251</v>
       </c>
       <c r="B134">
-        <v>24</v>
+        <v>2</v>
       </c>
       <c r="C134">
         <v>0</v>
@@ -2775,10 +2775,10 @@
     </row>
     <row r="135" spans="1:4">
       <c r="A135" s="2">
-        <v>46233</v>
+        <v>46251</v>
       </c>
       <c r="B135">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="C135">
         <v>0</v>
@@ -2789,10 +2789,10 @@
     </row>
     <row r="136" spans="1:4">
       <c r="A136" s="2">
-        <v>46233</v>
+        <v>46251</v>
       </c>
       <c r="B136">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="C136">
         <v>0</v>
@@ -2803,10 +2803,10 @@
     </row>
     <row r="137" spans="1:4">
       <c r="A137" s="2">
-        <v>46233</v>
+        <v>46251</v>
       </c>
       <c r="B137">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="C137">
         <v>0</v>
@@ -2817,10 +2817,10 @@
     </row>
     <row r="138" spans="1:4">
       <c r="A138" s="2">
-        <v>46233</v>
+        <v>46251</v>
       </c>
       <c r="B138">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="C138">
         <v>0</v>
@@ -2831,13 +2831,13 @@
     </row>
     <row r="139" spans="1:4">
       <c r="A139" s="2">
-        <v>46233</v>
+        <v>46251</v>
       </c>
       <c r="B139">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="C139">
-        <v>0</v>
+        <v>0.024</v>
       </c>
       <c r="D139" t="s">
         <v>141</v>
@@ -2845,13 +2845,13 @@
     </row>
     <row r="140" spans="1:4">
       <c r="A140" s="2">
-        <v>46233</v>
+        <v>46251</v>
       </c>
       <c r="B140">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="C140">
-        <v>0</v>
+        <v>0.251</v>
       </c>
       <c r="D140" t="s">
         <v>142</v>
@@ -2859,13 +2859,13 @@
     </row>
     <row r="141" spans="1:4">
       <c r="A141" s="2">
-        <v>46233</v>
+        <v>46251</v>
       </c>
       <c r="B141">
-        <v>7</v>
+        <v>9</v>
       </c>
       <c r="C141">
-        <v>0.046</v>
+        <v>0.9379999999999999</v>
       </c>
       <c r="D141" t="s">
         <v>143</v>
@@ -2873,13 +2873,13 @@
     </row>
     <row r="142" spans="1:4">
       <c r="A142" s="2">
-        <v>46233</v>
+        <v>46251</v>
       </c>
       <c r="B142">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="C142">
-        <v>0.365</v>
+        <v>1.705</v>
       </c>
       <c r="D142" t="s">
         <v>144</v>
@@ -2887,13 +2887,13 @@
     </row>
     <row r="143" spans="1:4">
       <c r="A143" s="2">
-        <v>46233</v>
+        <v>46251</v>
       </c>
       <c r="B143">
-        <v>9</v>
+        <v>11</v>
       </c>
       <c r="C143">
-        <v>1.037</v>
+        <v>2.32</v>
       </c>
       <c r="D143" t="s">
         <v>145</v>
@@ -2901,13 +2901,13 @@
     </row>
     <row r="144" spans="1:4">
       <c r="A144" s="2">
-        <v>46233</v>
+        <v>46251</v>
       </c>
       <c r="B144">
-        <v>10</v>
+        <v>12</v>
       </c>
       <c r="C144">
-        <v>1.786</v>
+        <v>2.772</v>
       </c>
       <c r="D144" t="s">
         <v>146</v>
@@ -2915,13 +2915,13 @@
     </row>
     <row r="145" spans="1:4">
       <c r="A145" s="2">
-        <v>46233</v>
+        <v>46251</v>
       </c>
       <c r="B145">
-        <v>11</v>
+        <v>13</v>
       </c>
       <c r="C145">
-        <v>2.343</v>
+        <v>3.079</v>
       </c>
       <c r="D145" t="s">
         <v>147</v>
@@ -2929,13 +2929,13 @@
     </row>
     <row r="146" spans="1:4">
       <c r="A146" s="2">
-        <v>46233</v>
+        <v>46251</v>
       </c>
       <c r="B146">
-        <v>12</v>
+        <v>14</v>
       </c>
       <c r="C146">
-        <v>2.64</v>
+        <v>3.136</v>
       </c>
       <c r="D146" t="s">
         <v>148</v>
@@ -2943,13 +2943,13 @@
     </row>
     <row r="147" spans="1:4">
       <c r="A147" s="2">
-        <v>46233</v>
+        <v>46251</v>
       </c>
       <c r="B147">
-        <v>13</v>
+        <v>15</v>
       </c>
       <c r="C147">
-        <v>2.874</v>
+        <v>2.981</v>
       </c>
       <c r="D147" t="s">
         <v>149</v>
@@ -2957,13 +2957,13 @@
     </row>
     <row r="148" spans="1:4">
       <c r="A148" s="2">
-        <v>46233</v>
+        <v>46251</v>
       </c>
       <c r="B148">
-        <v>14</v>
+        <v>16</v>
       </c>
       <c r="C148">
-        <v>3.058</v>
+        <v>2.62</v>
       </c>
       <c r="D148" t="s">
         <v>150</v>
@@ -2971,13 +2971,13 @@
     </row>
     <row r="149" spans="1:4">
       <c r="A149" s="2">
-        <v>46233</v>
+        <v>46251</v>
       </c>
       <c r="B149">
-        <v>15</v>
+        <v>17</v>
       </c>
       <c r="C149">
-        <v>3.031</v>
+        <v>2.04</v>
       </c>
       <c r="D149" t="s">
         <v>151</v>
@@ -2985,13 +2985,13 @@
     </row>
     <row r="150" spans="1:4">
       <c r="A150" s="2">
-        <v>46233</v>
+        <v>46251</v>
       </c>
       <c r="B150">
-        <v>16</v>
+        <v>18</v>
       </c>
       <c r="C150">
-        <v>2.562</v>
+        <v>1.483</v>
       </c>
       <c r="D150" t="s">
         <v>152</v>
@@ -2999,13 +2999,13 @@
     </row>
     <row r="151" spans="1:4">
       <c r="A151" s="2">
-        <v>46233</v>
+        <v>46251</v>
       </c>
       <c r="B151">
-        <v>17</v>
+        <v>19</v>
       </c>
       <c r="C151">
-        <v>1.98</v>
+        <v>0.641</v>
       </c>
       <c r="D151" t="s">
         <v>153</v>
@@ -3013,13 +3013,13 @@
     </row>
     <row r="152" spans="1:4">
       <c r="A152" s="2">
-        <v>46233</v>
+        <v>46251</v>
       </c>
       <c r="B152">
-        <v>18</v>
+        <v>20</v>
       </c>
       <c r="C152">
-        <v>1.378</v>
+        <v>0.151</v>
       </c>
       <c r="D152" t="s">
         <v>154</v>
@@ -3027,13 +3027,13 @@
     </row>
     <row r="153" spans="1:4">
       <c r="A153" s="2">
-        <v>46233</v>
+        <v>46251</v>
       </c>
       <c r="B153">
-        <v>19</v>
+        <v>21</v>
       </c>
       <c r="C153">
-        <v>0.747</v>
+        <v>0.011</v>
       </c>
       <c r="D153" t="s">
         <v>155</v>
@@ -3041,13 +3041,13 @@
     </row>
     <row r="154" spans="1:4">
       <c r="A154" s="2">
-        <v>46233</v>
+        <v>46251</v>
       </c>
       <c r="B154">
-        <v>20</v>
+        <v>22</v>
       </c>
       <c r="C154">
-        <v>0.248</v>
+        <v>0</v>
       </c>
       <c r="D154" t="s">
         <v>156</v>
@@ -3055,13 +3055,13 @@
     </row>
     <row r="155" spans="1:4">
       <c r="A155" s="2">
-        <v>46233</v>
+        <v>46251</v>
       </c>
       <c r="B155">
-        <v>21</v>
+        <v>23</v>
       </c>
       <c r="C155">
-        <v>0.048</v>
+        <v>0</v>
       </c>
       <c r="D155" t="s">
         <v>157</v>
@@ -3069,10 +3069,10 @@
     </row>
     <row r="156" spans="1:4">
       <c r="A156" s="2">
-        <v>46233</v>
+        <v>46251</v>
       </c>
       <c r="B156">
-        <v>22</v>
+        <v>24</v>
       </c>
       <c r="C156">
         <v>0</v>
@@ -3083,10 +3083,10 @@
     </row>
     <row r="157" spans="1:4">
       <c r="A157" s="2">
-        <v>46233</v>
+        <v>46252</v>
       </c>
       <c r="B157">
-        <v>23</v>
+        <v>1</v>
       </c>
       <c r="C157">
         <v>0</v>
@@ -3097,10 +3097,10 @@
     </row>
     <row r="158" spans="1:4">
       <c r="A158" s="2">
-        <v>46233</v>
+        <v>46252</v>
       </c>
       <c r="B158">
-        <v>24</v>
+        <v>2</v>
       </c>
       <c r="C158">
         <v>0</v>
@@ -3111,10 +3111,10 @@
     </row>
     <row r="159" spans="1:4">
       <c r="A159" s="2">
-        <v>46234</v>
+        <v>46252</v>
       </c>
       <c r="B159">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="C159">
         <v>0</v>
@@ -3125,10 +3125,10 @@
     </row>
     <row r="160" spans="1:4">
       <c r="A160" s="2">
-        <v>46234</v>
+        <v>46252</v>
       </c>
       <c r="B160">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="C160">
         <v>0</v>
@@ -3139,10 +3139,10 @@
     </row>
     <row r="161" spans="1:4">
       <c r="A161" s="2">
-        <v>46234</v>
+        <v>46252</v>
       </c>
       <c r="B161">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="C161">
         <v>0</v>
@@ -3153,10 +3153,10 @@
     </row>
     <row r="162" spans="1:4">
       <c r="A162" s="2">
-        <v>46234</v>
+        <v>46252</v>
       </c>
       <c r="B162">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="C162">
         <v>0</v>
@@ -3167,13 +3167,13 @@
     </row>
     <row r="163" spans="1:4">
       <c r="A163" s="2">
-        <v>46234</v>
+        <v>46252</v>
       </c>
       <c r="B163">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="C163">
-        <v>0</v>
+        <v>0.016</v>
       </c>
       <c r="D163" t="s">
         <v>165</v>
@@ -3181,13 +3181,13 @@
     </row>
     <row r="164" spans="1:4">
       <c r="A164" s="2">
-        <v>46234</v>
+        <v>46252</v>
       </c>
       <c r="B164">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="C164">
-        <v>0</v>
+        <v>0.229</v>
       </c>
       <c r="D164" t="s">
         <v>166</v>
@@ -3195,13 +3195,13 @@
     </row>
     <row r="165" spans="1:4">
       <c r="A165" s="2">
-        <v>46234</v>
+        <v>46252</v>
       </c>
       <c r="B165">
-        <v>7</v>
+        <v>9</v>
       </c>
       <c r="C165">
-        <v>0.039</v>
+        <v>0.918</v>
       </c>
       <c r="D165" t="s">
         <v>167</v>
@@ -3209,13 +3209,13 @@
     </row>
     <row r="166" spans="1:4">
       <c r="A166" s="2">
-        <v>46234</v>
+        <v>46252</v>
       </c>
       <c r="B166">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="C166">
-        <v>0.36</v>
+        <v>1.721</v>
       </c>
       <c r="D166" t="s">
         <v>168</v>
@@ -3223,13 +3223,13 @@
     </row>
     <row r="167" spans="1:4">
       <c r="A167" s="2">
-        <v>46234</v>
+        <v>46252</v>
       </c>
       <c r="B167">
-        <v>9</v>
+        <v>11</v>
       </c>
       <c r="C167">
-        <v>0.994</v>
+        <v>2.313</v>
       </c>
       <c r="D167" t="s">
         <v>169</v>
@@ -3237,13 +3237,13 @@
     </row>
     <row r="168" spans="1:4">
       <c r="A168" s="2">
-        <v>46234</v>
+        <v>46252</v>
       </c>
       <c r="B168">
-        <v>10</v>
+        <v>12</v>
       </c>
       <c r="C168">
-        <v>1.729</v>
+        <v>2.814</v>
       </c>
       <c r="D168" t="s">
         <v>170</v>
@@ -3251,13 +3251,13 @@
     </row>
     <row r="169" spans="1:4">
       <c r="A169" s="2">
-        <v>46234</v>
+        <v>46252</v>
       </c>
       <c r="B169">
-        <v>11</v>
+        <v>13</v>
       </c>
       <c r="C169">
-        <v>2.347</v>
+        <v>3.052</v>
       </c>
       <c r="D169" t="s">
         <v>171</v>
@@ -3265,13 +3265,13 @@
     </row>
     <row r="170" spans="1:4">
       <c r="A170" s="2">
-        <v>46234</v>
+        <v>46252</v>
       </c>
       <c r="B170">
-        <v>12</v>
+        <v>14</v>
       </c>
       <c r="C170">
-        <v>2.688</v>
+        <v>3.124</v>
       </c>
       <c r="D170" t="s">
         <v>172</v>

</xml_diff>